<commit_message>
Log B7 W1 T1 (Recovery-gate 2/5 session: Tier-A shape baseline + 90 negatives + light WPU)
</commit_message>
<xml_diff>
--- a/Training_3_B7.xlsx
+++ b/Training_3_B7.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1474" uniqueCount="830">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1499" uniqueCount="837">
   <si>
     <t>B7 — Performance-Block Dashboard (Advanced OAHS)</t>
   </si>
@@ -1958,13 +1958,34 @@
     <t>L</t>
   </si>
   <si>
-    <t>Demo: Straddle links, bester 6s, Q4 (Tier A besitzt)</t>
+    <t>Recovery-Gate 2/5; links meist &gt;5s, sauber</t>
+  </si>
+  <si>
+    <t>R</t>
+  </si>
+  <si>
+    <t>rechts 2-5s, inkonsistent</t>
+  </si>
+  <si>
+    <t>links &gt;5s</t>
+  </si>
+  <si>
+    <t>rechts 2-5s</t>
+  </si>
+  <si>
+    <t>links ~5s</t>
   </si>
   <si>
     <t>NA</t>
   </si>
   <si>
-    <t>Demo: 90 Cluster frisch, 3 saubere Reps @RPE7</t>
+    <t>2 Negativ</t>
+  </si>
+  <si>
+    <t>Negativ-Version (Recovery-Gate); RPE 6-7, Parallettes</t>
+  </si>
+  <si>
+    <t>Straps, leicht (Gate); 20 kg</t>
   </si>
   <si>
     <t>B7 — Nutrition Targets (Maintenance, KEIN Defizit)</t>
@@ -3749,7 +3770,7 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>766</v>
+        <v>773</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3759,7 +3780,7 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="12" t="s">
-        <v>767</v>
+        <v>774</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -3784,12 +3805,12 @@
         <v>153</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>768</v>
+        <v>775</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="9" t="s">
-        <v>769</v>
+        <v>776</v>
       </c>
       <c r="B4" s="11">
         <f>SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Skill90",'B7_Training_Log'!$C$2:$C$1000,1)+SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Planche",'B7_Training_Log'!$C$2:$C$1000,1)+SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Push",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -3814,7 +3835,7 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="9" t="s">
-        <v>770</v>
+        <v>777</v>
       </c>
       <c r="B5" s="11">
         <f>SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Pull",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -3839,7 +3860,7 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="9" t="s">
-        <v>771</v>
+        <v>778</v>
       </c>
       <c r="B6" s="11">
         <f>SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Legs",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -3864,7 +3885,7 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="9" t="s">
-        <v>772</v>
+        <v>779</v>
       </c>
       <c r="B7" s="10">
         <f>SUMIFS('B7_Training_Log'!$N$2:$N$1000,'B7_Training_Log'!$D$2:$D$1000,"90",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -3889,7 +3910,7 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="9" t="s">
-        <v>773</v>
+        <v>780</v>
       </c>
       <c r="B8" s="10">
         <f>COUNTIFS('B7_Training_Log'!$E$2:$E$1000,"SkillOAHS",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -3914,7 +3935,7 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="9" t="s">
-        <v>774</v>
+        <v>781</v>
       </c>
       <c r="B9" s="10">
         <f>MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_straddle",'B7_Training_Log'!$F$2:$F$1000,"L",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -3939,7 +3960,7 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="9" t="s">
-        <v>775</v>
+        <v>782</v>
       </c>
       <c r="B10" s="10">
         <f>MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_straddle",'B7_Training_Log'!$F$2:$F$1000,"R",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -3964,7 +3985,7 @@
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="9" t="s">
-        <v>776</v>
+        <v>783</v>
       </c>
       <c r="B11" s="10">
         <f>MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_diamond",'B7_Training_Log'!$F$2:$F$1000,"L",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -3989,7 +4010,7 @@
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="9" t="s">
-        <v>777</v>
+        <v>784</v>
       </c>
       <c r="B12" s="10">
         <f>MAX(MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_flag",'B7_Training_Log'!$C$2:$C$1000,1),MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_figa",'B7_Training_Log'!$C$2:$C$1000,1))</f>
@@ -4014,7 +4035,7 @@
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="9" t="s">
-        <v>778</v>
+        <v>785</v>
       </c>
       <c r="B13" s="11">
         <f>IFERROR(AVERAGEIFS('B7_Training_Log'!$J$2:$J$1000,'B7_Training_Log'!$C$2:$C$1000,1),0)</f>
@@ -4089,7 +4110,7 @@
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="9" t="s">
-        <v>779</v>
+        <v>786</v>
       </c>
       <c r="B16" s="10">
         <f>COUNTIFS('B7_Training_Log'!$K$2:$K$1000,"&gt;=4",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4114,7 +4135,7 @@
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="9" t="s">
-        <v>780</v>
+        <v>787</v>
       </c>
       <c r="B17" s="10">
         <f>COUNTIFS('B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4158,7 +4179,7 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
-        <v>781</v>
+        <v>788</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4166,7 +4187,7 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="5" t="s">
-        <v>782</v>
+        <v>789</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
@@ -4174,13 +4195,13 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="7" t="s">
-        <v>783</v>
+        <v>790</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>784</v>
+        <v>791</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>785</v>
+        <v>792</v>
       </c>
       <c r="D4" s="7"/>
     </row>
@@ -4189,10 +4210,10 @@
         <v>627</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>786</v>
+        <v>793</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>787</v>
+        <v>794</v>
       </c>
       <c r="D5" s="4"/>
     </row>
@@ -4201,10 +4222,10 @@
         <v>628</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>788</v>
+        <v>795</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>789</v>
+        <v>796</v>
       </c>
       <c r="D6" s="4"/>
     </row>
@@ -4213,10 +4234,10 @@
         <v>629</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>790</v>
+        <v>797</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>791</v>
+        <v>798</v>
       </c>
       <c r="D7" s="4"/>
     </row>
@@ -4225,10 +4246,10 @@
         <v>436</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>792</v>
+        <v>799</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>793</v>
+        <v>800</v>
       </c>
       <c r="D8" s="4"/>
     </row>
@@ -4237,10 +4258,10 @@
         <v>439</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>794</v>
+        <v>801</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>795</v>
+        <v>802</v>
       </c>
       <c r="D9" s="4"/>
     </row>
@@ -4249,10 +4270,10 @@
         <v>630</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>796</v>
+        <v>803</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>797</v>
+        <v>804</v>
       </c>
       <c r="D10" s="4"/>
     </row>
@@ -4261,10 +4282,10 @@
         <v>631</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>798</v>
+        <v>805</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>799</v>
+        <v>806</v>
       </c>
       <c r="D11" s="4"/>
     </row>
@@ -4273,10 +4294,10 @@
         <v>632</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>800</v>
+        <v>807</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>801</v>
+        <v>808</v>
       </c>
       <c r="D12" s="4"/>
     </row>
@@ -4285,10 +4306,10 @@
         <v>633</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>798</v>
+        <v>805</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>802</v>
+        <v>809</v>
       </c>
       <c r="D13" s="4"/>
     </row>
@@ -4297,10 +4318,10 @@
         <v>634</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>803</v>
+        <v>810</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>804</v>
+        <v>811</v>
       </c>
       <c r="D14" s="4"/>
     </row>
@@ -4309,10 +4330,10 @@
         <v>635</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>805</v>
+        <v>812</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>806</v>
+        <v>813</v>
       </c>
       <c r="D15" s="4"/>
     </row>
@@ -4321,10 +4342,10 @@
         <v>636</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>807</v>
+        <v>814</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>808</v>
+        <v>815</v>
       </c>
       <c r="D16" s="4"/>
     </row>
@@ -4333,10 +4354,10 @@
         <v>637</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>798</v>
+        <v>805</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>809</v>
+        <v>816</v>
       </c>
       <c r="D17" s="4"/>
     </row>
@@ -4345,10 +4366,10 @@
         <v>638</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>798</v>
+        <v>805</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>810</v>
+        <v>817</v>
       </c>
       <c r="D18" s="4"/>
     </row>
@@ -4357,10 +4378,10 @@
         <v>639</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>811</v>
+        <v>818</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>812</v>
+        <v>819</v>
       </c>
       <c r="D19" s="4"/>
     </row>
@@ -4369,10 +4390,10 @@
         <v>92</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>800</v>
+        <v>807</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>813</v>
+        <v>820</v>
       </c>
       <c r="D20" s="4"/>
     </row>
@@ -4381,16 +4402,16 @@
         <v>640</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>814</v>
+        <v>821</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>815</v>
+        <v>822</v>
       </c>
       <c r="D21" s="4"/>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="5" t="s">
-        <v>816</v>
+        <v>823</v>
       </c>
       <c r="B23" s="5"/>
       <c r="C23" s="5"/>
@@ -4398,7 +4419,7 @@
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="4" t="s">
-        <v>817</v>
+        <v>824</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -4406,7 +4427,7 @@
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="4" t="s">
-        <v>818</v>
+        <v>825</v>
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -4414,7 +4435,7 @@
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="4" t="s">
-        <v>819</v>
+        <v>826</v>
       </c>
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
@@ -4422,7 +4443,7 @@
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="4" t="s">
-        <v>820</v>
+        <v>827</v>
       </c>
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
@@ -4430,7 +4451,7 @@
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="4" t="s">
-        <v>821</v>
+        <v>828</v>
       </c>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
@@ -4438,7 +4459,7 @@
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="4" t="s">
-        <v>822</v>
+        <v>829</v>
       </c>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -4446,7 +4467,7 @@
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="4" t="s">
-        <v>823</v>
+        <v>830</v>
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -4454,7 +4475,7 @@
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="5" t="s">
-        <v>824</v>
+        <v>831</v>
       </c>
       <c r="B32" s="5"/>
       <c r="C32" s="5"/>
@@ -4462,7 +4483,7 @@
     </row>
     <row r="33" spans="1:4">
       <c r="A33" s="4" t="s">
-        <v>825</v>
+        <v>832</v>
       </c>
       <c r="B33" s="4"/>
       <c r="C33" s="4"/>
@@ -4470,7 +4491,7 @@
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="4" t="s">
-        <v>826</v>
+        <v>833</v>
       </c>
       <c r="B34" s="4"/>
       <c r="C34" s="4"/>
@@ -4478,7 +4499,7 @@
     </row>
     <row r="35" spans="1:4">
       <c r="A35" s="4" t="s">
-        <v>827</v>
+        <v>834</v>
       </c>
       <c r="B35" s="4"/>
       <c r="C35" s="4"/>
@@ -4486,7 +4507,7 @@
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="4" t="s">
-        <v>828</v>
+        <v>835</v>
       </c>
       <c r="B36" s="4"/>
       <c r="C36" s="4"/>
@@ -4494,7 +4515,7 @@
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="4" t="s">
-        <v>829</v>
+        <v>836</v>
       </c>
       <c r="B37" s="4"/>
       <c r="C37" s="4"/>
@@ -8476,7 +8497,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q3"/>
+  <dimension ref="A1:Q9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -8551,7 +8572,7 @@
     </row>
     <row r="2" spans="1:17">
       <c r="A2" s="25">
-        <v>46204</v>
+        <v>46211</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>94</v>
@@ -8570,7 +8591,7 @@
         <v>641</v>
       </c>
       <c r="G2" s="6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I2" s="6">
         <v>0</v>
@@ -8582,7 +8603,7 @@
         <v>6</v>
       </c>
       <c r="O2" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P2" s="4" t="s">
         <v>642</v>
@@ -8594,7 +8615,7 @@
     </row>
     <row r="3" spans="1:17">
       <c r="A3" s="25">
-        <v>46204</v>
+        <v>46211</v>
       </c>
       <c r="B3" s="6" t="s">
         <v>94</v>
@@ -8603,7 +8624,7 @@
         <v>1</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>444</v>
+        <v>596</v>
       </c>
       <c r="E3" s="6">
         <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D3,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
@@ -8613,34 +8634,286 @@
         <v>643</v>
       </c>
       <c r="G3" s="6">
-        <v>4</v>
-      </c>
-      <c r="H3" s="4" t="s">
-        <v>46</v>
+        <v>3</v>
       </c>
       <c r="I3" s="6">
         <v>0</v>
       </c>
-      <c r="J3" s="6">
-        <v>7</v>
-      </c>
-      <c r="K3" s="6">
-        <v>1</v>
-      </c>
       <c r="L3" s="6">
-        <v>4</v>
-      </c>
-      <c r="N3" s="6">
         <v>3</v>
       </c>
+      <c r="M3" s="6">
+        <v>5</v>
+      </c>
       <c r="O3" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P3" s="4" t="s">
         <v>644</v>
       </c>
       <c r="Q3" s="6">
         <f>IF($B3="","",$B3&amp;"_W"&amp;$C3)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17">
+      <c r="A4" s="25">
+        <v>46211</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="C4" s="6">
+        <v>1</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>599</v>
+      </c>
+      <c r="E4" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D4,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>641</v>
+      </c>
+      <c r="G4" s="6">
+        <v>3</v>
+      </c>
+      <c r="I4" s="6">
+        <v>0</v>
+      </c>
+      <c r="L4" s="6">
+        <v>4</v>
+      </c>
+      <c r="M4" s="6">
+        <v>6</v>
+      </c>
+      <c r="O4" s="6">
+        <v>2</v>
+      </c>
+      <c r="P4" s="4" t="s">
+        <v>645</v>
+      </c>
+      <c r="Q4" s="6">
+        <f>IF($B4="","",$B4&amp;"_W"&amp;$C4)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17">
+      <c r="A5" s="25">
+        <v>46211</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="C5" s="6">
+        <v>1</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>599</v>
+      </c>
+      <c r="E5" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D5,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>643</v>
+      </c>
+      <c r="G5" s="6">
+        <v>3</v>
+      </c>
+      <c r="I5" s="6">
+        <v>0</v>
+      </c>
+      <c r="L5" s="6">
+        <v>3</v>
+      </c>
+      <c r="M5" s="6">
+        <v>4</v>
+      </c>
+      <c r="O5" s="6">
+        <v>2</v>
+      </c>
+      <c r="P5" s="4" t="s">
+        <v>646</v>
+      </c>
+      <c r="Q5" s="6">
+        <f>IF($B5="","",$B5&amp;"_W"&amp;$C5)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17">
+      <c r="A6" s="25">
+        <v>46211</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="C6" s="6">
+        <v>1</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>602</v>
+      </c>
+      <c r="E6" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D6,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>641</v>
+      </c>
+      <c r="G6" s="6">
+        <v>3</v>
+      </c>
+      <c r="I6" s="6">
+        <v>0</v>
+      </c>
+      <c r="L6" s="6">
+        <v>4</v>
+      </c>
+      <c r="M6" s="6">
+        <v>5</v>
+      </c>
+      <c r="O6" s="6">
+        <v>2</v>
+      </c>
+      <c r="P6" s="4" t="s">
+        <v>647</v>
+      </c>
+      <c r="Q6" s="6">
+        <f>IF($B6="","",$B6&amp;"_W"&amp;$C6)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17">
+      <c r="A7" s="25">
+        <v>46211</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="C7" s="6">
+        <v>1</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>602</v>
+      </c>
+      <c r="E7" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D7,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>643</v>
+      </c>
+      <c r="G7" s="6">
+        <v>3</v>
+      </c>
+      <c r="I7" s="6">
+        <v>0</v>
+      </c>
+      <c r="L7" s="6">
+        <v>3</v>
+      </c>
+      <c r="M7" s="6">
+        <v>4</v>
+      </c>
+      <c r="O7" s="6">
+        <v>2</v>
+      </c>
+      <c r="P7" s="4" t="s">
+        <v>646</v>
+      </c>
+      <c r="Q7" s="6">
+        <f>IF($B7="","",$B7&amp;"_W"&amp;$C7)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17">
+      <c r="A8" s="25">
+        <v>46211</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="C8" s="6">
+        <v>1</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>444</v>
+      </c>
+      <c r="E8" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D8,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>648</v>
+      </c>
+      <c r="G8" s="6">
+        <v>3</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="I8" s="6">
+        <v>0</v>
+      </c>
+      <c r="J8" s="6">
+        <v>7</v>
+      </c>
+      <c r="L8" s="6">
+        <v>4</v>
+      </c>
+      <c r="O8" s="6">
+        <v>2</v>
+      </c>
+      <c r="P8" s="4" t="s">
+        <v>650</v>
+      </c>
+      <c r="Q8" s="6">
+        <f>IF($B8="","",$B8&amp;"_W"&amp;$C8)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17">
+      <c r="A9" s="25">
+        <v>46211</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="C9" s="6">
+        <v>1</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>481</v>
+      </c>
+      <c r="E9" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D9,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>648</v>
+      </c>
+      <c r="G9" s="6">
+        <v>2</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="I9" s="6">
+        <v>20</v>
+      </c>
+      <c r="J9" s="6">
+        <v>6</v>
+      </c>
+      <c r="O9" s="6">
+        <v>2</v>
+      </c>
+      <c r="P9" s="4" t="s">
+        <v>651</v>
+      </c>
+      <c r="Q9" s="6">
+        <f>IF($B9="","",$B9&amp;"_W"&amp;$C9)</f>
         <v>0</v>
       </c>
     </row>
@@ -8718,7 +8991,7 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>645</v>
+        <v>652</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -8729,20 +9002,20 @@
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="5" t="s">
-        <v>646</v>
+        <v>653</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="9" t="s">
-        <v>647</v>
+        <v>654</v>
       </c>
       <c r="B4" s="11">
         <v>81</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>655</v>
+        <v>662</v>
       </c>
       <c r="D4" s="4"/>
       <c r="E4" s="4"/>
@@ -8751,21 +9024,21 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="9" t="s">
-        <v>648</v>
+        <v>655</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>649</v>
+        <v>656</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="9" t="s">
-        <v>650</v>
+        <v>657</v>
       </c>
       <c r="B6" s="11">
         <v>2.2</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>656</v>
+        <v>663</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
@@ -8774,7 +9047,7 @@
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="9" t="s">
-        <v>651</v>
+        <v>658</v>
       </c>
       <c r="B7" s="11">
         <v>0.9</v>
@@ -8782,7 +9055,7 @@
     </row>
     <row r="8" spans="1:7">
       <c r="A8" s="9" t="s">
-        <v>652</v>
+        <v>659</v>
       </c>
       <c r="B8" s="10">
         <v>2700</v>
@@ -8790,7 +9063,7 @@
     </row>
     <row r="9" spans="1:7">
       <c r="A9" s="9" t="s">
-        <v>653</v>
+        <v>660</v>
       </c>
       <c r="B9" s="10">
         <f>ROUND(BW*B6,0)</f>
@@ -8799,7 +9072,7 @@
     </row>
     <row r="10" spans="1:7">
       <c r="A10" s="9" t="s">
-        <v>654</v>
+        <v>661</v>
       </c>
       <c r="B10" s="10">
         <f>ROUND(BW*B7,0)</f>
@@ -8808,7 +9081,7 @@
     </row>
     <row r="12" spans="1:7">
       <c r="A12" s="5" t="s">
-        <v>657</v>
+        <v>664</v>
       </c>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -8822,27 +9095,27 @@
         <v>85</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>658</v>
+        <v>665</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>659</v>
+        <v>666</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>660</v>
+        <v>667</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>661</v>
+        <v>668</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>662</v>
+        <v>669</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>663</v>
+        <v>670</v>
       </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" s="9" t="s">
-        <v>664</v>
+        <v>671</v>
       </c>
       <c r="B14" s="26">
         <v>250</v>
@@ -8864,7 +9137,7 @@
         <v>0</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>665</v>
+        <v>672</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -8891,12 +9164,12 @@
         <v>0</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>666</v>
+        <v>673</v>
       </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" s="9" t="s">
-        <v>667</v>
+        <v>674</v>
       </c>
       <c r="B16" s="26">
         <v>200</v>
@@ -8918,12 +9191,12 @@
         <v>0</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>668</v>
+        <v>675</v>
       </c>
     </row>
     <row r="17" spans="1:7">
       <c r="A17" s="9" t="s">
-        <v>669</v>
+        <v>676</v>
       </c>
       <c r="B17" s="26">
         <v>150</v>
@@ -8945,12 +9218,12 @@
         <v>0</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>670</v>
+        <v>677</v>
       </c>
     </row>
     <row r="18" spans="1:7">
       <c r="A18" s="9" t="s">
-        <v>671</v>
+        <v>678</v>
       </c>
       <c r="B18" s="26">
         <v>100</v>
@@ -8972,7 +9245,7 @@
         <v>0</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>672</v>
+        <v>679</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -8999,12 +9272,12 @@
         <v>0</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>673</v>
+        <v>680</v>
       </c>
     </row>
     <row r="21" spans="1:7">
       <c r="A21" s="5" t="s">
-        <v>674</v>
+        <v>681</v>
       </c>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
@@ -9015,7 +9288,7 @@
     </row>
     <row r="22" spans="1:7">
       <c r="A22" s="4" t="s">
-        <v>675</v>
+        <v>682</v>
       </c>
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
@@ -9026,7 +9299,7 @@
     </row>
     <row r="23" spans="1:7">
       <c r="A23" s="4" t="s">
-        <v>676</v>
+        <v>683</v>
       </c>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
@@ -9037,7 +9310,7 @@
     </row>
     <row r="24" spans="1:7">
       <c r="A24" s="4" t="s">
-        <v>677</v>
+        <v>684</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -9048,7 +9321,7 @@
     </row>
     <row r="25" spans="1:7">
       <c r="A25" s="4" t="s">
-        <v>678</v>
+        <v>685</v>
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -9093,7 +9366,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>679</v>
+        <v>686</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -9102,7 +9375,7 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="5" t="s">
-        <v>680</v>
+        <v>687</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
@@ -9111,126 +9384,126 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="7" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>682</v>
+        <v>689</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>683</v>
+        <v>690</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>684</v>
+        <v>691</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>685</v>
+        <v>692</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="9" t="s">
-        <v>686</v>
+        <v>693</v>
       </c>
       <c r="B5" s="22" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="C5" s="27" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
       <c r="D5" s="28" t="s">
-        <v>689</v>
+        <v>696</v>
       </c>
       <c r="E5" s="29" t="s">
-        <v>690</v>
+        <v>697</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="9" t="s">
-        <v>691</v>
+        <v>698</v>
       </c>
       <c r="B6" s="22" t="s">
-        <v>692</v>
+        <v>699</v>
       </c>
       <c r="C6" s="27" t="s">
-        <v>693</v>
+        <v>700</v>
       </c>
       <c r="D6" s="28" t="s">
-        <v>694</v>
+        <v>701</v>
       </c>
       <c r="E6" s="29" t="s">
-        <v>695</v>
+        <v>702</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="9" t="s">
-        <v>696</v>
+        <v>703</v>
       </c>
       <c r="B7" s="22" t="s">
-        <v>697</v>
+        <v>704</v>
       </c>
       <c r="C7" s="27" t="s">
-        <v>698</v>
+        <v>705</v>
       </c>
       <c r="D7" s="28" t="s">
-        <v>699</v>
+        <v>706</v>
       </c>
       <c r="E7" s="29" t="s">
-        <v>700</v>
+        <v>707</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="9" t="s">
-        <v>701</v>
+        <v>708</v>
       </c>
       <c r="B8" s="22" t="s">
-        <v>702</v>
+        <v>709</v>
       </c>
       <c r="C8" s="27" t="s">
-        <v>703</v>
+        <v>710</v>
       </c>
       <c r="D8" s="28" t="s">
-        <v>704</v>
+        <v>711</v>
       </c>
       <c r="E8" s="29" t="s">
-        <v>705</v>
+        <v>712</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="9" t="s">
-        <v>706</v>
+        <v>713</v>
       </c>
       <c r="B9" s="22" t="s">
-        <v>707</v>
+        <v>714</v>
       </c>
       <c r="C9" s="27" t="s">
-        <v>708</v>
+        <v>715</v>
       </c>
       <c r="D9" s="28" t="s">
-        <v>709</v>
+        <v>716</v>
       </c>
       <c r="E9" s="29" t="s">
-        <v>710</v>
+        <v>717</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="9" t="s">
-        <v>711</v>
+        <v>718</v>
       </c>
       <c r="B10" s="22" t="s">
-        <v>712</v>
+        <v>719</v>
       </c>
       <c r="C10" s="27" t="s">
-        <v>713</v>
+        <v>720</v>
       </c>
       <c r="D10" s="28" t="s">
-        <v>714</v>
+        <v>721</v>
       </c>
       <c r="E10" s="29" t="s">
-        <v>715</v>
+        <v>722</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="5" t="s">
-        <v>716</v>
+        <v>723</v>
       </c>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -9293,7 +9566,7 @@
     </row>
     <row r="20" spans="1:5">
       <c r="A20" s="5" t="s">
-        <v>717</v>
+        <v>724</v>
       </c>
       <c r="B20" s="5"/>
       <c r="C20" s="5"/>
@@ -9302,36 +9575,36 @@
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="7" t="s">
-        <v>718</v>
+        <v>725</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>719</v>
+        <v>726</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>720</v>
+        <v>727</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>721</v>
+        <v>728</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>722</v>
+        <v>729</v>
       </c>
     </row>
     <row r="22" spans="1:5">
       <c r="A22" s="14" t="s">
-        <v>723</v>
+        <v>730</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>724</v>
+        <v>731</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>725</v>
+        <v>732</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>726</v>
+        <v>733</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>727</v>
+        <v>734</v>
       </c>
     </row>
     <row r="23" spans="1:5">
@@ -9339,16 +9612,16 @@
         <v>46</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>728</v>
+        <v>735</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>729</v>
+        <v>736</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>730</v>
+        <v>737</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>731</v>
+        <v>738</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -9356,16 +9629,16 @@
         <v>33</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>732</v>
+        <v>739</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>733</v>
+        <v>740</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>734</v>
+        <v>741</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>735</v>
+        <v>742</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -9373,21 +9646,21 @@
         <v>36</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>736</v>
+        <v>743</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>737</v>
+        <v>744</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>738</v>
+        <v>745</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>739</v>
+        <v>746</v>
       </c>
     </row>
     <row r="27" spans="1:5">
       <c r="A27" s="5" t="s">
-        <v>740</v>
+        <v>747</v>
       </c>
       <c r="B27" s="5"/>
       <c r="C27" s="5"/>
@@ -9396,7 +9669,7 @@
     </row>
     <row r="28" spans="1:5">
       <c r="A28" s="4" t="s">
-        <v>741</v>
+        <v>748</v>
       </c>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
@@ -9405,7 +9678,7 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" s="4" t="s">
-        <v>742</v>
+        <v>749</v>
       </c>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -9414,7 +9687,7 @@
     </row>
     <row r="30" spans="1:5">
       <c r="A30" s="4" t="s">
-        <v>743</v>
+        <v>750</v>
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -9423,7 +9696,7 @@
     </row>
     <row r="31" spans="1:5">
       <c r="A31" s="4" t="s">
-        <v>744</v>
+        <v>751</v>
       </c>
       <c r="B31" s="4"/>
       <c r="C31" s="4"/>
@@ -9432,7 +9705,7 @@
     </row>
     <row r="32" spans="1:5">
       <c r="A32" s="4" t="s">
-        <v>745</v>
+        <v>752</v>
       </c>
       <c r="B32" s="4"/>
       <c r="C32" s="4"/>
@@ -9456,98 +9729,98 @@
         <v>423</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>746</v>
+        <v>753</v>
       </c>
       <c r="D35" s="7"/>
       <c r="E35" s="7"/>
     </row>
     <row r="36" spans="1:5">
       <c r="A36" s="4" t="s">
-        <v>747</v>
+        <v>754</v>
       </c>
       <c r="B36" s="24" t="s">
-        <v>748</v>
+        <v>755</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>749</v>
+        <v>756</v>
       </c>
       <c r="D36" s="4"/>
       <c r="E36" s="4"/>
     </row>
     <row r="37" spans="1:5">
       <c r="A37" s="4" t="s">
-        <v>750</v>
+        <v>757</v>
       </c>
       <c r="B37" s="24" t="s">
-        <v>751</v>
+        <v>758</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>752</v>
+        <v>759</v>
       </c>
       <c r="D37" s="4"/>
       <c r="E37" s="4"/>
     </row>
     <row r="38" spans="1:5">
       <c r="A38" s="4" t="s">
-        <v>753</v>
+        <v>760</v>
       </c>
       <c r="B38" s="24" t="s">
         <v>431</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>754</v>
+        <v>761</v>
       </c>
       <c r="D38" s="4"/>
       <c r="E38" s="4"/>
     </row>
     <row r="39" spans="1:5">
       <c r="A39" s="4" t="s">
-        <v>755</v>
+        <v>762</v>
       </c>
       <c r="B39" s="24" t="s">
-        <v>756</v>
+        <v>763</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>757</v>
+        <v>764</v>
       </c>
       <c r="D39" s="4"/>
       <c r="E39" s="4"/>
     </row>
     <row r="40" spans="1:5">
       <c r="A40" s="4" t="s">
-        <v>755</v>
+        <v>762</v>
       </c>
       <c r="B40" s="24" t="s">
-        <v>758</v>
+        <v>765</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>759</v>
+        <v>766</v>
       </c>
       <c r="D40" s="4"/>
       <c r="E40" s="4"/>
     </row>
     <row r="41" spans="1:5">
       <c r="A41" s="4" t="s">
-        <v>760</v>
+        <v>767</v>
       </c>
       <c r="B41" s="24" t="s">
-        <v>761</v>
+        <v>768</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>762</v>
+        <v>769</v>
       </c>
       <c r="D41" s="4"/>
       <c r="E41" s="4"/>
     </row>
     <row r="42" spans="1:5">
       <c r="A42" s="4" t="s">
-        <v>763</v>
+        <v>770</v>
       </c>
       <c r="B42" s="24" t="s">
-        <v>764</v>
+        <v>771</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>765</v>
+        <v>772</v>
       </c>
       <c r="D42" s="4"/>
       <c r="E42" s="4"/>

</xml_diff>

<commit_message>
Complete B7 W1 T1: add Tuck Planche + shoulder hygiene (ext rotation, scap pull-ups)
</commit_message>
<xml_diff>
--- a/Training_3_B7.xlsx
+++ b/Training_3_B7.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1499" uniqueCount="837">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1513" uniqueCount="841">
   <si>
     <t>B7 — Performance-Block Dashboard (Advanced OAHS)</t>
   </si>
@@ -1986,6 +1986,18 @@
   </si>
   <si>
     <t>Straps, leicht (Gate); 20 kg</t>
+  </si>
+  <si>
+    <t>Tuck Planche 2x8s</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>External Rotation, leichtes Band</t>
+  </si>
+  <si>
+    <t>Scap Pull-ups; linke Hand seitlich spuerbar (kein Schmerz)</t>
   </si>
   <si>
     <t>B7 — Nutrition Targets (Maintenance, KEIN Defizit)</t>
@@ -3770,7 +3782,7 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>773</v>
+        <v>777</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3780,7 +3792,7 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="12" t="s">
-        <v>774</v>
+        <v>778</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -3805,12 +3817,12 @@
         <v>153</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>775</v>
+        <v>779</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="9" t="s">
-        <v>776</v>
+        <v>780</v>
       </c>
       <c r="B4" s="11">
         <f>SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Skill90",'B7_Training_Log'!$C$2:$C$1000,1)+SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Planche",'B7_Training_Log'!$C$2:$C$1000,1)+SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Push",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -3835,7 +3847,7 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="9" t="s">
-        <v>777</v>
+        <v>781</v>
       </c>
       <c r="B5" s="11">
         <f>SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Pull",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -3860,7 +3872,7 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="9" t="s">
-        <v>778</v>
+        <v>782</v>
       </c>
       <c r="B6" s="11">
         <f>SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Legs",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -3885,7 +3897,7 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="9" t="s">
-        <v>779</v>
+        <v>783</v>
       </c>
       <c r="B7" s="10">
         <f>SUMIFS('B7_Training_Log'!$N$2:$N$1000,'B7_Training_Log'!$D$2:$D$1000,"90",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -3910,7 +3922,7 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="9" t="s">
-        <v>780</v>
+        <v>784</v>
       </c>
       <c r="B8" s="10">
         <f>COUNTIFS('B7_Training_Log'!$E$2:$E$1000,"SkillOAHS",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -3935,7 +3947,7 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="9" t="s">
-        <v>781</v>
+        <v>785</v>
       </c>
       <c r="B9" s="10">
         <f>MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_straddle",'B7_Training_Log'!$F$2:$F$1000,"L",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -3960,7 +3972,7 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="9" t="s">
-        <v>782</v>
+        <v>786</v>
       </c>
       <c r="B10" s="10">
         <f>MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_straddle",'B7_Training_Log'!$F$2:$F$1000,"R",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -3985,7 +3997,7 @@
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="9" t="s">
-        <v>783</v>
+        <v>787</v>
       </c>
       <c r="B11" s="10">
         <f>MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_diamond",'B7_Training_Log'!$F$2:$F$1000,"L",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4010,7 +4022,7 @@
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="9" t="s">
-        <v>784</v>
+        <v>788</v>
       </c>
       <c r="B12" s="10">
         <f>MAX(MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_flag",'B7_Training_Log'!$C$2:$C$1000,1),MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_figa",'B7_Training_Log'!$C$2:$C$1000,1))</f>
@@ -4035,7 +4047,7 @@
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="9" t="s">
-        <v>785</v>
+        <v>789</v>
       </c>
       <c r="B13" s="11">
         <f>IFERROR(AVERAGEIFS('B7_Training_Log'!$J$2:$J$1000,'B7_Training_Log'!$C$2:$C$1000,1),0)</f>
@@ -4110,7 +4122,7 @@
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="9" t="s">
-        <v>786</v>
+        <v>790</v>
       </c>
       <c r="B16" s="10">
         <f>COUNTIFS('B7_Training_Log'!$K$2:$K$1000,"&gt;=4",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4135,7 +4147,7 @@
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="9" t="s">
-        <v>787</v>
+        <v>791</v>
       </c>
       <c r="B17" s="10">
         <f>COUNTIFS('B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4179,7 +4191,7 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
-        <v>788</v>
+        <v>792</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4187,7 +4199,7 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="5" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
@@ -4195,13 +4207,13 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="7" t="s">
-        <v>790</v>
+        <v>794</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>791</v>
+        <v>795</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>792</v>
+        <v>796</v>
       </c>
       <c r="D4" s="7"/>
     </row>
@@ -4210,10 +4222,10 @@
         <v>627</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>793</v>
+        <v>797</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>794</v>
+        <v>798</v>
       </c>
       <c r="D5" s="4"/>
     </row>
@@ -4222,10 +4234,10 @@
         <v>628</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>795</v>
+        <v>799</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>796</v>
+        <v>800</v>
       </c>
       <c r="D6" s="4"/>
     </row>
@@ -4234,10 +4246,10 @@
         <v>629</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>797</v>
+        <v>801</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>798</v>
+        <v>802</v>
       </c>
       <c r="D7" s="4"/>
     </row>
@@ -4246,10 +4258,10 @@
         <v>436</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>799</v>
+        <v>803</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>800</v>
+        <v>804</v>
       </c>
       <c r="D8" s="4"/>
     </row>
@@ -4258,10 +4270,10 @@
         <v>439</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>801</v>
+        <v>805</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>802</v>
+        <v>806</v>
       </c>
       <c r="D9" s="4"/>
     </row>
@@ -4270,10 +4282,10 @@
         <v>630</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>803</v>
+        <v>807</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>804</v>
+        <v>808</v>
       </c>
       <c r="D10" s="4"/>
     </row>
@@ -4282,10 +4294,10 @@
         <v>631</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>805</v>
+        <v>809</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>806</v>
+        <v>810</v>
       </c>
       <c r="D11" s="4"/>
     </row>
@@ -4294,10 +4306,10 @@
         <v>632</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>807</v>
+        <v>811</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>808</v>
+        <v>812</v>
       </c>
       <c r="D12" s="4"/>
     </row>
@@ -4306,10 +4318,10 @@
         <v>633</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>805</v>
+        <v>809</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>809</v>
+        <v>813</v>
       </c>
       <c r="D13" s="4"/>
     </row>
@@ -4318,10 +4330,10 @@
         <v>634</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>810</v>
+        <v>814</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>811</v>
+        <v>815</v>
       </c>
       <c r="D14" s="4"/>
     </row>
@@ -4330,10 +4342,10 @@
         <v>635</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>812</v>
+        <v>816</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>813</v>
+        <v>817</v>
       </c>
       <c r="D15" s="4"/>
     </row>
@@ -4342,10 +4354,10 @@
         <v>636</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>814</v>
+        <v>818</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>815</v>
+        <v>819</v>
       </c>
       <c r="D16" s="4"/>
     </row>
@@ -4354,10 +4366,10 @@
         <v>637</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>805</v>
+        <v>809</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>816</v>
+        <v>820</v>
       </c>
       <c r="D17" s="4"/>
     </row>
@@ -4366,10 +4378,10 @@
         <v>638</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>805</v>
+        <v>809</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>817</v>
+        <v>821</v>
       </c>
       <c r="D18" s="4"/>
     </row>
@@ -4378,10 +4390,10 @@
         <v>639</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>818</v>
+        <v>822</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>819</v>
+        <v>823</v>
       </c>
       <c r="D19" s="4"/>
     </row>
@@ -4390,10 +4402,10 @@
         <v>92</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>807</v>
+        <v>811</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>820</v>
+        <v>824</v>
       </c>
       <c r="D20" s="4"/>
     </row>
@@ -4402,16 +4414,16 @@
         <v>640</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>821</v>
+        <v>825</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>822</v>
+        <v>826</v>
       </c>
       <c r="D21" s="4"/>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="5" t="s">
-        <v>823</v>
+        <v>827</v>
       </c>
       <c r="B23" s="5"/>
       <c r="C23" s="5"/>
@@ -4419,7 +4431,7 @@
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="4" t="s">
-        <v>824</v>
+        <v>828</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -4427,7 +4439,7 @@
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="4" t="s">
-        <v>825</v>
+        <v>829</v>
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -4435,7 +4447,7 @@
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="4" t="s">
-        <v>826</v>
+        <v>830</v>
       </c>
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
@@ -4443,7 +4455,7 @@
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="4" t="s">
-        <v>827</v>
+        <v>831</v>
       </c>
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
@@ -4451,7 +4463,7 @@
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="4" t="s">
-        <v>828</v>
+        <v>832</v>
       </c>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
@@ -4459,7 +4471,7 @@
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="4" t="s">
-        <v>829</v>
+        <v>833</v>
       </c>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -4467,7 +4479,7 @@
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="4" t="s">
-        <v>830</v>
+        <v>834</v>
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -4475,7 +4487,7 @@
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="5" t="s">
-        <v>831</v>
+        <v>835</v>
       </c>
       <c r="B32" s="5"/>
       <c r="C32" s="5"/>
@@ -4483,7 +4495,7 @@
     </row>
     <row r="33" spans="1:4">
       <c r="A33" s="4" t="s">
-        <v>832</v>
+        <v>836</v>
       </c>
       <c r="B33" s="4"/>
       <c r="C33" s="4"/>
@@ -4491,7 +4503,7 @@
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="4" t="s">
-        <v>833</v>
+        <v>837</v>
       </c>
       <c r="B34" s="4"/>
       <c r="C34" s="4"/>
@@ -4499,7 +4511,7 @@
     </row>
     <row r="35" spans="1:4">
       <c r="A35" s="4" t="s">
-        <v>834</v>
+        <v>838</v>
       </c>
       <c r="B35" s="4"/>
       <c r="C35" s="4"/>
@@ -4507,7 +4519,7 @@
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="4" t="s">
-        <v>835</v>
+        <v>839</v>
       </c>
       <c r="B36" s="4"/>
       <c r="C36" s="4"/>
@@ -4515,7 +4527,7 @@
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="4" t="s">
-        <v>836</v>
+        <v>840</v>
       </c>
       <c r="B37" s="4"/>
       <c r="C37" s="4"/>
@@ -8497,7 +8509,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q9"/>
+  <dimension ref="A1:Q12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -8914,6 +8926,132 @@
       </c>
       <c r="Q9" s="6">
         <f>IF($B9="","",$B9&amp;"_W"&amp;$C9)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17">
+      <c r="A10" s="25">
+        <v>46211</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="C10" s="6">
+        <v>1</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>478</v>
+      </c>
+      <c r="E10" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D10,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>648</v>
+      </c>
+      <c r="G10" s="6">
+        <v>2</v>
+      </c>
+      <c r="I10" s="6">
+        <v>0</v>
+      </c>
+      <c r="J10" s="6">
+        <v>6</v>
+      </c>
+      <c r="M10" s="6">
+        <v>8</v>
+      </c>
+      <c r="O10" s="6">
+        <v>2</v>
+      </c>
+      <c r="P10" s="4" t="s">
+        <v>652</v>
+      </c>
+      <c r="Q10" s="6">
+        <f>IF($B10="","",$B10&amp;"_W"&amp;$C10)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17">
+      <c r="A11" s="25">
+        <v>46211</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="C11" s="6">
+        <v>1</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>514</v>
+      </c>
+      <c r="E11" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D11,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>648</v>
+      </c>
+      <c r="G11" s="6">
+        <v>2</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>653</v>
+      </c>
+      <c r="J11" s="6">
+        <v>6</v>
+      </c>
+      <c r="O11" s="6">
+        <v>2</v>
+      </c>
+      <c r="P11" s="4" t="s">
+        <v>654</v>
+      </c>
+      <c r="Q11" s="6">
+        <f>IF($B11="","",$B11&amp;"_W"&amp;$C11)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17">
+      <c r="A12" s="25">
+        <v>46211</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="C12" s="6">
+        <v>1</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>509</v>
+      </c>
+      <c r="E12" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D12,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>648</v>
+      </c>
+      <c r="G12" s="6">
+        <v>2</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>653</v>
+      </c>
+      <c r="I12" s="6">
+        <v>0</v>
+      </c>
+      <c r="J12" s="6">
+        <v>6</v>
+      </c>
+      <c r="O12" s="6">
+        <v>2</v>
+      </c>
+      <c r="P12" s="4" t="s">
+        <v>655</v>
+      </c>
+      <c r="Q12" s="6">
+        <f>IF($B12="","",$B12&amp;"_W"&amp;$C12)</f>
         <v>0</v>
       </c>
     </row>
@@ -8991,7 +9129,7 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>652</v>
+        <v>656</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -9002,20 +9140,20 @@
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="5" t="s">
-        <v>653</v>
+        <v>657</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="9" t="s">
-        <v>654</v>
+        <v>658</v>
       </c>
       <c r="B4" s="11">
         <v>81</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>662</v>
+        <v>666</v>
       </c>
       <c r="D4" s="4"/>
       <c r="E4" s="4"/>
@@ -9024,21 +9162,21 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="9" t="s">
-        <v>655</v>
+        <v>659</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>656</v>
+        <v>660</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="9" t="s">
-        <v>657</v>
+        <v>661</v>
       </c>
       <c r="B6" s="11">
         <v>2.2</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>663</v>
+        <v>667</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
@@ -9047,7 +9185,7 @@
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="9" t="s">
-        <v>658</v>
+        <v>662</v>
       </c>
       <c r="B7" s="11">
         <v>0.9</v>
@@ -9055,7 +9193,7 @@
     </row>
     <row r="8" spans="1:7">
       <c r="A8" s="9" t="s">
-        <v>659</v>
+        <v>663</v>
       </c>
       <c r="B8" s="10">
         <v>2700</v>
@@ -9063,7 +9201,7 @@
     </row>
     <row r="9" spans="1:7">
       <c r="A9" s="9" t="s">
-        <v>660</v>
+        <v>664</v>
       </c>
       <c r="B9" s="10">
         <f>ROUND(BW*B6,0)</f>
@@ -9072,7 +9210,7 @@
     </row>
     <row r="10" spans="1:7">
       <c r="A10" s="9" t="s">
-        <v>661</v>
+        <v>665</v>
       </c>
       <c r="B10" s="10">
         <f>ROUND(BW*B7,0)</f>
@@ -9081,7 +9219,7 @@
     </row>
     <row r="12" spans="1:7">
       <c r="A12" s="5" t="s">
-        <v>664</v>
+        <v>668</v>
       </c>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -9095,27 +9233,27 @@
         <v>85</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>666</v>
+        <v>670</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>667</v>
+        <v>671</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>668</v>
+        <v>672</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>669</v>
+        <v>673</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>670</v>
+        <v>674</v>
       </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" s="9" t="s">
-        <v>671</v>
+        <v>675</v>
       </c>
       <c r="B14" s="26">
         <v>250</v>
@@ -9137,7 +9275,7 @@
         <v>0</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>672</v>
+        <v>676</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -9164,12 +9302,12 @@
         <v>0</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>673</v>
+        <v>677</v>
       </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" s="9" t="s">
-        <v>674</v>
+        <v>678</v>
       </c>
       <c r="B16" s="26">
         <v>200</v>
@@ -9191,12 +9329,12 @@
         <v>0</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>675</v>
+        <v>679</v>
       </c>
     </row>
     <row r="17" spans="1:7">
       <c r="A17" s="9" t="s">
-        <v>676</v>
+        <v>680</v>
       </c>
       <c r="B17" s="26">
         <v>150</v>
@@ -9218,12 +9356,12 @@
         <v>0</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>677</v>
+        <v>681</v>
       </c>
     </row>
     <row r="18" spans="1:7">
       <c r="A18" s="9" t="s">
-        <v>678</v>
+        <v>682</v>
       </c>
       <c r="B18" s="26">
         <v>100</v>
@@ -9245,7 +9383,7 @@
         <v>0</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>679</v>
+        <v>683</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -9272,12 +9410,12 @@
         <v>0</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>680</v>
+        <v>684</v>
       </c>
     </row>
     <row r="21" spans="1:7">
       <c r="A21" s="5" t="s">
-        <v>681</v>
+        <v>685</v>
       </c>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
@@ -9288,7 +9426,7 @@
     </row>
     <row r="22" spans="1:7">
       <c r="A22" s="4" t="s">
-        <v>682</v>
+        <v>686</v>
       </c>
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
@@ -9299,7 +9437,7 @@
     </row>
     <row r="23" spans="1:7">
       <c r="A23" s="4" t="s">
-        <v>683</v>
+        <v>687</v>
       </c>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
@@ -9310,7 +9448,7 @@
     </row>
     <row r="24" spans="1:7">
       <c r="A24" s="4" t="s">
-        <v>684</v>
+        <v>688</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -9321,7 +9459,7 @@
     </row>
     <row r="25" spans="1:7">
       <c r="A25" s="4" t="s">
-        <v>685</v>
+        <v>689</v>
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -9366,7 +9504,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>686</v>
+        <v>690</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -9375,7 +9513,7 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="5" t="s">
-        <v>687</v>
+        <v>691</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
@@ -9384,126 +9522,126 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="7" t="s">
-        <v>688</v>
+        <v>692</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>689</v>
+        <v>693</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>690</v>
+        <v>694</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>691</v>
+        <v>695</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>692</v>
+        <v>696</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="9" t="s">
-        <v>693</v>
+        <v>697</v>
       </c>
       <c r="B5" s="22" t="s">
-        <v>694</v>
+        <v>698</v>
       </c>
       <c r="C5" s="27" t="s">
-        <v>695</v>
+        <v>699</v>
       </c>
       <c r="D5" s="28" t="s">
-        <v>696</v>
+        <v>700</v>
       </c>
       <c r="E5" s="29" t="s">
-        <v>697</v>
+        <v>701</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="9" t="s">
-        <v>698</v>
+        <v>702</v>
       </c>
       <c r="B6" s="22" t="s">
-        <v>699</v>
+        <v>703</v>
       </c>
       <c r="C6" s="27" t="s">
-        <v>700</v>
+        <v>704</v>
       </c>
       <c r="D6" s="28" t="s">
-        <v>701</v>
+        <v>705</v>
       </c>
       <c r="E6" s="29" t="s">
-        <v>702</v>
+        <v>706</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="9" t="s">
-        <v>703</v>
+        <v>707</v>
       </c>
       <c r="B7" s="22" t="s">
-        <v>704</v>
+        <v>708</v>
       </c>
       <c r="C7" s="27" t="s">
-        <v>705</v>
+        <v>709</v>
       </c>
       <c r="D7" s="28" t="s">
-        <v>706</v>
+        <v>710</v>
       </c>
       <c r="E7" s="29" t="s">
-        <v>707</v>
+        <v>711</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="9" t="s">
-        <v>708</v>
+        <v>712</v>
       </c>
       <c r="B8" s="22" t="s">
-        <v>709</v>
+        <v>713</v>
       </c>
       <c r="C8" s="27" t="s">
-        <v>710</v>
+        <v>714</v>
       </c>
       <c r="D8" s="28" t="s">
-        <v>711</v>
+        <v>715</v>
       </c>
       <c r="E8" s="29" t="s">
-        <v>712</v>
+        <v>716</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="9" t="s">
-        <v>713</v>
+        <v>717</v>
       </c>
       <c r="B9" s="22" t="s">
-        <v>714</v>
+        <v>718</v>
       </c>
       <c r="C9" s="27" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
       <c r="D9" s="28" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="E9" s="29" t="s">
-        <v>717</v>
+        <v>721</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="9" t="s">
-        <v>718</v>
+        <v>722</v>
       </c>
       <c r="B10" s="22" t="s">
-        <v>719</v>
+        <v>723</v>
       </c>
       <c r="C10" s="27" t="s">
-        <v>720</v>
+        <v>724</v>
       </c>
       <c r="D10" s="28" t="s">
-        <v>721</v>
+        <v>725</v>
       </c>
       <c r="E10" s="29" t="s">
-        <v>722</v>
+        <v>726</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="5" t="s">
-        <v>723</v>
+        <v>727</v>
       </c>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -9566,7 +9704,7 @@
     </row>
     <row r="20" spans="1:5">
       <c r="A20" s="5" t="s">
-        <v>724</v>
+        <v>728</v>
       </c>
       <c r="B20" s="5"/>
       <c r="C20" s="5"/>
@@ -9575,36 +9713,36 @@
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="7" t="s">
-        <v>725</v>
+        <v>729</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>726</v>
+        <v>730</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>727</v>
+        <v>731</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>728</v>
+        <v>732</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>729</v>
+        <v>733</v>
       </c>
     </row>
     <row r="22" spans="1:5">
       <c r="A22" s="14" t="s">
-        <v>730</v>
+        <v>734</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>731</v>
+        <v>735</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>732</v>
+        <v>736</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>733</v>
+        <v>737</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>734</v>
+        <v>738</v>
       </c>
     </row>
     <row r="23" spans="1:5">
@@ -9612,16 +9750,16 @@
         <v>46</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>735</v>
+        <v>739</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>736</v>
+        <v>740</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>737</v>
+        <v>741</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>738</v>
+        <v>742</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -9629,16 +9767,16 @@
         <v>33</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>739</v>
+        <v>743</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>740</v>
+        <v>744</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>741</v>
+        <v>745</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>742</v>
+        <v>746</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -9646,21 +9784,21 @@
         <v>36</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>743</v>
+        <v>747</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>744</v>
+        <v>748</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>745</v>
+        <v>749</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>746</v>
+        <v>750</v>
       </c>
     </row>
     <row r="27" spans="1:5">
       <c r="A27" s="5" t="s">
-        <v>747</v>
+        <v>751</v>
       </c>
       <c r="B27" s="5"/>
       <c r="C27" s="5"/>
@@ -9669,7 +9807,7 @@
     </row>
     <row r="28" spans="1:5">
       <c r="A28" s="4" t="s">
-        <v>748</v>
+        <v>752</v>
       </c>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
@@ -9678,7 +9816,7 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" s="4" t="s">
-        <v>749</v>
+        <v>753</v>
       </c>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -9687,7 +9825,7 @@
     </row>
     <row r="30" spans="1:5">
       <c r="A30" s="4" t="s">
-        <v>750</v>
+        <v>754</v>
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -9696,7 +9834,7 @@
     </row>
     <row r="31" spans="1:5">
       <c r="A31" s="4" t="s">
-        <v>751</v>
+        <v>755</v>
       </c>
       <c r="B31" s="4"/>
       <c r="C31" s="4"/>
@@ -9705,7 +9843,7 @@
     </row>
     <row r="32" spans="1:5">
       <c r="A32" s="4" t="s">
-        <v>752</v>
+        <v>756</v>
       </c>
       <c r="B32" s="4"/>
       <c r="C32" s="4"/>
@@ -9729,98 +9867,98 @@
         <v>423</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>753</v>
+        <v>757</v>
       </c>
       <c r="D35" s="7"/>
       <c r="E35" s="7"/>
     </row>
     <row r="36" spans="1:5">
       <c r="A36" s="4" t="s">
-        <v>754</v>
+        <v>758</v>
       </c>
       <c r="B36" s="24" t="s">
-        <v>755</v>
+        <v>759</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>756</v>
+        <v>760</v>
       </c>
       <c r="D36" s="4"/>
       <c r="E36" s="4"/>
     </row>
     <row r="37" spans="1:5">
       <c r="A37" s="4" t="s">
-        <v>757</v>
+        <v>761</v>
       </c>
       <c r="B37" s="24" t="s">
-        <v>758</v>
+        <v>762</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>759</v>
+        <v>763</v>
       </c>
       <c r="D37" s="4"/>
       <c r="E37" s="4"/>
     </row>
     <row r="38" spans="1:5">
       <c r="A38" s="4" t="s">
-        <v>760</v>
+        <v>764</v>
       </c>
       <c r="B38" s="24" t="s">
         <v>431</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>761</v>
+        <v>765</v>
       </c>
       <c r="D38" s="4"/>
       <c r="E38" s="4"/>
     </row>
     <row r="39" spans="1:5">
       <c r="A39" s="4" t="s">
-        <v>762</v>
+        <v>766</v>
       </c>
       <c r="B39" s="24" t="s">
-        <v>763</v>
+        <v>767</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>764</v>
+        <v>768</v>
       </c>
       <c r="D39" s="4"/>
       <c r="E39" s="4"/>
     </row>
     <row r="40" spans="1:5">
       <c r="A40" s="4" t="s">
-        <v>762</v>
+        <v>766</v>
       </c>
       <c r="B40" s="24" t="s">
-        <v>765</v>
+        <v>769</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>766</v>
+        <v>770</v>
       </c>
       <c r="D40" s="4"/>
       <c r="E40" s="4"/>
     </row>
     <row r="41" spans="1:5">
       <c r="A41" s="4" t="s">
-        <v>767</v>
+        <v>771</v>
       </c>
       <c r="B41" s="24" t="s">
-        <v>768</v>
+        <v>772</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>769</v>
+        <v>773</v>
       </c>
       <c r="D41" s="4"/>
       <c r="E41" s="4"/>
     </row>
     <row r="42" spans="1:5">
       <c r="A42" s="4" t="s">
-        <v>770</v>
+        <v>774</v>
       </c>
       <c r="B42" s="24" t="s">
-        <v>771</v>
+        <v>775</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>772</v>
+        <v>776</v>
       </c>
       <c r="D42" s="4"/>
       <c r="E42" s="4"/>

</xml_diff>

<commit_message>
Log B7 W1 T2 (Recovery 3): Tier-A shapes 8s progress incl right side + pull/core
</commit_message>
<xml_diff>
--- a/Training_3_B7.xlsx
+++ b/Training_3_B7.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1513" uniqueCount="841">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1560" uniqueCount="854">
   <si>
     <t>B7 — Performance-Block Dashboard (Advanced OAHS)</t>
   </si>
@@ -1998,6 +1998,45 @@
   </si>
   <si>
     <t>Scap Pull-ups; linke Hand seitlich spuerbar (kein Schmerz)</t>
+  </si>
+  <si>
+    <t>8s 2/3 links; Schulter bereits bei 8s-Holds muede</t>
+  </si>
+  <si>
+    <t>8s 2/3 rechts - verbessert!</t>
+  </si>
+  <si>
+    <t>8s 2/3 links</t>
+  </si>
+  <si>
+    <t>8s 1/3 rechts</t>
+  </si>
+  <si>
+    <t>kein 8s, 4-6s, letzter Satz muede</t>
+  </si>
+  <si>
+    <t>kein 8s, 4-6s, muede</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>Seated/Chest Row</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>Reverse Butterfly</t>
+  </si>
+  <si>
+    <t>30s</t>
+  </si>
+  <si>
+    <t>3x30s</t>
   </si>
   <si>
     <t>B7 — Nutrition Targets (Maintenance, KEIN Defizit)</t>
@@ -3782,7 +3821,7 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>777</v>
+        <v>790</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3792,7 +3831,7 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="12" t="s">
-        <v>778</v>
+        <v>791</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -3817,12 +3856,12 @@
         <v>153</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>779</v>
+        <v>792</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="9" t="s">
-        <v>780</v>
+        <v>793</v>
       </c>
       <c r="B4" s="11">
         <f>SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Skill90",'B7_Training_Log'!$C$2:$C$1000,1)+SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Planche",'B7_Training_Log'!$C$2:$C$1000,1)+SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Push",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -3847,7 +3886,7 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="9" t="s">
-        <v>781</v>
+        <v>794</v>
       </c>
       <c r="B5" s="11">
         <f>SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Pull",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -3872,7 +3911,7 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="9" t="s">
-        <v>782</v>
+        <v>795</v>
       </c>
       <c r="B6" s="11">
         <f>SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Legs",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -3897,7 +3936,7 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="9" t="s">
-        <v>783</v>
+        <v>796</v>
       </c>
       <c r="B7" s="10">
         <f>SUMIFS('B7_Training_Log'!$N$2:$N$1000,'B7_Training_Log'!$D$2:$D$1000,"90",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -3922,7 +3961,7 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="9" t="s">
-        <v>784</v>
+        <v>797</v>
       </c>
       <c r="B8" s="10">
         <f>COUNTIFS('B7_Training_Log'!$E$2:$E$1000,"SkillOAHS",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -3947,7 +3986,7 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="9" t="s">
-        <v>785</v>
+        <v>798</v>
       </c>
       <c r="B9" s="10">
         <f>MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_straddle",'B7_Training_Log'!$F$2:$F$1000,"L",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -3972,7 +4011,7 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="9" t="s">
-        <v>786</v>
+        <v>799</v>
       </c>
       <c r="B10" s="10">
         <f>MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_straddle",'B7_Training_Log'!$F$2:$F$1000,"R",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -3997,7 +4036,7 @@
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="9" t="s">
-        <v>787</v>
+        <v>800</v>
       </c>
       <c r="B11" s="10">
         <f>MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_diamond",'B7_Training_Log'!$F$2:$F$1000,"L",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4022,7 +4061,7 @@
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="9" t="s">
-        <v>788</v>
+        <v>801</v>
       </c>
       <c r="B12" s="10">
         <f>MAX(MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_flag",'B7_Training_Log'!$C$2:$C$1000,1),MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_figa",'B7_Training_Log'!$C$2:$C$1000,1))</f>
@@ -4047,7 +4086,7 @@
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="9" t="s">
-        <v>789</v>
+        <v>802</v>
       </c>
       <c r="B13" s="11">
         <f>IFERROR(AVERAGEIFS('B7_Training_Log'!$J$2:$J$1000,'B7_Training_Log'!$C$2:$C$1000,1),0)</f>
@@ -4122,7 +4161,7 @@
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="9" t="s">
-        <v>790</v>
+        <v>803</v>
       </c>
       <c r="B16" s="10">
         <f>COUNTIFS('B7_Training_Log'!$K$2:$K$1000,"&gt;=4",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4147,7 +4186,7 @@
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="9" t="s">
-        <v>791</v>
+        <v>804</v>
       </c>
       <c r="B17" s="10">
         <f>COUNTIFS('B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4191,7 +4230,7 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
-        <v>792</v>
+        <v>805</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4199,7 +4238,7 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="5" t="s">
-        <v>793</v>
+        <v>806</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
@@ -4207,13 +4246,13 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="7" t="s">
-        <v>794</v>
+        <v>807</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>795</v>
+        <v>808</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>796</v>
+        <v>809</v>
       </c>
       <c r="D4" s="7"/>
     </row>
@@ -4222,10 +4261,10 @@
         <v>627</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>797</v>
+        <v>810</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>798</v>
+        <v>811</v>
       </c>
       <c r="D5" s="4"/>
     </row>
@@ -4234,10 +4273,10 @@
         <v>628</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>799</v>
+        <v>812</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>800</v>
+        <v>813</v>
       </c>
       <c r="D6" s="4"/>
     </row>
@@ -4246,10 +4285,10 @@
         <v>629</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>801</v>
+        <v>814</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>802</v>
+        <v>815</v>
       </c>
       <c r="D7" s="4"/>
     </row>
@@ -4258,10 +4297,10 @@
         <v>436</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>803</v>
+        <v>816</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>804</v>
+        <v>817</v>
       </c>
       <c r="D8" s="4"/>
     </row>
@@ -4270,10 +4309,10 @@
         <v>439</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>805</v>
+        <v>818</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>806</v>
+        <v>819</v>
       </c>
       <c r="D9" s="4"/>
     </row>
@@ -4282,10 +4321,10 @@
         <v>630</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>807</v>
+        <v>820</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>808</v>
+        <v>821</v>
       </c>
       <c r="D10" s="4"/>
     </row>
@@ -4294,10 +4333,10 @@
         <v>631</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>809</v>
+        <v>822</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>810</v>
+        <v>823</v>
       </c>
       <c r="D11" s="4"/>
     </row>
@@ -4306,10 +4345,10 @@
         <v>632</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>811</v>
+        <v>824</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>812</v>
+        <v>825</v>
       </c>
       <c r="D12" s="4"/>
     </row>
@@ -4318,10 +4357,10 @@
         <v>633</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>809</v>
+        <v>822</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>813</v>
+        <v>826</v>
       </c>
       <c r="D13" s="4"/>
     </row>
@@ -4330,10 +4369,10 @@
         <v>634</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>814</v>
+        <v>827</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>815</v>
+        <v>828</v>
       </c>
       <c r="D14" s="4"/>
     </row>
@@ -4342,10 +4381,10 @@
         <v>635</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>816</v>
+        <v>829</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>817</v>
+        <v>830</v>
       </c>
       <c r="D15" s="4"/>
     </row>
@@ -4354,10 +4393,10 @@
         <v>636</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>818</v>
+        <v>831</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>819</v>
+        <v>832</v>
       </c>
       <c r="D16" s="4"/>
     </row>
@@ -4366,10 +4405,10 @@
         <v>637</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>809</v>
+        <v>822</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>820</v>
+        <v>833</v>
       </c>
       <c r="D17" s="4"/>
     </row>
@@ -4378,10 +4417,10 @@
         <v>638</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>809</v>
+        <v>822</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>821</v>
+        <v>834</v>
       </c>
       <c r="D18" s="4"/>
     </row>
@@ -4390,10 +4429,10 @@
         <v>639</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>822</v>
+        <v>835</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>823</v>
+        <v>836</v>
       </c>
       <c r="D19" s="4"/>
     </row>
@@ -4402,10 +4441,10 @@
         <v>92</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>811</v>
+        <v>824</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>824</v>
+        <v>837</v>
       </c>
       <c r="D20" s="4"/>
     </row>
@@ -4414,16 +4453,16 @@
         <v>640</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>825</v>
+        <v>838</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>826</v>
+        <v>839</v>
       </c>
       <c r="D21" s="4"/>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="5" t="s">
-        <v>827</v>
+        <v>840</v>
       </c>
       <c r="B23" s="5"/>
       <c r="C23" s="5"/>
@@ -4431,7 +4470,7 @@
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="4" t="s">
-        <v>828</v>
+        <v>841</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -4439,7 +4478,7 @@
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="4" t="s">
-        <v>829</v>
+        <v>842</v>
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -4447,7 +4486,7 @@
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="4" t="s">
-        <v>830</v>
+        <v>843</v>
       </c>
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
@@ -4455,7 +4494,7 @@
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="4" t="s">
-        <v>831</v>
+        <v>844</v>
       </c>
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
@@ -4463,7 +4502,7 @@
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="4" t="s">
-        <v>832</v>
+        <v>845</v>
       </c>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
@@ -4471,7 +4510,7 @@
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="4" t="s">
-        <v>833</v>
+        <v>846</v>
       </c>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -4479,7 +4518,7 @@
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="4" t="s">
-        <v>834</v>
+        <v>847</v>
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -4487,7 +4526,7 @@
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="5" t="s">
-        <v>835</v>
+        <v>848</v>
       </c>
       <c r="B32" s="5"/>
       <c r="C32" s="5"/>
@@ -4495,7 +4534,7 @@
     </row>
     <row r="33" spans="1:4">
       <c r="A33" s="4" t="s">
-        <v>836</v>
+        <v>849</v>
       </c>
       <c r="B33" s="4"/>
       <c r="C33" s="4"/>
@@ -4503,7 +4542,7 @@
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="4" t="s">
-        <v>837</v>
+        <v>850</v>
       </c>
       <c r="B34" s="4"/>
       <c r="C34" s="4"/>
@@ -4511,7 +4550,7 @@
     </row>
     <row r="35" spans="1:4">
       <c r="A35" s="4" t="s">
-        <v>838</v>
+        <v>851</v>
       </c>
       <c r="B35" s="4"/>
       <c r="C35" s="4"/>
@@ -4519,7 +4558,7 @@
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="4" t="s">
-        <v>839</v>
+        <v>852</v>
       </c>
       <c r="B36" s="4"/>
       <c r="C36" s="4"/>
@@ -4527,7 +4566,7 @@
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="4" t="s">
-        <v>840</v>
+        <v>853</v>
       </c>
       <c r="B37" s="4"/>
       <c r="C37" s="4"/>
@@ -8509,7 +8548,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q12"/>
+  <dimension ref="A1:Q23"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -9052,6 +9091,473 @@
       </c>
       <c r="Q12" s="6">
         <f>IF($B12="","",$B12&amp;"_W"&amp;$C12)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17">
+      <c r="A13" s="25">
+        <v>46212</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="C13" s="6">
+        <v>1</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>596</v>
+      </c>
+      <c r="E13" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D13,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>641</v>
+      </c>
+      <c r="G13" s="6">
+        <v>3</v>
+      </c>
+      <c r="I13" s="6">
+        <v>0</v>
+      </c>
+      <c r="L13" s="6">
+        <v>4</v>
+      </c>
+      <c r="M13" s="6">
+        <v>8</v>
+      </c>
+      <c r="O13" s="6">
+        <v>3</v>
+      </c>
+      <c r="P13" s="4" t="s">
+        <v>656</v>
+      </c>
+      <c r="Q13" s="6">
+        <f>IF($B13="","",$B13&amp;"_W"&amp;$C13)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17">
+      <c r="A14" s="25">
+        <v>46212</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="C14" s="6">
+        <v>1</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>596</v>
+      </c>
+      <c r="E14" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D14,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>643</v>
+      </c>
+      <c r="G14" s="6">
+        <v>3</v>
+      </c>
+      <c r="I14" s="6">
+        <v>0</v>
+      </c>
+      <c r="L14" s="6">
+        <v>4</v>
+      </c>
+      <c r="M14" s="6">
+        <v>8</v>
+      </c>
+      <c r="O14" s="6">
+        <v>3</v>
+      </c>
+      <c r="P14" s="4" t="s">
+        <v>657</v>
+      </c>
+      <c r="Q14" s="6">
+        <f>IF($B14="","",$B14&amp;"_W"&amp;$C14)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17">
+      <c r="A15" s="25">
+        <v>46212</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="C15" s="6">
+        <v>1</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>599</v>
+      </c>
+      <c r="E15" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D15,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>641</v>
+      </c>
+      <c r="G15" s="6">
+        <v>3</v>
+      </c>
+      <c r="I15" s="6">
+        <v>0</v>
+      </c>
+      <c r="L15" s="6">
+        <v>4</v>
+      </c>
+      <c r="M15" s="6">
+        <v>8</v>
+      </c>
+      <c r="O15" s="6">
+        <v>3</v>
+      </c>
+      <c r="P15" s="4" t="s">
+        <v>658</v>
+      </c>
+      <c r="Q15" s="6">
+        <f>IF($B15="","",$B15&amp;"_W"&amp;$C15)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17">
+      <c r="A16" s="25">
+        <v>46212</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="C16" s="6">
+        <v>1</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>599</v>
+      </c>
+      <c r="E16" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D16,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F16" s="6" t="s">
+        <v>643</v>
+      </c>
+      <c r="G16" s="6">
+        <v>3</v>
+      </c>
+      <c r="I16" s="6">
+        <v>0</v>
+      </c>
+      <c r="L16" s="6">
+        <v>3</v>
+      </c>
+      <c r="M16" s="6">
+        <v>8</v>
+      </c>
+      <c r="O16" s="6">
+        <v>3</v>
+      </c>
+      <c r="P16" s="4" t="s">
+        <v>659</v>
+      </c>
+      <c r="Q16" s="6">
+        <f>IF($B16="","",$B16&amp;"_W"&amp;$C16)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17">
+      <c r="A17" s="25">
+        <v>46212</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="C17" s="6">
+        <v>1</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>602</v>
+      </c>
+      <c r="E17" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D17,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F17" s="6" t="s">
+        <v>641</v>
+      </c>
+      <c r="G17" s="6">
+        <v>3</v>
+      </c>
+      <c r="I17" s="6">
+        <v>0</v>
+      </c>
+      <c r="L17" s="6">
+        <v>3</v>
+      </c>
+      <c r="M17" s="6">
+        <v>6</v>
+      </c>
+      <c r="O17" s="6">
+        <v>3</v>
+      </c>
+      <c r="P17" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="Q17" s="6">
+        <f>IF($B17="","",$B17&amp;"_W"&amp;$C17)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:17">
+      <c r="A18" s="25">
+        <v>46212</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="C18" s="6">
+        <v>1</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>602</v>
+      </c>
+      <c r="E18" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D18,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>643</v>
+      </c>
+      <c r="G18" s="6">
+        <v>3</v>
+      </c>
+      <c r="I18" s="6">
+        <v>0</v>
+      </c>
+      <c r="L18" s="6">
+        <v>3</v>
+      </c>
+      <c r="M18" s="6">
+        <v>6</v>
+      </c>
+      <c r="O18" s="6">
+        <v>3</v>
+      </c>
+      <c r="P18" s="4" t="s">
+        <v>661</v>
+      </c>
+      <c r="Q18" s="6">
+        <f>IF($B18="","",$B18&amp;"_W"&amp;$C18)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:17">
+      <c r="A19" s="25">
+        <v>46212</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="C19" s="6">
+        <v>1</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>494</v>
+      </c>
+      <c r="E19" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D19,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F19" s="6" t="s">
+        <v>648</v>
+      </c>
+      <c r="G19" s="6">
+        <v>3</v>
+      </c>
+      <c r="H19" s="4" t="s">
+        <v>662</v>
+      </c>
+      <c r="I19" s="6">
+        <v>90</v>
+      </c>
+      <c r="J19" s="6">
+        <v>7</v>
+      </c>
+      <c r="O19" s="6">
+        <v>3</v>
+      </c>
+      <c r="P19" s="4" t="s">
+        <v>663</v>
+      </c>
+      <c r="Q19" s="6">
+        <f>IF($B19="","",$B19&amp;"_W"&amp;$C19)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17">
+      <c r="A20" s="25">
+        <v>46212</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="C20" s="6">
+        <v>1</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>491</v>
+      </c>
+      <c r="E20" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D20,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F20" s="6" t="s">
+        <v>648</v>
+      </c>
+      <c r="G20" s="6">
+        <v>3</v>
+      </c>
+      <c r="H20" s="4" t="s">
+        <v>664</v>
+      </c>
+      <c r="I20" s="6">
+        <v>70</v>
+      </c>
+      <c r="J20" s="6">
+        <v>7</v>
+      </c>
+      <c r="O20" s="6">
+        <v>3</v>
+      </c>
+      <c r="Q20" s="6">
+        <f>IF($B20="","",$B20&amp;"_W"&amp;$C20)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:17">
+      <c r="A21" s="25">
+        <v>46212</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="C21" s="6">
+        <v>1</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>501</v>
+      </c>
+      <c r="E21" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D21,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F21" s="6" t="s">
+        <v>648</v>
+      </c>
+      <c r="G21" s="6">
+        <v>2</v>
+      </c>
+      <c r="H21" s="4" t="s">
+        <v>665</v>
+      </c>
+      <c r="I21" s="6">
+        <v>25</v>
+      </c>
+      <c r="J21" s="6">
+        <v>6</v>
+      </c>
+      <c r="O21" s="6">
+        <v>3</v>
+      </c>
+      <c r="P21" s="4" t="s">
+        <v>666</v>
+      </c>
+      <c r="Q21" s="6">
+        <f>IF($B21="","",$B21&amp;"_W"&amp;$C21)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:17">
+      <c r="A22" s="25">
+        <v>46212</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="C22" s="6">
+        <v>1</v>
+      </c>
+      <c r="D22" s="6" t="s">
+        <v>505</v>
+      </c>
+      <c r="E22" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D22,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F22" s="6" t="s">
+        <v>648</v>
+      </c>
+      <c r="G22" s="6">
+        <v>2</v>
+      </c>
+      <c r="H22" s="4" t="s">
+        <v>665</v>
+      </c>
+      <c r="I22" s="6">
+        <v>25</v>
+      </c>
+      <c r="J22" s="6">
+        <v>7</v>
+      </c>
+      <c r="O22" s="6">
+        <v>3</v>
+      </c>
+      <c r="Q22" s="6">
+        <f>IF($B22="","",$B22&amp;"_W"&amp;$C22)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:17">
+      <c r="A23" s="25">
+        <v>46212</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="C23" s="6">
+        <v>1</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>577</v>
+      </c>
+      <c r="E23" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D23,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F23" s="6" t="s">
+        <v>648</v>
+      </c>
+      <c r="G23" s="6">
+        <v>3</v>
+      </c>
+      <c r="H23" s="4" t="s">
+        <v>667</v>
+      </c>
+      <c r="J23" s="6">
+        <v>8</v>
+      </c>
+      <c r="M23" s="6">
+        <v>30</v>
+      </c>
+      <c r="O23" s="6">
+        <v>3</v>
+      </c>
+      <c r="P23" s="4" t="s">
+        <v>668</v>
+      </c>
+      <c r="Q23" s="6">
+        <f>IF($B23="","",$B23&amp;"_W"&amp;$C23)</f>
         <v>0</v>
       </c>
     </row>
@@ -9129,7 +9635,7 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>656</v>
+        <v>669</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -9140,20 +9646,20 @@
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="5" t="s">
-        <v>657</v>
+        <v>670</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="9" t="s">
-        <v>658</v>
+        <v>671</v>
       </c>
       <c r="B4" s="11">
         <v>81</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>666</v>
+        <v>679</v>
       </c>
       <c r="D4" s="4"/>
       <c r="E4" s="4"/>
@@ -9162,21 +9668,21 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="9" t="s">
-        <v>659</v>
+        <v>672</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>660</v>
+        <v>673</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="9" t="s">
-        <v>661</v>
+        <v>674</v>
       </c>
       <c r="B6" s="11">
         <v>2.2</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>667</v>
+        <v>680</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
@@ -9185,7 +9691,7 @@
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="9" t="s">
-        <v>662</v>
+        <v>675</v>
       </c>
       <c r="B7" s="11">
         <v>0.9</v>
@@ -9193,7 +9699,7 @@
     </row>
     <row r="8" spans="1:7">
       <c r="A8" s="9" t="s">
-        <v>663</v>
+        <v>676</v>
       </c>
       <c r="B8" s="10">
         <v>2700</v>
@@ -9201,7 +9707,7 @@
     </row>
     <row r="9" spans="1:7">
       <c r="A9" s="9" t="s">
-        <v>664</v>
+        <v>677</v>
       </c>
       <c r="B9" s="10">
         <f>ROUND(BW*B6,0)</f>
@@ -9210,7 +9716,7 @@
     </row>
     <row r="10" spans="1:7">
       <c r="A10" s="9" t="s">
-        <v>665</v>
+        <v>678</v>
       </c>
       <c r="B10" s="10">
         <f>ROUND(BW*B7,0)</f>
@@ -9219,7 +9725,7 @@
     </row>
     <row r="12" spans="1:7">
       <c r="A12" s="5" t="s">
-        <v>668</v>
+        <v>681</v>
       </c>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -9233,27 +9739,27 @@
         <v>85</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>669</v>
+        <v>682</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>670</v>
+        <v>683</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>671</v>
+        <v>684</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>672</v>
+        <v>685</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>673</v>
+        <v>686</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>674</v>
+        <v>687</v>
       </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" s="9" t="s">
-        <v>675</v>
+        <v>688</v>
       </c>
       <c r="B14" s="26">
         <v>250</v>
@@ -9275,7 +9781,7 @@
         <v>0</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>676</v>
+        <v>689</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -9302,12 +9808,12 @@
         <v>0</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>677</v>
+        <v>690</v>
       </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" s="9" t="s">
-        <v>678</v>
+        <v>691</v>
       </c>
       <c r="B16" s="26">
         <v>200</v>
@@ -9329,12 +9835,12 @@
         <v>0</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>679</v>
+        <v>692</v>
       </c>
     </row>
     <row r="17" spans="1:7">
       <c r="A17" s="9" t="s">
-        <v>680</v>
+        <v>693</v>
       </c>
       <c r="B17" s="26">
         <v>150</v>
@@ -9356,12 +9862,12 @@
         <v>0</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>681</v>
+        <v>694</v>
       </c>
     </row>
     <row r="18" spans="1:7">
       <c r="A18" s="9" t="s">
-        <v>682</v>
+        <v>695</v>
       </c>
       <c r="B18" s="26">
         <v>100</v>
@@ -9383,7 +9889,7 @@
         <v>0</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>683</v>
+        <v>696</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -9410,12 +9916,12 @@
         <v>0</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>684</v>
+        <v>697</v>
       </c>
     </row>
     <row r="21" spans="1:7">
       <c r="A21" s="5" t="s">
-        <v>685</v>
+        <v>698</v>
       </c>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
@@ -9426,7 +9932,7 @@
     </row>
     <row r="22" spans="1:7">
       <c r="A22" s="4" t="s">
-        <v>686</v>
+        <v>699</v>
       </c>
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
@@ -9437,7 +9943,7 @@
     </row>
     <row r="23" spans="1:7">
       <c r="A23" s="4" t="s">
-        <v>687</v>
+        <v>700</v>
       </c>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
@@ -9448,7 +9954,7 @@
     </row>
     <row r="24" spans="1:7">
       <c r="A24" s="4" t="s">
-        <v>688</v>
+        <v>701</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -9459,7 +9965,7 @@
     </row>
     <row r="25" spans="1:7">
       <c r="A25" s="4" t="s">
-        <v>689</v>
+        <v>702</v>
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -9504,7 +10010,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>690</v>
+        <v>703</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -9513,7 +10019,7 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="5" t="s">
-        <v>691</v>
+        <v>704</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
@@ -9522,126 +10028,126 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="7" t="s">
-        <v>692</v>
+        <v>705</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>693</v>
+        <v>706</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>694</v>
+        <v>707</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>695</v>
+        <v>708</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>696</v>
+        <v>709</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="9" t="s">
-        <v>697</v>
+        <v>710</v>
       </c>
       <c r="B5" s="22" t="s">
-        <v>698</v>
+        <v>711</v>
       </c>
       <c r="C5" s="27" t="s">
-        <v>699</v>
+        <v>712</v>
       </c>
       <c r="D5" s="28" t="s">
-        <v>700</v>
+        <v>713</v>
       </c>
       <c r="E5" s="29" t="s">
-        <v>701</v>
+        <v>714</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="9" t="s">
-        <v>702</v>
+        <v>715</v>
       </c>
       <c r="B6" s="22" t="s">
-        <v>703</v>
+        <v>716</v>
       </c>
       <c r="C6" s="27" t="s">
-        <v>704</v>
+        <v>717</v>
       </c>
       <c r="D6" s="28" t="s">
-        <v>705</v>
+        <v>718</v>
       </c>
       <c r="E6" s="29" t="s">
-        <v>706</v>
+        <v>719</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="9" t="s">
-        <v>707</v>
+        <v>720</v>
       </c>
       <c r="B7" s="22" t="s">
-        <v>708</v>
+        <v>721</v>
       </c>
       <c r="C7" s="27" t="s">
-        <v>709</v>
+        <v>722</v>
       </c>
       <c r="D7" s="28" t="s">
-        <v>710</v>
+        <v>723</v>
       </c>
       <c r="E7" s="29" t="s">
-        <v>711</v>
+        <v>724</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="9" t="s">
-        <v>712</v>
+        <v>725</v>
       </c>
       <c r="B8" s="22" t="s">
-        <v>713</v>
+        <v>726</v>
       </c>
       <c r="C8" s="27" t="s">
-        <v>714</v>
+        <v>727</v>
       </c>
       <c r="D8" s="28" t="s">
-        <v>715</v>
+        <v>728</v>
       </c>
       <c r="E8" s="29" t="s">
-        <v>716</v>
+        <v>729</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="9" t="s">
-        <v>717</v>
+        <v>730</v>
       </c>
       <c r="B9" s="22" t="s">
-        <v>718</v>
+        <v>731</v>
       </c>
       <c r="C9" s="27" t="s">
-        <v>719</v>
+        <v>732</v>
       </c>
       <c r="D9" s="28" t="s">
-        <v>720</v>
+        <v>733</v>
       </c>
       <c r="E9" s="29" t="s">
-        <v>721</v>
+        <v>734</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="9" t="s">
-        <v>722</v>
+        <v>735</v>
       </c>
       <c r="B10" s="22" t="s">
-        <v>723</v>
+        <v>736</v>
       </c>
       <c r="C10" s="27" t="s">
-        <v>724</v>
+        <v>737</v>
       </c>
       <c r="D10" s="28" t="s">
-        <v>725</v>
+        <v>738</v>
       </c>
       <c r="E10" s="29" t="s">
-        <v>726</v>
+        <v>739</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="5" t="s">
-        <v>727</v>
+        <v>740</v>
       </c>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -9704,7 +10210,7 @@
     </row>
     <row r="20" spans="1:5">
       <c r="A20" s="5" t="s">
-        <v>728</v>
+        <v>741</v>
       </c>
       <c r="B20" s="5"/>
       <c r="C20" s="5"/>
@@ -9713,36 +10219,36 @@
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="7" t="s">
-        <v>729</v>
+        <v>742</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>730</v>
+        <v>743</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>731</v>
+        <v>744</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>732</v>
+        <v>745</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>733</v>
+        <v>746</v>
       </c>
     </row>
     <row r="22" spans="1:5">
       <c r="A22" s="14" t="s">
-        <v>734</v>
+        <v>747</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>735</v>
+        <v>748</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>736</v>
+        <v>749</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>737</v>
+        <v>750</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>738</v>
+        <v>751</v>
       </c>
     </row>
     <row r="23" spans="1:5">
@@ -9750,16 +10256,16 @@
         <v>46</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>739</v>
+        <v>752</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>740</v>
+        <v>753</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>741</v>
+        <v>754</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>742</v>
+        <v>755</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -9767,16 +10273,16 @@
         <v>33</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>743</v>
+        <v>756</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>744</v>
+        <v>757</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>745</v>
+        <v>758</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>746</v>
+        <v>759</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -9784,21 +10290,21 @@
         <v>36</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>747</v>
+        <v>760</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>748</v>
+        <v>761</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>749</v>
+        <v>762</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>750</v>
+        <v>763</v>
       </c>
     </row>
     <row r="27" spans="1:5">
       <c r="A27" s="5" t="s">
-        <v>751</v>
+        <v>764</v>
       </c>
       <c r="B27" s="5"/>
       <c r="C27" s="5"/>
@@ -9807,7 +10313,7 @@
     </row>
     <row r="28" spans="1:5">
       <c r="A28" s="4" t="s">
-        <v>752</v>
+        <v>765</v>
       </c>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
@@ -9816,7 +10322,7 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" s="4" t="s">
-        <v>753</v>
+        <v>766</v>
       </c>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -9825,7 +10331,7 @@
     </row>
     <row r="30" spans="1:5">
       <c r="A30" s="4" t="s">
-        <v>754</v>
+        <v>767</v>
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -9834,7 +10340,7 @@
     </row>
     <row r="31" spans="1:5">
       <c r="A31" s="4" t="s">
-        <v>755</v>
+        <v>768</v>
       </c>
       <c r="B31" s="4"/>
       <c r="C31" s="4"/>
@@ -9843,7 +10349,7 @@
     </row>
     <row r="32" spans="1:5">
       <c r="A32" s="4" t="s">
-        <v>756</v>
+        <v>769</v>
       </c>
       <c r="B32" s="4"/>
       <c r="C32" s="4"/>
@@ -9867,98 +10373,98 @@
         <v>423</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>757</v>
+        <v>770</v>
       </c>
       <c r="D35" s="7"/>
       <c r="E35" s="7"/>
     </row>
     <row r="36" spans="1:5">
       <c r="A36" s="4" t="s">
-        <v>758</v>
+        <v>771</v>
       </c>
       <c r="B36" s="24" t="s">
-        <v>759</v>
+        <v>772</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>760</v>
+        <v>773</v>
       </c>
       <c r="D36" s="4"/>
       <c r="E36" s="4"/>
     </row>
     <row r="37" spans="1:5">
       <c r="A37" s="4" t="s">
-        <v>761</v>
+        <v>774</v>
       </c>
       <c r="B37" s="24" t="s">
-        <v>762</v>
+        <v>775</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>763</v>
+        <v>776</v>
       </c>
       <c r="D37" s="4"/>
       <c r="E37" s="4"/>
     </row>
     <row r="38" spans="1:5">
       <c r="A38" s="4" t="s">
-        <v>764</v>
+        <v>777</v>
       </c>
       <c r="B38" s="24" t="s">
         <v>431</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>765</v>
+        <v>778</v>
       </c>
       <c r="D38" s="4"/>
       <c r="E38" s="4"/>
     </row>
     <row r="39" spans="1:5">
       <c r="A39" s="4" t="s">
-        <v>766</v>
+        <v>779</v>
       </c>
       <c r="B39" s="24" t="s">
-        <v>767</v>
+        <v>780</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>768</v>
+        <v>781</v>
       </c>
       <c r="D39" s="4"/>
       <c r="E39" s="4"/>
     </row>
     <row r="40" spans="1:5">
       <c r="A40" s="4" t="s">
-        <v>766</v>
+        <v>779</v>
       </c>
       <c r="B40" s="24" t="s">
-        <v>769</v>
+        <v>782</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>770</v>
+        <v>783</v>
       </c>
       <c r="D40" s="4"/>
       <c r="E40" s="4"/>
     </row>
     <row r="41" spans="1:5">
       <c r="A41" s="4" t="s">
-        <v>771</v>
+        <v>784</v>
       </c>
       <c r="B41" s="24" t="s">
-        <v>772</v>
+        <v>785</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>773</v>
+        <v>786</v>
       </c>
       <c r="D41" s="4"/>
       <c r="E41" s="4"/>
     </row>
     <row r="42" spans="1:5">
       <c r="A42" s="4" t="s">
-        <v>774</v>
+        <v>787</v>
       </c>
       <c r="B42" s="24" t="s">
-        <v>775</v>
+        <v>788</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>776</v>
+        <v>789</v>
       </c>
       <c r="D42" s="4"/>
       <c r="E42" s="4"/>

</xml_diff>

<commit_message>
Log B7 W1 T3 (Recovery 4): legs + legs-together line/supported skill; note RPE creep on BSS/ham curl
</commit_message>
<xml_diff>
--- a/Training_3_B7.xlsx
+++ b/Training_3_B7.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1560" uniqueCount="854">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1594" uniqueCount="861">
   <si>
     <t>B7 — Performance-Block Dashboard (Advanced OAHS)</t>
   </si>
@@ -2037,6 +2037,27 @@
   </si>
   <si>
     <t>3x30s</t>
+  </si>
+  <si>
+    <t>20+s Line-Holds</t>
+  </si>
+  <si>
+    <t>Legs-together Weight-Shifts, 2/Seite (Line-Arbeit)</t>
+  </si>
+  <si>
+    <t>SUPPORTED (2 Finger), 8s - KEIN freier Hold</t>
+  </si>
+  <si>
+    <t>8,7,7</t>
+  </si>
+  <si>
+    <t>RPE eher 8 (ueber Cap 7)</t>
+  </si>
+  <si>
+    <t>12,10,10</t>
+  </si>
+  <si>
+    <t>RPE 8 (ueber Cap 7)</t>
   </si>
   <si>
     <t>B7 — Nutrition Targets (Maintenance, KEIN Defizit)</t>
@@ -3821,7 +3842,7 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>790</v>
+        <v>797</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3831,7 +3852,7 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="12" t="s">
-        <v>791</v>
+        <v>798</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -3856,12 +3877,12 @@
         <v>153</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>792</v>
+        <v>799</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="9" t="s">
-        <v>793</v>
+        <v>800</v>
       </c>
       <c r="B4" s="11">
         <f>SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Skill90",'B7_Training_Log'!$C$2:$C$1000,1)+SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Planche",'B7_Training_Log'!$C$2:$C$1000,1)+SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Push",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -3886,7 +3907,7 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="9" t="s">
-        <v>794</v>
+        <v>801</v>
       </c>
       <c r="B5" s="11">
         <f>SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Pull",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -3911,7 +3932,7 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="9" t="s">
-        <v>795</v>
+        <v>802</v>
       </c>
       <c r="B6" s="11">
         <f>SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Legs",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -3936,7 +3957,7 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="9" t="s">
-        <v>796</v>
+        <v>803</v>
       </c>
       <c r="B7" s="10">
         <f>SUMIFS('B7_Training_Log'!$N$2:$N$1000,'B7_Training_Log'!$D$2:$D$1000,"90",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -3961,7 +3982,7 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="9" t="s">
-        <v>797</v>
+        <v>804</v>
       </c>
       <c r="B8" s="10">
         <f>COUNTIFS('B7_Training_Log'!$E$2:$E$1000,"SkillOAHS",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -3986,7 +4007,7 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="9" t="s">
-        <v>798</v>
+        <v>805</v>
       </c>
       <c r="B9" s="10">
         <f>MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_straddle",'B7_Training_Log'!$F$2:$F$1000,"L",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4011,7 +4032,7 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="9" t="s">
-        <v>799</v>
+        <v>806</v>
       </c>
       <c r="B10" s="10">
         <f>MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_straddle",'B7_Training_Log'!$F$2:$F$1000,"R",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4036,7 +4057,7 @@
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="9" t="s">
-        <v>800</v>
+        <v>807</v>
       </c>
       <c r="B11" s="10">
         <f>MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_diamond",'B7_Training_Log'!$F$2:$F$1000,"L",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4061,7 +4082,7 @@
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="9" t="s">
-        <v>801</v>
+        <v>808</v>
       </c>
       <c r="B12" s="10">
         <f>MAX(MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_flag",'B7_Training_Log'!$C$2:$C$1000,1),MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_figa",'B7_Training_Log'!$C$2:$C$1000,1))</f>
@@ -4086,7 +4107,7 @@
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="9" t="s">
-        <v>802</v>
+        <v>809</v>
       </c>
       <c r="B13" s="11">
         <f>IFERROR(AVERAGEIFS('B7_Training_Log'!$J$2:$J$1000,'B7_Training_Log'!$C$2:$C$1000,1),0)</f>
@@ -4161,7 +4182,7 @@
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="9" t="s">
-        <v>803</v>
+        <v>810</v>
       </c>
       <c r="B16" s="10">
         <f>COUNTIFS('B7_Training_Log'!$K$2:$K$1000,"&gt;=4",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4186,7 +4207,7 @@
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="9" t="s">
-        <v>804</v>
+        <v>811</v>
       </c>
       <c r="B17" s="10">
         <f>COUNTIFS('B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4230,7 +4251,7 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
-        <v>805</v>
+        <v>812</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4238,7 +4259,7 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="5" t="s">
-        <v>806</v>
+        <v>813</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
@@ -4246,13 +4267,13 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="7" t="s">
-        <v>807</v>
+        <v>814</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>808</v>
+        <v>815</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>809</v>
+        <v>816</v>
       </c>
       <c r="D4" s="7"/>
     </row>
@@ -4261,10 +4282,10 @@
         <v>627</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>810</v>
+        <v>817</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>811</v>
+        <v>818</v>
       </c>
       <c r="D5" s="4"/>
     </row>
@@ -4273,10 +4294,10 @@
         <v>628</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>812</v>
+        <v>819</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>813</v>
+        <v>820</v>
       </c>
       <c r="D6" s="4"/>
     </row>
@@ -4285,10 +4306,10 @@
         <v>629</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>814</v>
+        <v>821</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>815</v>
+        <v>822</v>
       </c>
       <c r="D7" s="4"/>
     </row>
@@ -4297,10 +4318,10 @@
         <v>436</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>816</v>
+        <v>823</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>817</v>
+        <v>824</v>
       </c>
       <c r="D8" s="4"/>
     </row>
@@ -4309,10 +4330,10 @@
         <v>439</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>818</v>
+        <v>825</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>819</v>
+        <v>826</v>
       </c>
       <c r="D9" s="4"/>
     </row>
@@ -4321,10 +4342,10 @@
         <v>630</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>820</v>
+        <v>827</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>821</v>
+        <v>828</v>
       </c>
       <c r="D10" s="4"/>
     </row>
@@ -4333,10 +4354,10 @@
         <v>631</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>822</v>
+        <v>829</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>823</v>
+        <v>830</v>
       </c>
       <c r="D11" s="4"/>
     </row>
@@ -4345,10 +4366,10 @@
         <v>632</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>824</v>
+        <v>831</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>825</v>
+        <v>832</v>
       </c>
       <c r="D12" s="4"/>
     </row>
@@ -4357,10 +4378,10 @@
         <v>633</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>822</v>
+        <v>829</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>826</v>
+        <v>833</v>
       </c>
       <c r="D13" s="4"/>
     </row>
@@ -4369,10 +4390,10 @@
         <v>634</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>827</v>
+        <v>834</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>828</v>
+        <v>835</v>
       </c>
       <c r="D14" s="4"/>
     </row>
@@ -4381,10 +4402,10 @@
         <v>635</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>829</v>
+        <v>836</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>830</v>
+        <v>837</v>
       </c>
       <c r="D15" s="4"/>
     </row>
@@ -4393,10 +4414,10 @@
         <v>636</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>831</v>
+        <v>838</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>832</v>
+        <v>839</v>
       </c>
       <c r="D16" s="4"/>
     </row>
@@ -4405,10 +4426,10 @@
         <v>637</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>822</v>
+        <v>829</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>833</v>
+        <v>840</v>
       </c>
       <c r="D17" s="4"/>
     </row>
@@ -4417,10 +4438,10 @@
         <v>638</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>822</v>
+        <v>829</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>834</v>
+        <v>841</v>
       </c>
       <c r="D18" s="4"/>
     </row>
@@ -4429,10 +4450,10 @@
         <v>639</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>835</v>
+        <v>842</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>836</v>
+        <v>843</v>
       </c>
       <c r="D19" s="4"/>
     </row>
@@ -4441,10 +4462,10 @@
         <v>92</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>824</v>
+        <v>831</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>837</v>
+        <v>844</v>
       </c>
       <c r="D20" s="4"/>
     </row>
@@ -4453,16 +4474,16 @@
         <v>640</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>838</v>
+        <v>845</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>839</v>
+        <v>846</v>
       </c>
       <c r="D21" s="4"/>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="5" t="s">
-        <v>840</v>
+        <v>847</v>
       </c>
       <c r="B23" s="5"/>
       <c r="C23" s="5"/>
@@ -4470,7 +4491,7 @@
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="4" t="s">
-        <v>841</v>
+        <v>848</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -4478,7 +4499,7 @@
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="4" t="s">
-        <v>842</v>
+        <v>849</v>
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -4486,7 +4507,7 @@
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="4" t="s">
-        <v>843</v>
+        <v>850</v>
       </c>
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
@@ -4494,7 +4515,7 @@
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="4" t="s">
-        <v>844</v>
+        <v>851</v>
       </c>
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
@@ -4502,7 +4523,7 @@
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="4" t="s">
-        <v>845</v>
+        <v>852</v>
       </c>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
@@ -4510,7 +4531,7 @@
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="4" t="s">
-        <v>846</v>
+        <v>853</v>
       </c>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -4518,7 +4539,7 @@
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="4" t="s">
-        <v>847</v>
+        <v>854</v>
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -4526,7 +4547,7 @@
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="5" t="s">
-        <v>848</v>
+        <v>855</v>
       </c>
       <c r="B32" s="5"/>
       <c r="C32" s="5"/>
@@ -4534,7 +4555,7 @@
     </row>
     <row r="33" spans="1:4">
       <c r="A33" s="4" t="s">
-        <v>849</v>
+        <v>856</v>
       </c>
       <c r="B33" s="4"/>
       <c r="C33" s="4"/>
@@ -4542,7 +4563,7 @@
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="4" t="s">
-        <v>850</v>
+        <v>857</v>
       </c>
       <c r="B34" s="4"/>
       <c r="C34" s="4"/>
@@ -4550,7 +4571,7 @@
     </row>
     <row r="35" spans="1:4">
       <c r="A35" s="4" t="s">
-        <v>851</v>
+        <v>858</v>
       </c>
       <c r="B35" s="4"/>
       <c r="C35" s="4"/>
@@ -4558,7 +4579,7 @@
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="4" t="s">
-        <v>852</v>
+        <v>859</v>
       </c>
       <c r="B36" s="4"/>
       <c r="C36" s="4"/>
@@ -4566,7 +4587,7 @@
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="4" t="s">
-        <v>853</v>
+        <v>860</v>
       </c>
       <c r="B37" s="4"/>
       <c r="C37" s="4"/>
@@ -8548,7 +8569,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q23"/>
+  <dimension ref="A1:Q31"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -9558,6 +9579,338 @@
       </c>
       <c r="Q23" s="6">
         <f>IF($B23="","",$B23&amp;"_W"&amp;$C23)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:17">
+      <c r="A24" s="25">
+        <v>46214</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="C24" s="6">
+        <v>1</v>
+      </c>
+      <c r="D24" s="6" t="s">
+        <v>459</v>
+      </c>
+      <c r="E24" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D24,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F24" s="6" t="s">
+        <v>648</v>
+      </c>
+      <c r="G24" s="6">
+        <v>3</v>
+      </c>
+      <c r="I24" s="6">
+        <v>0</v>
+      </c>
+      <c r="L24" s="6">
+        <v>4</v>
+      </c>
+      <c r="M24" s="6">
+        <v>20</v>
+      </c>
+      <c r="O24" s="6">
+        <v>4</v>
+      </c>
+      <c r="P24" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="Q24" s="6">
+        <f>IF($B24="","",$B24&amp;"_W"&amp;$C24)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:17">
+      <c r="A25" s="25">
+        <v>46214</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="C25" s="6">
+        <v>1</v>
+      </c>
+      <c r="D25" s="6" t="s">
+        <v>608</v>
+      </c>
+      <c r="E25" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D25,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F25" s="6" t="s">
+        <v>648</v>
+      </c>
+      <c r="G25" s="6">
+        <v>2</v>
+      </c>
+      <c r="I25" s="6">
+        <v>0</v>
+      </c>
+      <c r="O25" s="6">
+        <v>4</v>
+      </c>
+      <c r="P25" s="4" t="s">
+        <v>670</v>
+      </c>
+      <c r="Q25" s="6">
+        <f>IF($B25="","",$B25&amp;"_W"&amp;$C25)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:17">
+      <c r="A26" s="25">
+        <v>46214</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="C26" s="6">
+        <v>1</v>
+      </c>
+      <c r="D26" s="6" t="s">
+        <v>608</v>
+      </c>
+      <c r="E26" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D26,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F26" s="6" t="s">
+        <v>641</v>
+      </c>
+      <c r="G26" s="6">
+        <v>3</v>
+      </c>
+      <c r="I26" s="6">
+        <v>0</v>
+      </c>
+      <c r="L26" s="6">
+        <v>3</v>
+      </c>
+      <c r="M26" s="6">
+        <v>8</v>
+      </c>
+      <c r="O26" s="6">
+        <v>4</v>
+      </c>
+      <c r="P26" s="4" t="s">
+        <v>671</v>
+      </c>
+      <c r="Q26" s="6">
+        <f>IF($B26="","",$B26&amp;"_W"&amp;$C26)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:17">
+      <c r="A27" s="25">
+        <v>46214</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="C27" s="6">
+        <v>1</v>
+      </c>
+      <c r="D27" s="6" t="s">
+        <v>608</v>
+      </c>
+      <c r="E27" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D27,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F27" s="6" t="s">
+        <v>643</v>
+      </c>
+      <c r="G27" s="6">
+        <v>3</v>
+      </c>
+      <c r="I27" s="6">
+        <v>0</v>
+      </c>
+      <c r="L27" s="6">
+        <v>3</v>
+      </c>
+      <c r="M27" s="6">
+        <v>8</v>
+      </c>
+      <c r="O27" s="6">
+        <v>4</v>
+      </c>
+      <c r="P27" s="4" t="s">
+        <v>671</v>
+      </c>
+      <c r="Q27" s="6">
+        <f>IF($B27="","",$B27&amp;"_W"&amp;$C27)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:17">
+      <c r="A28" s="25">
+        <v>46214</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="C28" s="6">
+        <v>1</v>
+      </c>
+      <c r="D28" s="6" t="s">
+        <v>544</v>
+      </c>
+      <c r="E28" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D28,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F28" s="6" t="s">
+        <v>648</v>
+      </c>
+      <c r="G28" s="6">
+        <v>3</v>
+      </c>
+      <c r="H28" s="4" t="s">
+        <v>672</v>
+      </c>
+      <c r="I28" s="6">
+        <v>40</v>
+      </c>
+      <c r="J28" s="6">
+        <v>8</v>
+      </c>
+      <c r="O28" s="6">
+        <v>4</v>
+      </c>
+      <c r="P28" s="4" t="s">
+        <v>673</v>
+      </c>
+      <c r="Q28" s="6">
+        <f>IF($B28="","",$B28&amp;"_W"&amp;$C28)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:17">
+      <c r="A29" s="25">
+        <v>46214</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="C29" s="6">
+        <v>1</v>
+      </c>
+      <c r="D29" s="6" t="s">
+        <v>547</v>
+      </c>
+      <c r="E29" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D29,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F29" s="6" t="s">
+        <v>648</v>
+      </c>
+      <c r="G29" s="6">
+        <v>3</v>
+      </c>
+      <c r="H29" s="4" t="s">
+        <v>653</v>
+      </c>
+      <c r="I29" s="6">
+        <v>70</v>
+      </c>
+      <c r="J29" s="6">
+        <v>7</v>
+      </c>
+      <c r="O29" s="6">
+        <v>4</v>
+      </c>
+      <c r="Q29" s="6">
+        <f>IF($B29="","",$B29&amp;"_W"&amp;$C29)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:17">
+      <c r="A30" s="25">
+        <v>46214</v>
+      </c>
+      <c r="B30" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="C30" s="6">
+        <v>1</v>
+      </c>
+      <c r="D30" s="6" t="s">
+        <v>550</v>
+      </c>
+      <c r="E30" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D30,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F30" s="6" t="s">
+        <v>648</v>
+      </c>
+      <c r="G30" s="6">
+        <v>3</v>
+      </c>
+      <c r="H30" s="4" t="s">
+        <v>674</v>
+      </c>
+      <c r="I30" s="6">
+        <v>50</v>
+      </c>
+      <c r="J30" s="6">
+        <v>8</v>
+      </c>
+      <c r="O30" s="6">
+        <v>4</v>
+      </c>
+      <c r="P30" s="4" t="s">
+        <v>675</v>
+      </c>
+      <c r="Q30" s="6">
+        <f>IF($B30="","",$B30&amp;"_W"&amp;$C30)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:17">
+      <c r="A31" s="25">
+        <v>46214</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="C31" s="6">
+        <v>1</v>
+      </c>
+      <c r="D31" s="6" t="s">
+        <v>560</v>
+      </c>
+      <c r="E31" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D31,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F31" s="6" t="s">
+        <v>648</v>
+      </c>
+      <c r="G31" s="6">
+        <v>3</v>
+      </c>
+      <c r="H31" s="4" t="s">
+        <v>665</v>
+      </c>
+      <c r="I31" s="6">
+        <v>70</v>
+      </c>
+      <c r="J31" s="6">
+        <v>7</v>
+      </c>
+      <c r="O31" s="6">
+        <v>4</v>
+      </c>
+      <c r="Q31" s="6">
+        <f>IF($B31="","",$B31&amp;"_W"&amp;$C31)</f>
         <v>0</v>
       </c>
     </row>
@@ -9635,7 +9988,7 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>669</v>
+        <v>676</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -9646,20 +9999,20 @@
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="5" t="s">
-        <v>670</v>
+        <v>677</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="9" t="s">
-        <v>671</v>
+        <v>678</v>
       </c>
       <c r="B4" s="11">
         <v>81</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>679</v>
+        <v>686</v>
       </c>
       <c r="D4" s="4"/>
       <c r="E4" s="4"/>
@@ -9668,21 +10021,21 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="9" t="s">
-        <v>672</v>
+        <v>679</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>673</v>
+        <v>680</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="9" t="s">
-        <v>674</v>
+        <v>681</v>
       </c>
       <c r="B6" s="11">
         <v>2.2</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>680</v>
+        <v>687</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
@@ -9691,7 +10044,7 @@
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="9" t="s">
-        <v>675</v>
+        <v>682</v>
       </c>
       <c r="B7" s="11">
         <v>0.9</v>
@@ -9699,7 +10052,7 @@
     </row>
     <row r="8" spans="1:7">
       <c r="A8" s="9" t="s">
-        <v>676</v>
+        <v>683</v>
       </c>
       <c r="B8" s="10">
         <v>2700</v>
@@ -9707,7 +10060,7 @@
     </row>
     <row r="9" spans="1:7">
       <c r="A9" s="9" t="s">
-        <v>677</v>
+        <v>684</v>
       </c>
       <c r="B9" s="10">
         <f>ROUND(BW*B6,0)</f>
@@ -9716,7 +10069,7 @@
     </row>
     <row r="10" spans="1:7">
       <c r="A10" s="9" t="s">
-        <v>678</v>
+        <v>685</v>
       </c>
       <c r="B10" s="10">
         <f>ROUND(BW*B7,0)</f>
@@ -9725,7 +10078,7 @@
     </row>
     <row r="12" spans="1:7">
       <c r="A12" s="5" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -9739,27 +10092,27 @@
         <v>85</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>682</v>
+        <v>689</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>683</v>
+        <v>690</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>684</v>
+        <v>691</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>685</v>
+        <v>692</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>686</v>
+        <v>693</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" s="9" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
       <c r="B14" s="26">
         <v>250</v>
@@ -9781,7 +10134,7 @@
         <v>0</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>689</v>
+        <v>696</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -9808,12 +10161,12 @@
         <v>0</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>690</v>
+        <v>697</v>
       </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" s="9" t="s">
-        <v>691</v>
+        <v>698</v>
       </c>
       <c r="B16" s="26">
         <v>200</v>
@@ -9835,12 +10188,12 @@
         <v>0</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>692</v>
+        <v>699</v>
       </c>
     </row>
     <row r="17" spans="1:7">
       <c r="A17" s="9" t="s">
-        <v>693</v>
+        <v>700</v>
       </c>
       <c r="B17" s="26">
         <v>150</v>
@@ -9862,12 +10215,12 @@
         <v>0</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>694</v>
+        <v>701</v>
       </c>
     </row>
     <row r="18" spans="1:7">
       <c r="A18" s="9" t="s">
-        <v>695</v>
+        <v>702</v>
       </c>
       <c r="B18" s="26">
         <v>100</v>
@@ -9889,7 +10242,7 @@
         <v>0</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>696</v>
+        <v>703</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -9916,12 +10269,12 @@
         <v>0</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>697</v>
+        <v>704</v>
       </c>
     </row>
     <row r="21" spans="1:7">
       <c r="A21" s="5" t="s">
-        <v>698</v>
+        <v>705</v>
       </c>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
@@ -9932,7 +10285,7 @@
     </row>
     <row r="22" spans="1:7">
       <c r="A22" s="4" t="s">
-        <v>699</v>
+        <v>706</v>
       </c>
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
@@ -9943,7 +10296,7 @@
     </row>
     <row r="23" spans="1:7">
       <c r="A23" s="4" t="s">
-        <v>700</v>
+        <v>707</v>
       </c>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
@@ -9954,7 +10307,7 @@
     </row>
     <row r="24" spans="1:7">
       <c r="A24" s="4" t="s">
-        <v>701</v>
+        <v>708</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -9965,7 +10318,7 @@
     </row>
     <row r="25" spans="1:7">
       <c r="A25" s="4" t="s">
-        <v>702</v>
+        <v>709</v>
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -10010,7 +10363,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>703</v>
+        <v>710</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -10019,7 +10372,7 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="5" t="s">
-        <v>704</v>
+        <v>711</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
@@ -10028,126 +10381,126 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="7" t="s">
-        <v>705</v>
+        <v>712</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>706</v>
+        <v>713</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>707</v>
+        <v>714</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>708</v>
+        <v>715</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>709</v>
+        <v>716</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="9" t="s">
-        <v>710</v>
+        <v>717</v>
       </c>
       <c r="B5" s="22" t="s">
-        <v>711</v>
+        <v>718</v>
       </c>
       <c r="C5" s="27" t="s">
-        <v>712</v>
+        <v>719</v>
       </c>
       <c r="D5" s="28" t="s">
-        <v>713</v>
+        <v>720</v>
       </c>
       <c r="E5" s="29" t="s">
-        <v>714</v>
+        <v>721</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="9" t="s">
-        <v>715</v>
+        <v>722</v>
       </c>
       <c r="B6" s="22" t="s">
-        <v>716</v>
+        <v>723</v>
       </c>
       <c r="C6" s="27" t="s">
-        <v>717</v>
+        <v>724</v>
       </c>
       <c r="D6" s="28" t="s">
-        <v>718</v>
+        <v>725</v>
       </c>
       <c r="E6" s="29" t="s">
-        <v>719</v>
+        <v>726</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="9" t="s">
-        <v>720</v>
+        <v>727</v>
       </c>
       <c r="B7" s="22" t="s">
-        <v>721</v>
+        <v>728</v>
       </c>
       <c r="C7" s="27" t="s">
-        <v>722</v>
+        <v>729</v>
       </c>
       <c r="D7" s="28" t="s">
-        <v>723</v>
+        <v>730</v>
       </c>
       <c r="E7" s="29" t="s">
-        <v>724</v>
+        <v>731</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="9" t="s">
-        <v>725</v>
+        <v>732</v>
       </c>
       <c r="B8" s="22" t="s">
-        <v>726</v>
+        <v>733</v>
       </c>
       <c r="C8" s="27" t="s">
-        <v>727</v>
+        <v>734</v>
       </c>
       <c r="D8" s="28" t="s">
-        <v>728</v>
+        <v>735</v>
       </c>
       <c r="E8" s="29" t="s">
-        <v>729</v>
+        <v>736</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="9" t="s">
-        <v>730</v>
+        <v>737</v>
       </c>
       <c r="B9" s="22" t="s">
-        <v>731</v>
+        <v>738</v>
       </c>
       <c r="C9" s="27" t="s">
-        <v>732</v>
+        <v>739</v>
       </c>
       <c r="D9" s="28" t="s">
-        <v>733</v>
+        <v>740</v>
       </c>
       <c r="E9" s="29" t="s">
-        <v>734</v>
+        <v>741</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="9" t="s">
-        <v>735</v>
+        <v>742</v>
       </c>
       <c r="B10" s="22" t="s">
-        <v>736</v>
+        <v>743</v>
       </c>
       <c r="C10" s="27" t="s">
-        <v>737</v>
+        <v>744</v>
       </c>
       <c r="D10" s="28" t="s">
-        <v>738</v>
+        <v>745</v>
       </c>
       <c r="E10" s="29" t="s">
-        <v>739</v>
+        <v>746</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="5" t="s">
-        <v>740</v>
+        <v>747</v>
       </c>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -10210,7 +10563,7 @@
     </row>
     <row r="20" spans="1:5">
       <c r="A20" s="5" t="s">
-        <v>741</v>
+        <v>748</v>
       </c>
       <c r="B20" s="5"/>
       <c r="C20" s="5"/>
@@ -10219,36 +10572,36 @@
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="7" t="s">
-        <v>742</v>
+        <v>749</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>743</v>
+        <v>750</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>744</v>
+        <v>751</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>745</v>
+        <v>752</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>746</v>
+        <v>753</v>
       </c>
     </row>
     <row r="22" spans="1:5">
       <c r="A22" s="14" t="s">
-        <v>747</v>
+        <v>754</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>748</v>
+        <v>755</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>749</v>
+        <v>756</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>750</v>
+        <v>757</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>751</v>
+        <v>758</v>
       </c>
     </row>
     <row r="23" spans="1:5">
@@ -10256,16 +10609,16 @@
         <v>46</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>752</v>
+        <v>759</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>753</v>
+        <v>760</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>754</v>
+        <v>761</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>755</v>
+        <v>762</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -10273,16 +10626,16 @@
         <v>33</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>756</v>
+        <v>763</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>757</v>
+        <v>764</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>758</v>
+        <v>765</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>759</v>
+        <v>766</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -10290,21 +10643,21 @@
         <v>36</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>760</v>
+        <v>767</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>761</v>
+        <v>768</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>762</v>
+        <v>769</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>763</v>
+        <v>770</v>
       </c>
     </row>
     <row r="27" spans="1:5">
       <c r="A27" s="5" t="s">
-        <v>764</v>
+        <v>771</v>
       </c>
       <c r="B27" s="5"/>
       <c r="C27" s="5"/>
@@ -10313,7 +10666,7 @@
     </row>
     <row r="28" spans="1:5">
       <c r="A28" s="4" t="s">
-        <v>765</v>
+        <v>772</v>
       </c>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
@@ -10322,7 +10675,7 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" s="4" t="s">
-        <v>766</v>
+        <v>773</v>
       </c>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -10331,7 +10684,7 @@
     </row>
     <row r="30" spans="1:5">
       <c r="A30" s="4" t="s">
-        <v>767</v>
+        <v>774</v>
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -10340,7 +10693,7 @@
     </row>
     <row r="31" spans="1:5">
       <c r="A31" s="4" t="s">
-        <v>768</v>
+        <v>775</v>
       </c>
       <c r="B31" s="4"/>
       <c r="C31" s="4"/>
@@ -10349,7 +10702,7 @@
     </row>
     <row r="32" spans="1:5">
       <c r="A32" s="4" t="s">
-        <v>769</v>
+        <v>776</v>
       </c>
       <c r="B32" s="4"/>
       <c r="C32" s="4"/>
@@ -10373,98 +10726,98 @@
         <v>423</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>770</v>
+        <v>777</v>
       </c>
       <c r="D35" s="7"/>
       <c r="E35" s="7"/>
     </row>
     <row r="36" spans="1:5">
       <c r="A36" s="4" t="s">
-        <v>771</v>
+        <v>778</v>
       </c>
       <c r="B36" s="24" t="s">
-        <v>772</v>
+        <v>779</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>773</v>
+        <v>780</v>
       </c>
       <c r="D36" s="4"/>
       <c r="E36" s="4"/>
     </row>
     <row r="37" spans="1:5">
       <c r="A37" s="4" t="s">
-        <v>774</v>
+        <v>781</v>
       </c>
       <c r="B37" s="24" t="s">
-        <v>775</v>
+        <v>782</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>776</v>
+        <v>783</v>
       </c>
       <c r="D37" s="4"/>
       <c r="E37" s="4"/>
     </row>
     <row r="38" spans="1:5">
       <c r="A38" s="4" t="s">
-        <v>777</v>
+        <v>784</v>
       </c>
       <c r="B38" s="24" t="s">
         <v>431</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>778</v>
+        <v>785</v>
       </c>
       <c r="D38" s="4"/>
       <c r="E38" s="4"/>
     </row>
     <row r="39" spans="1:5">
       <c r="A39" s="4" t="s">
-        <v>779</v>
+        <v>786</v>
       </c>
       <c r="B39" s="24" t="s">
-        <v>780</v>
+        <v>787</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>781</v>
+        <v>788</v>
       </c>
       <c r="D39" s="4"/>
       <c r="E39" s="4"/>
     </row>
     <row r="40" spans="1:5">
       <c r="A40" s="4" t="s">
-        <v>779</v>
+        <v>786</v>
       </c>
       <c r="B40" s="24" t="s">
-        <v>782</v>
+        <v>789</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>783</v>
+        <v>790</v>
       </c>
       <c r="D40" s="4"/>
       <c r="E40" s="4"/>
     </row>
     <row r="41" spans="1:5">
       <c r="A41" s="4" t="s">
-        <v>784</v>
+        <v>791</v>
       </c>
       <c r="B41" s="24" t="s">
-        <v>785</v>
+        <v>792</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>786</v>
+        <v>793</v>
       </c>
       <c r="D41" s="4"/>
       <c r="E41" s="4"/>
     </row>
     <row r="42" spans="1:5">
       <c r="A42" s="4" t="s">
-        <v>787</v>
+        <v>794</v>
       </c>
       <c r="B42" s="24" t="s">
-        <v>788</v>
+        <v>795</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>789</v>
+        <v>796</v>
       </c>
       <c r="D42" s="4"/>
       <c r="E42" s="4"/>

</xml_diff>

<commit_message>
Log B7 W1: Rest instead of T4 (symptoms: hay fever, headache, circulation, twitching)
</commit_message>
<xml_diff>
--- a/Training_3_B7.xlsx
+++ b/Training_3_B7.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1612" uniqueCount="870">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1616" uniqueCount="871">
   <si>
     <t>B7 — Performance-Block Dashboard (Advanced OAHS)</t>
   </si>
@@ -2085,6 +2085,9 @@
   </si>
   <si>
     <t>RPE 8 (ueber Cap 7)</t>
+  </si>
+  <si>
+    <t>Symptome: Heuschnupfen, Kopfschmerz (unueblich), Kreislauf/zittrig, Muskelzuckungen, Stress -&gt; Rest statt T4</t>
   </si>
   <si>
     <t>B7 — Nutrition Targets (Maintenance, KEIN Defizit)</t>
@@ -3895,7 +3898,7 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>806</v>
+        <v>807</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3905,7 +3908,7 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="12" t="s">
-        <v>807</v>
+        <v>808</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -3930,12 +3933,12 @@
         <v>155</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>808</v>
+        <v>809</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="9" t="s">
-        <v>809</v>
+        <v>810</v>
       </c>
       <c r="B4" s="11">
         <f>SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Skill90",'B7_Training_Log'!$C$2:$C$1000,1)+SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Planche",'B7_Training_Log'!$C$2:$C$1000,1)+SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Push",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -3960,7 +3963,7 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="9" t="s">
-        <v>810</v>
+        <v>811</v>
       </c>
       <c r="B5" s="11">
         <f>SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Pull",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -3985,7 +3988,7 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="9" t="s">
-        <v>811</v>
+        <v>812</v>
       </c>
       <c r="B6" s="11">
         <f>SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Legs",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4010,7 +4013,7 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="9" t="s">
-        <v>812</v>
+        <v>813</v>
       </c>
       <c r="B7" s="10">
         <f>SUMIFS('B7_Training_Log'!$N$2:$N$1000,'B7_Training_Log'!$D$2:$D$1000,"90",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4035,7 +4038,7 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="9" t="s">
-        <v>813</v>
+        <v>814</v>
       </c>
       <c r="B8" s="10">
         <f>COUNTIFS('B7_Training_Log'!$E$2:$E$1000,"SkillOAHS",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4060,7 +4063,7 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="9" t="s">
-        <v>814</v>
+        <v>815</v>
       </c>
       <c r="B9" s="10">
         <f>MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_straddle",'B7_Training_Log'!$F$2:$F$1000,"L",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4085,7 +4088,7 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="9" t="s">
-        <v>815</v>
+        <v>816</v>
       </c>
       <c r="B10" s="10">
         <f>MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_straddle",'B7_Training_Log'!$F$2:$F$1000,"R",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4110,7 +4113,7 @@
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="9" t="s">
-        <v>816</v>
+        <v>817</v>
       </c>
       <c r="B11" s="10">
         <f>MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_diamond",'B7_Training_Log'!$F$2:$F$1000,"L",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4135,7 +4138,7 @@
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="9" t="s">
-        <v>817</v>
+        <v>818</v>
       </c>
       <c r="B12" s="10">
         <f>MAX(MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_flag",'B7_Training_Log'!$C$2:$C$1000,1),MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_figa",'B7_Training_Log'!$C$2:$C$1000,1))</f>
@@ -4160,7 +4163,7 @@
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="9" t="s">
-        <v>818</v>
+        <v>819</v>
       </c>
       <c r="B13" s="11">
         <f>IFERROR(AVERAGEIFS('B7_Training_Log'!$J$2:$J$1000,'B7_Training_Log'!$C$2:$C$1000,1),0)</f>
@@ -4235,7 +4238,7 @@
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="9" t="s">
-        <v>819</v>
+        <v>820</v>
       </c>
       <c r="B16" s="10">
         <f>COUNTIFS('B7_Training_Log'!$K$2:$K$1000,"&gt;=4",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4260,7 +4263,7 @@
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="9" t="s">
-        <v>820</v>
+        <v>821</v>
       </c>
       <c r="B17" s="10">
         <f>COUNTIFS('B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4304,7 +4307,7 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
-        <v>821</v>
+        <v>822</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4312,7 +4315,7 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="5" t="s">
-        <v>822</v>
+        <v>823</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
@@ -4320,13 +4323,13 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="7" t="s">
-        <v>823</v>
+        <v>824</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>824</v>
+        <v>825</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>825</v>
+        <v>826</v>
       </c>
       <c r="D4" s="7"/>
     </row>
@@ -4335,10 +4338,10 @@
         <v>636</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>826</v>
+        <v>827</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>827</v>
+        <v>828</v>
       </c>
       <c r="D5" s="4"/>
     </row>
@@ -4347,10 +4350,10 @@
         <v>637</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>828</v>
+        <v>829</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>829</v>
+        <v>830</v>
       </c>
       <c r="D6" s="4"/>
     </row>
@@ -4359,10 +4362,10 @@
         <v>638</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>830</v>
+        <v>831</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>831</v>
+        <v>832</v>
       </c>
       <c r="D7" s="4"/>
     </row>
@@ -4371,10 +4374,10 @@
         <v>445</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>832</v>
+        <v>833</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>833</v>
+        <v>834</v>
       </c>
       <c r="D8" s="4"/>
     </row>
@@ -4383,10 +4386,10 @@
         <v>448</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>834</v>
+        <v>835</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>835</v>
+        <v>836</v>
       </c>
       <c r="D9" s="4"/>
     </row>
@@ -4395,10 +4398,10 @@
         <v>639</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>836</v>
+        <v>837</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>837</v>
+        <v>838</v>
       </c>
       <c r="D10" s="4"/>
     </row>
@@ -4407,10 +4410,10 @@
         <v>640</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>838</v>
+        <v>839</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>839</v>
+        <v>840</v>
       </c>
       <c r="D11" s="4"/>
     </row>
@@ -4419,10 +4422,10 @@
         <v>641</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>840</v>
+        <v>841</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>841</v>
+        <v>842</v>
       </c>
       <c r="D12" s="4"/>
     </row>
@@ -4431,10 +4434,10 @@
         <v>642</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>838</v>
+        <v>839</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>842</v>
+        <v>843</v>
       </c>
       <c r="D13" s="4"/>
     </row>
@@ -4443,10 +4446,10 @@
         <v>643</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>843</v>
+        <v>844</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>844</v>
+        <v>845</v>
       </c>
       <c r="D14" s="4"/>
     </row>
@@ -4455,10 +4458,10 @@
         <v>644</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>845</v>
+        <v>846</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>846</v>
+        <v>847</v>
       </c>
       <c r="D15" s="4"/>
     </row>
@@ -4467,10 +4470,10 @@
         <v>645</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>847</v>
+        <v>848</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>848</v>
+        <v>849</v>
       </c>
       <c r="D16" s="4"/>
     </row>
@@ -4479,10 +4482,10 @@
         <v>646</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>838</v>
+        <v>839</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>849</v>
+        <v>850</v>
       </c>
       <c r="D17" s="4"/>
     </row>
@@ -4491,10 +4494,10 @@
         <v>647</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>838</v>
+        <v>839</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>850</v>
+        <v>851</v>
       </c>
       <c r="D18" s="4"/>
     </row>
@@ -4503,10 +4506,10 @@
         <v>648</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>851</v>
+        <v>852</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>852</v>
+        <v>853</v>
       </c>
       <c r="D19" s="4"/>
     </row>
@@ -4515,10 +4518,10 @@
         <v>94</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>840</v>
+        <v>841</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>853</v>
+        <v>854</v>
       </c>
       <c r="D20" s="4"/>
     </row>
@@ -4527,16 +4530,16 @@
         <v>649</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>854</v>
+        <v>855</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>855</v>
+        <v>856</v>
       </c>
       <c r="D21" s="4"/>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="5" t="s">
-        <v>856</v>
+        <v>857</v>
       </c>
       <c r="B23" s="5"/>
       <c r="C23" s="5"/>
@@ -4544,7 +4547,7 @@
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="4" t="s">
-        <v>857</v>
+        <v>858</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -4552,7 +4555,7 @@
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="4" t="s">
-        <v>858</v>
+        <v>859</v>
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -4560,7 +4563,7 @@
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="4" t="s">
-        <v>859</v>
+        <v>860</v>
       </c>
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
@@ -4568,7 +4571,7 @@
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="4" t="s">
-        <v>860</v>
+        <v>861</v>
       </c>
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
@@ -4576,7 +4579,7 @@
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="4" t="s">
-        <v>861</v>
+        <v>862</v>
       </c>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
@@ -4584,7 +4587,7 @@
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="4" t="s">
-        <v>862</v>
+        <v>863</v>
       </c>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -4592,7 +4595,7 @@
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="4" t="s">
-        <v>863</v>
+        <v>864</v>
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -4600,7 +4603,7 @@
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="5" t="s">
-        <v>864</v>
+        <v>865</v>
       </c>
       <c r="B32" s="5"/>
       <c r="C32" s="5"/>
@@ -4608,7 +4611,7 @@
     </row>
     <row r="33" spans="1:4">
       <c r="A33" s="4" t="s">
-        <v>865</v>
+        <v>866</v>
       </c>
       <c r="B33" s="4"/>
       <c r="C33" s="4"/>
@@ -4616,7 +4619,7 @@
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="4" t="s">
-        <v>866</v>
+        <v>867</v>
       </c>
       <c r="B34" s="4"/>
       <c r="C34" s="4"/>
@@ -4624,7 +4627,7 @@
     </row>
     <row r="35" spans="1:4">
       <c r="A35" s="4" t="s">
-        <v>867</v>
+        <v>868</v>
       </c>
       <c r="B35" s="4"/>
       <c r="C35" s="4"/>
@@ -4632,7 +4635,7 @@
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="4" t="s">
-        <v>868</v>
+        <v>869</v>
       </c>
       <c r="B36" s="4"/>
       <c r="C36" s="4"/>
@@ -4640,7 +4643,7 @@
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="4" t="s">
-        <v>869</v>
+        <v>870</v>
       </c>
       <c r="B37" s="4"/>
       <c r="C37" s="4"/>
@@ -8670,7 +8673,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q31"/>
+  <dimension ref="A1:Q32"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -10012,6 +10015,37 @@
       </c>
       <c r="Q31" s="6">
         <f>IF($B31="","",$B31&amp;"_W"&amp;$C31)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:17">
+      <c r="A32" s="25">
+        <v>46215</v>
+      </c>
+      <c r="B32" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="C32" s="6">
+        <v>1</v>
+      </c>
+      <c r="D32" s="6" t="s">
+        <v>602</v>
+      </c>
+      <c r="E32" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D32,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F32" s="6" t="s">
+        <v>657</v>
+      </c>
+      <c r="O32" s="6">
+        <v>2</v>
+      </c>
+      <c r="P32" s="4" t="s">
+        <v>685</v>
+      </c>
+      <c r="Q32" s="6">
+        <f>IF($B32="","",$B32&amp;"_W"&amp;$C32)</f>
         <v>0</v>
       </c>
     </row>
@@ -10089,7 +10123,7 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>685</v>
+        <v>686</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -10100,20 +10134,20 @@
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="5" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="9" t="s">
-        <v>687</v>
+        <v>688</v>
       </c>
       <c r="B4" s="11">
         <v>81</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="D4" s="4"/>
       <c r="E4" s="4"/>
@@ -10122,21 +10156,21 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="9" t="s">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>689</v>
+        <v>690</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="9" t="s">
-        <v>690</v>
+        <v>691</v>
       </c>
       <c r="B6" s="11">
         <v>2.2</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
@@ -10145,7 +10179,7 @@
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="9" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="B7" s="11">
         <v>0.9</v>
@@ -10153,7 +10187,7 @@
     </row>
     <row r="8" spans="1:7">
       <c r="A8" s="9" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="B8" s="10">
         <v>2700</v>
@@ -10161,7 +10195,7 @@
     </row>
     <row r="9" spans="1:7">
       <c r="A9" s="9" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="B9" s="10">
         <f>ROUND(BW*B6,0)</f>
@@ -10170,7 +10204,7 @@
     </row>
     <row r="10" spans="1:7">
       <c r="A10" s="9" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="B10" s="10">
         <f>ROUND(BW*B7,0)</f>
@@ -10179,7 +10213,7 @@
     </row>
     <row r="12" spans="1:7">
       <c r="A12" s="5" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -10193,27 +10227,27 @@
         <v>87</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" s="9" t="s">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="B14" s="26">
         <v>250</v>
@@ -10235,7 +10269,7 @@
         <v>0</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -10262,12 +10296,12 @@
         <v>0</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>706</v>
+        <v>707</v>
       </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" s="9" t="s">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="B16" s="26">
         <v>200</v>
@@ -10289,12 +10323,12 @@
         <v>0</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
     </row>
     <row r="17" spans="1:7">
       <c r="A17" s="9" t="s">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="B17" s="26">
         <v>150</v>
@@ -10316,12 +10350,12 @@
         <v>0</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>710</v>
+        <v>711</v>
       </c>
     </row>
     <row r="18" spans="1:7">
       <c r="A18" s="9" t="s">
-        <v>711</v>
+        <v>712</v>
       </c>
       <c r="B18" s="26">
         <v>100</v>
@@ -10343,7 +10377,7 @@
         <v>0</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>712</v>
+        <v>713</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -10370,12 +10404,12 @@
         <v>0</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>713</v>
+        <v>714</v>
       </c>
     </row>
     <row r="21" spans="1:7">
       <c r="A21" s="5" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
@@ -10386,7 +10420,7 @@
     </row>
     <row r="22" spans="1:7">
       <c r="A22" s="4" t="s">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
@@ -10397,7 +10431,7 @@
     </row>
     <row r="23" spans="1:7">
       <c r="A23" s="4" t="s">
-        <v>716</v>
+        <v>717</v>
       </c>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
@@ -10408,7 +10442,7 @@
     </row>
     <row r="24" spans="1:7">
       <c r="A24" s="4" t="s">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -10419,7 +10453,7 @@
     </row>
     <row r="25" spans="1:7">
       <c r="A25" s="4" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -10464,7 +10498,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -10473,7 +10507,7 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="5" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
@@ -10482,126 +10516,126 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="7" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="9" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="B5" s="22" t="s">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="C5" s="27" t="s">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="D5" s="28" t="s">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="E5" s="29" t="s">
-        <v>730</v>
+        <v>731</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="9" t="s">
-        <v>731</v>
+        <v>732</v>
       </c>
       <c r="B6" s="22" t="s">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="C6" s="27" t="s">
-        <v>733</v>
+        <v>734</v>
       </c>
       <c r="D6" s="28" t="s">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="E6" s="29" t="s">
-        <v>735</v>
+        <v>736</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="9" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="B7" s="22" t="s">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="C7" s="27" t="s">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="D7" s="28" t="s">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="E7" s="29" t="s">
-        <v>740</v>
+        <v>741</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="9" t="s">
-        <v>741</v>
+        <v>742</v>
       </c>
       <c r="B8" s="22" t="s">
-        <v>742</v>
+        <v>743</v>
       </c>
       <c r="C8" s="27" t="s">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="D8" s="28" t="s">
-        <v>744</v>
+        <v>745</v>
       </c>
       <c r="E8" s="29" t="s">
-        <v>745</v>
+        <v>746</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="9" t="s">
-        <v>746</v>
+        <v>747</v>
       </c>
       <c r="B9" s="22" t="s">
-        <v>747</v>
+        <v>748</v>
       </c>
       <c r="C9" s="27" t="s">
-        <v>748</v>
+        <v>749</v>
       </c>
       <c r="D9" s="28" t="s">
-        <v>749</v>
+        <v>750</v>
       </c>
       <c r="E9" s="29" t="s">
-        <v>750</v>
+        <v>751</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="9" t="s">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="B10" s="22" t="s">
-        <v>752</v>
+        <v>753</v>
       </c>
       <c r="C10" s="27" t="s">
-        <v>753</v>
+        <v>754</v>
       </c>
       <c r="D10" s="28" t="s">
-        <v>754</v>
+        <v>755</v>
       </c>
       <c r="E10" s="29" t="s">
-        <v>755</v>
+        <v>756</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="5" t="s">
-        <v>756</v>
+        <v>757</v>
       </c>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -10673,7 +10707,7 @@
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="5" t="s">
-        <v>757</v>
+        <v>758</v>
       </c>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
@@ -10682,36 +10716,36 @@
     </row>
     <row r="22" spans="1:5">
       <c r="A22" s="7" t="s">
-        <v>758</v>
+        <v>759</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>759</v>
+        <v>760</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>760</v>
+        <v>761</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>761</v>
+        <v>762</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>762</v>
+        <v>763</v>
       </c>
     </row>
     <row r="23" spans="1:5">
       <c r="A23" s="14" t="s">
-        <v>763</v>
+        <v>764</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>764</v>
+        <v>765</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>766</v>
+        <v>767</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>767</v>
+        <v>768</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -10719,16 +10753,16 @@
         <v>48</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>768</v>
+        <v>769</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>769</v>
+        <v>770</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>770</v>
+        <v>771</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>771</v>
+        <v>772</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -10736,16 +10770,16 @@
         <v>35</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>772</v>
+        <v>773</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>773</v>
+        <v>774</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>774</v>
+        <v>775</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>775</v>
+        <v>776</v>
       </c>
     </row>
     <row r="26" spans="1:5">
@@ -10753,21 +10787,21 @@
         <v>38</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>776</v>
+        <v>777</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>777</v>
+        <v>778</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>778</v>
+        <v>779</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>779</v>
+        <v>780</v>
       </c>
     </row>
     <row r="28" spans="1:5">
       <c r="A28" s="5" t="s">
-        <v>780</v>
+        <v>781</v>
       </c>
       <c r="B28" s="5"/>
       <c r="C28" s="5"/>
@@ -10776,7 +10810,7 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" s="4" t="s">
-        <v>781</v>
+        <v>782</v>
       </c>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -10785,7 +10819,7 @@
     </row>
     <row r="30" spans="1:5">
       <c r="A30" s="4" t="s">
-        <v>782</v>
+        <v>783</v>
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -10794,7 +10828,7 @@
     </row>
     <row r="31" spans="1:5">
       <c r="A31" s="4" t="s">
-        <v>783</v>
+        <v>784</v>
       </c>
       <c r="B31" s="4"/>
       <c r="C31" s="4"/>
@@ -10803,7 +10837,7 @@
     </row>
     <row r="32" spans="1:5">
       <c r="A32" s="4" t="s">
-        <v>784</v>
+        <v>785</v>
       </c>
       <c r="B32" s="4"/>
       <c r="C32" s="4"/>
@@ -10812,7 +10846,7 @@
     </row>
     <row r="33" spans="1:5">
       <c r="A33" s="4" t="s">
-        <v>785</v>
+        <v>786</v>
       </c>
       <c r="B33" s="4"/>
       <c r="C33" s="4"/>
@@ -10836,98 +10870,98 @@
         <v>432</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>786</v>
+        <v>787</v>
       </c>
       <c r="D36" s="7"/>
       <c r="E36" s="7"/>
     </row>
     <row r="37" spans="1:5">
       <c r="A37" s="4" t="s">
-        <v>787</v>
+        <v>788</v>
       </c>
       <c r="B37" s="24" t="s">
-        <v>788</v>
+        <v>789</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>789</v>
+        <v>790</v>
       </c>
       <c r="D37" s="4"/>
       <c r="E37" s="4"/>
     </row>
     <row r="38" spans="1:5">
       <c r="A38" s="4" t="s">
-        <v>790</v>
+        <v>791</v>
       </c>
       <c r="B38" s="24" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>792</v>
+        <v>793</v>
       </c>
       <c r="D38" s="4"/>
       <c r="E38" s="4"/>
     </row>
     <row r="39" spans="1:5">
       <c r="A39" s="4" t="s">
-        <v>793</v>
+        <v>794</v>
       </c>
       <c r="B39" s="24" t="s">
         <v>440</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>794</v>
+        <v>795</v>
       </c>
       <c r="D39" s="4"/>
       <c r="E39" s="4"/>
     </row>
     <row r="40" spans="1:5">
       <c r="A40" s="4" t="s">
-        <v>795</v>
+        <v>796</v>
       </c>
       <c r="B40" s="24" t="s">
-        <v>796</v>
+        <v>797</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>797</v>
+        <v>798</v>
       </c>
       <c r="D40" s="4"/>
       <c r="E40" s="4"/>
     </row>
     <row r="41" spans="1:5">
       <c r="A41" s="4" t="s">
-        <v>795</v>
+        <v>796</v>
       </c>
       <c r="B41" s="24" t="s">
-        <v>798</v>
+        <v>799</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>799</v>
+        <v>800</v>
       </c>
       <c r="D41" s="4"/>
       <c r="E41" s="4"/>
     </row>
     <row r="42" spans="1:5">
       <c r="A42" s="4" t="s">
-        <v>800</v>
+        <v>801</v>
       </c>
       <c r="B42" s="24" t="s">
-        <v>801</v>
+        <v>802</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>802</v>
+        <v>803</v>
       </c>
       <c r="D42" s="4"/>
       <c r="E42" s="4"/>
     </row>
     <row r="43" spans="1:5">
       <c r="A43" s="4" t="s">
-        <v>803</v>
+        <v>804</v>
       </c>
       <c r="B43" s="24" t="s">
-        <v>804</v>
+        <v>805</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>805</v>
+        <v>806</v>
       </c>
       <c r="D43" s="4"/>
       <c r="E43" s="4"/>

</xml_diff>

<commit_message>
Log B7 W1 T4 (Recovery 4, home): straddle+diamond flag lean holds, 90 negatives, pike, band biceps
</commit_message>
<xml_diff>
--- a/Training_3_B7.xlsx
+++ b/Training_3_B7.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1640" uniqueCount="880">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1662" uniqueCount="887">
   <si>
     <t>B7 — Performance-Block Dashboard (Advanced OAHS)</t>
   </si>
@@ -2115,6 +2115,27 @@
   </si>
   <si>
     <t>Symptome: Heuschnupfen, Kopfschmerz (unueblich), Kreislauf/zittrig, Muskelzuckungen, Stress -&gt; Rest statt T4</t>
+  </si>
+  <si>
+    <t>Straddle: OAHS-Holds + Return zum Center; sonst kurzer Straddle Flag Lean Hold</t>
+  </si>
+  <si>
+    <t>Diamond Flag Lean Hold</t>
+  </si>
+  <si>
+    <t>3,2,2 Negativ</t>
+  </si>
+  <si>
+    <t>Negative, Parallettes</t>
+  </si>
+  <si>
+    <t>7,6,6</t>
+  </si>
+  <si>
+    <t>Pike Push-ups feet elevated</t>
+  </si>
+  <si>
+    <t>Blaues Band (Pull-Ersatz daheim); Row entfiel (kein Equipment)</t>
   </si>
   <si>
     <t>B7 — Nutrition Targets (Maintenance, KEIN Defizit)</t>
@@ -3925,7 +3946,7 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>816</v>
+        <v>823</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3935,7 +3956,7 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="12" t="s">
-        <v>817</v>
+        <v>824</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -3960,12 +3981,12 @@
         <v>155</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>818</v>
+        <v>825</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="9" t="s">
-        <v>819</v>
+        <v>826</v>
       </c>
       <c r="B4" s="11">
         <f>SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Skill90",'B7_Training_Log'!$C$2:$C$1000,1)+SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Planche",'B7_Training_Log'!$C$2:$C$1000,1)+SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Push",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -3990,7 +4011,7 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="9" t="s">
-        <v>820</v>
+        <v>827</v>
       </c>
       <c r="B5" s="11">
         <f>SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Pull",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4015,7 +4036,7 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="9" t="s">
-        <v>821</v>
+        <v>828</v>
       </c>
       <c r="B6" s="11">
         <f>SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Legs",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4040,7 +4061,7 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="9" t="s">
-        <v>822</v>
+        <v>829</v>
       </c>
       <c r="B7" s="10">
         <f>SUMIFS('B7_Training_Log'!$N$2:$N$1000,'B7_Training_Log'!$D$2:$D$1000,"90",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4065,7 +4086,7 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="9" t="s">
-        <v>823</v>
+        <v>830</v>
       </c>
       <c r="B8" s="10">
         <f>COUNTIFS('B7_Training_Log'!$E$2:$E$1000,"SkillOAHS",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4090,7 +4111,7 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="9" t="s">
-        <v>824</v>
+        <v>831</v>
       </c>
       <c r="B9" s="10">
         <f>MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_straddle",'B7_Training_Log'!$F$2:$F$1000,"L",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4115,7 +4136,7 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="9" t="s">
-        <v>825</v>
+        <v>832</v>
       </c>
       <c r="B10" s="10">
         <f>MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_straddle",'B7_Training_Log'!$F$2:$F$1000,"R",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4140,7 +4161,7 @@
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="9" t="s">
-        <v>826</v>
+        <v>833</v>
       </c>
       <c r="B11" s="10">
         <f>MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_diamond",'B7_Training_Log'!$F$2:$F$1000,"L",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4165,7 +4186,7 @@
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="9" t="s">
-        <v>827</v>
+        <v>834</v>
       </c>
       <c r="B12" s="10">
         <f>MAX(MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_flag",'B7_Training_Log'!$C$2:$C$1000,1),MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_figa",'B7_Training_Log'!$C$2:$C$1000,1))</f>
@@ -4190,7 +4211,7 @@
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="9" t="s">
-        <v>828</v>
+        <v>835</v>
       </c>
       <c r="B13" s="11">
         <f>IFERROR(AVERAGEIFS('B7_Training_Log'!$J$2:$J$1000,'B7_Training_Log'!$C$2:$C$1000,1),0)</f>
@@ -4265,7 +4286,7 @@
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="9" t="s">
-        <v>829</v>
+        <v>836</v>
       </c>
       <c r="B16" s="10">
         <f>COUNTIFS('B7_Training_Log'!$K$2:$K$1000,"&gt;=4",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4290,7 +4311,7 @@
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="9" t="s">
-        <v>830</v>
+        <v>837</v>
       </c>
       <c r="B17" s="10">
         <f>COUNTIFS('B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4334,7 +4355,7 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
-        <v>831</v>
+        <v>838</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4342,7 +4363,7 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="5" t="s">
-        <v>832</v>
+        <v>839</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
@@ -4350,13 +4371,13 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="7" t="s">
-        <v>833</v>
+        <v>840</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>834</v>
+        <v>841</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>835</v>
+        <v>842</v>
       </c>
       <c r="D4" s="7"/>
     </row>
@@ -4365,10 +4386,10 @@
         <v>645</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>836</v>
+        <v>843</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>837</v>
+        <v>844</v>
       </c>
       <c r="D5" s="4"/>
     </row>
@@ -4377,10 +4398,10 @@
         <v>646</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>838</v>
+        <v>845</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>839</v>
+        <v>846</v>
       </c>
       <c r="D6" s="4"/>
     </row>
@@ -4389,10 +4410,10 @@
         <v>647</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>840</v>
+        <v>847</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>841</v>
+        <v>848</v>
       </c>
       <c r="D7" s="4"/>
     </row>
@@ -4401,10 +4422,10 @@
         <v>454</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>842</v>
+        <v>849</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>843</v>
+        <v>850</v>
       </c>
       <c r="D8" s="4"/>
     </row>
@@ -4413,10 +4434,10 @@
         <v>457</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>844</v>
+        <v>851</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>845</v>
+        <v>852</v>
       </c>
       <c r="D9" s="4"/>
     </row>
@@ -4425,10 +4446,10 @@
         <v>648</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>846</v>
+        <v>853</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>847</v>
+        <v>854</v>
       </c>
       <c r="D10" s="4"/>
     </row>
@@ -4437,10 +4458,10 @@
         <v>649</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>848</v>
+        <v>855</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>849</v>
+        <v>856</v>
       </c>
       <c r="D11" s="4"/>
     </row>
@@ -4449,10 +4470,10 @@
         <v>650</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>850</v>
+        <v>857</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>851</v>
+        <v>858</v>
       </c>
       <c r="D12" s="4"/>
     </row>
@@ -4461,10 +4482,10 @@
         <v>651</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>848</v>
+        <v>855</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>852</v>
+        <v>859</v>
       </c>
       <c r="D13" s="4"/>
     </row>
@@ -4473,10 +4494,10 @@
         <v>652</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>853</v>
+        <v>860</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>854</v>
+        <v>861</v>
       </c>
       <c r="D14" s="4"/>
     </row>
@@ -4485,10 +4506,10 @@
         <v>653</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>855</v>
+        <v>862</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>856</v>
+        <v>863</v>
       </c>
       <c r="D15" s="4"/>
     </row>
@@ -4497,10 +4518,10 @@
         <v>654</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>857</v>
+        <v>864</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>858</v>
+        <v>865</v>
       </c>
       <c r="D16" s="4"/>
     </row>
@@ -4509,10 +4530,10 @@
         <v>655</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>848</v>
+        <v>855</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>859</v>
+        <v>866</v>
       </c>
       <c r="D17" s="4"/>
     </row>
@@ -4521,10 +4542,10 @@
         <v>656</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>848</v>
+        <v>855</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>860</v>
+        <v>867</v>
       </c>
       <c r="D18" s="4"/>
     </row>
@@ -4533,10 +4554,10 @@
         <v>657</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>861</v>
+        <v>868</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>862</v>
+        <v>869</v>
       </c>
       <c r="D19" s="4"/>
     </row>
@@ -4545,10 +4566,10 @@
         <v>94</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>850</v>
+        <v>857</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>863</v>
+        <v>870</v>
       </c>
       <c r="D20" s="4"/>
     </row>
@@ -4557,16 +4578,16 @@
         <v>658</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>864</v>
+        <v>871</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>865</v>
+        <v>872</v>
       </c>
       <c r="D21" s="4"/>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="5" t="s">
-        <v>866</v>
+        <v>873</v>
       </c>
       <c r="B23" s="5"/>
       <c r="C23" s="5"/>
@@ -4574,7 +4595,7 @@
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="4" t="s">
-        <v>867</v>
+        <v>874</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -4582,7 +4603,7 @@
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="4" t="s">
-        <v>868</v>
+        <v>875</v>
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -4590,7 +4611,7 @@
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="4" t="s">
-        <v>869</v>
+        <v>876</v>
       </c>
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
@@ -4598,7 +4619,7 @@
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="4" t="s">
-        <v>870</v>
+        <v>877</v>
       </c>
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
@@ -4606,7 +4627,7 @@
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="4" t="s">
-        <v>871</v>
+        <v>878</v>
       </c>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
@@ -4614,7 +4635,7 @@
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="4" t="s">
-        <v>872</v>
+        <v>879</v>
       </c>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -4622,7 +4643,7 @@
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="4" t="s">
-        <v>873</v>
+        <v>880</v>
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -4630,7 +4651,7 @@
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="5" t="s">
-        <v>874</v>
+        <v>881</v>
       </c>
       <c r="B32" s="5"/>
       <c r="C32" s="5"/>
@@ -4638,7 +4659,7 @@
     </row>
     <row r="33" spans="1:4">
       <c r="A33" s="4" t="s">
-        <v>875</v>
+        <v>882</v>
       </c>
       <c r="B33" s="4"/>
       <c r="C33" s="4"/>
@@ -4646,7 +4667,7 @@
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="4" t="s">
-        <v>876</v>
+        <v>883</v>
       </c>
       <c r="B34" s="4"/>
       <c r="C34" s="4"/>
@@ -4654,7 +4675,7 @@
     </row>
     <row r="35" spans="1:4">
       <c r="A35" s="4" t="s">
-        <v>877</v>
+        <v>884</v>
       </c>
       <c r="B35" s="4"/>
       <c r="C35" s="4"/>
@@ -4662,7 +4683,7 @@
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="4" t="s">
-        <v>878</v>
+        <v>885</v>
       </c>
       <c r="B36" s="4"/>
       <c r="C36" s="4"/>
@@ -4670,7 +4691,7 @@
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="4" t="s">
-        <v>879</v>
+        <v>886</v>
       </c>
       <c r="B37" s="4"/>
       <c r="C37" s="4"/>
@@ -8776,7 +8797,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q32"/>
+  <dimension ref="A1:Q37"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -10149,6 +10170,218 @@
       </c>
       <c r="Q32" s="6">
         <f>IF($B32="","",$B32&amp;"_W"&amp;$C32)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:17">
+      <c r="A33" s="25">
+        <v>46217</v>
+      </c>
+      <c r="B33" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="C33" s="6">
+        <v>1</v>
+      </c>
+      <c r="D33" s="6" t="s">
+        <v>641</v>
+      </c>
+      <c r="E33" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D33,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F33" s="6" t="s">
+        <v>666</v>
+      </c>
+      <c r="G33" s="6">
+        <v>4</v>
+      </c>
+      <c r="I33" s="6">
+        <v>0</v>
+      </c>
+      <c r="L33" s="6">
+        <v>3</v>
+      </c>
+      <c r="M33" s="6">
+        <v>3</v>
+      </c>
+      <c r="O33" s="6">
+        <v>4</v>
+      </c>
+      <c r="P33" s="4" t="s">
+        <v>695</v>
+      </c>
+      <c r="Q33" s="6">
+        <f>IF($B33="","",$B33&amp;"_W"&amp;$C33)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:17">
+      <c r="A34" s="25">
+        <v>46217</v>
+      </c>
+      <c r="B34" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="C34" s="6">
+        <v>1</v>
+      </c>
+      <c r="D34" s="6" t="s">
+        <v>641</v>
+      </c>
+      <c r="E34" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D34,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F34" s="6" t="s">
+        <v>666</v>
+      </c>
+      <c r="G34" s="6">
+        <v>3</v>
+      </c>
+      <c r="I34" s="6">
+        <v>0</v>
+      </c>
+      <c r="L34" s="6">
+        <v>3</v>
+      </c>
+      <c r="M34" s="6">
+        <v>3</v>
+      </c>
+      <c r="O34" s="6">
+        <v>4</v>
+      </c>
+      <c r="P34" s="4" t="s">
+        <v>696</v>
+      </c>
+      <c r="Q34" s="6">
+        <f>IF($B34="","",$B34&amp;"_W"&amp;$C34)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:17">
+      <c r="A35" s="25">
+        <v>46217</v>
+      </c>
+      <c r="B35" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="C35" s="6">
+        <v>1</v>
+      </c>
+      <c r="D35" s="6" t="s">
+        <v>462</v>
+      </c>
+      <c r="E35" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D35,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F35" s="6" t="s">
+        <v>666</v>
+      </c>
+      <c r="G35" s="6">
+        <v>3</v>
+      </c>
+      <c r="H35" s="4" t="s">
+        <v>697</v>
+      </c>
+      <c r="I35" s="6">
+        <v>0</v>
+      </c>
+      <c r="J35" s="6">
+        <v>7</v>
+      </c>
+      <c r="L35" s="6">
+        <v>4</v>
+      </c>
+      <c r="O35" s="6">
+        <v>4</v>
+      </c>
+      <c r="P35" s="4" t="s">
+        <v>698</v>
+      </c>
+      <c r="Q35" s="6">
+        <f>IF($B35="","",$B35&amp;"_W"&amp;$C35)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:17">
+      <c r="A36" s="25">
+        <v>46217</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="C36" s="6">
+        <v>1</v>
+      </c>
+      <c r="D36" s="6" t="s">
+        <v>540</v>
+      </c>
+      <c r="E36" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D36,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F36" s="6" t="s">
+        <v>666</v>
+      </c>
+      <c r="G36" s="6">
+        <v>3</v>
+      </c>
+      <c r="H36" s="4" t="s">
+        <v>699</v>
+      </c>
+      <c r="I36" s="6">
+        <v>0</v>
+      </c>
+      <c r="J36" s="6">
+        <v>7</v>
+      </c>
+      <c r="O36" s="6">
+        <v>4</v>
+      </c>
+      <c r="P36" s="4" t="s">
+        <v>700</v>
+      </c>
+      <c r="Q36" s="6">
+        <f>IF($B36="","",$B36&amp;"_W"&amp;$C36)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:17">
+      <c r="A37" s="25">
+        <v>46217</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="C37" s="6">
+        <v>1</v>
+      </c>
+      <c r="D37" s="6" t="s">
+        <v>558</v>
+      </c>
+      <c r="E37" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D37,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F37" s="6" t="s">
+        <v>666</v>
+      </c>
+      <c r="G37" s="6">
+        <v>3</v>
+      </c>
+      <c r="J37" s="6">
+        <v>7</v>
+      </c>
+      <c r="O37" s="6">
+        <v>4</v>
+      </c>
+      <c r="P37" s="4" t="s">
+        <v>701</v>
+      </c>
+      <c r="Q37" s="6">
+        <f>IF($B37="","",$B37&amp;"_W"&amp;$C37)</f>
         <v>0</v>
       </c>
     </row>
@@ -10226,7 +10459,7 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>695</v>
+        <v>702</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -10237,20 +10470,20 @@
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="5" t="s">
-        <v>696</v>
+        <v>703</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="9" t="s">
-        <v>697</v>
+        <v>704</v>
       </c>
       <c r="B4" s="11">
         <v>81</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>705</v>
+        <v>712</v>
       </c>
       <c r="D4" s="4"/>
       <c r="E4" s="4"/>
@@ -10259,21 +10492,21 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="9" t="s">
-        <v>698</v>
+        <v>705</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>699</v>
+        <v>706</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="9" t="s">
-        <v>700</v>
+        <v>707</v>
       </c>
       <c r="B6" s="11">
         <v>2.2</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>706</v>
+        <v>713</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
@@ -10282,7 +10515,7 @@
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="9" t="s">
-        <v>701</v>
+        <v>708</v>
       </c>
       <c r="B7" s="11">
         <v>0.9</v>
@@ -10290,7 +10523,7 @@
     </row>
     <row r="8" spans="1:7">
       <c r="A8" s="9" t="s">
-        <v>702</v>
+        <v>709</v>
       </c>
       <c r="B8" s="10">
         <v>2700</v>
@@ -10298,7 +10531,7 @@
     </row>
     <row r="9" spans="1:7">
       <c r="A9" s="9" t="s">
-        <v>703</v>
+        <v>710</v>
       </c>
       <c r="B9" s="10">
         <f>ROUND(BW*B6,0)</f>
@@ -10307,7 +10540,7 @@
     </row>
     <row r="10" spans="1:7">
       <c r="A10" s="9" t="s">
-        <v>704</v>
+        <v>711</v>
       </c>
       <c r="B10" s="10">
         <f>ROUND(BW*B7,0)</f>
@@ -10316,7 +10549,7 @@
     </row>
     <row r="12" spans="1:7">
       <c r="A12" s="5" t="s">
-        <v>707</v>
+        <v>714</v>
       </c>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -10330,27 +10563,27 @@
         <v>87</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>708</v>
+        <v>715</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>709</v>
+        <v>716</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>710</v>
+        <v>717</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>711</v>
+        <v>718</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>712</v>
+        <v>719</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>713</v>
+        <v>720</v>
       </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" s="9" t="s">
-        <v>714</v>
+        <v>721</v>
       </c>
       <c r="B14" s="26">
         <v>250</v>
@@ -10372,7 +10605,7 @@
         <v>0</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>715</v>
+        <v>722</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -10399,12 +10632,12 @@
         <v>0</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>716</v>
+        <v>723</v>
       </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" s="9" t="s">
-        <v>717</v>
+        <v>724</v>
       </c>
       <c r="B16" s="26">
         <v>200</v>
@@ -10426,12 +10659,12 @@
         <v>0</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>718</v>
+        <v>725</v>
       </c>
     </row>
     <row r="17" spans="1:7">
       <c r="A17" s="9" t="s">
-        <v>719</v>
+        <v>726</v>
       </c>
       <c r="B17" s="26">
         <v>150</v>
@@ -10453,12 +10686,12 @@
         <v>0</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>720</v>
+        <v>727</v>
       </c>
     </row>
     <row r="18" spans="1:7">
       <c r="A18" s="9" t="s">
-        <v>721</v>
+        <v>728</v>
       </c>
       <c r="B18" s="26">
         <v>100</v>
@@ -10480,7 +10713,7 @@
         <v>0</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>722</v>
+        <v>729</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -10507,12 +10740,12 @@
         <v>0</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>723</v>
+        <v>730</v>
       </c>
     </row>
     <row r="21" spans="1:7">
       <c r="A21" s="5" t="s">
-        <v>724</v>
+        <v>731</v>
       </c>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
@@ -10523,7 +10756,7 @@
     </row>
     <row r="22" spans="1:7">
       <c r="A22" s="4" t="s">
-        <v>725</v>
+        <v>732</v>
       </c>
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
@@ -10534,7 +10767,7 @@
     </row>
     <row r="23" spans="1:7">
       <c r="A23" s="4" t="s">
-        <v>726</v>
+        <v>733</v>
       </c>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
@@ -10545,7 +10778,7 @@
     </row>
     <row r="24" spans="1:7">
       <c r="A24" s="4" t="s">
-        <v>727</v>
+        <v>734</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -10556,7 +10789,7 @@
     </row>
     <row r="25" spans="1:7">
       <c r="A25" s="4" t="s">
-        <v>728</v>
+        <v>735</v>
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -10601,7 +10834,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>729</v>
+        <v>736</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -10610,7 +10843,7 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="5" t="s">
-        <v>730</v>
+        <v>737</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
@@ -10619,126 +10852,126 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="7" t="s">
-        <v>731</v>
+        <v>738</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>732</v>
+        <v>739</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>733</v>
+        <v>740</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>734</v>
+        <v>741</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>735</v>
+        <v>742</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="9" t="s">
-        <v>736</v>
+        <v>743</v>
       </c>
       <c r="B5" s="22" t="s">
-        <v>737</v>
+        <v>744</v>
       </c>
       <c r="C5" s="27" t="s">
-        <v>738</v>
+        <v>745</v>
       </c>
       <c r="D5" s="28" t="s">
-        <v>739</v>
+        <v>746</v>
       </c>
       <c r="E5" s="29" t="s">
-        <v>740</v>
+        <v>747</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="9" t="s">
-        <v>741</v>
+        <v>748</v>
       </c>
       <c r="B6" s="22" t="s">
-        <v>742</v>
+        <v>749</v>
       </c>
       <c r="C6" s="27" t="s">
-        <v>743</v>
+        <v>750</v>
       </c>
       <c r="D6" s="28" t="s">
-        <v>744</v>
+        <v>751</v>
       </c>
       <c r="E6" s="29" t="s">
-        <v>745</v>
+        <v>752</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="9" t="s">
-        <v>746</v>
+        <v>753</v>
       </c>
       <c r="B7" s="22" t="s">
-        <v>747</v>
+        <v>754</v>
       </c>
       <c r="C7" s="27" t="s">
-        <v>748</v>
+        <v>755</v>
       </c>
       <c r="D7" s="28" t="s">
-        <v>749</v>
+        <v>756</v>
       </c>
       <c r="E7" s="29" t="s">
-        <v>750</v>
+        <v>757</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="9" t="s">
-        <v>751</v>
+        <v>758</v>
       </c>
       <c r="B8" s="22" t="s">
-        <v>752</v>
+        <v>759</v>
       </c>
       <c r="C8" s="27" t="s">
-        <v>753</v>
+        <v>760</v>
       </c>
       <c r="D8" s="28" t="s">
-        <v>754</v>
+        <v>761</v>
       </c>
       <c r="E8" s="29" t="s">
-        <v>755</v>
+        <v>762</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="9" t="s">
-        <v>756</v>
+        <v>763</v>
       </c>
       <c r="B9" s="22" t="s">
-        <v>757</v>
+        <v>764</v>
       </c>
       <c r="C9" s="27" t="s">
-        <v>758</v>
+        <v>765</v>
       </c>
       <c r="D9" s="28" t="s">
-        <v>759</v>
+        <v>766</v>
       </c>
       <c r="E9" s="29" t="s">
-        <v>760</v>
+        <v>767</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="9" t="s">
-        <v>761</v>
+        <v>768</v>
       </c>
       <c r="B10" s="22" t="s">
-        <v>762</v>
+        <v>769</v>
       </c>
       <c r="C10" s="27" t="s">
-        <v>763</v>
+        <v>770</v>
       </c>
       <c r="D10" s="28" t="s">
-        <v>764</v>
+        <v>771</v>
       </c>
       <c r="E10" s="29" t="s">
-        <v>765</v>
+        <v>772</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="5" t="s">
-        <v>766</v>
+        <v>773</v>
       </c>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -10810,7 +11043,7 @@
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="5" t="s">
-        <v>767</v>
+        <v>774</v>
       </c>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
@@ -10819,36 +11052,36 @@
     </row>
     <row r="22" spans="1:5">
       <c r="A22" s="7" t="s">
-        <v>768</v>
+        <v>775</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>769</v>
+        <v>776</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>770</v>
+        <v>777</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>771</v>
+        <v>778</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>772</v>
+        <v>779</v>
       </c>
     </row>
     <row r="23" spans="1:5">
       <c r="A23" s="14" t="s">
-        <v>773</v>
+        <v>780</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>774</v>
+        <v>781</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>775</v>
+        <v>782</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>776</v>
+        <v>783</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>777</v>
+        <v>784</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -10856,16 +11089,16 @@
         <v>48</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>778</v>
+        <v>785</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>779</v>
+        <v>786</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>780</v>
+        <v>787</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>781</v>
+        <v>788</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -10873,16 +11106,16 @@
         <v>35</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>782</v>
+        <v>789</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>783</v>
+        <v>790</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>784</v>
+        <v>791</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>785</v>
+        <v>792</v>
       </c>
     </row>
     <row r="26" spans="1:5">
@@ -10890,21 +11123,21 @@
         <v>38</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>786</v>
+        <v>793</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>787</v>
+        <v>794</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>788</v>
+        <v>795</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>789</v>
+        <v>796</v>
       </c>
     </row>
     <row r="28" spans="1:5">
       <c r="A28" s="5" t="s">
-        <v>790</v>
+        <v>797</v>
       </c>
       <c r="B28" s="5"/>
       <c r="C28" s="5"/>
@@ -10913,7 +11146,7 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" s="4" t="s">
-        <v>791</v>
+        <v>798</v>
       </c>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -10922,7 +11155,7 @@
     </row>
     <row r="30" spans="1:5">
       <c r="A30" s="4" t="s">
-        <v>792</v>
+        <v>799</v>
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -10931,7 +11164,7 @@
     </row>
     <row r="31" spans="1:5">
       <c r="A31" s="4" t="s">
-        <v>793</v>
+        <v>800</v>
       </c>
       <c r="B31" s="4"/>
       <c r="C31" s="4"/>
@@ -10940,7 +11173,7 @@
     </row>
     <row r="32" spans="1:5">
       <c r="A32" s="4" t="s">
-        <v>794</v>
+        <v>801</v>
       </c>
       <c r="B32" s="4"/>
       <c r="C32" s="4"/>
@@ -10949,7 +11182,7 @@
     </row>
     <row r="33" spans="1:5">
       <c r="A33" s="4" t="s">
-        <v>795</v>
+        <v>802</v>
       </c>
       <c r="B33" s="4"/>
       <c r="C33" s="4"/>
@@ -10973,98 +11206,98 @@
         <v>441</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>796</v>
+        <v>803</v>
       </c>
       <c r="D36" s="7"/>
       <c r="E36" s="7"/>
     </row>
     <row r="37" spans="1:5">
       <c r="A37" s="4" t="s">
-        <v>797</v>
+        <v>804</v>
       </c>
       <c r="B37" s="24" t="s">
-        <v>798</v>
+        <v>805</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>799</v>
+        <v>806</v>
       </c>
       <c r="D37" s="4"/>
       <c r="E37" s="4"/>
     </row>
     <row r="38" spans="1:5">
       <c r="A38" s="4" t="s">
-        <v>800</v>
+        <v>807</v>
       </c>
       <c r="B38" s="24" t="s">
-        <v>801</v>
+        <v>808</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>802</v>
+        <v>809</v>
       </c>
       <c r="D38" s="4"/>
       <c r="E38" s="4"/>
     </row>
     <row r="39" spans="1:5">
       <c r="A39" s="4" t="s">
-        <v>803</v>
+        <v>810</v>
       </c>
       <c r="B39" s="24" t="s">
         <v>449</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>804</v>
+        <v>811</v>
       </c>
       <c r="D39" s="4"/>
       <c r="E39" s="4"/>
     </row>
     <row r="40" spans="1:5">
       <c r="A40" s="4" t="s">
-        <v>805</v>
+        <v>812</v>
       </c>
       <c r="B40" s="24" t="s">
-        <v>806</v>
+        <v>813</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>807</v>
+        <v>814</v>
       </c>
       <c r="D40" s="4"/>
       <c r="E40" s="4"/>
     </row>
     <row r="41" spans="1:5">
       <c r="A41" s="4" t="s">
-        <v>805</v>
+        <v>812</v>
       </c>
       <c r="B41" s="24" t="s">
-        <v>808</v>
+        <v>815</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>809</v>
+        <v>816</v>
       </c>
       <c r="D41" s="4"/>
       <c r="E41" s="4"/>
     </row>
     <row r="42" spans="1:5">
       <c r="A42" s="4" t="s">
-        <v>810</v>
+        <v>817</v>
       </c>
       <c r="B42" s="24" t="s">
-        <v>811</v>
+        <v>818</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>812</v>
+        <v>819</v>
       </c>
       <c r="D42" s="4"/>
       <c r="E42" s="4"/>
     </row>
     <row r="43" spans="1:5">
       <c r="A43" s="4" t="s">
-        <v>813</v>
+        <v>820</v>
       </c>
       <c r="B43" s="24" t="s">
-        <v>814</v>
+        <v>821</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>815</v>
+        <v>822</v>
       </c>
       <c r="D43" s="4"/>
       <c r="E43" s="4"/>

</xml_diff>

<commit_message>
Log B7 W2 T2 (Recovery 5): OAHS shapes rebuilding post-vacation, pull volume; chest row corrected to 100kg
</commit_message>
<xml_diff>
--- a/Training_3_B7.xlsx
+++ b/Training_3_B7.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1714" uniqueCount="906">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1762" uniqueCount="915">
   <si>
     <t>B7 — Performance-Block Dashboard (Advanced OAHS)</t>
   </si>
@@ -2193,6 +2193,33 @@
   </si>
   <si>
     <t>Endurance-Versuch improvisiert (Sprossenwand), nicht smooth -&gt; Protokoll auf C2W-Holds umgestellt</t>
+  </si>
+  <si>
+    <t>alle 3 Saetze 5s+ (Balance noch off nach Krankheits-Andeutung)</t>
+  </si>
+  <si>
+    <t>~3s+</t>
+  </si>
+  <si>
+    <t>2 Saetze 5s+, 1 Satz 3s</t>
+  </si>
+  <si>
+    <t>alle ~2-3s</t>
+  </si>
+  <si>
+    <t>2 Versuche &gt;5s</t>
+  </si>
+  <si>
+    <t>1x 5s + 1 trash; 3. Satz beidseitig trash -&gt; gestoppt (Fatigue)</t>
+  </si>
+  <si>
+    <t>korrigiert: 100 kg (vorher 90 falsch gerechnet) -&gt; keine echte Steigerung, nur korrektes Gewicht</t>
+  </si>
+  <si>
+    <t>haette ~3 mehr geschafft (eher RPE 7)</t>
+  </si>
+  <si>
+    <t>DB bent-over 2 kg (Maschine besetzt)</t>
   </si>
   <si>
     <t>B7 — Nutrition Targets (Maintenance, KEIN Defizit)</t>
@@ -4003,7 +4030,7 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>842</v>
+        <v>851</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4013,7 +4040,7 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="12" t="s">
-        <v>843</v>
+        <v>852</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -4038,12 +4065,12 @@
         <v>155</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>844</v>
+        <v>853</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="9" t="s">
-        <v>845</v>
+        <v>854</v>
       </c>
       <c r="B4" s="11">
         <f>SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Skill90",'B7_Training_Log'!$C$2:$C$1000,1)+SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Planche",'B7_Training_Log'!$C$2:$C$1000,1)+SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Push",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4068,7 +4095,7 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="9" t="s">
-        <v>846</v>
+        <v>855</v>
       </c>
       <c r="B5" s="11">
         <f>SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Pull",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4093,7 +4120,7 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="9" t="s">
-        <v>847</v>
+        <v>856</v>
       </c>
       <c r="B6" s="11">
         <f>SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Legs",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4118,7 +4145,7 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="9" t="s">
-        <v>848</v>
+        <v>857</v>
       </c>
       <c r="B7" s="10">
         <f>SUMIFS('B7_Training_Log'!$N$2:$N$1000,'B7_Training_Log'!$D$2:$D$1000,"90",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4143,7 +4170,7 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="9" t="s">
-        <v>849</v>
+        <v>858</v>
       </c>
       <c r="B8" s="10">
         <f>COUNTIFS('B7_Training_Log'!$E$2:$E$1000,"SkillOAHS",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4168,7 +4195,7 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="9" t="s">
-        <v>850</v>
+        <v>859</v>
       </c>
       <c r="B9" s="10">
         <f>MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_straddle",'B7_Training_Log'!$F$2:$F$1000,"L",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4193,7 +4220,7 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="9" t="s">
-        <v>851</v>
+        <v>860</v>
       </c>
       <c r="B10" s="10">
         <f>MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_straddle",'B7_Training_Log'!$F$2:$F$1000,"R",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4218,7 +4245,7 @@
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="9" t="s">
-        <v>852</v>
+        <v>861</v>
       </c>
       <c r="B11" s="10">
         <f>MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_diamond",'B7_Training_Log'!$F$2:$F$1000,"L",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4243,7 +4270,7 @@
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="9" t="s">
-        <v>853</v>
+        <v>862</v>
       </c>
       <c r="B12" s="10">
         <f>MAX(MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_flag",'B7_Training_Log'!$C$2:$C$1000,1),MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_figa",'B7_Training_Log'!$C$2:$C$1000,1))</f>
@@ -4268,7 +4295,7 @@
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="9" t="s">
-        <v>854</v>
+        <v>863</v>
       </c>
       <c r="B13" s="11">
         <f>IFERROR(AVERAGEIFS('B7_Training_Log'!$J$2:$J$1000,'B7_Training_Log'!$C$2:$C$1000,1),0)</f>
@@ -4343,7 +4370,7 @@
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="9" t="s">
-        <v>855</v>
+        <v>864</v>
       </c>
       <c r="B16" s="10">
         <f>COUNTIFS('B7_Training_Log'!$K$2:$K$1000,"&gt;=4",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4368,7 +4395,7 @@
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="9" t="s">
-        <v>856</v>
+        <v>865</v>
       </c>
       <c r="B17" s="10">
         <f>COUNTIFS('B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4412,7 +4439,7 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
-        <v>857</v>
+        <v>866</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4420,7 +4447,7 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="5" t="s">
-        <v>858</v>
+        <v>867</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
@@ -4428,13 +4455,13 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="7" t="s">
-        <v>859</v>
+        <v>868</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>860</v>
+        <v>869</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>861</v>
+        <v>870</v>
       </c>
       <c r="D4" s="7"/>
     </row>
@@ -4443,10 +4470,10 @@
         <v>651</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>862</v>
+        <v>871</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>863</v>
+        <v>872</v>
       </c>
       <c r="D5" s="4"/>
     </row>
@@ -4455,10 +4482,10 @@
         <v>652</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>864</v>
+        <v>873</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>865</v>
+        <v>874</v>
       </c>
       <c r="D6" s="4"/>
     </row>
@@ -4467,10 +4494,10 @@
         <v>653</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>866</v>
+        <v>875</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>867</v>
+        <v>876</v>
       </c>
       <c r="D7" s="4"/>
     </row>
@@ -4479,10 +4506,10 @@
         <v>460</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>868</v>
+        <v>877</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>869</v>
+        <v>878</v>
       </c>
       <c r="D8" s="4"/>
     </row>
@@ -4491,10 +4518,10 @@
         <v>463</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>870</v>
+        <v>879</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>871</v>
+        <v>880</v>
       </c>
       <c r="D9" s="4"/>
     </row>
@@ -4503,10 +4530,10 @@
         <v>654</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>872</v>
+        <v>881</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>873</v>
+        <v>882</v>
       </c>
       <c r="D10" s="4"/>
     </row>
@@ -4515,10 +4542,10 @@
         <v>655</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>874</v>
+        <v>883</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>875</v>
+        <v>884</v>
       </c>
       <c r="D11" s="4"/>
     </row>
@@ -4527,10 +4554,10 @@
         <v>656</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>876</v>
+        <v>885</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>877</v>
+        <v>886</v>
       </c>
       <c r="D12" s="4"/>
     </row>
@@ -4539,10 +4566,10 @@
         <v>657</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>874</v>
+        <v>883</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>878</v>
+        <v>887</v>
       </c>
       <c r="D13" s="4"/>
     </row>
@@ -4551,10 +4578,10 @@
         <v>658</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>879</v>
+        <v>888</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>880</v>
+        <v>889</v>
       </c>
       <c r="D14" s="4"/>
     </row>
@@ -4563,10 +4590,10 @@
         <v>659</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>881</v>
+        <v>890</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>882</v>
+        <v>891</v>
       </c>
       <c r="D15" s="4"/>
     </row>
@@ -4575,10 +4602,10 @@
         <v>660</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>883</v>
+        <v>892</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>884</v>
+        <v>893</v>
       </c>
       <c r="D16" s="4"/>
     </row>
@@ -4587,10 +4614,10 @@
         <v>661</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>874</v>
+        <v>883</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>885</v>
+        <v>894</v>
       </c>
       <c r="D17" s="4"/>
     </row>
@@ -4599,10 +4626,10 @@
         <v>662</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>874</v>
+        <v>883</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>886</v>
+        <v>895</v>
       </c>
       <c r="D18" s="4"/>
     </row>
@@ -4611,10 +4638,10 @@
         <v>663</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>887</v>
+        <v>896</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>888</v>
+        <v>897</v>
       </c>
       <c r="D19" s="4"/>
     </row>
@@ -4623,10 +4650,10 @@
         <v>94</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>876</v>
+        <v>885</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>889</v>
+        <v>898</v>
       </c>
       <c r="D20" s="4"/>
     </row>
@@ -4635,16 +4662,16 @@
         <v>664</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>890</v>
+        <v>899</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>891</v>
+        <v>900</v>
       </c>
       <c r="D21" s="4"/>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="5" t="s">
-        <v>892</v>
+        <v>901</v>
       </c>
       <c r="B23" s="5"/>
       <c r="C23" s="5"/>
@@ -4652,7 +4679,7 @@
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="4" t="s">
-        <v>893</v>
+        <v>902</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -4660,7 +4687,7 @@
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="4" t="s">
-        <v>894</v>
+        <v>903</v>
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -4668,7 +4695,7 @@
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="4" t="s">
-        <v>895</v>
+        <v>904</v>
       </c>
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
@@ -4676,7 +4703,7 @@
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="4" t="s">
-        <v>896</v>
+        <v>905</v>
       </c>
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
@@ -4684,7 +4711,7 @@
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="4" t="s">
-        <v>897</v>
+        <v>906</v>
       </c>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
@@ -4692,7 +4719,7 @@
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="4" t="s">
-        <v>898</v>
+        <v>907</v>
       </c>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -4700,7 +4727,7 @@
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="4" t="s">
-        <v>899</v>
+        <v>908</v>
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -4708,7 +4735,7 @@
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="5" t="s">
-        <v>900</v>
+        <v>909</v>
       </c>
       <c r="B32" s="5"/>
       <c r="C32" s="5"/>
@@ -4716,7 +4743,7 @@
     </row>
     <row r="33" spans="1:4">
       <c r="A33" s="4" t="s">
-        <v>901</v>
+        <v>910</v>
       </c>
       <c r="B33" s="4"/>
       <c r="C33" s="4"/>
@@ -4724,7 +4751,7 @@
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="4" t="s">
-        <v>902</v>
+        <v>911</v>
       </c>
       <c r="B34" s="4"/>
       <c r="C34" s="4"/>
@@ -4732,7 +4759,7 @@
     </row>
     <row r="35" spans="1:4">
       <c r="A35" s="4" t="s">
-        <v>903</v>
+        <v>912</v>
       </c>
       <c r="B35" s="4"/>
       <c r="C35" s="4"/>
@@ -4740,7 +4767,7 @@
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="4" t="s">
-        <v>904</v>
+        <v>913</v>
       </c>
       <c r="B36" s="4"/>
       <c r="C36" s="4"/>
@@ -4748,7 +4775,7 @@
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="4" t="s">
-        <v>905</v>
+        <v>914</v>
       </c>
       <c r="B37" s="4"/>
       <c r="C37" s="4"/>
@@ -8854,7 +8881,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q49"/>
+  <dimension ref="A1:Q60"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -10925,6 +10952,476 @@
       </c>
       <c r="Q49" s="6">
         <f>IF($B49="","",$B49&amp;"_W"&amp;$C49)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:17">
+      <c r="A50" s="25">
+        <v>46235</v>
+      </c>
+      <c r="B50" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C50" s="6">
+        <v>2</v>
+      </c>
+      <c r="D50" s="6" t="s">
+        <v>620</v>
+      </c>
+      <c r="E50" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D50,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F50" s="6" t="s">
+        <v>665</v>
+      </c>
+      <c r="G50" s="6">
+        <v>3</v>
+      </c>
+      <c r="I50" s="6">
+        <v>0</v>
+      </c>
+      <c r="L50" s="6">
+        <v>4</v>
+      </c>
+      <c r="M50" s="6">
+        <v>5</v>
+      </c>
+      <c r="O50" s="6">
+        <v>5</v>
+      </c>
+      <c r="P50" s="4" t="s">
+        <v>721</v>
+      </c>
+      <c r="Q50" s="6">
+        <f>IF($B50="","",$B50&amp;"_W"&amp;$C50)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:17">
+      <c r="A51" s="25">
+        <v>46235</v>
+      </c>
+      <c r="B51" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C51" s="6">
+        <v>2</v>
+      </c>
+      <c r="D51" s="6" t="s">
+        <v>620</v>
+      </c>
+      <c r="E51" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D51,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F51" s="6" t="s">
+        <v>667</v>
+      </c>
+      <c r="G51" s="6">
+        <v>3</v>
+      </c>
+      <c r="I51" s="6">
+        <v>0</v>
+      </c>
+      <c r="L51" s="6">
+        <v>3</v>
+      </c>
+      <c r="M51" s="6">
+        <v>3</v>
+      </c>
+      <c r="O51" s="6">
+        <v>5</v>
+      </c>
+      <c r="P51" s="4" t="s">
+        <v>722</v>
+      </c>
+      <c r="Q51" s="6">
+        <f>IF($B51="","",$B51&amp;"_W"&amp;$C51)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:17">
+      <c r="A52" s="25">
+        <v>46235</v>
+      </c>
+      <c r="B52" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C52" s="6">
+        <v>2</v>
+      </c>
+      <c r="D52" s="6" t="s">
+        <v>626</v>
+      </c>
+      <c r="E52" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D52,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F52" s="6" t="s">
+        <v>665</v>
+      </c>
+      <c r="G52" s="6">
+        <v>3</v>
+      </c>
+      <c r="I52" s="6">
+        <v>0</v>
+      </c>
+      <c r="L52" s="6">
+        <v>3</v>
+      </c>
+      <c r="M52" s="6">
+        <v>5</v>
+      </c>
+      <c r="O52" s="6">
+        <v>5</v>
+      </c>
+      <c r="P52" s="4" t="s">
+        <v>723</v>
+      </c>
+      <c r="Q52" s="6">
+        <f>IF($B52="","",$B52&amp;"_W"&amp;$C52)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:17">
+      <c r="A53" s="25">
+        <v>46235</v>
+      </c>
+      <c r="B53" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C53" s="6">
+        <v>2</v>
+      </c>
+      <c r="D53" s="6" t="s">
+        <v>626</v>
+      </c>
+      <c r="E53" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D53,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F53" s="6" t="s">
+        <v>667</v>
+      </c>
+      <c r="G53" s="6">
+        <v>3</v>
+      </c>
+      <c r="I53" s="6">
+        <v>0</v>
+      </c>
+      <c r="L53" s="6">
+        <v>2</v>
+      </c>
+      <c r="M53" s="6">
+        <v>3</v>
+      </c>
+      <c r="O53" s="6">
+        <v>5</v>
+      </c>
+      <c r="P53" s="4" t="s">
+        <v>724</v>
+      </c>
+      <c r="Q53" s="6">
+        <f>IF($B53="","",$B53&amp;"_W"&amp;$C53)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:17">
+      <c r="A54" s="25">
+        <v>46235</v>
+      </c>
+      <c r="B54" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C54" s="6">
+        <v>2</v>
+      </c>
+      <c r="D54" s="6" t="s">
+        <v>623</v>
+      </c>
+      <c r="E54" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D54,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F54" s="6" t="s">
+        <v>665</v>
+      </c>
+      <c r="G54" s="6">
+        <v>2</v>
+      </c>
+      <c r="I54" s="6">
+        <v>0</v>
+      </c>
+      <c r="L54" s="6">
+        <v>3</v>
+      </c>
+      <c r="M54" s="6">
+        <v>5</v>
+      </c>
+      <c r="O54" s="6">
+        <v>5</v>
+      </c>
+      <c r="P54" s="4" t="s">
+        <v>725</v>
+      </c>
+      <c r="Q54" s="6">
+        <f>IF($B54="","",$B54&amp;"_W"&amp;$C54)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:17">
+      <c r="A55" s="25">
+        <v>46235</v>
+      </c>
+      <c r="B55" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C55" s="6">
+        <v>2</v>
+      </c>
+      <c r="D55" s="6" t="s">
+        <v>623</v>
+      </c>
+      <c r="E55" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D55,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F55" s="6" t="s">
+        <v>667</v>
+      </c>
+      <c r="G55" s="6">
+        <v>2</v>
+      </c>
+      <c r="I55" s="6">
+        <v>0</v>
+      </c>
+      <c r="L55" s="6">
+        <v>2</v>
+      </c>
+      <c r="M55" s="6">
+        <v>5</v>
+      </c>
+      <c r="O55" s="6">
+        <v>5</v>
+      </c>
+      <c r="P55" s="4" t="s">
+        <v>726</v>
+      </c>
+      <c r="Q55" s="6">
+        <f>IF($B55="","",$B55&amp;"_W"&amp;$C55)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:17">
+      <c r="A56" s="25">
+        <v>46235</v>
+      </c>
+      <c r="B56" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C56" s="6">
+        <v>2</v>
+      </c>
+      <c r="D56" s="6" t="s">
+        <v>518</v>
+      </c>
+      <c r="E56" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D56,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F56" s="6" t="s">
+        <v>672</v>
+      </c>
+      <c r="G56" s="6">
+        <v>3</v>
+      </c>
+      <c r="H56" s="4" t="s">
+        <v>686</v>
+      </c>
+      <c r="I56" s="6">
+        <v>100</v>
+      </c>
+      <c r="J56" s="6">
+        <v>7</v>
+      </c>
+      <c r="O56" s="6">
+        <v>5</v>
+      </c>
+      <c r="P56" s="4" t="s">
+        <v>727</v>
+      </c>
+      <c r="Q56" s="6">
+        <f>IF($B56="","",$B56&amp;"_W"&amp;$C56)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:17">
+      <c r="A57" s="25">
+        <v>46235</v>
+      </c>
+      <c r="B57" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C57" s="6">
+        <v>2</v>
+      </c>
+      <c r="D57" s="6" t="s">
+        <v>515</v>
+      </c>
+      <c r="E57" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D57,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F57" s="6" t="s">
+        <v>672</v>
+      </c>
+      <c r="G57" s="6">
+        <v>3</v>
+      </c>
+      <c r="H57" s="4" t="s">
+        <v>688</v>
+      </c>
+      <c r="I57" s="6">
+        <v>70</v>
+      </c>
+      <c r="J57" s="6">
+        <v>7</v>
+      </c>
+      <c r="O57" s="6">
+        <v>5</v>
+      </c>
+      <c r="Q57" s="6">
+        <f>IF($B57="","",$B57&amp;"_W"&amp;$C57)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:17">
+      <c r="A58" s="25">
+        <v>46235</v>
+      </c>
+      <c r="B58" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C58" s="6">
+        <v>2</v>
+      </c>
+      <c r="D58" s="6" t="s">
+        <v>529</v>
+      </c>
+      <c r="E58" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D58,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F58" s="6" t="s">
+        <v>672</v>
+      </c>
+      <c r="G58" s="6">
+        <v>3</v>
+      </c>
+      <c r="H58" s="4" t="s">
+        <v>677</v>
+      </c>
+      <c r="I58" s="6">
+        <v>30</v>
+      </c>
+      <c r="J58" s="6">
+        <v>7</v>
+      </c>
+      <c r="O58" s="6">
+        <v>5</v>
+      </c>
+      <c r="P58" s="4" t="s">
+        <v>728</v>
+      </c>
+      <c r="Q58" s="6">
+        <f>IF($B58="","",$B58&amp;"_W"&amp;$C58)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:17">
+      <c r="A59" s="25">
+        <v>46235</v>
+      </c>
+      <c r="B59" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C59" s="6">
+        <v>2</v>
+      </c>
+      <c r="D59" s="6" t="s">
+        <v>525</v>
+      </c>
+      <c r="E59" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D59,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F59" s="6" t="s">
+        <v>672</v>
+      </c>
+      <c r="G59" s="6">
+        <v>2</v>
+      </c>
+      <c r="H59" s="4" t="s">
+        <v>677</v>
+      </c>
+      <c r="I59" s="6">
+        <v>2</v>
+      </c>
+      <c r="J59" s="6">
+        <v>7</v>
+      </c>
+      <c r="O59" s="6">
+        <v>5</v>
+      </c>
+      <c r="P59" s="4" t="s">
+        <v>729</v>
+      </c>
+      <c r="Q59" s="6">
+        <f>IF($B59="","",$B59&amp;"_W"&amp;$C59)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:17">
+      <c r="A60" s="25">
+        <v>46235</v>
+      </c>
+      <c r="B60" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C60" s="6">
+        <v>2</v>
+      </c>
+      <c r="D60" s="6" t="s">
+        <v>601</v>
+      </c>
+      <c r="E60" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D60,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F60" s="6" t="s">
+        <v>672</v>
+      </c>
+      <c r="G60" s="6">
+        <v>3</v>
+      </c>
+      <c r="H60" s="4" t="s">
+        <v>691</v>
+      </c>
+      <c r="J60" s="6">
+        <v>7</v>
+      </c>
+      <c r="M60" s="6">
+        <v>30</v>
+      </c>
+      <c r="O60" s="6">
+        <v>5</v>
+      </c>
+      <c r="P60" s="4" t="s">
+        <v>692</v>
+      </c>
+      <c r="Q60" s="6">
+        <f>IF($B60="","",$B60&amp;"_W"&amp;$C60)</f>
         <v>0</v>
       </c>
     </row>
@@ -11002,7 +11499,7 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>721</v>
+        <v>730</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -11013,20 +11510,20 @@
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="5" t="s">
-        <v>722</v>
+        <v>731</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="9" t="s">
-        <v>723</v>
+        <v>732</v>
       </c>
       <c r="B4" s="11">
         <v>81</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>731</v>
+        <v>740</v>
       </c>
       <c r="D4" s="4"/>
       <c r="E4" s="4"/>
@@ -11035,21 +11532,21 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="9" t="s">
-        <v>724</v>
+        <v>733</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>725</v>
+        <v>734</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="9" t="s">
-        <v>726</v>
+        <v>735</v>
       </c>
       <c r="B6" s="11">
         <v>2.2</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>732</v>
+        <v>741</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
@@ -11058,7 +11555,7 @@
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="9" t="s">
-        <v>727</v>
+        <v>736</v>
       </c>
       <c r="B7" s="11">
         <v>0.9</v>
@@ -11066,7 +11563,7 @@
     </row>
     <row r="8" spans="1:7">
       <c r="A8" s="9" t="s">
-        <v>728</v>
+        <v>737</v>
       </c>
       <c r="B8" s="10">
         <v>2700</v>
@@ -11074,7 +11571,7 @@
     </row>
     <row r="9" spans="1:7">
       <c r="A9" s="9" t="s">
-        <v>729</v>
+        <v>738</v>
       </c>
       <c r="B9" s="10">
         <f>ROUND(BW*B6,0)</f>
@@ -11083,7 +11580,7 @@
     </row>
     <row r="10" spans="1:7">
       <c r="A10" s="9" t="s">
-        <v>730</v>
+        <v>739</v>
       </c>
       <c r="B10" s="10">
         <f>ROUND(BW*B7,0)</f>
@@ -11092,7 +11589,7 @@
     </row>
     <row r="12" spans="1:7">
       <c r="A12" s="5" t="s">
-        <v>733</v>
+        <v>742</v>
       </c>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -11106,27 +11603,27 @@
         <v>87</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>734</v>
+        <v>743</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>735</v>
+        <v>744</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>736</v>
+        <v>745</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>737</v>
+        <v>746</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>738</v>
+        <v>747</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>739</v>
+        <v>748</v>
       </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" s="9" t="s">
-        <v>740</v>
+        <v>749</v>
       </c>
       <c r="B14" s="26">
         <v>250</v>
@@ -11148,7 +11645,7 @@
         <v>0</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>741</v>
+        <v>750</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -11175,12 +11672,12 @@
         <v>0</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>742</v>
+        <v>751</v>
       </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" s="9" t="s">
-        <v>743</v>
+        <v>752</v>
       </c>
       <c r="B16" s="26">
         <v>200</v>
@@ -11202,12 +11699,12 @@
         <v>0</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>744</v>
+        <v>753</v>
       </c>
     </row>
     <row r="17" spans="1:7">
       <c r="A17" s="9" t="s">
-        <v>745</v>
+        <v>754</v>
       </c>
       <c r="B17" s="26">
         <v>150</v>
@@ -11229,12 +11726,12 @@
         <v>0</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>746</v>
+        <v>755</v>
       </c>
     </row>
     <row r="18" spans="1:7">
       <c r="A18" s="9" t="s">
-        <v>747</v>
+        <v>756</v>
       </c>
       <c r="B18" s="26">
         <v>100</v>
@@ -11256,7 +11753,7 @@
         <v>0</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>748</v>
+        <v>757</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -11283,12 +11780,12 @@
         <v>0</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>749</v>
+        <v>758</v>
       </c>
     </row>
     <row r="21" spans="1:7">
       <c r="A21" s="5" t="s">
-        <v>750</v>
+        <v>759</v>
       </c>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
@@ -11299,7 +11796,7 @@
     </row>
     <row r="22" spans="1:7">
       <c r="A22" s="4" t="s">
-        <v>751</v>
+        <v>760</v>
       </c>
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
@@ -11310,7 +11807,7 @@
     </row>
     <row r="23" spans="1:7">
       <c r="A23" s="4" t="s">
-        <v>752</v>
+        <v>761</v>
       </c>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
@@ -11321,7 +11818,7 @@
     </row>
     <row r="24" spans="1:7">
       <c r="A24" s="4" t="s">
-        <v>753</v>
+        <v>762</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -11332,7 +11829,7 @@
     </row>
     <row r="25" spans="1:7">
       <c r="A25" s="4" t="s">
-        <v>754</v>
+        <v>763</v>
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -11377,7 +11874,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>755</v>
+        <v>764</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -11386,7 +11883,7 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="5" t="s">
-        <v>756</v>
+        <v>765</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
@@ -11395,126 +11892,126 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="7" t="s">
-        <v>757</v>
+        <v>766</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>758</v>
+        <v>767</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>759</v>
+        <v>768</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>760</v>
+        <v>769</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>761</v>
+        <v>770</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="9" t="s">
-        <v>762</v>
+        <v>771</v>
       </c>
       <c r="B5" s="22" t="s">
-        <v>763</v>
+        <v>772</v>
       </c>
       <c r="C5" s="27" t="s">
-        <v>764</v>
+        <v>773</v>
       </c>
       <c r="D5" s="28" t="s">
-        <v>765</v>
+        <v>774</v>
       </c>
       <c r="E5" s="29" t="s">
-        <v>766</v>
+        <v>775</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="9" t="s">
-        <v>767</v>
+        <v>776</v>
       </c>
       <c r="B6" s="22" t="s">
-        <v>768</v>
+        <v>777</v>
       </c>
       <c r="C6" s="27" t="s">
-        <v>769</v>
+        <v>778</v>
       </c>
       <c r="D6" s="28" t="s">
-        <v>770</v>
+        <v>779</v>
       </c>
       <c r="E6" s="29" t="s">
-        <v>771</v>
+        <v>780</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="9" t="s">
-        <v>772</v>
+        <v>781</v>
       </c>
       <c r="B7" s="22" t="s">
-        <v>773</v>
+        <v>782</v>
       </c>
       <c r="C7" s="27" t="s">
-        <v>774</v>
+        <v>783</v>
       </c>
       <c r="D7" s="28" t="s">
-        <v>775</v>
+        <v>784</v>
       </c>
       <c r="E7" s="29" t="s">
-        <v>776</v>
+        <v>785</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="9" t="s">
-        <v>777</v>
+        <v>786</v>
       </c>
       <c r="B8" s="22" t="s">
-        <v>778</v>
+        <v>787</v>
       </c>
       <c r="C8" s="27" t="s">
-        <v>779</v>
+        <v>788</v>
       </c>
       <c r="D8" s="28" t="s">
-        <v>780</v>
+        <v>789</v>
       </c>
       <c r="E8" s="29" t="s">
-        <v>781</v>
+        <v>790</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="9" t="s">
-        <v>782</v>
+        <v>791</v>
       </c>
       <c r="B9" s="22" t="s">
-        <v>783</v>
+        <v>792</v>
       </c>
       <c r="C9" s="27" t="s">
-        <v>784</v>
+        <v>793</v>
       </c>
       <c r="D9" s="28" t="s">
-        <v>785</v>
+        <v>794</v>
       </c>
       <c r="E9" s="29" t="s">
-        <v>786</v>
+        <v>795</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="9" t="s">
-        <v>787</v>
+        <v>796</v>
       </c>
       <c r="B10" s="22" t="s">
-        <v>788</v>
+        <v>797</v>
       </c>
       <c r="C10" s="27" t="s">
-        <v>789</v>
+        <v>798</v>
       </c>
       <c r="D10" s="28" t="s">
-        <v>790</v>
+        <v>799</v>
       </c>
       <c r="E10" s="29" t="s">
-        <v>791</v>
+        <v>800</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="5" t="s">
-        <v>792</v>
+        <v>801</v>
       </c>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -11586,7 +12083,7 @@
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="5" t="s">
-        <v>793</v>
+        <v>802</v>
       </c>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
@@ -11595,36 +12092,36 @@
     </row>
     <row r="22" spans="1:5">
       <c r="A22" s="7" t="s">
-        <v>794</v>
+        <v>803</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>795</v>
+        <v>804</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>796</v>
+        <v>805</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>797</v>
+        <v>806</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>798</v>
+        <v>807</v>
       </c>
     </row>
     <row r="23" spans="1:5">
       <c r="A23" s="14" t="s">
-        <v>799</v>
+        <v>808</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>800</v>
+        <v>809</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>801</v>
+        <v>810</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>802</v>
+        <v>811</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>803</v>
+        <v>812</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -11632,16 +12129,16 @@
         <v>48</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>804</v>
+        <v>813</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>805</v>
+        <v>814</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>806</v>
+        <v>815</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>807</v>
+        <v>816</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -11649,16 +12146,16 @@
         <v>35</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>808</v>
+        <v>817</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>809</v>
+        <v>818</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>810</v>
+        <v>819</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>811</v>
+        <v>820</v>
       </c>
     </row>
     <row r="26" spans="1:5">
@@ -11666,21 +12163,21 @@
         <v>38</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>812</v>
+        <v>821</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>813</v>
+        <v>822</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>814</v>
+        <v>823</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>815</v>
+        <v>824</v>
       </c>
     </row>
     <row r="28" spans="1:5">
       <c r="A28" s="5" t="s">
-        <v>816</v>
+        <v>825</v>
       </c>
       <c r="B28" s="5"/>
       <c r="C28" s="5"/>
@@ -11689,7 +12186,7 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" s="4" t="s">
-        <v>817</v>
+        <v>826</v>
       </c>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -11698,7 +12195,7 @@
     </row>
     <row r="30" spans="1:5">
       <c r="A30" s="4" t="s">
-        <v>818</v>
+        <v>827</v>
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -11707,7 +12204,7 @@
     </row>
     <row r="31" spans="1:5">
       <c r="A31" s="4" t="s">
-        <v>819</v>
+        <v>828</v>
       </c>
       <c r="B31" s="4"/>
       <c r="C31" s="4"/>
@@ -11716,7 +12213,7 @@
     </row>
     <row r="32" spans="1:5">
       <c r="A32" s="4" t="s">
-        <v>820</v>
+        <v>829</v>
       </c>
       <c r="B32" s="4"/>
       <c r="C32" s="4"/>
@@ -11725,7 +12222,7 @@
     </row>
     <row r="33" spans="1:5">
       <c r="A33" s="4" t="s">
-        <v>821</v>
+        <v>830</v>
       </c>
       <c r="B33" s="4"/>
       <c r="C33" s="4"/>
@@ -11749,98 +12246,98 @@
         <v>447</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>822</v>
+        <v>831</v>
       </c>
       <c r="D36" s="7"/>
       <c r="E36" s="7"/>
     </row>
     <row r="37" spans="1:5">
       <c r="A37" s="4" t="s">
-        <v>823</v>
+        <v>832</v>
       </c>
       <c r="B37" s="24" t="s">
-        <v>824</v>
+        <v>833</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>825</v>
+        <v>834</v>
       </c>
       <c r="D37" s="4"/>
       <c r="E37" s="4"/>
     </row>
     <row r="38" spans="1:5">
       <c r="A38" s="4" t="s">
-        <v>826</v>
+        <v>835</v>
       </c>
       <c r="B38" s="24" t="s">
-        <v>827</v>
+        <v>836</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>828</v>
+        <v>837</v>
       </c>
       <c r="D38" s="4"/>
       <c r="E38" s="4"/>
     </row>
     <row r="39" spans="1:5">
       <c r="A39" s="4" t="s">
-        <v>829</v>
+        <v>838</v>
       </c>
       <c r="B39" s="24" t="s">
         <v>455</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>830</v>
+        <v>839</v>
       </c>
       <c r="D39" s="4"/>
       <c r="E39" s="4"/>
     </row>
     <row r="40" spans="1:5">
       <c r="A40" s="4" t="s">
-        <v>831</v>
+        <v>840</v>
       </c>
       <c r="B40" s="24" t="s">
-        <v>832</v>
+        <v>841</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>833</v>
+        <v>842</v>
       </c>
       <c r="D40" s="4"/>
       <c r="E40" s="4"/>
     </row>
     <row r="41" spans="1:5">
       <c r="A41" s="4" t="s">
-        <v>831</v>
+        <v>840</v>
       </c>
       <c r="B41" s="24" t="s">
-        <v>834</v>
+        <v>843</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>835</v>
+        <v>844</v>
       </c>
       <c r="D41" s="4"/>
       <c r="E41" s="4"/>
     </row>
     <row r="42" spans="1:5">
       <c r="A42" s="4" t="s">
-        <v>836</v>
+        <v>845</v>
       </c>
       <c r="B42" s="24" t="s">
-        <v>837</v>
+        <v>846</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>838</v>
+        <v>847</v>
       </c>
       <c r="D42" s="4"/>
       <c r="E42" s="4"/>
     </row>
     <row r="43" spans="1:5">
       <c r="A43" s="4" t="s">
-        <v>839</v>
+        <v>848</v>
       </c>
       <c r="B43" s="24" t="s">
-        <v>840</v>
+        <v>849</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>841</v>
+        <v>850</v>
       </c>
       <c r="D43" s="4"/>
       <c r="E43" s="4"/>

</xml_diff>

<commit_message>
Log B7 W2 T3 (legs rebound: BSS 40kg@RPE7; 2x50s freestanding handstand endurance)
</commit_message>
<xml_diff>
--- a/Training_3_B7.xlsx
+++ b/Training_3_B7.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1786" uniqueCount="936">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1816" uniqueCount="941">
   <si>
     <t>B7 — Performance-Block Dashboard (Advanced OAHS)</t>
   </si>
@@ -2283,6 +2283,21 @@
   </si>
   <si>
     <t>DB bent-over 2 kg (Maschine besetzt)</t>
+  </si>
+  <si>
+    <t>Taegliche Mikrodosis A-C gemacht (Fingerdruck-Kalibrierung + Weight-Shift)</t>
+  </si>
+  <si>
+    <t>40 kg jetzt @ RPE 7 (vorher 40 = RPE 8) -&gt; Rebound</t>
+  </si>
+  <si>
+    <t>80 kg (75 gabs nicht) -&gt; RPE 8, leicht ueber Cap; naechstes Mal 80x10</t>
+  </si>
+  <si>
+    <t>2 Runden Core-Zirkel (Anti-Bewegung)</t>
+  </si>
+  <si>
+    <t>Handstand-Endurance FREISTEHEND 2x50s (stark!)</t>
   </si>
   <si>
     <t>B7 — Nutrition Targets (Maintenance, KEIN Defizit)</t>
@@ -4093,7 +4108,7 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>872</v>
+        <v>877</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4103,7 +4118,7 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="12" t="s">
-        <v>873</v>
+        <v>878</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -4128,12 +4143,12 @@
         <v>155</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>874</v>
+        <v>879</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="9" t="s">
-        <v>875</v>
+        <v>880</v>
       </c>
       <c r="B4" s="11">
         <f>SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Skill90",'B7_Training_Log'!$C$2:$C$1000,1)+SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Planche",'B7_Training_Log'!$C$2:$C$1000,1)+SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Push",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4158,7 +4173,7 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="9" t="s">
-        <v>876</v>
+        <v>881</v>
       </c>
       <c r="B5" s="11">
         <f>SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Pull",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4183,7 +4198,7 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="9" t="s">
-        <v>877</v>
+        <v>882</v>
       </c>
       <c r="B6" s="11">
         <f>SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Legs",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4208,7 +4223,7 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="9" t="s">
-        <v>878</v>
+        <v>883</v>
       </c>
       <c r="B7" s="10">
         <f>SUMIFS('B7_Training_Log'!$N$2:$N$1000,'B7_Training_Log'!$D$2:$D$1000,"90",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4233,7 +4248,7 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="9" t="s">
-        <v>879</v>
+        <v>884</v>
       </c>
       <c r="B8" s="10">
         <f>COUNTIFS('B7_Training_Log'!$E$2:$E$1000,"SkillOAHS",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4258,7 +4273,7 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="9" t="s">
-        <v>880</v>
+        <v>885</v>
       </c>
       <c r="B9" s="10">
         <f>MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_straddle",'B7_Training_Log'!$F$2:$F$1000,"L",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4283,7 +4298,7 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="9" t="s">
-        <v>881</v>
+        <v>886</v>
       </c>
       <c r="B10" s="10">
         <f>MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_straddle",'B7_Training_Log'!$F$2:$F$1000,"R",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4308,7 +4323,7 @@
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="9" t="s">
-        <v>882</v>
+        <v>887</v>
       </c>
       <c r="B11" s="10">
         <f>MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_diamond",'B7_Training_Log'!$F$2:$F$1000,"L",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4333,7 +4348,7 @@
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="9" t="s">
-        <v>883</v>
+        <v>888</v>
       </c>
       <c r="B12" s="10">
         <f>MAX(MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_flag",'B7_Training_Log'!$C$2:$C$1000,1),MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_figa",'B7_Training_Log'!$C$2:$C$1000,1))</f>
@@ -4358,7 +4373,7 @@
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="9" t="s">
-        <v>884</v>
+        <v>889</v>
       </c>
       <c r="B13" s="11">
         <f>IFERROR(AVERAGEIFS('B7_Training_Log'!$J$2:$J$1000,'B7_Training_Log'!$C$2:$C$1000,1),0)</f>
@@ -4433,7 +4448,7 @@
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="9" t="s">
-        <v>885</v>
+        <v>890</v>
       </c>
       <c r="B16" s="10">
         <f>COUNTIFS('B7_Training_Log'!$K$2:$K$1000,"&gt;=4",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4458,7 +4473,7 @@
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="9" t="s">
-        <v>886</v>
+        <v>891</v>
       </c>
       <c r="B17" s="10">
         <f>COUNTIFS('B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4502,7 +4517,7 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
-        <v>887</v>
+        <v>892</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4510,7 +4525,7 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="5" t="s">
-        <v>888</v>
+        <v>893</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
@@ -4518,13 +4533,13 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="7" t="s">
-        <v>889</v>
+        <v>894</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>890</v>
+        <v>895</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>891</v>
+        <v>896</v>
       </c>
       <c r="D4" s="7"/>
     </row>
@@ -4533,10 +4548,10 @@
         <v>672</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>892</v>
+        <v>897</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>893</v>
+        <v>898</v>
       </c>
       <c r="D5" s="4"/>
     </row>
@@ -4545,10 +4560,10 @@
         <v>673</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>894</v>
+        <v>899</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>895</v>
+        <v>900</v>
       </c>
       <c r="D6" s="4"/>
     </row>
@@ -4557,10 +4572,10 @@
         <v>674</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>896</v>
+        <v>901</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>897</v>
+        <v>902</v>
       </c>
       <c r="D7" s="4"/>
     </row>
@@ -4569,10 +4584,10 @@
         <v>481</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>898</v>
+        <v>903</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>899</v>
+        <v>904</v>
       </c>
       <c r="D8" s="4"/>
     </row>
@@ -4581,10 +4596,10 @@
         <v>484</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>900</v>
+        <v>905</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>901</v>
+        <v>906</v>
       </c>
       <c r="D9" s="4"/>
     </row>
@@ -4593,10 +4608,10 @@
         <v>675</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>902</v>
+        <v>907</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>903</v>
+        <v>908</v>
       </c>
       <c r="D10" s="4"/>
     </row>
@@ -4605,10 +4620,10 @@
         <v>676</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>904</v>
+        <v>909</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>905</v>
+        <v>910</v>
       </c>
       <c r="D11" s="4"/>
     </row>
@@ -4617,10 +4632,10 @@
         <v>677</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>906</v>
+        <v>911</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>907</v>
+        <v>912</v>
       </c>
       <c r="D12" s="4"/>
     </row>
@@ -4629,10 +4644,10 @@
         <v>678</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>904</v>
+        <v>909</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>908</v>
+        <v>913</v>
       </c>
       <c r="D13" s="4"/>
     </row>
@@ -4641,10 +4656,10 @@
         <v>679</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>909</v>
+        <v>914</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>910</v>
+        <v>915</v>
       </c>
       <c r="D14" s="4"/>
     </row>
@@ -4653,10 +4668,10 @@
         <v>680</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>911</v>
+        <v>916</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>912</v>
+        <v>917</v>
       </c>
       <c r="D15" s="4"/>
     </row>
@@ -4665,10 +4680,10 @@
         <v>681</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>913</v>
+        <v>918</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>914</v>
+        <v>919</v>
       </c>
       <c r="D16" s="4"/>
     </row>
@@ -4677,10 +4692,10 @@
         <v>682</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>904</v>
+        <v>909</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>915</v>
+        <v>920</v>
       </c>
       <c r="D17" s="4"/>
     </row>
@@ -4689,10 +4704,10 @@
         <v>683</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>904</v>
+        <v>909</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>916</v>
+        <v>921</v>
       </c>
       <c r="D18" s="4"/>
     </row>
@@ -4701,10 +4716,10 @@
         <v>684</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>917</v>
+        <v>922</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>918</v>
+        <v>923</v>
       </c>
       <c r="D19" s="4"/>
     </row>
@@ -4713,10 +4728,10 @@
         <v>94</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>906</v>
+        <v>911</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>919</v>
+        <v>924</v>
       </c>
       <c r="D20" s="4"/>
     </row>
@@ -4725,16 +4740,16 @@
         <v>685</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>920</v>
+        <v>925</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>921</v>
+        <v>926</v>
       </c>
       <c r="D21" s="4"/>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="5" t="s">
-        <v>922</v>
+        <v>927</v>
       </c>
       <c r="B23" s="5"/>
       <c r="C23" s="5"/>
@@ -4742,7 +4757,7 @@
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="4" t="s">
-        <v>923</v>
+        <v>928</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -4750,7 +4765,7 @@
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="4" t="s">
-        <v>924</v>
+        <v>929</v>
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -4758,7 +4773,7 @@
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="4" t="s">
-        <v>925</v>
+        <v>930</v>
       </c>
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
@@ -4766,7 +4781,7 @@
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="4" t="s">
-        <v>926</v>
+        <v>931</v>
       </c>
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
@@ -4774,7 +4789,7 @@
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="4" t="s">
-        <v>927</v>
+        <v>932</v>
       </c>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
@@ -4782,7 +4797,7 @@
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="4" t="s">
-        <v>928</v>
+        <v>933</v>
       </c>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -4790,7 +4805,7 @@
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="4" t="s">
-        <v>929</v>
+        <v>934</v>
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -4798,7 +4813,7 @@
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="5" t="s">
-        <v>930</v>
+        <v>935</v>
       </c>
       <c r="B32" s="5"/>
       <c r="C32" s="5"/>
@@ -4806,7 +4821,7 @@
     </row>
     <row r="33" spans="1:4">
       <c r="A33" s="4" t="s">
-        <v>931</v>
+        <v>936</v>
       </c>
       <c r="B33" s="4"/>
       <c r="C33" s="4"/>
@@ -4814,7 +4829,7 @@
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="4" t="s">
-        <v>932</v>
+        <v>937</v>
       </c>
       <c r="B34" s="4"/>
       <c r="C34" s="4"/>
@@ -4822,7 +4837,7 @@
     </row>
     <row r="35" spans="1:4">
       <c r="A35" s="4" t="s">
-        <v>933</v>
+        <v>938</v>
       </c>
       <c r="B35" s="4"/>
       <c r="C35" s="4"/>
@@ -4830,7 +4845,7 @@
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="4" t="s">
-        <v>934</v>
+        <v>939</v>
       </c>
       <c r="B36" s="4"/>
       <c r="C36" s="4"/>
@@ -4838,7 +4853,7 @@
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="4" t="s">
-        <v>935</v>
+        <v>940</v>
       </c>
       <c r="B37" s="4"/>
       <c r="C37" s="4"/>
@@ -9066,7 +9081,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q60"/>
+  <dimension ref="A1:Q67"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -11607,6 +11622,286 @@
       </c>
       <c r="Q60" s="6">
         <f>IF($B60="","",$B60&amp;"_W"&amp;$C60)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:17">
+      <c r="A61" s="25">
+        <v>46236</v>
+      </c>
+      <c r="B61" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="C61" s="6">
+        <v>2</v>
+      </c>
+      <c r="D61" s="6" t="s">
+        <v>495</v>
+      </c>
+      <c r="E61" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D61,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F61" s="6" t="s">
+        <v>693</v>
+      </c>
+      <c r="G61" s="6">
+        <v>1</v>
+      </c>
+      <c r="I61" s="6">
+        <v>0</v>
+      </c>
+      <c r="O61" s="6">
+        <v>4</v>
+      </c>
+      <c r="P61" s="4" t="s">
+        <v>751</v>
+      </c>
+      <c r="Q61" s="6">
+        <f>IF($B61="","",$B61&amp;"_W"&amp;$C61)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:17">
+      <c r="A62" s="25">
+        <v>46236</v>
+      </c>
+      <c r="B62" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="C62" s="6">
+        <v>2</v>
+      </c>
+      <c r="D62" s="6" t="s">
+        <v>589</v>
+      </c>
+      <c r="E62" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D62,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F62" s="6" t="s">
+        <v>693</v>
+      </c>
+      <c r="G62" s="6">
+        <v>3</v>
+      </c>
+      <c r="H62" s="4" t="s">
+        <v>709</v>
+      </c>
+      <c r="I62" s="6">
+        <v>40</v>
+      </c>
+      <c r="J62" s="6">
+        <v>7</v>
+      </c>
+      <c r="O62" s="6">
+        <v>4</v>
+      </c>
+      <c r="P62" s="4" t="s">
+        <v>752</v>
+      </c>
+      <c r="Q62" s="6">
+        <f>IF($B62="","",$B62&amp;"_W"&amp;$C62)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:17">
+      <c r="A63" s="25">
+        <v>46236</v>
+      </c>
+      <c r="B63" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="C63" s="6">
+        <v>2</v>
+      </c>
+      <c r="D63" s="6" t="s">
+        <v>592</v>
+      </c>
+      <c r="E63" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D63,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F63" s="6" t="s">
+        <v>693</v>
+      </c>
+      <c r="G63" s="6">
+        <v>3</v>
+      </c>
+      <c r="H63" s="4" t="s">
+        <v>698</v>
+      </c>
+      <c r="I63" s="6">
+        <v>80</v>
+      </c>
+      <c r="J63" s="6">
+        <v>8</v>
+      </c>
+      <c r="O63" s="6">
+        <v>4</v>
+      </c>
+      <c r="P63" s="4" t="s">
+        <v>753</v>
+      </c>
+      <c r="Q63" s="6">
+        <f>IF($B63="","",$B63&amp;"_W"&amp;$C63)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:17">
+      <c r="A64" s="25">
+        <v>46236</v>
+      </c>
+      <c r="B64" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="C64" s="6">
+        <v>2</v>
+      </c>
+      <c r="D64" s="6" t="s">
+        <v>595</v>
+      </c>
+      <c r="E64" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D64,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F64" s="6" t="s">
+        <v>693</v>
+      </c>
+      <c r="G64" s="6">
+        <v>3</v>
+      </c>
+      <c r="H64" s="4" t="s">
+        <v>707</v>
+      </c>
+      <c r="I64" s="6">
+        <v>45</v>
+      </c>
+      <c r="J64" s="6">
+        <v>7</v>
+      </c>
+      <c r="O64" s="6">
+        <v>4</v>
+      </c>
+      <c r="Q64" s="6">
+        <f>IF($B64="","",$B64&amp;"_W"&amp;$C64)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:17">
+      <c r="A65" s="25">
+        <v>46236</v>
+      </c>
+      <c r="B65" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="C65" s="6">
+        <v>2</v>
+      </c>
+      <c r="D65" s="6" t="s">
+        <v>605</v>
+      </c>
+      <c r="E65" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D65,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F65" s="6" t="s">
+        <v>693</v>
+      </c>
+      <c r="G65" s="6">
+        <v>3</v>
+      </c>
+      <c r="H65" s="4" t="s">
+        <v>710</v>
+      </c>
+      <c r="I65" s="6">
+        <v>80</v>
+      </c>
+      <c r="J65" s="6">
+        <v>7</v>
+      </c>
+      <c r="O65" s="6">
+        <v>4</v>
+      </c>
+      <c r="Q65" s="6">
+        <f>IF($B65="","",$B65&amp;"_W"&amp;$C65)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="1:17">
+      <c r="A66" s="25">
+        <v>46236</v>
+      </c>
+      <c r="B66" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="C66" s="6">
+        <v>2</v>
+      </c>
+      <c r="D66" s="6" t="s">
+        <v>610</v>
+      </c>
+      <c r="E66" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D66,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F66" s="6" t="s">
+        <v>693</v>
+      </c>
+      <c r="G66" s="6">
+        <v>2</v>
+      </c>
+      <c r="O66" s="6">
+        <v>4</v>
+      </c>
+      <c r="P66" s="4" t="s">
+        <v>754</v>
+      </c>
+      <c r="Q66" s="6">
+        <f>IF($B66="","",$B66&amp;"_W"&amp;$C66)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:17">
+      <c r="A67" s="25">
+        <v>46236</v>
+      </c>
+      <c r="B67" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="C67" s="6">
+        <v>2</v>
+      </c>
+      <c r="D67" s="6" t="s">
+        <v>504</v>
+      </c>
+      <c r="E67" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D67,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F67" s="6" t="s">
+        <v>693</v>
+      </c>
+      <c r="G67" s="6">
+        <v>2</v>
+      </c>
+      <c r="I67" s="6">
+        <v>0</v>
+      </c>
+      <c r="L67" s="6">
+        <v>4</v>
+      </c>
+      <c r="M67" s="6">
+        <v>50</v>
+      </c>
+      <c r="O67" s="6">
+        <v>4</v>
+      </c>
+      <c r="P67" s="4" t="s">
+        <v>755</v>
+      </c>
+      <c r="Q67" s="6">
+        <f>IF($B67="","",$B67&amp;"_W"&amp;$C67)</f>
         <v>0</v>
       </c>
     </row>
@@ -11684,7 +11979,7 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>751</v>
+        <v>756</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -11695,20 +11990,20 @@
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="5" t="s">
-        <v>752</v>
+        <v>757</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="9" t="s">
-        <v>753</v>
+        <v>758</v>
       </c>
       <c r="B4" s="11">
         <v>81</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>761</v>
+        <v>766</v>
       </c>
       <c r="D4" s="4"/>
       <c r="E4" s="4"/>
@@ -11717,21 +12012,21 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="9" t="s">
-        <v>754</v>
+        <v>759</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>755</v>
+        <v>760</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="9" t="s">
-        <v>756</v>
+        <v>761</v>
       </c>
       <c r="B6" s="11">
         <v>2.2</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>762</v>
+        <v>767</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
@@ -11740,7 +12035,7 @@
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="9" t="s">
-        <v>757</v>
+        <v>762</v>
       </c>
       <c r="B7" s="11">
         <v>0.9</v>
@@ -11748,7 +12043,7 @@
     </row>
     <row r="8" spans="1:7">
       <c r="A8" s="9" t="s">
-        <v>758</v>
+        <v>763</v>
       </c>
       <c r="B8" s="10">
         <v>2700</v>
@@ -11756,7 +12051,7 @@
     </row>
     <row r="9" spans="1:7">
       <c r="A9" s="9" t="s">
-        <v>759</v>
+        <v>764</v>
       </c>
       <c r="B9" s="10">
         <f>ROUND(BW*B6,0)</f>
@@ -11765,7 +12060,7 @@
     </row>
     <row r="10" spans="1:7">
       <c r="A10" s="9" t="s">
-        <v>760</v>
+        <v>765</v>
       </c>
       <c r="B10" s="10">
         <f>ROUND(BW*B7,0)</f>
@@ -11774,7 +12069,7 @@
     </row>
     <row r="12" spans="1:7">
       <c r="A12" s="5" t="s">
-        <v>763</v>
+        <v>768</v>
       </c>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -11788,27 +12083,27 @@
         <v>87</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>764</v>
+        <v>769</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>765</v>
+        <v>770</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>766</v>
+        <v>771</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>767</v>
+        <v>772</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>768</v>
+        <v>773</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>769</v>
+        <v>774</v>
       </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" s="9" t="s">
-        <v>770</v>
+        <v>775</v>
       </c>
       <c r="B14" s="26">
         <v>250</v>
@@ -11830,7 +12125,7 @@
         <v>0</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>771</v>
+        <v>776</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -11857,12 +12152,12 @@
         <v>0</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>772</v>
+        <v>777</v>
       </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" s="9" t="s">
-        <v>773</v>
+        <v>778</v>
       </c>
       <c r="B16" s="26">
         <v>200</v>
@@ -11884,12 +12179,12 @@
         <v>0</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>774</v>
+        <v>779</v>
       </c>
     </row>
     <row r="17" spans="1:7">
       <c r="A17" s="9" t="s">
-        <v>775</v>
+        <v>780</v>
       </c>
       <c r="B17" s="26">
         <v>150</v>
@@ -11911,12 +12206,12 @@
         <v>0</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>776</v>
+        <v>781</v>
       </c>
     </row>
     <row r="18" spans="1:7">
       <c r="A18" s="9" t="s">
-        <v>777</v>
+        <v>782</v>
       </c>
       <c r="B18" s="26">
         <v>100</v>
@@ -11938,7 +12233,7 @@
         <v>0</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>778</v>
+        <v>783</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -11965,12 +12260,12 @@
         <v>0</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>779</v>
+        <v>784</v>
       </c>
     </row>
     <row r="21" spans="1:7">
       <c r="A21" s="5" t="s">
-        <v>780</v>
+        <v>785</v>
       </c>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
@@ -11981,7 +12276,7 @@
     </row>
     <row r="22" spans="1:7">
       <c r="A22" s="4" t="s">
-        <v>781</v>
+        <v>786</v>
       </c>
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
@@ -11992,7 +12287,7 @@
     </row>
     <row r="23" spans="1:7">
       <c r="A23" s="4" t="s">
-        <v>782</v>
+        <v>787</v>
       </c>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
@@ -12003,7 +12298,7 @@
     </row>
     <row r="24" spans="1:7">
       <c r="A24" s="4" t="s">
-        <v>783</v>
+        <v>788</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -12014,7 +12309,7 @@
     </row>
     <row r="25" spans="1:7">
       <c r="A25" s="4" t="s">
-        <v>784</v>
+        <v>789</v>
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -12059,7 +12354,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>785</v>
+        <v>790</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -12068,7 +12363,7 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="5" t="s">
-        <v>786</v>
+        <v>791</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
@@ -12077,126 +12372,126 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="7" t="s">
-        <v>787</v>
+        <v>792</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>788</v>
+        <v>793</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>789</v>
+        <v>794</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>790</v>
+        <v>795</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>791</v>
+        <v>796</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="9" t="s">
-        <v>792</v>
+        <v>797</v>
       </c>
       <c r="B5" s="22" t="s">
-        <v>793</v>
+        <v>798</v>
       </c>
       <c r="C5" s="27" t="s">
-        <v>794</v>
+        <v>799</v>
       </c>
       <c r="D5" s="28" t="s">
-        <v>795</v>
+        <v>800</v>
       </c>
       <c r="E5" s="29" t="s">
-        <v>796</v>
+        <v>801</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="9" t="s">
-        <v>797</v>
+        <v>802</v>
       </c>
       <c r="B6" s="22" t="s">
-        <v>798</v>
+        <v>803</v>
       </c>
       <c r="C6" s="27" t="s">
-        <v>799</v>
+        <v>804</v>
       </c>
       <c r="D6" s="28" t="s">
-        <v>800</v>
+        <v>805</v>
       </c>
       <c r="E6" s="29" t="s">
-        <v>801</v>
+        <v>806</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="9" t="s">
-        <v>802</v>
+        <v>807</v>
       </c>
       <c r="B7" s="22" t="s">
-        <v>803</v>
+        <v>808</v>
       </c>
       <c r="C7" s="27" t="s">
-        <v>804</v>
+        <v>809</v>
       </c>
       <c r="D7" s="28" t="s">
-        <v>805</v>
+        <v>810</v>
       </c>
       <c r="E7" s="29" t="s">
-        <v>806</v>
+        <v>811</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="9" t="s">
-        <v>807</v>
+        <v>812</v>
       </c>
       <c r="B8" s="22" t="s">
-        <v>808</v>
+        <v>813</v>
       </c>
       <c r="C8" s="27" t="s">
-        <v>809</v>
+        <v>814</v>
       </c>
       <c r="D8" s="28" t="s">
-        <v>810</v>
+        <v>815</v>
       </c>
       <c r="E8" s="29" t="s">
-        <v>811</v>
+        <v>816</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="9" t="s">
-        <v>812</v>
+        <v>817</v>
       </c>
       <c r="B9" s="22" t="s">
-        <v>813</v>
+        <v>818</v>
       </c>
       <c r="C9" s="27" t="s">
-        <v>814</v>
+        <v>819</v>
       </c>
       <c r="D9" s="28" t="s">
-        <v>815</v>
+        <v>820</v>
       </c>
       <c r="E9" s="29" t="s">
-        <v>816</v>
+        <v>821</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="9" t="s">
-        <v>817</v>
+        <v>822</v>
       </c>
       <c r="B10" s="22" t="s">
-        <v>818</v>
+        <v>823</v>
       </c>
       <c r="C10" s="27" t="s">
-        <v>819</v>
+        <v>824</v>
       </c>
       <c r="D10" s="28" t="s">
-        <v>820</v>
+        <v>825</v>
       </c>
       <c r="E10" s="29" t="s">
-        <v>821</v>
+        <v>826</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="5" t="s">
-        <v>822</v>
+        <v>827</v>
       </c>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -12268,7 +12563,7 @@
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="5" t="s">
-        <v>823</v>
+        <v>828</v>
       </c>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
@@ -12277,36 +12572,36 @@
     </row>
     <row r="22" spans="1:5">
       <c r="A22" s="7" t="s">
-        <v>824</v>
+        <v>829</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>825</v>
+        <v>830</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>826</v>
+        <v>831</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>827</v>
+        <v>832</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>828</v>
+        <v>833</v>
       </c>
     </row>
     <row r="23" spans="1:5">
       <c r="A23" s="14" t="s">
-        <v>829</v>
+        <v>834</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>830</v>
+        <v>835</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>831</v>
+        <v>836</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>832</v>
+        <v>837</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>833</v>
+        <v>838</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -12314,16 +12609,16 @@
         <v>48</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>834</v>
+        <v>839</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>835</v>
+        <v>840</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>836</v>
+        <v>841</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>837</v>
+        <v>842</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -12331,16 +12626,16 @@
         <v>35</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>838</v>
+        <v>843</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>839</v>
+        <v>844</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>840</v>
+        <v>845</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>841</v>
+        <v>846</v>
       </c>
     </row>
     <row r="26" spans="1:5">
@@ -12348,21 +12643,21 @@
         <v>38</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>842</v>
+        <v>847</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>843</v>
+        <v>848</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>844</v>
+        <v>849</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>845</v>
+        <v>850</v>
       </c>
     </row>
     <row r="28" spans="1:5">
       <c r="A28" s="5" t="s">
-        <v>846</v>
+        <v>851</v>
       </c>
       <c r="B28" s="5"/>
       <c r="C28" s="5"/>
@@ -12371,7 +12666,7 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" s="4" t="s">
-        <v>847</v>
+        <v>852</v>
       </c>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -12380,7 +12675,7 @@
     </row>
     <row r="30" spans="1:5">
       <c r="A30" s="4" t="s">
-        <v>848</v>
+        <v>853</v>
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -12389,7 +12684,7 @@
     </row>
     <row r="31" spans="1:5">
       <c r="A31" s="4" t="s">
-        <v>849</v>
+        <v>854</v>
       </c>
       <c r="B31" s="4"/>
       <c r="C31" s="4"/>
@@ -12398,7 +12693,7 @@
     </row>
     <row r="32" spans="1:5">
       <c r="A32" s="4" t="s">
-        <v>850</v>
+        <v>855</v>
       </c>
       <c r="B32" s="4"/>
       <c r="C32" s="4"/>
@@ -12407,7 +12702,7 @@
     </row>
     <row r="33" spans="1:5">
       <c r="A33" s="4" t="s">
-        <v>851</v>
+        <v>856</v>
       </c>
       <c r="B33" s="4"/>
       <c r="C33" s="4"/>
@@ -12431,98 +12726,98 @@
         <v>462</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>852</v>
+        <v>857</v>
       </c>
       <c r="D36" s="7"/>
       <c r="E36" s="7"/>
     </row>
     <row r="37" spans="1:5">
       <c r="A37" s="4" t="s">
-        <v>853</v>
+        <v>858</v>
       </c>
       <c r="B37" s="24" t="s">
-        <v>854</v>
+        <v>859</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>855</v>
+        <v>860</v>
       </c>
       <c r="D37" s="4"/>
       <c r="E37" s="4"/>
     </row>
     <row r="38" spans="1:5">
       <c r="A38" s="4" t="s">
-        <v>856</v>
+        <v>861</v>
       </c>
       <c r="B38" s="24" t="s">
-        <v>857</v>
+        <v>862</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>858</v>
+        <v>863</v>
       </c>
       <c r="D38" s="4"/>
       <c r="E38" s="4"/>
     </row>
     <row r="39" spans="1:5">
       <c r="A39" s="4" t="s">
-        <v>859</v>
+        <v>864</v>
       </c>
       <c r="B39" s="24" t="s">
         <v>470</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>860</v>
+        <v>865</v>
       </c>
       <c r="D39" s="4"/>
       <c r="E39" s="4"/>
     </row>
     <row r="40" spans="1:5">
       <c r="A40" s="4" t="s">
-        <v>861</v>
+        <v>866</v>
       </c>
       <c r="B40" s="24" t="s">
-        <v>862</v>
+        <v>867</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>863</v>
+        <v>868</v>
       </c>
       <c r="D40" s="4"/>
       <c r="E40" s="4"/>
     </row>
     <row r="41" spans="1:5">
       <c r="A41" s="4" t="s">
-        <v>861</v>
+        <v>866</v>
       </c>
       <c r="B41" s="24" t="s">
-        <v>864</v>
+        <v>869</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>865</v>
+        <v>870</v>
       </c>
       <c r="D41" s="4"/>
       <c r="E41" s="4"/>
     </row>
     <row r="42" spans="1:5">
       <c r="A42" s="4" t="s">
-        <v>866</v>
+        <v>871</v>
       </c>
       <c r="B42" s="24" t="s">
-        <v>867</v>
+        <v>872</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>868</v>
+        <v>873</v>
       </c>
       <c r="D42" s="4"/>
       <c r="E42" s="4"/>
     </row>
     <row r="43" spans="1:5">
       <c r="A43" s="4" t="s">
-        <v>869</v>
+        <v>874</v>
       </c>
       <c r="B43" s="24" t="s">
-        <v>870</v>
+        <v>875</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>871</v>
+        <v>876</v>
       </c>
       <c r="D43" s="4"/>
       <c r="E43" s="4"/>

</xml_diff>

<commit_message>
Log B7 W2 T4 (Recovery 3->2, trash session: flag L 2-3s/R 1s, 90 balance off)
</commit_message>
<xml_diff>
--- a/Training_3_B7.xlsx
+++ b/Training_3_B7.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1816" uniqueCount="941">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1839" uniqueCount="946">
   <si>
     <t>B7 — Performance-Block Dashboard (Advanced OAHS)</t>
   </si>
@@ -2298,6 +2298,21 @@
   </si>
   <si>
     <t>Handstand-Endurance FREISTEHEND 2x50s (stark!)</t>
+  </si>
+  <si>
+    <t>Straddle: unsupported Lean+Return + Freeze; links 2-3s Freeze manchmal; ein paar Fallouts</t>
+  </si>
+  <si>
+    <t>rechts max 1s Freeze+Return, froh es zu schaffen; Fallouts</t>
+  </si>
+  <si>
+    <t>Trash-Tag; Balance mies (untypisch), S2 fast Kontrollverlust; nur Negative, abgebrochen damit RPE nicht explodiert</t>
+  </si>
+  <si>
+    <t>ging noch (Balance/Last reduziert)</t>
+  </si>
+  <si>
+    <t>Chest-supported Row</t>
   </si>
   <si>
     <t>B7 — Nutrition Targets (Maintenance, KEIN Defizit)</t>
@@ -4108,7 +4123,7 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>877</v>
+        <v>882</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4118,7 +4133,7 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="12" t="s">
-        <v>878</v>
+        <v>883</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -4143,12 +4158,12 @@
         <v>155</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>879</v>
+        <v>884</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="9" t="s">
-        <v>880</v>
+        <v>885</v>
       </c>
       <c r="B4" s="11">
         <f>SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Skill90",'B7_Training_Log'!$C$2:$C$1000,1)+SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Planche",'B7_Training_Log'!$C$2:$C$1000,1)+SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Push",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4173,7 +4188,7 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="9" t="s">
-        <v>881</v>
+        <v>886</v>
       </c>
       <c r="B5" s="11">
         <f>SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Pull",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4198,7 +4213,7 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="9" t="s">
-        <v>882</v>
+        <v>887</v>
       </c>
       <c r="B6" s="11">
         <f>SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Legs",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4223,7 +4238,7 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="9" t="s">
-        <v>883</v>
+        <v>888</v>
       </c>
       <c r="B7" s="10">
         <f>SUMIFS('B7_Training_Log'!$N$2:$N$1000,'B7_Training_Log'!$D$2:$D$1000,"90",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4248,7 +4263,7 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="9" t="s">
-        <v>884</v>
+        <v>889</v>
       </c>
       <c r="B8" s="10">
         <f>COUNTIFS('B7_Training_Log'!$E$2:$E$1000,"SkillOAHS",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4273,7 +4288,7 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="9" t="s">
-        <v>885</v>
+        <v>890</v>
       </c>
       <c r="B9" s="10">
         <f>MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_straddle",'B7_Training_Log'!$F$2:$F$1000,"L",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4298,7 +4313,7 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="9" t="s">
-        <v>886</v>
+        <v>891</v>
       </c>
       <c r="B10" s="10">
         <f>MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_straddle",'B7_Training_Log'!$F$2:$F$1000,"R",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4323,7 +4338,7 @@
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="9" t="s">
-        <v>887</v>
+        <v>892</v>
       </c>
       <c r="B11" s="10">
         <f>MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_diamond",'B7_Training_Log'!$F$2:$F$1000,"L",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4348,7 +4363,7 @@
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="9" t="s">
-        <v>888</v>
+        <v>893</v>
       </c>
       <c r="B12" s="10">
         <f>MAX(MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_flag",'B7_Training_Log'!$C$2:$C$1000,1),MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_figa",'B7_Training_Log'!$C$2:$C$1000,1))</f>
@@ -4373,7 +4388,7 @@
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="9" t="s">
-        <v>889</v>
+        <v>894</v>
       </c>
       <c r="B13" s="11">
         <f>IFERROR(AVERAGEIFS('B7_Training_Log'!$J$2:$J$1000,'B7_Training_Log'!$C$2:$C$1000,1),0)</f>
@@ -4448,7 +4463,7 @@
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="9" t="s">
-        <v>890</v>
+        <v>895</v>
       </c>
       <c r="B16" s="10">
         <f>COUNTIFS('B7_Training_Log'!$K$2:$K$1000,"&gt;=4",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4473,7 +4488,7 @@
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="9" t="s">
-        <v>891</v>
+        <v>896</v>
       </c>
       <c r="B17" s="10">
         <f>COUNTIFS('B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4517,7 +4532,7 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
-        <v>892</v>
+        <v>897</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4525,7 +4540,7 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="5" t="s">
-        <v>893</v>
+        <v>898</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
@@ -4533,13 +4548,13 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="7" t="s">
-        <v>894</v>
+        <v>899</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>895</v>
+        <v>900</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>896</v>
+        <v>901</v>
       </c>
       <c r="D4" s="7"/>
     </row>
@@ -4548,10 +4563,10 @@
         <v>672</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>897</v>
+        <v>902</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>898</v>
+        <v>903</v>
       </c>
       <c r="D5" s="4"/>
     </row>
@@ -4560,10 +4575,10 @@
         <v>673</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>899</v>
+        <v>904</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>900</v>
+        <v>905</v>
       </c>
       <c r="D6" s="4"/>
     </row>
@@ -4572,10 +4587,10 @@
         <v>674</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>901</v>
+        <v>906</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>902</v>
+        <v>907</v>
       </c>
       <c r="D7" s="4"/>
     </row>
@@ -4584,10 +4599,10 @@
         <v>481</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>903</v>
+        <v>908</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>904</v>
+        <v>909</v>
       </c>
       <c r="D8" s="4"/>
     </row>
@@ -4596,10 +4611,10 @@
         <v>484</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>905</v>
+        <v>910</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>906</v>
+        <v>911</v>
       </c>
       <c r="D9" s="4"/>
     </row>
@@ -4608,10 +4623,10 @@
         <v>675</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>907</v>
+        <v>912</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>908</v>
+        <v>913</v>
       </c>
       <c r="D10" s="4"/>
     </row>
@@ -4620,10 +4635,10 @@
         <v>676</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>909</v>
+        <v>914</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>910</v>
+        <v>915</v>
       </c>
       <c r="D11" s="4"/>
     </row>
@@ -4632,10 +4647,10 @@
         <v>677</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>911</v>
+        <v>916</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>912</v>
+        <v>917</v>
       </c>
       <c r="D12" s="4"/>
     </row>
@@ -4644,10 +4659,10 @@
         <v>678</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>909</v>
+        <v>914</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>913</v>
+        <v>918</v>
       </c>
       <c r="D13" s="4"/>
     </row>
@@ -4656,10 +4671,10 @@
         <v>679</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>914</v>
+        <v>919</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>915</v>
+        <v>920</v>
       </c>
       <c r="D14" s="4"/>
     </row>
@@ -4668,10 +4683,10 @@
         <v>680</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>916</v>
+        <v>921</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>917</v>
+        <v>922</v>
       </c>
       <c r="D15" s="4"/>
     </row>
@@ -4680,10 +4695,10 @@
         <v>681</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>918</v>
+        <v>923</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>919</v>
+        <v>924</v>
       </c>
       <c r="D16" s="4"/>
     </row>
@@ -4692,10 +4707,10 @@
         <v>682</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>909</v>
+        <v>914</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>920</v>
+        <v>925</v>
       </c>
       <c r="D17" s="4"/>
     </row>
@@ -4704,10 +4719,10 @@
         <v>683</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>909</v>
+        <v>914</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>921</v>
+        <v>926</v>
       </c>
       <c r="D18" s="4"/>
     </row>
@@ -4716,10 +4731,10 @@
         <v>684</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>922</v>
+        <v>927</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>923</v>
+        <v>928</v>
       </c>
       <c r="D19" s="4"/>
     </row>
@@ -4728,10 +4743,10 @@
         <v>94</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>911</v>
+        <v>916</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>924</v>
+        <v>929</v>
       </c>
       <c r="D20" s="4"/>
     </row>
@@ -4740,16 +4755,16 @@
         <v>685</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>925</v>
+        <v>930</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>926</v>
+        <v>931</v>
       </c>
       <c r="D21" s="4"/>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="5" t="s">
-        <v>927</v>
+        <v>932</v>
       </c>
       <c r="B23" s="5"/>
       <c r="C23" s="5"/>
@@ -4757,7 +4772,7 @@
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="4" t="s">
-        <v>928</v>
+        <v>933</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -4765,7 +4780,7 @@
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="4" t="s">
-        <v>929</v>
+        <v>934</v>
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -4773,7 +4788,7 @@
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="4" t="s">
-        <v>930</v>
+        <v>935</v>
       </c>
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
@@ -4781,7 +4796,7 @@
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="4" t="s">
-        <v>931</v>
+        <v>936</v>
       </c>
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
@@ -4789,7 +4804,7 @@
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="4" t="s">
-        <v>932</v>
+        <v>937</v>
       </c>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
@@ -4797,7 +4812,7 @@
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="4" t="s">
-        <v>933</v>
+        <v>938</v>
       </c>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -4805,7 +4820,7 @@
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="4" t="s">
-        <v>934</v>
+        <v>939</v>
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -4813,7 +4828,7 @@
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="5" t="s">
-        <v>935</v>
+        <v>940</v>
       </c>
       <c r="B32" s="5"/>
       <c r="C32" s="5"/>
@@ -4821,7 +4836,7 @@
     </row>
     <row r="33" spans="1:4">
       <c r="A33" s="4" t="s">
-        <v>936</v>
+        <v>941</v>
       </c>
       <c r="B33" s="4"/>
       <c r="C33" s="4"/>
@@ -4829,7 +4844,7 @@
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="4" t="s">
-        <v>937</v>
+        <v>942</v>
       </c>
       <c r="B34" s="4"/>
       <c r="C34" s="4"/>
@@ -4837,7 +4852,7 @@
     </row>
     <row r="35" spans="1:4">
       <c r="A35" s="4" t="s">
-        <v>938</v>
+        <v>943</v>
       </c>
       <c r="B35" s="4"/>
       <c r="C35" s="4"/>
@@ -4845,7 +4860,7 @@
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="4" t="s">
-        <v>939</v>
+        <v>944</v>
       </c>
       <c r="B36" s="4"/>
       <c r="C36" s="4"/>
@@ -4853,7 +4868,7 @@
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="4" t="s">
-        <v>940</v>
+        <v>945</v>
       </c>
       <c r="B37" s="4"/>
       <c r="C37" s="4"/>
@@ -9081,7 +9096,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q67"/>
+  <dimension ref="A1:Q72"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -11902,6 +11917,227 @@
       </c>
       <c r="Q67" s="6">
         <f>IF($B67="","",$B67&amp;"_W"&amp;$C67)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" spans="1:17">
+      <c r="A68" s="25">
+        <v>46238</v>
+      </c>
+      <c r="B68" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="C68" s="6">
+        <v>2</v>
+      </c>
+      <c r="D68" s="6" t="s">
+        <v>668</v>
+      </c>
+      <c r="E68" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D68,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F68" s="6" t="s">
+        <v>686</v>
+      </c>
+      <c r="G68" s="6">
+        <v>4</v>
+      </c>
+      <c r="I68" s="6">
+        <v>0</v>
+      </c>
+      <c r="L68" s="6">
+        <v>3</v>
+      </c>
+      <c r="M68" s="6">
+        <v>3</v>
+      </c>
+      <c r="O68" s="6">
+        <v>2</v>
+      </c>
+      <c r="P68" s="4" t="s">
+        <v>756</v>
+      </c>
+      <c r="Q68" s="6">
+        <f>IF($B68="","",$B68&amp;"_W"&amp;$C68)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:17">
+      <c r="A69" s="25">
+        <v>46238</v>
+      </c>
+      <c r="B69" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="C69" s="6">
+        <v>2</v>
+      </c>
+      <c r="D69" s="6" t="s">
+        <v>668</v>
+      </c>
+      <c r="E69" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D69,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F69" s="6" t="s">
+        <v>688</v>
+      </c>
+      <c r="G69" s="6">
+        <v>4</v>
+      </c>
+      <c r="I69" s="6">
+        <v>0</v>
+      </c>
+      <c r="L69" s="6">
+        <v>2</v>
+      </c>
+      <c r="M69" s="6">
+        <v>1</v>
+      </c>
+      <c r="O69" s="6">
+        <v>2</v>
+      </c>
+      <c r="P69" s="4" t="s">
+        <v>757</v>
+      </c>
+      <c r="Q69" s="6">
+        <f>IF($B69="","",$B69&amp;"_W"&amp;$C69)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:17">
+      <c r="A70" s="25">
+        <v>46238</v>
+      </c>
+      <c r="B70" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="C70" s="6">
+        <v>2</v>
+      </c>
+      <c r="D70" s="6" t="s">
+        <v>489</v>
+      </c>
+      <c r="E70" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D70,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F70" s="6" t="s">
+        <v>693</v>
+      </c>
+      <c r="G70" s="6">
+        <v>3</v>
+      </c>
+      <c r="H70" s="4" t="s">
+        <v>694</v>
+      </c>
+      <c r="I70" s="6">
+        <v>0</v>
+      </c>
+      <c r="J70" s="6">
+        <v>9</v>
+      </c>
+      <c r="L70" s="6">
+        <v>1</v>
+      </c>
+      <c r="N70" s="6">
+        <v>0</v>
+      </c>
+      <c r="O70" s="6">
+        <v>2</v>
+      </c>
+      <c r="P70" s="4" t="s">
+        <v>758</v>
+      </c>
+      <c r="Q70" s="6">
+        <f>IF($B70="","",$B70&amp;"_W"&amp;$C70)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="1:17">
+      <c r="A71" s="25">
+        <v>46238</v>
+      </c>
+      <c r="B71" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="C71" s="6">
+        <v>2</v>
+      </c>
+      <c r="D71" s="6" t="s">
+        <v>567</v>
+      </c>
+      <c r="E71" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D71,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F71" s="6" t="s">
+        <v>693</v>
+      </c>
+      <c r="G71" s="6">
+        <v>3</v>
+      </c>
+      <c r="H71" s="4" t="s">
+        <v>739</v>
+      </c>
+      <c r="I71" s="6">
+        <v>0</v>
+      </c>
+      <c r="J71" s="6">
+        <v>7</v>
+      </c>
+      <c r="O71" s="6">
+        <v>2</v>
+      </c>
+      <c r="P71" s="4" t="s">
+        <v>759</v>
+      </c>
+      <c r="Q71" s="6">
+        <f>IF($B71="","",$B71&amp;"_W"&amp;$C71)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="1:17">
+      <c r="A72" s="25">
+        <v>46238</v>
+      </c>
+      <c r="B72" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="C72" s="6">
+        <v>2</v>
+      </c>
+      <c r="D72" s="6" t="s">
+        <v>539</v>
+      </c>
+      <c r="E72" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D72,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F72" s="6" t="s">
+        <v>693</v>
+      </c>
+      <c r="G72" s="6">
+        <v>2</v>
+      </c>
+      <c r="H72" s="4" t="s">
+        <v>707</v>
+      </c>
+      <c r="I72" s="6">
+        <v>100</v>
+      </c>
+      <c r="J72" s="6">
+        <v>7</v>
+      </c>
+      <c r="O72" s="6">
+        <v>2</v>
+      </c>
+      <c r="P72" s="4" t="s">
+        <v>760</v>
+      </c>
+      <c r="Q72" s="6">
+        <f>IF($B72="","",$B72&amp;"_W"&amp;$C72)</f>
         <v>0</v>
       </c>
     </row>
@@ -11979,7 +12215,7 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>756</v>
+        <v>761</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -11990,20 +12226,20 @@
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="5" t="s">
-        <v>757</v>
+        <v>762</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="9" t="s">
-        <v>758</v>
+        <v>763</v>
       </c>
       <c r="B4" s="11">
         <v>81</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>766</v>
+        <v>771</v>
       </c>
       <c r="D4" s="4"/>
       <c r="E4" s="4"/>
@@ -12012,21 +12248,21 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="9" t="s">
-        <v>759</v>
+        <v>764</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>760</v>
+        <v>765</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="9" t="s">
-        <v>761</v>
+        <v>766</v>
       </c>
       <c r="B6" s="11">
         <v>2.2</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>767</v>
+        <v>772</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
@@ -12035,7 +12271,7 @@
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="9" t="s">
-        <v>762</v>
+        <v>767</v>
       </c>
       <c r="B7" s="11">
         <v>0.9</v>
@@ -12043,7 +12279,7 @@
     </row>
     <row r="8" spans="1:7">
       <c r="A8" s="9" t="s">
-        <v>763</v>
+        <v>768</v>
       </c>
       <c r="B8" s="10">
         <v>2700</v>
@@ -12051,7 +12287,7 @@
     </row>
     <row r="9" spans="1:7">
       <c r="A9" s="9" t="s">
-        <v>764</v>
+        <v>769</v>
       </c>
       <c r="B9" s="10">
         <f>ROUND(BW*B6,0)</f>
@@ -12060,7 +12296,7 @@
     </row>
     <row r="10" spans="1:7">
       <c r="A10" s="9" t="s">
-        <v>765</v>
+        <v>770</v>
       </c>
       <c r="B10" s="10">
         <f>ROUND(BW*B7,0)</f>
@@ -12069,7 +12305,7 @@
     </row>
     <row r="12" spans="1:7">
       <c r="A12" s="5" t="s">
-        <v>768</v>
+        <v>773</v>
       </c>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -12083,27 +12319,27 @@
         <v>87</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>769</v>
+        <v>774</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>770</v>
+        <v>775</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>771</v>
+        <v>776</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>772</v>
+        <v>777</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>773</v>
+        <v>778</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>774</v>
+        <v>779</v>
       </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" s="9" t="s">
-        <v>775</v>
+        <v>780</v>
       </c>
       <c r="B14" s="26">
         <v>250</v>
@@ -12125,7 +12361,7 @@
         <v>0</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>776</v>
+        <v>781</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -12152,12 +12388,12 @@
         <v>0</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>777</v>
+        <v>782</v>
       </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" s="9" t="s">
-        <v>778</v>
+        <v>783</v>
       </c>
       <c r="B16" s="26">
         <v>200</v>
@@ -12179,12 +12415,12 @@
         <v>0</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>779</v>
+        <v>784</v>
       </c>
     </row>
     <row r="17" spans="1:7">
       <c r="A17" s="9" t="s">
-        <v>780</v>
+        <v>785</v>
       </c>
       <c r="B17" s="26">
         <v>150</v>
@@ -12206,12 +12442,12 @@
         <v>0</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>781</v>
+        <v>786</v>
       </c>
     </row>
     <row r="18" spans="1:7">
       <c r="A18" s="9" t="s">
-        <v>782</v>
+        <v>787</v>
       </c>
       <c r="B18" s="26">
         <v>100</v>
@@ -12233,7 +12469,7 @@
         <v>0</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>783</v>
+        <v>788</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -12260,12 +12496,12 @@
         <v>0</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>784</v>
+        <v>789</v>
       </c>
     </row>
     <row r="21" spans="1:7">
       <c r="A21" s="5" t="s">
-        <v>785</v>
+        <v>790</v>
       </c>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
@@ -12276,7 +12512,7 @@
     </row>
     <row r="22" spans="1:7">
       <c r="A22" s="4" t="s">
-        <v>786</v>
+        <v>791</v>
       </c>
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
@@ -12287,7 +12523,7 @@
     </row>
     <row r="23" spans="1:7">
       <c r="A23" s="4" t="s">
-        <v>787</v>
+        <v>792</v>
       </c>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
@@ -12298,7 +12534,7 @@
     </row>
     <row r="24" spans="1:7">
       <c r="A24" s="4" t="s">
-        <v>788</v>
+        <v>793</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -12309,7 +12545,7 @@
     </row>
     <row r="25" spans="1:7">
       <c r="A25" s="4" t="s">
-        <v>789</v>
+        <v>794</v>
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -12354,7 +12590,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>790</v>
+        <v>795</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -12363,7 +12599,7 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="5" t="s">
-        <v>791</v>
+        <v>796</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
@@ -12372,126 +12608,126 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="7" t="s">
-        <v>792</v>
+        <v>797</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>793</v>
+        <v>798</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>794</v>
+        <v>799</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>795</v>
+        <v>800</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>796</v>
+        <v>801</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="9" t="s">
-        <v>797</v>
+        <v>802</v>
       </c>
       <c r="B5" s="22" t="s">
-        <v>798</v>
+        <v>803</v>
       </c>
       <c r="C5" s="27" t="s">
-        <v>799</v>
+        <v>804</v>
       </c>
       <c r="D5" s="28" t="s">
-        <v>800</v>
+        <v>805</v>
       </c>
       <c r="E5" s="29" t="s">
-        <v>801</v>
+        <v>806</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="9" t="s">
-        <v>802</v>
+        <v>807</v>
       </c>
       <c r="B6" s="22" t="s">
-        <v>803</v>
+        <v>808</v>
       </c>
       <c r="C6" s="27" t="s">
-        <v>804</v>
+        <v>809</v>
       </c>
       <c r="D6" s="28" t="s">
-        <v>805</v>
+        <v>810</v>
       </c>
       <c r="E6" s="29" t="s">
-        <v>806</v>
+        <v>811</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="9" t="s">
-        <v>807</v>
+        <v>812</v>
       </c>
       <c r="B7" s="22" t="s">
-        <v>808</v>
+        <v>813</v>
       </c>
       <c r="C7" s="27" t="s">
-        <v>809</v>
+        <v>814</v>
       </c>
       <c r="D7" s="28" t="s">
-        <v>810</v>
+        <v>815</v>
       </c>
       <c r="E7" s="29" t="s">
-        <v>811</v>
+        <v>816</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="9" t="s">
-        <v>812</v>
+        <v>817</v>
       </c>
       <c r="B8" s="22" t="s">
-        <v>813</v>
+        <v>818</v>
       </c>
       <c r="C8" s="27" t="s">
-        <v>814</v>
+        <v>819</v>
       </c>
       <c r="D8" s="28" t="s">
-        <v>815</v>
+        <v>820</v>
       </c>
       <c r="E8" s="29" t="s">
-        <v>816</v>
+        <v>821</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="9" t="s">
-        <v>817</v>
+        <v>822</v>
       </c>
       <c r="B9" s="22" t="s">
-        <v>818</v>
+        <v>823</v>
       </c>
       <c r="C9" s="27" t="s">
-        <v>819</v>
+        <v>824</v>
       </c>
       <c r="D9" s="28" t="s">
-        <v>820</v>
+        <v>825</v>
       </c>
       <c r="E9" s="29" t="s">
-        <v>821</v>
+        <v>826</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="9" t="s">
-        <v>822</v>
+        <v>827</v>
       </c>
       <c r="B10" s="22" t="s">
-        <v>823</v>
+        <v>828</v>
       </c>
       <c r="C10" s="27" t="s">
-        <v>824</v>
+        <v>829</v>
       </c>
       <c r="D10" s="28" t="s">
-        <v>825</v>
+        <v>830</v>
       </c>
       <c r="E10" s="29" t="s">
-        <v>826</v>
+        <v>831</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="5" t="s">
-        <v>827</v>
+        <v>832</v>
       </c>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -12563,7 +12799,7 @@
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="5" t="s">
-        <v>828</v>
+        <v>833</v>
       </c>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
@@ -12572,36 +12808,36 @@
     </row>
     <row r="22" spans="1:5">
       <c r="A22" s="7" t="s">
-        <v>829</v>
+        <v>834</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>830</v>
+        <v>835</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>831</v>
+        <v>836</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>832</v>
+        <v>837</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>833</v>
+        <v>838</v>
       </c>
     </row>
     <row r="23" spans="1:5">
       <c r="A23" s="14" t="s">
-        <v>834</v>
+        <v>839</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>835</v>
+        <v>840</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>836</v>
+        <v>841</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>837</v>
+        <v>842</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>838</v>
+        <v>843</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -12609,16 +12845,16 @@
         <v>48</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>839</v>
+        <v>844</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>840</v>
+        <v>845</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>841</v>
+        <v>846</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>842</v>
+        <v>847</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -12626,16 +12862,16 @@
         <v>35</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>843</v>
+        <v>848</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>844</v>
+        <v>849</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>845</v>
+        <v>850</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>846</v>
+        <v>851</v>
       </c>
     </row>
     <row r="26" spans="1:5">
@@ -12643,21 +12879,21 @@
         <v>38</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>847</v>
+        <v>852</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>848</v>
+        <v>853</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>849</v>
+        <v>854</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>850</v>
+        <v>855</v>
       </c>
     </row>
     <row r="28" spans="1:5">
       <c r="A28" s="5" t="s">
-        <v>851</v>
+        <v>856</v>
       </c>
       <c r="B28" s="5"/>
       <c r="C28" s="5"/>
@@ -12666,7 +12902,7 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" s="4" t="s">
-        <v>852</v>
+        <v>857</v>
       </c>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -12675,7 +12911,7 @@
     </row>
     <row r="30" spans="1:5">
       <c r="A30" s="4" t="s">
-        <v>853</v>
+        <v>858</v>
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -12684,7 +12920,7 @@
     </row>
     <row r="31" spans="1:5">
       <c r="A31" s="4" t="s">
-        <v>854</v>
+        <v>859</v>
       </c>
       <c r="B31" s="4"/>
       <c r="C31" s="4"/>
@@ -12693,7 +12929,7 @@
     </row>
     <row r="32" spans="1:5">
       <c r="A32" s="4" t="s">
-        <v>855</v>
+        <v>860</v>
       </c>
       <c r="B32" s="4"/>
       <c r="C32" s="4"/>
@@ -12702,7 +12938,7 @@
     </row>
     <row r="33" spans="1:5">
       <c r="A33" s="4" t="s">
-        <v>856</v>
+        <v>861</v>
       </c>
       <c r="B33" s="4"/>
       <c r="C33" s="4"/>
@@ -12726,98 +12962,98 @@
         <v>462</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>857</v>
+        <v>862</v>
       </c>
       <c r="D36" s="7"/>
       <c r="E36" s="7"/>
     </row>
     <row r="37" spans="1:5">
       <c r="A37" s="4" t="s">
-        <v>858</v>
+        <v>863</v>
       </c>
       <c r="B37" s="24" t="s">
-        <v>859</v>
+        <v>864</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>860</v>
+        <v>865</v>
       </c>
       <c r="D37" s="4"/>
       <c r="E37" s="4"/>
     </row>
     <row r="38" spans="1:5">
       <c r="A38" s="4" t="s">
-        <v>861</v>
+        <v>866</v>
       </c>
       <c r="B38" s="24" t="s">
-        <v>862</v>
+        <v>867</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>863</v>
+        <v>868</v>
       </c>
       <c r="D38" s="4"/>
       <c r="E38" s="4"/>
     </row>
     <row r="39" spans="1:5">
       <c r="A39" s="4" t="s">
-        <v>864</v>
+        <v>869</v>
       </c>
       <c r="B39" s="24" t="s">
         <v>470</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>865</v>
+        <v>870</v>
       </c>
       <c r="D39" s="4"/>
       <c r="E39" s="4"/>
     </row>
     <row r="40" spans="1:5">
       <c r="A40" s="4" t="s">
-        <v>866</v>
+        <v>871</v>
       </c>
       <c r="B40" s="24" t="s">
-        <v>867</v>
+        <v>872</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>868</v>
+        <v>873</v>
       </c>
       <c r="D40" s="4"/>
       <c r="E40" s="4"/>
     </row>
     <row r="41" spans="1:5">
       <c r="A41" s="4" t="s">
-        <v>866</v>
+        <v>871</v>
       </c>
       <c r="B41" s="24" t="s">
-        <v>869</v>
+        <v>874</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>870</v>
+        <v>875</v>
       </c>
       <c r="D41" s="4"/>
       <c r="E41" s="4"/>
     </row>
     <row r="42" spans="1:5">
       <c r="A42" s="4" t="s">
-        <v>871</v>
+        <v>876</v>
       </c>
       <c r="B42" s="24" t="s">
-        <v>872</v>
+        <v>877</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>873</v>
+        <v>878</v>
       </c>
       <c r="D42" s="4"/>
       <c r="E42" s="4"/>
     </row>
     <row r="43" spans="1:5">
       <c r="A43" s="4" t="s">
-        <v>874</v>
+        <v>879</v>
       </c>
       <c r="B43" s="24" t="s">
-        <v>875</v>
+        <v>880</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>876</v>
+        <v>881</v>
       </c>
       <c r="D43" s="4"/>
       <c r="E43" s="4"/>

</xml_diff>

<commit_message>
Log B7 W2 T5 (Recovery ~4-5, strong rebound) - W2 complete
</commit_message>
<xml_diff>
--- a/Training_3_B7.xlsx
+++ b/Training_3_B7.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1839" uniqueCount="946">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1887" uniqueCount="957">
   <si>
     <t>B7 — Performance-Block Dashboard (Advanced OAHS)</t>
   </si>
@@ -2313,6 +2313,39 @@
   </si>
   <si>
     <t>Chest-supported Row</t>
+  </si>
+  <si>
+    <t>Mikrodosis: Legs-together OHNE Noodle-Support, ging gut (Tier-B-Signal)</t>
+  </si>
+  <si>
+    <t>kontrolliert, kein Failure (Recovery ~4-5)</t>
+  </si>
+  <si>
+    <t>leicht (RPE 5-6) -&gt; Progressionspotenzial</t>
+  </si>
+  <si>
+    <t>hohe Parallettes, Fuesse erhoeht</t>
+  </si>
+  <si>
+    <t>Kabelzug (besserer Pump)</t>
+  </si>
+  <si>
+    <t>10,9,8</t>
+  </si>
+  <si>
+    <t>Gewicht nicht genannt (~8 kg?)</t>
+  </si>
+  <si>
+    <t>Maschine</t>
+  </si>
+  <si>
+    <t>12,10</t>
+  </si>
+  <si>
+    <t>Kabel 23,5+1,75</t>
+  </si>
+  <si>
+    <t>Kabel 16,5+1,75</t>
   </si>
   <si>
     <t>B7 — Nutrition Targets (Maintenance, KEIN Defizit)</t>
@@ -4123,7 +4156,7 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>882</v>
+        <v>893</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4133,7 +4166,7 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="12" t="s">
-        <v>883</v>
+        <v>894</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -4158,12 +4191,12 @@
         <v>155</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>884</v>
+        <v>895</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="9" t="s">
-        <v>885</v>
+        <v>896</v>
       </c>
       <c r="B4" s="11">
         <f>SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Skill90",'B7_Training_Log'!$C$2:$C$1000,1)+SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Planche",'B7_Training_Log'!$C$2:$C$1000,1)+SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Push",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4188,7 +4221,7 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="9" t="s">
-        <v>886</v>
+        <v>897</v>
       </c>
       <c r="B5" s="11">
         <f>SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Pull",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4213,7 +4246,7 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="9" t="s">
-        <v>887</v>
+        <v>898</v>
       </c>
       <c r="B6" s="11">
         <f>SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Legs",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4238,7 +4271,7 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="9" t="s">
-        <v>888</v>
+        <v>899</v>
       </c>
       <c r="B7" s="10">
         <f>SUMIFS('B7_Training_Log'!$N$2:$N$1000,'B7_Training_Log'!$D$2:$D$1000,"90",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4263,7 +4296,7 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="9" t="s">
-        <v>889</v>
+        <v>900</v>
       </c>
       <c r="B8" s="10">
         <f>COUNTIFS('B7_Training_Log'!$E$2:$E$1000,"SkillOAHS",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4288,7 +4321,7 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="9" t="s">
-        <v>890</v>
+        <v>901</v>
       </c>
       <c r="B9" s="10">
         <f>MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_straddle",'B7_Training_Log'!$F$2:$F$1000,"L",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4313,7 +4346,7 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="9" t="s">
-        <v>891</v>
+        <v>902</v>
       </c>
       <c r="B10" s="10">
         <f>MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_straddle",'B7_Training_Log'!$F$2:$F$1000,"R",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4338,7 +4371,7 @@
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="9" t="s">
-        <v>892</v>
+        <v>903</v>
       </c>
       <c r="B11" s="10">
         <f>MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_diamond",'B7_Training_Log'!$F$2:$F$1000,"L",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4363,7 +4396,7 @@
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="9" t="s">
-        <v>893</v>
+        <v>904</v>
       </c>
       <c r="B12" s="10">
         <f>MAX(MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_flag",'B7_Training_Log'!$C$2:$C$1000,1),MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_figa",'B7_Training_Log'!$C$2:$C$1000,1))</f>
@@ -4388,7 +4421,7 @@
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="9" t="s">
-        <v>894</v>
+        <v>905</v>
       </c>
       <c r="B13" s="11">
         <f>IFERROR(AVERAGEIFS('B7_Training_Log'!$J$2:$J$1000,'B7_Training_Log'!$C$2:$C$1000,1),0)</f>
@@ -4463,7 +4496,7 @@
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="9" t="s">
-        <v>895</v>
+        <v>906</v>
       </c>
       <c r="B16" s="10">
         <f>COUNTIFS('B7_Training_Log'!$K$2:$K$1000,"&gt;=4",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4488,7 +4521,7 @@
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="9" t="s">
-        <v>896</v>
+        <v>907</v>
       </c>
       <c r="B17" s="10">
         <f>COUNTIFS('B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4532,7 +4565,7 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
-        <v>897</v>
+        <v>908</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4540,7 +4573,7 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="5" t="s">
-        <v>898</v>
+        <v>909</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
@@ -4548,13 +4581,13 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="7" t="s">
-        <v>899</v>
+        <v>910</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>900</v>
+        <v>911</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>901</v>
+        <v>912</v>
       </c>
       <c r="D4" s="7"/>
     </row>
@@ -4563,10 +4596,10 @@
         <v>672</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>902</v>
+        <v>913</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>903</v>
+        <v>914</v>
       </c>
       <c r="D5" s="4"/>
     </row>
@@ -4575,10 +4608,10 @@
         <v>673</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>904</v>
+        <v>915</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>905</v>
+        <v>916</v>
       </c>
       <c r="D6" s="4"/>
     </row>
@@ -4587,10 +4620,10 @@
         <v>674</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>906</v>
+        <v>917</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>907</v>
+        <v>918</v>
       </c>
       <c r="D7" s="4"/>
     </row>
@@ -4599,10 +4632,10 @@
         <v>481</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>908</v>
+        <v>919</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>909</v>
+        <v>920</v>
       </c>
       <c r="D8" s="4"/>
     </row>
@@ -4611,10 +4644,10 @@
         <v>484</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>910</v>
+        <v>921</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>911</v>
+        <v>922</v>
       </c>
       <c r="D9" s="4"/>
     </row>
@@ -4623,10 +4656,10 @@
         <v>675</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>912</v>
+        <v>923</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>913</v>
+        <v>924</v>
       </c>
       <c r="D10" s="4"/>
     </row>
@@ -4635,10 +4668,10 @@
         <v>676</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>914</v>
+        <v>925</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>915</v>
+        <v>926</v>
       </c>
       <c r="D11" s="4"/>
     </row>
@@ -4647,10 +4680,10 @@
         <v>677</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>916</v>
+        <v>927</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>917</v>
+        <v>928</v>
       </c>
       <c r="D12" s="4"/>
     </row>
@@ -4659,10 +4692,10 @@
         <v>678</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>914</v>
+        <v>925</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>918</v>
+        <v>929</v>
       </c>
       <c r="D13" s="4"/>
     </row>
@@ -4671,10 +4704,10 @@
         <v>679</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>919</v>
+        <v>930</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>920</v>
+        <v>931</v>
       </c>
       <c r="D14" s="4"/>
     </row>
@@ -4683,10 +4716,10 @@
         <v>680</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>921</v>
+        <v>932</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>922</v>
+        <v>933</v>
       </c>
       <c r="D15" s="4"/>
     </row>
@@ -4695,10 +4728,10 @@
         <v>681</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>923</v>
+        <v>934</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>924</v>
+        <v>935</v>
       </c>
       <c r="D16" s="4"/>
     </row>
@@ -4707,10 +4740,10 @@
         <v>682</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>914</v>
+        <v>925</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>925</v>
+        <v>936</v>
       </c>
       <c r="D17" s="4"/>
     </row>
@@ -4719,10 +4752,10 @@
         <v>683</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>914</v>
+        <v>925</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>926</v>
+        <v>937</v>
       </c>
       <c r="D18" s="4"/>
     </row>
@@ -4731,10 +4764,10 @@
         <v>684</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>927</v>
+        <v>938</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>928</v>
+        <v>939</v>
       </c>
       <c r="D19" s="4"/>
     </row>
@@ -4743,10 +4776,10 @@
         <v>94</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>916</v>
+        <v>927</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>929</v>
+        <v>940</v>
       </c>
       <c r="D20" s="4"/>
     </row>
@@ -4755,16 +4788,16 @@
         <v>685</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>930</v>
+        <v>941</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>931</v>
+        <v>942</v>
       </c>
       <c r="D21" s="4"/>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="5" t="s">
-        <v>932</v>
+        <v>943</v>
       </c>
       <c r="B23" s="5"/>
       <c r="C23" s="5"/>
@@ -4772,7 +4805,7 @@
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="4" t="s">
-        <v>933</v>
+        <v>944</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -4780,7 +4813,7 @@
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="4" t="s">
-        <v>934</v>
+        <v>945</v>
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -4788,7 +4821,7 @@
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="4" t="s">
-        <v>935</v>
+        <v>946</v>
       </c>
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
@@ -4796,7 +4829,7 @@
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="4" t="s">
-        <v>936</v>
+        <v>947</v>
       </c>
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
@@ -4804,7 +4837,7 @@
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="4" t="s">
-        <v>937</v>
+        <v>948</v>
       </c>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
@@ -4812,7 +4845,7 @@
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="4" t="s">
-        <v>938</v>
+        <v>949</v>
       </c>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -4820,7 +4853,7 @@
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="4" t="s">
-        <v>939</v>
+        <v>950</v>
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -4828,7 +4861,7 @@
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="5" t="s">
-        <v>940</v>
+        <v>951</v>
       </c>
       <c r="B32" s="5"/>
       <c r="C32" s="5"/>
@@ -4836,7 +4869,7 @@
     </row>
     <row r="33" spans="1:4">
       <c r="A33" s="4" t="s">
-        <v>941</v>
+        <v>952</v>
       </c>
       <c r="B33" s="4"/>
       <c r="C33" s="4"/>
@@ -4844,7 +4877,7 @@
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="4" t="s">
-        <v>942</v>
+        <v>953</v>
       </c>
       <c r="B34" s="4"/>
       <c r="C34" s="4"/>
@@ -4852,7 +4885,7 @@
     </row>
     <row r="35" spans="1:4">
       <c r="A35" s="4" t="s">
-        <v>943</v>
+        <v>954</v>
       </c>
       <c r="B35" s="4"/>
       <c r="C35" s="4"/>
@@ -4860,7 +4893,7 @@
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="4" t="s">
-        <v>944</v>
+        <v>955</v>
       </c>
       <c r="B36" s="4"/>
       <c r="C36" s="4"/>
@@ -4868,7 +4901,7 @@
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="4" t="s">
-        <v>945</v>
+        <v>956</v>
       </c>
       <c r="B37" s="4"/>
       <c r="C37" s="4"/>
@@ -9096,7 +9129,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q72"/>
+  <dimension ref="A1:Q82"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -12138,6 +12171,427 @@
       </c>
       <c r="Q72" s="6">
         <f>IF($B72="","",$B72&amp;"_W"&amp;$C72)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" spans="1:17">
+      <c r="A73" s="25">
+        <v>46239</v>
+      </c>
+      <c r="B73" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="C73" s="6">
+        <v>2</v>
+      </c>
+      <c r="D73" s="6" t="s">
+        <v>653</v>
+      </c>
+      <c r="E73" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D73,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F73" s="6" t="s">
+        <v>693</v>
+      </c>
+      <c r="G73" s="6">
+        <v>2</v>
+      </c>
+      <c r="I73" s="6">
+        <v>0</v>
+      </c>
+      <c r="L73" s="6">
+        <v>3</v>
+      </c>
+      <c r="O73" s="6">
+        <v>4</v>
+      </c>
+      <c r="P73" s="4" t="s">
+        <v>761</v>
+      </c>
+      <c r="Q73" s="6">
+        <f>IF($B73="","",$B73&amp;"_W"&amp;$C73)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="1:17">
+      <c r="A74" s="25">
+        <v>46239</v>
+      </c>
+      <c r="B74" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="C74" s="6">
+        <v>2</v>
+      </c>
+      <c r="D74" s="6" t="s">
+        <v>489</v>
+      </c>
+      <c r="E74" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D74,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F74" s="6" t="s">
+        <v>693</v>
+      </c>
+      <c r="G74" s="6">
+        <v>3</v>
+      </c>
+      <c r="H74" s="4" t="s">
+        <v>694</v>
+      </c>
+      <c r="I74" s="6">
+        <v>0</v>
+      </c>
+      <c r="J74" s="6">
+        <v>7</v>
+      </c>
+      <c r="O74" s="6">
+        <v>4</v>
+      </c>
+      <c r="P74" s="4" t="s">
+        <v>762</v>
+      </c>
+      <c r="Q74" s="6">
+        <f>IF($B74="","",$B74&amp;"_W"&amp;$C74)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="1:17">
+      <c r="A75" s="25">
+        <v>46239</v>
+      </c>
+      <c r="B75" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="C75" s="6">
+        <v>2</v>
+      </c>
+      <c r="D75" s="6" t="s">
+        <v>570</v>
+      </c>
+      <c r="E75" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D75,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F75" s="6" t="s">
+        <v>693</v>
+      </c>
+      <c r="G75" s="6">
+        <v>3</v>
+      </c>
+      <c r="H75" s="4" t="s">
+        <v>698</v>
+      </c>
+      <c r="I75" s="6">
+        <v>0</v>
+      </c>
+      <c r="J75" s="6">
+        <v>6</v>
+      </c>
+      <c r="O75" s="6">
+        <v>4</v>
+      </c>
+      <c r="P75" s="4" t="s">
+        <v>763</v>
+      </c>
+      <c r="Q75" s="6">
+        <f>IF($B75="","",$B75&amp;"_W"&amp;$C75)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" spans="1:17">
+      <c r="A76" s="25">
+        <v>46239</v>
+      </c>
+      <c r="B76" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="C76" s="6">
+        <v>2</v>
+      </c>
+      <c r="D76" s="6" t="s">
+        <v>574</v>
+      </c>
+      <c r="E76" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D76,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F76" s="6" t="s">
+        <v>693</v>
+      </c>
+      <c r="G76" s="6">
+        <v>2</v>
+      </c>
+      <c r="H76" s="4" t="s">
+        <v>707</v>
+      </c>
+      <c r="I76" s="6">
+        <v>0</v>
+      </c>
+      <c r="J76" s="6">
+        <v>7</v>
+      </c>
+      <c r="O76" s="6">
+        <v>4</v>
+      </c>
+      <c r="P76" s="4" t="s">
+        <v>764</v>
+      </c>
+      <c r="Q76" s="6">
+        <f>IF($B76="","",$B76&amp;"_W"&amp;$C76)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77" spans="1:17">
+      <c r="A77" s="25">
+        <v>46239</v>
+      </c>
+      <c r="B77" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="C77" s="6">
+        <v>2</v>
+      </c>
+      <c r="D77" s="6" t="s">
+        <v>539</v>
+      </c>
+      <c r="E77" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D77,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F77" s="6" t="s">
+        <v>693</v>
+      </c>
+      <c r="G77" s="6">
+        <v>3</v>
+      </c>
+      <c r="H77" s="4" t="s">
+        <v>707</v>
+      </c>
+      <c r="I77" s="6">
+        <v>80</v>
+      </c>
+      <c r="J77" s="6">
+        <v>7</v>
+      </c>
+      <c r="O77" s="6">
+        <v>4</v>
+      </c>
+      <c r="P77" s="4" t="s">
+        <v>765</v>
+      </c>
+      <c r="Q77" s="6">
+        <f>IF($B77="","",$B77&amp;"_W"&amp;$C77)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" spans="1:17">
+      <c r="A78" s="25">
+        <v>46239</v>
+      </c>
+      <c r="B78" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="C78" s="6">
+        <v>2</v>
+      </c>
+      <c r="D78" s="6" t="s">
+        <v>536</v>
+      </c>
+      <c r="E78" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D78,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F78" s="6" t="s">
+        <v>693</v>
+      </c>
+      <c r="G78" s="6">
+        <v>3</v>
+      </c>
+      <c r="H78" s="4" t="s">
+        <v>766</v>
+      </c>
+      <c r="I78" s="6">
+        <v>70</v>
+      </c>
+      <c r="J78" s="6">
+        <v>7</v>
+      </c>
+      <c r="O78" s="6">
+        <v>4</v>
+      </c>
+      <c r="Q78" s="6">
+        <f>IF($B78="","",$B78&amp;"_W"&amp;$C78)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" spans="1:17">
+      <c r="A79" s="25">
+        <v>46239</v>
+      </c>
+      <c r="B79" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="C79" s="6">
+        <v>2</v>
+      </c>
+      <c r="D79" s="6" t="s">
+        <v>577</v>
+      </c>
+      <c r="E79" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D79,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F79" s="6" t="s">
+        <v>693</v>
+      </c>
+      <c r="G79" s="6">
+        <v>3</v>
+      </c>
+      <c r="H79" s="4" t="s">
+        <v>698</v>
+      </c>
+      <c r="J79" s="6">
+        <v>7</v>
+      </c>
+      <c r="O79" s="6">
+        <v>4</v>
+      </c>
+      <c r="P79" s="4" t="s">
+        <v>767</v>
+      </c>
+      <c r="Q79" s="6">
+        <f>IF($B79="","",$B79&amp;"_W"&amp;$C79)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80" spans="1:17">
+      <c r="A80" s="25">
+        <v>46239</v>
+      </c>
+      <c r="B80" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="C80" s="6">
+        <v>2</v>
+      </c>
+      <c r="D80" s="6" t="s">
+        <v>546</v>
+      </c>
+      <c r="E80" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D80,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F80" s="6" t="s">
+        <v>693</v>
+      </c>
+      <c r="G80" s="6">
+        <v>3</v>
+      </c>
+      <c r="H80" s="4" t="s">
+        <v>698</v>
+      </c>
+      <c r="I80" s="6">
+        <v>30</v>
+      </c>
+      <c r="J80" s="6">
+        <v>7</v>
+      </c>
+      <c r="O80" s="6">
+        <v>4</v>
+      </c>
+      <c r="P80" s="4" t="s">
+        <v>768</v>
+      </c>
+      <c r="Q80" s="6">
+        <f>IF($B80="","",$B80&amp;"_W"&amp;$C80)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" spans="1:17">
+      <c r="A81" s="25">
+        <v>46239</v>
+      </c>
+      <c r="B81" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="C81" s="6">
+        <v>2</v>
+      </c>
+      <c r="D81" s="6" t="s">
+        <v>585</v>
+      </c>
+      <c r="E81" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D81,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F81" s="6" t="s">
+        <v>693</v>
+      </c>
+      <c r="G81" s="6">
+        <v>2</v>
+      </c>
+      <c r="H81" s="4" t="s">
+        <v>769</v>
+      </c>
+      <c r="I81" s="6">
+        <v>25.25</v>
+      </c>
+      <c r="J81" s="6">
+        <v>7</v>
+      </c>
+      <c r="O81" s="6">
+        <v>4</v>
+      </c>
+      <c r="P81" s="4" t="s">
+        <v>770</v>
+      </c>
+      <c r="Q81" s="6">
+        <f>IF($B81="","",$B81&amp;"_W"&amp;$C81)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82" spans="1:17">
+      <c r="A82" s="25">
+        <v>46239</v>
+      </c>
+      <c r="B82" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="C82" s="6">
+        <v>2</v>
+      </c>
+      <c r="D82" s="6" t="s">
+        <v>581</v>
+      </c>
+      <c r="E82" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D82,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F82" s="6" t="s">
+        <v>693</v>
+      </c>
+      <c r="G82" s="6">
+        <v>2</v>
+      </c>
+      <c r="H82" s="4" t="s">
+        <v>698</v>
+      </c>
+      <c r="I82" s="6">
+        <v>18.25</v>
+      </c>
+      <c r="J82" s="6">
+        <v>7</v>
+      </c>
+      <c r="O82" s="6">
+        <v>4</v>
+      </c>
+      <c r="P82" s="4" t="s">
+        <v>771</v>
+      </c>
+      <c r="Q82" s="6">
+        <f>IF($B82="","",$B82&amp;"_W"&amp;$C82)</f>
         <v>0</v>
       </c>
     </row>
@@ -12215,7 +12669,7 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>761</v>
+        <v>772</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -12226,20 +12680,20 @@
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="5" t="s">
-        <v>762</v>
+        <v>773</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="9" t="s">
-        <v>763</v>
+        <v>774</v>
       </c>
       <c r="B4" s="11">
         <v>81</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>771</v>
+        <v>782</v>
       </c>
       <c r="D4" s="4"/>
       <c r="E4" s="4"/>
@@ -12248,21 +12702,21 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="9" t="s">
-        <v>764</v>
+        <v>775</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>765</v>
+        <v>776</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="9" t="s">
-        <v>766</v>
+        <v>777</v>
       </c>
       <c r="B6" s="11">
         <v>2.2</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>772</v>
+        <v>783</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
@@ -12271,7 +12725,7 @@
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="9" t="s">
-        <v>767</v>
+        <v>778</v>
       </c>
       <c r="B7" s="11">
         <v>0.9</v>
@@ -12279,7 +12733,7 @@
     </row>
     <row r="8" spans="1:7">
       <c r="A8" s="9" t="s">
-        <v>768</v>
+        <v>779</v>
       </c>
       <c r="B8" s="10">
         <v>2700</v>
@@ -12287,7 +12741,7 @@
     </row>
     <row r="9" spans="1:7">
       <c r="A9" s="9" t="s">
-        <v>769</v>
+        <v>780</v>
       </c>
       <c r="B9" s="10">
         <f>ROUND(BW*B6,0)</f>
@@ -12296,7 +12750,7 @@
     </row>
     <row r="10" spans="1:7">
       <c r="A10" s="9" t="s">
-        <v>770</v>
+        <v>781</v>
       </c>
       <c r="B10" s="10">
         <f>ROUND(BW*B7,0)</f>
@@ -12305,7 +12759,7 @@
     </row>
     <row r="12" spans="1:7">
       <c r="A12" s="5" t="s">
-        <v>773</v>
+        <v>784</v>
       </c>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -12319,27 +12773,27 @@
         <v>87</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>774</v>
+        <v>785</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>775</v>
+        <v>786</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>776</v>
+        <v>787</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>777</v>
+        <v>788</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>778</v>
+        <v>789</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>779</v>
+        <v>790</v>
       </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" s="9" t="s">
-        <v>780</v>
+        <v>791</v>
       </c>
       <c r="B14" s="26">
         <v>250</v>
@@ -12361,7 +12815,7 @@
         <v>0</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>781</v>
+        <v>792</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -12388,12 +12842,12 @@
         <v>0</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>782</v>
+        <v>793</v>
       </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" s="9" t="s">
-        <v>783</v>
+        <v>794</v>
       </c>
       <c r="B16" s="26">
         <v>200</v>
@@ -12415,12 +12869,12 @@
         <v>0</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>784</v>
+        <v>795</v>
       </c>
     </row>
     <row r="17" spans="1:7">
       <c r="A17" s="9" t="s">
-        <v>785</v>
+        <v>796</v>
       </c>
       <c r="B17" s="26">
         <v>150</v>
@@ -12442,12 +12896,12 @@
         <v>0</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>786</v>
+        <v>797</v>
       </c>
     </row>
     <row r="18" spans="1:7">
       <c r="A18" s="9" t="s">
-        <v>787</v>
+        <v>798</v>
       </c>
       <c r="B18" s="26">
         <v>100</v>
@@ -12469,7 +12923,7 @@
         <v>0</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>788</v>
+        <v>799</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -12496,12 +12950,12 @@
         <v>0</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>789</v>
+        <v>800</v>
       </c>
     </row>
     <row r="21" spans="1:7">
       <c r="A21" s="5" t="s">
-        <v>790</v>
+        <v>801</v>
       </c>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
@@ -12512,7 +12966,7 @@
     </row>
     <row r="22" spans="1:7">
       <c r="A22" s="4" t="s">
-        <v>791</v>
+        <v>802</v>
       </c>
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
@@ -12523,7 +12977,7 @@
     </row>
     <row r="23" spans="1:7">
       <c r="A23" s="4" t="s">
-        <v>792</v>
+        <v>803</v>
       </c>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
@@ -12534,7 +12988,7 @@
     </row>
     <row r="24" spans="1:7">
       <c r="A24" s="4" t="s">
-        <v>793</v>
+        <v>804</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -12545,7 +12999,7 @@
     </row>
     <row r="25" spans="1:7">
       <c r="A25" s="4" t="s">
-        <v>794</v>
+        <v>805</v>
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -12590,7 +13044,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>795</v>
+        <v>806</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -12599,7 +13053,7 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="5" t="s">
-        <v>796</v>
+        <v>807</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
@@ -12608,126 +13062,126 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="7" t="s">
-        <v>797</v>
+        <v>808</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>798</v>
+        <v>809</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>799</v>
+        <v>810</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>800</v>
+        <v>811</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>801</v>
+        <v>812</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="9" t="s">
-        <v>802</v>
+        <v>813</v>
       </c>
       <c r="B5" s="22" t="s">
-        <v>803</v>
+        <v>814</v>
       </c>
       <c r="C5" s="27" t="s">
-        <v>804</v>
+        <v>815</v>
       </c>
       <c r="D5" s="28" t="s">
-        <v>805</v>
+        <v>816</v>
       </c>
       <c r="E5" s="29" t="s">
-        <v>806</v>
+        <v>817</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="9" t="s">
-        <v>807</v>
+        <v>818</v>
       </c>
       <c r="B6" s="22" t="s">
-        <v>808</v>
+        <v>819</v>
       </c>
       <c r="C6" s="27" t="s">
-        <v>809</v>
+        <v>820</v>
       </c>
       <c r="D6" s="28" t="s">
-        <v>810</v>
+        <v>821</v>
       </c>
       <c r="E6" s="29" t="s">
-        <v>811</v>
+        <v>822</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="9" t="s">
-        <v>812</v>
+        <v>823</v>
       </c>
       <c r="B7" s="22" t="s">
-        <v>813</v>
+        <v>824</v>
       </c>
       <c r="C7" s="27" t="s">
-        <v>814</v>
+        <v>825</v>
       </c>
       <c r="D7" s="28" t="s">
-        <v>815</v>
+        <v>826</v>
       </c>
       <c r="E7" s="29" t="s">
-        <v>816</v>
+        <v>827</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="9" t="s">
-        <v>817</v>
+        <v>828</v>
       </c>
       <c r="B8" s="22" t="s">
-        <v>818</v>
+        <v>829</v>
       </c>
       <c r="C8" s="27" t="s">
-        <v>819</v>
+        <v>830</v>
       </c>
       <c r="D8" s="28" t="s">
-        <v>820</v>
+        <v>831</v>
       </c>
       <c r="E8" s="29" t="s">
-        <v>821</v>
+        <v>832</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="9" t="s">
-        <v>822</v>
+        <v>833</v>
       </c>
       <c r="B9" s="22" t="s">
-        <v>823</v>
+        <v>834</v>
       </c>
       <c r="C9" s="27" t="s">
-        <v>824</v>
+        <v>835</v>
       </c>
       <c r="D9" s="28" t="s">
-        <v>825</v>
+        <v>836</v>
       </c>
       <c r="E9" s="29" t="s">
-        <v>826</v>
+        <v>837</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="9" t="s">
-        <v>827</v>
+        <v>838</v>
       </c>
       <c r="B10" s="22" t="s">
-        <v>828</v>
+        <v>839</v>
       </c>
       <c r="C10" s="27" t="s">
-        <v>829</v>
+        <v>840</v>
       </c>
       <c r="D10" s="28" t="s">
-        <v>830</v>
+        <v>841</v>
       </c>
       <c r="E10" s="29" t="s">
-        <v>831</v>
+        <v>842</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="5" t="s">
-        <v>832</v>
+        <v>843</v>
       </c>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -12799,7 +13253,7 @@
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="5" t="s">
-        <v>833</v>
+        <v>844</v>
       </c>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
@@ -12808,36 +13262,36 @@
     </row>
     <row r="22" spans="1:5">
       <c r="A22" s="7" t="s">
-        <v>834</v>
+        <v>845</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>835</v>
+        <v>846</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>836</v>
+        <v>847</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>837</v>
+        <v>848</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>838</v>
+        <v>849</v>
       </c>
     </row>
     <row r="23" spans="1:5">
       <c r="A23" s="14" t="s">
-        <v>839</v>
+        <v>850</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>840</v>
+        <v>851</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>841</v>
+        <v>852</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>842</v>
+        <v>853</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>843</v>
+        <v>854</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -12845,16 +13299,16 @@
         <v>48</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>844</v>
+        <v>855</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>845</v>
+        <v>856</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>846</v>
+        <v>857</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>847</v>
+        <v>858</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -12862,16 +13316,16 @@
         <v>35</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>848</v>
+        <v>859</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>849</v>
+        <v>860</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>850</v>
+        <v>861</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>851</v>
+        <v>862</v>
       </c>
     </row>
     <row r="26" spans="1:5">
@@ -12879,21 +13333,21 @@
         <v>38</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>852</v>
+        <v>863</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>853</v>
+        <v>864</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>854</v>
+        <v>865</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>855</v>
+        <v>866</v>
       </c>
     </row>
     <row r="28" spans="1:5">
       <c r="A28" s="5" t="s">
-        <v>856</v>
+        <v>867</v>
       </c>
       <c r="B28" s="5"/>
       <c r="C28" s="5"/>
@@ -12902,7 +13356,7 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" s="4" t="s">
-        <v>857</v>
+        <v>868</v>
       </c>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -12911,7 +13365,7 @@
     </row>
     <row r="30" spans="1:5">
       <c r="A30" s="4" t="s">
-        <v>858</v>
+        <v>869</v>
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -12920,7 +13374,7 @@
     </row>
     <row r="31" spans="1:5">
       <c r="A31" s="4" t="s">
-        <v>859</v>
+        <v>870</v>
       </c>
       <c r="B31" s="4"/>
       <c r="C31" s="4"/>
@@ -12929,7 +13383,7 @@
     </row>
     <row r="32" spans="1:5">
       <c r="A32" s="4" t="s">
-        <v>860</v>
+        <v>871</v>
       </c>
       <c r="B32" s="4"/>
       <c r="C32" s="4"/>
@@ -12938,7 +13392,7 @@
     </row>
     <row r="33" spans="1:5">
       <c r="A33" s="4" t="s">
-        <v>861</v>
+        <v>872</v>
       </c>
       <c r="B33" s="4"/>
       <c r="C33" s="4"/>
@@ -12962,98 +13416,98 @@
         <v>462</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>862</v>
+        <v>873</v>
       </c>
       <c r="D36" s="7"/>
       <c r="E36" s="7"/>
     </row>
     <row r="37" spans="1:5">
       <c r="A37" s="4" t="s">
-        <v>863</v>
+        <v>874</v>
       </c>
       <c r="B37" s="24" t="s">
-        <v>864</v>
+        <v>875</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>865</v>
+        <v>876</v>
       </c>
       <c r="D37" s="4"/>
       <c r="E37" s="4"/>
     </row>
     <row r="38" spans="1:5">
       <c r="A38" s="4" t="s">
-        <v>866</v>
+        <v>877</v>
       </c>
       <c r="B38" s="24" t="s">
-        <v>867</v>
+        <v>878</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>868</v>
+        <v>879</v>
       </c>
       <c r="D38" s="4"/>
       <c r="E38" s="4"/>
     </row>
     <row r="39" spans="1:5">
       <c r="A39" s="4" t="s">
-        <v>869</v>
+        <v>880</v>
       </c>
       <c r="B39" s="24" t="s">
         <v>470</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>870</v>
+        <v>881</v>
       </c>
       <c r="D39" s="4"/>
       <c r="E39" s="4"/>
     </row>
     <row r="40" spans="1:5">
       <c r="A40" s="4" t="s">
-        <v>871</v>
+        <v>882</v>
       </c>
       <c r="B40" s="24" t="s">
-        <v>872</v>
+        <v>883</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>873</v>
+        <v>884</v>
       </c>
       <c r="D40" s="4"/>
       <c r="E40" s="4"/>
     </row>
     <row r="41" spans="1:5">
       <c r="A41" s="4" t="s">
-        <v>871</v>
+        <v>882</v>
       </c>
       <c r="B41" s="24" t="s">
-        <v>874</v>
+        <v>885</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>875</v>
+        <v>886</v>
       </c>
       <c r="D41" s="4"/>
       <c r="E41" s="4"/>
     </row>
     <row r="42" spans="1:5">
       <c r="A42" s="4" t="s">
-        <v>876</v>
+        <v>887</v>
       </c>
       <c r="B42" s="24" t="s">
-        <v>877</v>
+        <v>888</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>878</v>
+        <v>889</v>
       </c>
       <c r="D42" s="4"/>
       <c r="E42" s="4"/>
     </row>
     <row r="43" spans="1:5">
       <c r="A43" s="4" t="s">
-        <v>879</v>
+        <v>890</v>
       </c>
       <c r="B43" s="24" t="s">
-        <v>880</v>
+        <v>891</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>881</v>
+        <v>892</v>
       </c>
       <c r="D43" s="4"/>
       <c r="E43" s="4"/>

</xml_diff>

<commit_message>
Log B7 W3 T1 (Recovery 3): skill/strength off (likely BW up post-vacation/AYCE), endurance up to 3x60s
</commit_message>
<xml_diff>
--- a/Training_3_B7.xlsx
+++ b/Training_3_B7.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1887" uniqueCount="957">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1926" uniqueCount="965">
   <si>
     <t>B7 — Performance-Block Dashboard (Advanced OAHS)</t>
   </si>
@@ -2346,6 +2346,30 @@
   </si>
   <si>
     <t>Kabel 16,5+1,75</t>
+  </si>
+  <si>
+    <t>1-2 Holds 4s+ aber sehr shaky; schwaechstes Level seit langem</t>
+  </si>
+  <si>
+    <t>max ~1s Freeze dann Fall</t>
+  </si>
+  <si>
+    <t>shaky</t>
+  </si>
+  <si>
+    <t>3 Singles ok + 2 Fails</t>
+  </si>
+  <si>
+    <t>Weg rauf Kampf, Momentum noetig; fuehlte sich nach WENIGER Kraft an (evtl. schwerer/BW hoch), nicht Ansteuerung</t>
+  </si>
+  <si>
+    <t>Tuck Planche 8/8/6 s</t>
+  </si>
+  <si>
+    <t>Wide grip; recht schwach @RPE8 (evtl. BW hoch)</t>
+  </si>
+  <si>
+    <t>Endurance freistehend Parallettes 3x60s - steigt weiter (2x50 -&gt; 3x60)!</t>
   </si>
   <si>
     <t>B7 — Nutrition Targets (Maintenance, KEIN Defizit)</t>
@@ -4156,7 +4180,7 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>893</v>
+        <v>901</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4166,7 +4190,7 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="12" t="s">
-        <v>894</v>
+        <v>902</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -4191,12 +4215,12 @@
         <v>155</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>895</v>
+        <v>903</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="9" t="s">
-        <v>896</v>
+        <v>904</v>
       </c>
       <c r="B4" s="11">
         <f>SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Skill90",'B7_Training_Log'!$C$2:$C$1000,1)+SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Planche",'B7_Training_Log'!$C$2:$C$1000,1)+SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Push",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4221,7 +4245,7 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="9" t="s">
-        <v>897</v>
+        <v>905</v>
       </c>
       <c r="B5" s="11">
         <f>SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Pull",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4246,7 +4270,7 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="9" t="s">
-        <v>898</v>
+        <v>906</v>
       </c>
       <c r="B6" s="11">
         <f>SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Legs",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4271,7 +4295,7 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="9" t="s">
-        <v>899</v>
+        <v>907</v>
       </c>
       <c r="B7" s="10">
         <f>SUMIFS('B7_Training_Log'!$N$2:$N$1000,'B7_Training_Log'!$D$2:$D$1000,"90",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4296,7 +4320,7 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="9" t="s">
-        <v>900</v>
+        <v>908</v>
       </c>
       <c r="B8" s="10">
         <f>COUNTIFS('B7_Training_Log'!$E$2:$E$1000,"SkillOAHS",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4321,7 +4345,7 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="9" t="s">
-        <v>901</v>
+        <v>909</v>
       </c>
       <c r="B9" s="10">
         <f>MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_straddle",'B7_Training_Log'!$F$2:$F$1000,"L",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4346,7 +4370,7 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="9" t="s">
-        <v>902</v>
+        <v>910</v>
       </c>
       <c r="B10" s="10">
         <f>MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_straddle",'B7_Training_Log'!$F$2:$F$1000,"R",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4371,7 +4395,7 @@
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="9" t="s">
-        <v>903</v>
+        <v>911</v>
       </c>
       <c r="B11" s="10">
         <f>MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_diamond",'B7_Training_Log'!$F$2:$F$1000,"L",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4396,7 +4420,7 @@
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="9" t="s">
-        <v>904</v>
+        <v>912</v>
       </c>
       <c r="B12" s="10">
         <f>MAX(MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_flag",'B7_Training_Log'!$C$2:$C$1000,1),MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_figa",'B7_Training_Log'!$C$2:$C$1000,1))</f>
@@ -4421,7 +4445,7 @@
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="9" t="s">
-        <v>905</v>
+        <v>913</v>
       </c>
       <c r="B13" s="11">
         <f>IFERROR(AVERAGEIFS('B7_Training_Log'!$J$2:$J$1000,'B7_Training_Log'!$C$2:$C$1000,1),0)</f>
@@ -4496,7 +4520,7 @@
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="9" t="s">
-        <v>906</v>
+        <v>914</v>
       </c>
       <c r="B16" s="10">
         <f>COUNTIFS('B7_Training_Log'!$K$2:$K$1000,"&gt;=4",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4521,7 +4545,7 @@
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="9" t="s">
-        <v>907</v>
+        <v>915</v>
       </c>
       <c r="B17" s="10">
         <f>COUNTIFS('B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4565,7 +4589,7 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
-        <v>908</v>
+        <v>916</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4573,7 +4597,7 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="5" t="s">
-        <v>909</v>
+        <v>917</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
@@ -4581,13 +4605,13 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="7" t="s">
-        <v>910</v>
+        <v>918</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>911</v>
+        <v>919</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>912</v>
+        <v>920</v>
       </c>
       <c r="D4" s="7"/>
     </row>
@@ -4596,10 +4620,10 @@
         <v>672</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>913</v>
+        <v>921</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>914</v>
+        <v>922</v>
       </c>
       <c r="D5" s="4"/>
     </row>
@@ -4608,10 +4632,10 @@
         <v>673</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>915</v>
+        <v>923</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>916</v>
+        <v>924</v>
       </c>
       <c r="D6" s="4"/>
     </row>
@@ -4620,10 +4644,10 @@
         <v>674</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>917</v>
+        <v>925</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>918</v>
+        <v>926</v>
       </c>
       <c r="D7" s="4"/>
     </row>
@@ -4632,10 +4656,10 @@
         <v>481</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>919</v>
+        <v>927</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>920</v>
+        <v>928</v>
       </c>
       <c r="D8" s="4"/>
     </row>
@@ -4644,10 +4668,10 @@
         <v>484</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>921</v>
+        <v>929</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>922</v>
+        <v>930</v>
       </c>
       <c r="D9" s="4"/>
     </row>
@@ -4656,10 +4680,10 @@
         <v>675</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>923</v>
+        <v>931</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>924</v>
+        <v>932</v>
       </c>
       <c r="D10" s="4"/>
     </row>
@@ -4668,10 +4692,10 @@
         <v>676</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>925</v>
+        <v>933</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>926</v>
+        <v>934</v>
       </c>
       <c r="D11" s="4"/>
     </row>
@@ -4680,10 +4704,10 @@
         <v>677</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>927</v>
+        <v>935</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>928</v>
+        <v>936</v>
       </c>
       <c r="D12" s="4"/>
     </row>
@@ -4692,10 +4716,10 @@
         <v>678</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>925</v>
+        <v>933</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>929</v>
+        <v>937</v>
       </c>
       <c r="D13" s="4"/>
     </row>
@@ -4704,10 +4728,10 @@
         <v>679</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>930</v>
+        <v>938</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>931</v>
+        <v>939</v>
       </c>
       <c r="D14" s="4"/>
     </row>
@@ -4716,10 +4740,10 @@
         <v>680</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>932</v>
+        <v>940</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>933</v>
+        <v>941</v>
       </c>
       <c r="D15" s="4"/>
     </row>
@@ -4728,10 +4752,10 @@
         <v>681</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>934</v>
+        <v>942</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>935</v>
+        <v>943</v>
       </c>
       <c r="D16" s="4"/>
     </row>
@@ -4740,10 +4764,10 @@
         <v>682</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>925</v>
+        <v>933</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>936</v>
+        <v>944</v>
       </c>
       <c r="D17" s="4"/>
     </row>
@@ -4752,10 +4776,10 @@
         <v>683</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>925</v>
+        <v>933</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>937</v>
+        <v>945</v>
       </c>
       <c r="D18" s="4"/>
     </row>
@@ -4764,10 +4788,10 @@
         <v>684</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>938</v>
+        <v>946</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>939</v>
+        <v>947</v>
       </c>
       <c r="D19" s="4"/>
     </row>
@@ -4776,10 +4800,10 @@
         <v>94</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>927</v>
+        <v>935</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>940</v>
+        <v>948</v>
       </c>
       <c r="D20" s="4"/>
     </row>
@@ -4788,16 +4812,16 @@
         <v>685</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>941</v>
+        <v>949</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>942</v>
+        <v>950</v>
       </c>
       <c r="D21" s="4"/>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="5" t="s">
-        <v>943</v>
+        <v>951</v>
       </c>
       <c r="B23" s="5"/>
       <c r="C23" s="5"/>
@@ -4805,7 +4829,7 @@
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="4" t="s">
-        <v>944</v>
+        <v>952</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -4813,7 +4837,7 @@
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="4" t="s">
-        <v>945</v>
+        <v>953</v>
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -4821,7 +4845,7 @@
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="4" t="s">
-        <v>946</v>
+        <v>954</v>
       </c>
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
@@ -4829,7 +4853,7 @@
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="4" t="s">
-        <v>947</v>
+        <v>955</v>
       </c>
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
@@ -4837,7 +4861,7 @@
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="4" t="s">
-        <v>948</v>
+        <v>956</v>
       </c>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
@@ -4845,7 +4869,7 @@
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="4" t="s">
-        <v>949</v>
+        <v>957</v>
       </c>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -4853,7 +4877,7 @@
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="4" t="s">
-        <v>950</v>
+        <v>958</v>
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -4861,7 +4885,7 @@
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="5" t="s">
-        <v>951</v>
+        <v>959</v>
       </c>
       <c r="B32" s="5"/>
       <c r="C32" s="5"/>
@@ -4869,7 +4893,7 @@
     </row>
     <row r="33" spans="1:4">
       <c r="A33" s="4" t="s">
-        <v>952</v>
+        <v>960</v>
       </c>
       <c r="B33" s="4"/>
       <c r="C33" s="4"/>
@@ -4877,7 +4901,7 @@
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="4" t="s">
-        <v>953</v>
+        <v>961</v>
       </c>
       <c r="B34" s="4"/>
       <c r="C34" s="4"/>
@@ -4885,7 +4909,7 @@
     </row>
     <row r="35" spans="1:4">
       <c r="A35" s="4" t="s">
-        <v>954</v>
+        <v>962</v>
       </c>
       <c r="B35" s="4"/>
       <c r="C35" s="4"/>
@@ -4893,7 +4917,7 @@
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="4" t="s">
-        <v>955</v>
+        <v>963</v>
       </c>
       <c r="B36" s="4"/>
       <c r="C36" s="4"/>
@@ -4901,7 +4925,7 @@
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="4" t="s">
-        <v>956</v>
+        <v>964</v>
       </c>
       <c r="B37" s="4"/>
       <c r="C37" s="4"/>
@@ -9129,7 +9153,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q82"/>
+  <dimension ref="A1:Q92"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -12592,6 +12616,430 @@
       </c>
       <c r="Q82" s="6">
         <f>IF($B82="","",$B82&amp;"_W"&amp;$C82)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83" spans="1:17">
+      <c r="A83" s="25">
+        <v>46241</v>
+      </c>
+      <c r="B83" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="C83" s="6">
+        <v>3</v>
+      </c>
+      <c r="D83" s="6" t="s">
+        <v>641</v>
+      </c>
+      <c r="E83" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D83,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F83" s="6" t="s">
+        <v>686</v>
+      </c>
+      <c r="G83" s="6">
+        <v>3</v>
+      </c>
+      <c r="I83" s="6">
+        <v>0</v>
+      </c>
+      <c r="L83" s="6">
+        <v>2</v>
+      </c>
+      <c r="M83" s="6">
+        <v>4</v>
+      </c>
+      <c r="O83" s="6">
+        <v>3</v>
+      </c>
+      <c r="P83" s="4" t="s">
+        <v>772</v>
+      </c>
+      <c r="Q83" s="6">
+        <f>IF($B83="","",$B83&amp;"_W"&amp;$C83)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84" spans="1:17">
+      <c r="A84" s="25">
+        <v>46241</v>
+      </c>
+      <c r="B84" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="C84" s="6">
+        <v>3</v>
+      </c>
+      <c r="D84" s="6" t="s">
+        <v>641</v>
+      </c>
+      <c r="E84" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D84,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F84" s="6" t="s">
+        <v>688</v>
+      </c>
+      <c r="G84" s="6">
+        <v>3</v>
+      </c>
+      <c r="I84" s="6">
+        <v>0</v>
+      </c>
+      <c r="L84" s="6">
+        <v>1</v>
+      </c>
+      <c r="M84" s="6">
+        <v>1</v>
+      </c>
+      <c r="O84" s="6">
+        <v>3</v>
+      </c>
+      <c r="P84" s="4" t="s">
+        <v>773</v>
+      </c>
+      <c r="Q84" s="6">
+        <f>IF($B84="","",$B84&amp;"_W"&amp;$C84)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85" spans="1:17">
+      <c r="A85" s="25">
+        <v>46241</v>
+      </c>
+      <c r="B85" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="C85" s="6">
+        <v>3</v>
+      </c>
+      <c r="D85" s="6" t="s">
+        <v>647</v>
+      </c>
+      <c r="E85" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D85,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F85" s="6" t="s">
+        <v>686</v>
+      </c>
+      <c r="G85" s="6">
+        <v>3</v>
+      </c>
+      <c r="I85" s="6">
+        <v>0</v>
+      </c>
+      <c r="L85" s="6">
+        <v>2</v>
+      </c>
+      <c r="M85" s="6">
+        <v>4</v>
+      </c>
+      <c r="O85" s="6">
+        <v>3</v>
+      </c>
+      <c r="P85" s="4" t="s">
+        <v>774</v>
+      </c>
+      <c r="Q85" s="6">
+        <f>IF($B85="","",$B85&amp;"_W"&amp;$C85)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86" spans="1:17">
+      <c r="A86" s="25">
+        <v>46241</v>
+      </c>
+      <c r="B86" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="C86" s="6">
+        <v>3</v>
+      </c>
+      <c r="D86" s="6" t="s">
+        <v>647</v>
+      </c>
+      <c r="E86" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D86,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F86" s="6" t="s">
+        <v>688</v>
+      </c>
+      <c r="G86" s="6">
+        <v>3</v>
+      </c>
+      <c r="I86" s="6">
+        <v>0</v>
+      </c>
+      <c r="L86" s="6">
+        <v>1</v>
+      </c>
+      <c r="M86" s="6">
+        <v>1</v>
+      </c>
+      <c r="O86" s="6">
+        <v>3</v>
+      </c>
+      <c r="Q86" s="6">
+        <f>IF($B86="","",$B86&amp;"_W"&amp;$C86)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87" spans="1:17">
+      <c r="A87" s="25">
+        <v>46241</v>
+      </c>
+      <c r="B87" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="C87" s="6">
+        <v>3</v>
+      </c>
+      <c r="D87" s="6" t="s">
+        <v>644</v>
+      </c>
+      <c r="E87" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D87,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F87" s="6" t="s">
+        <v>686</v>
+      </c>
+      <c r="G87" s="6">
+        <v>2</v>
+      </c>
+      <c r="I87" s="6">
+        <v>0</v>
+      </c>
+      <c r="L87" s="6">
+        <v>2</v>
+      </c>
+      <c r="M87" s="6">
+        <v>4</v>
+      </c>
+      <c r="O87" s="6">
+        <v>3</v>
+      </c>
+      <c r="Q87" s="6">
+        <f>IF($B87="","",$B87&amp;"_W"&amp;$C87)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" spans="1:17">
+      <c r="A88" s="25">
+        <v>46241</v>
+      </c>
+      <c r="B88" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="C88" s="6">
+        <v>3</v>
+      </c>
+      <c r="D88" s="6" t="s">
+        <v>644</v>
+      </c>
+      <c r="E88" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D88,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F88" s="6" t="s">
+        <v>688</v>
+      </c>
+      <c r="G88" s="6">
+        <v>2</v>
+      </c>
+      <c r="I88" s="6">
+        <v>0</v>
+      </c>
+      <c r="L88" s="6">
+        <v>1</v>
+      </c>
+      <c r="M88" s="6">
+        <v>1</v>
+      </c>
+      <c r="O88" s="6">
+        <v>3</v>
+      </c>
+      <c r="Q88" s="6">
+        <f>IF($B88="","",$B88&amp;"_W"&amp;$C88)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89" spans="1:17">
+      <c r="A89" s="25">
+        <v>46241</v>
+      </c>
+      <c r="B89" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="C89" s="6">
+        <v>3</v>
+      </c>
+      <c r="D89" s="6" t="s">
+        <v>489</v>
+      </c>
+      <c r="E89" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D89,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F89" s="6" t="s">
+        <v>693</v>
+      </c>
+      <c r="G89" s="6">
+        <v>5</v>
+      </c>
+      <c r="H89" s="4" t="s">
+        <v>775</v>
+      </c>
+      <c r="I89" s="6">
+        <v>0</v>
+      </c>
+      <c r="J89" s="6">
+        <v>8</v>
+      </c>
+      <c r="N89" s="6">
+        <v>3</v>
+      </c>
+      <c r="O89" s="6">
+        <v>3</v>
+      </c>
+      <c r="P89" s="4" t="s">
+        <v>776</v>
+      </c>
+      <c r="Q89" s="6">
+        <f>IF($B89="","",$B89&amp;"_W"&amp;$C89)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90" spans="1:17">
+      <c r="A90" s="25">
+        <v>46241</v>
+      </c>
+      <c r="B90" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="C90" s="6">
+        <v>3</v>
+      </c>
+      <c r="D90" s="6" t="s">
+        <v>523</v>
+      </c>
+      <c r="E90" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D90,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F90" s="6" t="s">
+        <v>693</v>
+      </c>
+      <c r="G90" s="6">
+        <v>3</v>
+      </c>
+      <c r="I90" s="6">
+        <v>0</v>
+      </c>
+      <c r="J90" s="6">
+        <v>7</v>
+      </c>
+      <c r="M90" s="6">
+        <v>8</v>
+      </c>
+      <c r="O90" s="6">
+        <v>3</v>
+      </c>
+      <c r="P90" s="4" t="s">
+        <v>777</v>
+      </c>
+      <c r="Q90" s="6">
+        <f>IF($B90="","",$B90&amp;"_W"&amp;$C90)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91" spans="1:17">
+      <c r="A91" s="25">
+        <v>46241</v>
+      </c>
+      <c r="B91" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="C91" s="6">
+        <v>3</v>
+      </c>
+      <c r="D91" s="6" t="s">
+        <v>526</v>
+      </c>
+      <c r="E91" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D91,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F91" s="6" t="s">
+        <v>693</v>
+      </c>
+      <c r="G91" s="6">
+        <v>3</v>
+      </c>
+      <c r="H91" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="I91" s="6">
+        <v>35</v>
+      </c>
+      <c r="J91" s="6">
+        <v>8</v>
+      </c>
+      <c r="O91" s="6">
+        <v>3</v>
+      </c>
+      <c r="P91" s="4" t="s">
+        <v>778</v>
+      </c>
+      <c r="Q91" s="6">
+        <f>IF($B91="","",$B91&amp;"_W"&amp;$C91)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92" spans="1:17">
+      <c r="A92" s="25">
+        <v>46241</v>
+      </c>
+      <c r="B92" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="C92" s="6">
+        <v>3</v>
+      </c>
+      <c r="D92" s="6" t="s">
+        <v>504</v>
+      </c>
+      <c r="E92" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D92,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F92" s="6" t="s">
+        <v>693</v>
+      </c>
+      <c r="G92" s="6">
+        <v>3</v>
+      </c>
+      <c r="I92" s="6">
+        <v>0</v>
+      </c>
+      <c r="L92" s="6">
+        <v>4</v>
+      </c>
+      <c r="M92" s="6">
+        <v>60</v>
+      </c>
+      <c r="O92" s="6">
+        <v>3</v>
+      </c>
+      <c r="P92" s="4" t="s">
+        <v>779</v>
+      </c>
+      <c r="Q92" s="6">
+        <f>IF($B92="","",$B92&amp;"_W"&amp;$C92)</f>
         <v>0</v>
       </c>
     </row>
@@ -12669,7 +13117,7 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>772</v>
+        <v>780</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -12680,20 +13128,20 @@
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="5" t="s">
-        <v>773</v>
+        <v>781</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="9" t="s">
-        <v>774</v>
+        <v>782</v>
       </c>
       <c r="B4" s="11">
         <v>81</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>782</v>
+        <v>790</v>
       </c>
       <c r="D4" s="4"/>
       <c r="E4" s="4"/>
@@ -12702,21 +13150,21 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="9" t="s">
-        <v>775</v>
+        <v>783</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>776</v>
+        <v>784</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="9" t="s">
-        <v>777</v>
+        <v>785</v>
       </c>
       <c r="B6" s="11">
         <v>2.2</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>783</v>
+        <v>791</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
@@ -12725,7 +13173,7 @@
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="9" t="s">
-        <v>778</v>
+        <v>786</v>
       </c>
       <c r="B7" s="11">
         <v>0.9</v>
@@ -12733,7 +13181,7 @@
     </row>
     <row r="8" spans="1:7">
       <c r="A8" s="9" t="s">
-        <v>779</v>
+        <v>787</v>
       </c>
       <c r="B8" s="10">
         <v>2700</v>
@@ -12741,7 +13189,7 @@
     </row>
     <row r="9" spans="1:7">
       <c r="A9" s="9" t="s">
-        <v>780</v>
+        <v>788</v>
       </c>
       <c r="B9" s="10">
         <f>ROUND(BW*B6,0)</f>
@@ -12750,7 +13198,7 @@
     </row>
     <row r="10" spans="1:7">
       <c r="A10" s="9" t="s">
-        <v>781</v>
+        <v>789</v>
       </c>
       <c r="B10" s="10">
         <f>ROUND(BW*B7,0)</f>
@@ -12759,7 +13207,7 @@
     </row>
     <row r="12" spans="1:7">
       <c r="A12" s="5" t="s">
-        <v>784</v>
+        <v>792</v>
       </c>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -12773,27 +13221,27 @@
         <v>87</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>785</v>
+        <v>793</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>786</v>
+        <v>794</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>787</v>
+        <v>795</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>788</v>
+        <v>796</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>789</v>
+        <v>797</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>790</v>
+        <v>798</v>
       </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" s="9" t="s">
-        <v>791</v>
+        <v>799</v>
       </c>
       <c r="B14" s="26">
         <v>250</v>
@@ -12815,7 +13263,7 @@
         <v>0</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>792</v>
+        <v>800</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -12842,12 +13290,12 @@
         <v>0</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>793</v>
+        <v>801</v>
       </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" s="9" t="s">
-        <v>794</v>
+        <v>802</v>
       </c>
       <c r="B16" s="26">
         <v>200</v>
@@ -12869,12 +13317,12 @@
         <v>0</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>795</v>
+        <v>803</v>
       </c>
     </row>
     <row r="17" spans="1:7">
       <c r="A17" s="9" t="s">
-        <v>796</v>
+        <v>804</v>
       </c>
       <c r="B17" s="26">
         <v>150</v>
@@ -12896,12 +13344,12 @@
         <v>0</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>797</v>
+        <v>805</v>
       </c>
     </row>
     <row r="18" spans="1:7">
       <c r="A18" s="9" t="s">
-        <v>798</v>
+        <v>806</v>
       </c>
       <c r="B18" s="26">
         <v>100</v>
@@ -12923,7 +13371,7 @@
         <v>0</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>799</v>
+        <v>807</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -12950,12 +13398,12 @@
         <v>0</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>800</v>
+        <v>808</v>
       </c>
     </row>
     <row r="21" spans="1:7">
       <c r="A21" s="5" t="s">
-        <v>801</v>
+        <v>809</v>
       </c>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
@@ -12966,7 +13414,7 @@
     </row>
     <row r="22" spans="1:7">
       <c r="A22" s="4" t="s">
-        <v>802</v>
+        <v>810</v>
       </c>
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
@@ -12977,7 +13425,7 @@
     </row>
     <row r="23" spans="1:7">
       <c r="A23" s="4" t="s">
-        <v>803</v>
+        <v>811</v>
       </c>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
@@ -12988,7 +13436,7 @@
     </row>
     <row r="24" spans="1:7">
       <c r="A24" s="4" t="s">
-        <v>804</v>
+        <v>812</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -12999,7 +13447,7 @@
     </row>
     <row r="25" spans="1:7">
       <c r="A25" s="4" t="s">
-        <v>805</v>
+        <v>813</v>
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -13044,7 +13492,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>806</v>
+        <v>814</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -13053,7 +13501,7 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="5" t="s">
-        <v>807</v>
+        <v>815</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
@@ -13062,126 +13510,126 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="7" t="s">
-        <v>808</v>
+        <v>816</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>809</v>
+        <v>817</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>810</v>
+        <v>818</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>811</v>
+        <v>819</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>812</v>
+        <v>820</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="9" t="s">
-        <v>813</v>
+        <v>821</v>
       </c>
       <c r="B5" s="22" t="s">
-        <v>814</v>
+        <v>822</v>
       </c>
       <c r="C5" s="27" t="s">
-        <v>815</v>
+        <v>823</v>
       </c>
       <c r="D5" s="28" t="s">
-        <v>816</v>
+        <v>824</v>
       </c>
       <c r="E5" s="29" t="s">
-        <v>817</v>
+        <v>825</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="9" t="s">
-        <v>818</v>
+        <v>826</v>
       </c>
       <c r="B6" s="22" t="s">
-        <v>819</v>
+        <v>827</v>
       </c>
       <c r="C6" s="27" t="s">
-        <v>820</v>
+        <v>828</v>
       </c>
       <c r="D6" s="28" t="s">
-        <v>821</v>
+        <v>829</v>
       </c>
       <c r="E6" s="29" t="s">
-        <v>822</v>
+        <v>830</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="9" t="s">
-        <v>823</v>
+        <v>831</v>
       </c>
       <c r="B7" s="22" t="s">
-        <v>824</v>
+        <v>832</v>
       </c>
       <c r="C7" s="27" t="s">
-        <v>825</v>
+        <v>833</v>
       </c>
       <c r="D7" s="28" t="s">
-        <v>826</v>
+        <v>834</v>
       </c>
       <c r="E7" s="29" t="s">
-        <v>827</v>
+        <v>835</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="9" t="s">
-        <v>828</v>
+        <v>836</v>
       </c>
       <c r="B8" s="22" t="s">
-        <v>829</v>
+        <v>837</v>
       </c>
       <c r="C8" s="27" t="s">
-        <v>830</v>
+        <v>838</v>
       </c>
       <c r="D8" s="28" t="s">
-        <v>831</v>
+        <v>839</v>
       </c>
       <c r="E8" s="29" t="s">
-        <v>832</v>
+        <v>840</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="9" t="s">
-        <v>833</v>
+        <v>841</v>
       </c>
       <c r="B9" s="22" t="s">
-        <v>834</v>
+        <v>842</v>
       </c>
       <c r="C9" s="27" t="s">
-        <v>835</v>
+        <v>843</v>
       </c>
       <c r="D9" s="28" t="s">
-        <v>836</v>
+        <v>844</v>
       </c>
       <c r="E9" s="29" t="s">
-        <v>837</v>
+        <v>845</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="9" t="s">
-        <v>838</v>
+        <v>846</v>
       </c>
       <c r="B10" s="22" t="s">
-        <v>839</v>
+        <v>847</v>
       </c>
       <c r="C10" s="27" t="s">
-        <v>840</v>
+        <v>848</v>
       </c>
       <c r="D10" s="28" t="s">
-        <v>841</v>
+        <v>849</v>
       </c>
       <c r="E10" s="29" t="s">
-        <v>842</v>
+        <v>850</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="5" t="s">
-        <v>843</v>
+        <v>851</v>
       </c>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -13253,7 +13701,7 @@
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="5" t="s">
-        <v>844</v>
+        <v>852</v>
       </c>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
@@ -13262,36 +13710,36 @@
     </row>
     <row r="22" spans="1:5">
       <c r="A22" s="7" t="s">
-        <v>845</v>
+        <v>853</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>846</v>
+        <v>854</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>847</v>
+        <v>855</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>848</v>
+        <v>856</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>849</v>
+        <v>857</v>
       </c>
     </row>
     <row r="23" spans="1:5">
       <c r="A23" s="14" t="s">
-        <v>850</v>
+        <v>858</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>851</v>
+        <v>859</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>852</v>
+        <v>860</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>853</v>
+        <v>861</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>854</v>
+        <v>862</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -13299,16 +13747,16 @@
         <v>48</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>855</v>
+        <v>863</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>856</v>
+        <v>864</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>857</v>
+        <v>865</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>858</v>
+        <v>866</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -13316,16 +13764,16 @@
         <v>35</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>859</v>
+        <v>867</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>860</v>
+        <v>868</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>861</v>
+        <v>869</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>862</v>
+        <v>870</v>
       </c>
     </row>
     <row r="26" spans="1:5">
@@ -13333,21 +13781,21 @@
         <v>38</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>863</v>
+        <v>871</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>864</v>
+        <v>872</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>865</v>
+        <v>873</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>866</v>
+        <v>874</v>
       </c>
     </row>
     <row r="28" spans="1:5">
       <c r="A28" s="5" t="s">
-        <v>867</v>
+        <v>875</v>
       </c>
       <c r="B28" s="5"/>
       <c r="C28" s="5"/>
@@ -13356,7 +13804,7 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" s="4" t="s">
-        <v>868</v>
+        <v>876</v>
       </c>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -13365,7 +13813,7 @@
     </row>
     <row r="30" spans="1:5">
       <c r="A30" s="4" t="s">
-        <v>869</v>
+        <v>877</v>
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -13374,7 +13822,7 @@
     </row>
     <row r="31" spans="1:5">
       <c r="A31" s="4" t="s">
-        <v>870</v>
+        <v>878</v>
       </c>
       <c r="B31" s="4"/>
       <c r="C31" s="4"/>
@@ -13383,7 +13831,7 @@
     </row>
     <row r="32" spans="1:5">
       <c r="A32" s="4" t="s">
-        <v>871</v>
+        <v>879</v>
       </c>
       <c r="B32" s="4"/>
       <c r="C32" s="4"/>
@@ -13392,7 +13840,7 @@
     </row>
     <row r="33" spans="1:5">
       <c r="A33" s="4" t="s">
-        <v>872</v>
+        <v>880</v>
       </c>
       <c r="B33" s="4"/>
       <c r="C33" s="4"/>
@@ -13416,98 +13864,98 @@
         <v>462</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>873</v>
+        <v>881</v>
       </c>
       <c r="D36" s="7"/>
       <c r="E36" s="7"/>
     </row>
     <row r="37" spans="1:5">
       <c r="A37" s="4" t="s">
-        <v>874</v>
+        <v>882</v>
       </c>
       <c r="B37" s="24" t="s">
-        <v>875</v>
+        <v>883</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>876</v>
+        <v>884</v>
       </c>
       <c r="D37" s="4"/>
       <c r="E37" s="4"/>
     </row>
     <row r="38" spans="1:5">
       <c r="A38" s="4" t="s">
-        <v>877</v>
+        <v>885</v>
       </c>
       <c r="B38" s="24" t="s">
-        <v>878</v>
+        <v>886</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>879</v>
+        <v>887</v>
       </c>
       <c r="D38" s="4"/>
       <c r="E38" s="4"/>
     </row>
     <row r="39" spans="1:5">
       <c r="A39" s="4" t="s">
-        <v>880</v>
+        <v>888</v>
       </c>
       <c r="B39" s="24" t="s">
         <v>470</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>881</v>
+        <v>889</v>
       </c>
       <c r="D39" s="4"/>
       <c r="E39" s="4"/>
     </row>
     <row r="40" spans="1:5">
       <c r="A40" s="4" t="s">
-        <v>882</v>
+        <v>890</v>
       </c>
       <c r="B40" s="24" t="s">
-        <v>883</v>
+        <v>891</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>884</v>
+        <v>892</v>
       </c>
       <c r="D40" s="4"/>
       <c r="E40" s="4"/>
     </row>
     <row r="41" spans="1:5">
       <c r="A41" s="4" t="s">
-        <v>882</v>
+        <v>890</v>
       </c>
       <c r="B41" s="24" t="s">
-        <v>885</v>
+        <v>893</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>886</v>
+        <v>894</v>
       </c>
       <c r="D41" s="4"/>
       <c r="E41" s="4"/>
     </row>
     <row r="42" spans="1:5">
       <c r="A42" s="4" t="s">
-        <v>887</v>
+        <v>895</v>
       </c>
       <c r="B42" s="24" t="s">
-        <v>888</v>
+        <v>896</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>889</v>
+        <v>897</v>
       </c>
       <c r="D42" s="4"/>
       <c r="E42" s="4"/>
     </row>
     <row r="43" spans="1:5">
       <c r="A43" s="4" t="s">
-        <v>890</v>
+        <v>898</v>
       </c>
       <c r="B43" s="24" t="s">
-        <v>891</v>
+        <v>899</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>892</v>
+        <v>900</v>
       </c>
       <c r="D43" s="4"/>
       <c r="E43" s="4"/>

</xml_diff>

<commit_message>
Log B7 W3 T2 (Recovery 3): skill rebound (R 5s back), pulldown 70->75 & hollow 30->35s progressed
</commit_message>
<xml_diff>
--- a/Training_3_B7.xlsx
+++ b/Training_3_B7.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1926" uniqueCount="965">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1974" uniqueCount="977">
   <si>
     <t>B7 — Performance-Block Dashboard (Advanced OAHS)</t>
   </si>
@@ -2370,6 +2370,42 @@
   </si>
   <si>
     <t>Endurance freistehend Parallettes 3x60s - steigt weiter (2x50 -&gt; 3x60)!</t>
+  </si>
+  <si>
+    <t>4-5s+ Holds</t>
+  </si>
+  <si>
+    <t>5s/3s/1-2s variabel - aber 5s zurueck (gestern nur 1s)</t>
+  </si>
+  <si>
+    <t>konstant 3s+</t>
+  </si>
+  <si>
+    <t>~2s</t>
+  </si>
+  <si>
+    <t>schoene 5s+ Holds</t>
+  </si>
+  <si>
+    <t>5s/3s/2s</t>
+  </si>
+  <si>
+    <t>Kabel; 80x8 aber RPE 7 (letzte 80x10@7) -&gt; Schulter-sore/Fatigue, kein Progress heute</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>PROGRESS 70-&gt;75 (letzte 70x10,9,8@7)</t>
+  </si>
+  <si>
+    <t>bewusst gehalten (Schulter-sore)</t>
+  </si>
+  <si>
+    <t>35s</t>
+  </si>
+  <si>
+    <t>Zeit-Progress 30-&gt;35s</t>
   </si>
   <si>
     <t>B7 — Nutrition Targets (Maintenance, KEIN Defizit)</t>
@@ -4180,7 +4216,7 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>901</v>
+        <v>913</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4190,7 +4226,7 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="12" t="s">
-        <v>902</v>
+        <v>914</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -4215,12 +4251,12 @@
         <v>155</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>903</v>
+        <v>915</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="9" t="s">
-        <v>904</v>
+        <v>916</v>
       </c>
       <c r="B4" s="11">
         <f>SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Skill90",'B7_Training_Log'!$C$2:$C$1000,1)+SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Planche",'B7_Training_Log'!$C$2:$C$1000,1)+SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Push",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4245,7 +4281,7 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="9" t="s">
-        <v>905</v>
+        <v>917</v>
       </c>
       <c r="B5" s="11">
         <f>SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Pull",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4270,7 +4306,7 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="9" t="s">
-        <v>906</v>
+        <v>918</v>
       </c>
       <c r="B6" s="11">
         <f>SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Legs",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4295,7 +4331,7 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="9" t="s">
-        <v>907</v>
+        <v>919</v>
       </c>
       <c r="B7" s="10">
         <f>SUMIFS('B7_Training_Log'!$N$2:$N$1000,'B7_Training_Log'!$D$2:$D$1000,"90",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4320,7 +4356,7 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="9" t="s">
-        <v>908</v>
+        <v>920</v>
       </c>
       <c r="B8" s="10">
         <f>COUNTIFS('B7_Training_Log'!$E$2:$E$1000,"SkillOAHS",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4345,7 +4381,7 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="9" t="s">
-        <v>909</v>
+        <v>921</v>
       </c>
       <c r="B9" s="10">
         <f>MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_straddle",'B7_Training_Log'!$F$2:$F$1000,"L",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4370,7 +4406,7 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="9" t="s">
-        <v>910</v>
+        <v>922</v>
       </c>
       <c r="B10" s="10">
         <f>MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_straddle",'B7_Training_Log'!$F$2:$F$1000,"R",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4395,7 +4431,7 @@
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="9" t="s">
-        <v>911</v>
+        <v>923</v>
       </c>
       <c r="B11" s="10">
         <f>MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_diamond",'B7_Training_Log'!$F$2:$F$1000,"L",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4420,7 +4456,7 @@
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="9" t="s">
-        <v>912</v>
+        <v>924</v>
       </c>
       <c r="B12" s="10">
         <f>MAX(MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_flag",'B7_Training_Log'!$C$2:$C$1000,1),MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_figa",'B7_Training_Log'!$C$2:$C$1000,1))</f>
@@ -4445,7 +4481,7 @@
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="9" t="s">
-        <v>913</v>
+        <v>925</v>
       </c>
       <c r="B13" s="11">
         <f>IFERROR(AVERAGEIFS('B7_Training_Log'!$J$2:$J$1000,'B7_Training_Log'!$C$2:$C$1000,1),0)</f>
@@ -4520,7 +4556,7 @@
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="9" t="s">
-        <v>914</v>
+        <v>926</v>
       </c>
       <c r="B16" s="10">
         <f>COUNTIFS('B7_Training_Log'!$K$2:$K$1000,"&gt;=4",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4545,7 +4581,7 @@
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="9" t="s">
-        <v>915</v>
+        <v>927</v>
       </c>
       <c r="B17" s="10">
         <f>COUNTIFS('B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4589,7 +4625,7 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
-        <v>916</v>
+        <v>928</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4597,7 +4633,7 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="5" t="s">
-        <v>917</v>
+        <v>929</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
@@ -4605,13 +4641,13 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="7" t="s">
-        <v>918</v>
+        <v>930</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>919</v>
+        <v>931</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>920</v>
+        <v>932</v>
       </c>
       <c r="D4" s="7"/>
     </row>
@@ -4620,10 +4656,10 @@
         <v>672</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>921</v>
+        <v>933</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>922</v>
+        <v>934</v>
       </c>
       <c r="D5" s="4"/>
     </row>
@@ -4632,10 +4668,10 @@
         <v>673</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>923</v>
+        <v>935</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>924</v>
+        <v>936</v>
       </c>
       <c r="D6" s="4"/>
     </row>
@@ -4644,10 +4680,10 @@
         <v>674</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>925</v>
+        <v>937</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>926</v>
+        <v>938</v>
       </c>
       <c r="D7" s="4"/>
     </row>
@@ -4656,10 +4692,10 @@
         <v>481</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>927</v>
+        <v>939</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>928</v>
+        <v>940</v>
       </c>
       <c r="D8" s="4"/>
     </row>
@@ -4668,10 +4704,10 @@
         <v>484</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>929</v>
+        <v>941</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>930</v>
+        <v>942</v>
       </c>
       <c r="D9" s="4"/>
     </row>
@@ -4680,10 +4716,10 @@
         <v>675</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>931</v>
+        <v>943</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>932</v>
+        <v>944</v>
       </c>
       <c r="D10" s="4"/>
     </row>
@@ -4692,10 +4728,10 @@
         <v>676</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>933</v>
+        <v>945</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>934</v>
+        <v>946</v>
       </c>
       <c r="D11" s="4"/>
     </row>
@@ -4704,10 +4740,10 @@
         <v>677</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>935</v>
+        <v>947</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>936</v>
+        <v>948</v>
       </c>
       <c r="D12" s="4"/>
     </row>
@@ -4716,10 +4752,10 @@
         <v>678</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>933</v>
+        <v>945</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>937</v>
+        <v>949</v>
       </c>
       <c r="D13" s="4"/>
     </row>
@@ -4728,10 +4764,10 @@
         <v>679</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>938</v>
+        <v>950</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>939</v>
+        <v>951</v>
       </c>
       <c r="D14" s="4"/>
     </row>
@@ -4740,10 +4776,10 @@
         <v>680</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>940</v>
+        <v>952</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>941</v>
+        <v>953</v>
       </c>
       <c r="D15" s="4"/>
     </row>
@@ -4752,10 +4788,10 @@
         <v>681</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>942</v>
+        <v>954</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>943</v>
+        <v>955</v>
       </c>
       <c r="D16" s="4"/>
     </row>
@@ -4764,10 +4800,10 @@
         <v>682</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>933</v>
+        <v>945</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>944</v>
+        <v>956</v>
       </c>
       <c r="D17" s="4"/>
     </row>
@@ -4776,10 +4812,10 @@
         <v>683</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>933</v>
+        <v>945</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>945</v>
+        <v>957</v>
       </c>
       <c r="D18" s="4"/>
     </row>
@@ -4788,10 +4824,10 @@
         <v>684</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>946</v>
+        <v>958</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>947</v>
+        <v>959</v>
       </c>
       <c r="D19" s="4"/>
     </row>
@@ -4800,10 +4836,10 @@
         <v>94</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>935</v>
+        <v>947</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>948</v>
+        <v>960</v>
       </c>
       <c r="D20" s="4"/>
     </row>
@@ -4812,16 +4848,16 @@
         <v>685</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>949</v>
+        <v>961</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>950</v>
+        <v>962</v>
       </c>
       <c r="D21" s="4"/>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="5" t="s">
-        <v>951</v>
+        <v>963</v>
       </c>
       <c r="B23" s="5"/>
       <c r="C23" s="5"/>
@@ -4829,7 +4865,7 @@
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="4" t="s">
-        <v>952</v>
+        <v>964</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -4837,7 +4873,7 @@
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="4" t="s">
-        <v>953</v>
+        <v>965</v>
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -4845,7 +4881,7 @@
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="4" t="s">
-        <v>954</v>
+        <v>966</v>
       </c>
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
@@ -4853,7 +4889,7 @@
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="4" t="s">
-        <v>955</v>
+        <v>967</v>
       </c>
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
@@ -4861,7 +4897,7 @@
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="4" t="s">
-        <v>956</v>
+        <v>968</v>
       </c>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
@@ -4869,7 +4905,7 @@
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="4" t="s">
-        <v>957</v>
+        <v>969</v>
       </c>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -4877,7 +4913,7 @@
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="4" t="s">
-        <v>958</v>
+        <v>970</v>
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -4885,7 +4921,7 @@
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="5" t="s">
-        <v>959</v>
+        <v>971</v>
       </c>
       <c r="B32" s="5"/>
       <c r="C32" s="5"/>
@@ -4893,7 +4929,7 @@
     </row>
     <row r="33" spans="1:4">
       <c r="A33" s="4" t="s">
-        <v>960</v>
+        <v>972</v>
       </c>
       <c r="B33" s="4"/>
       <c r="C33" s="4"/>
@@ -4901,7 +4937,7 @@
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="4" t="s">
-        <v>961</v>
+        <v>973</v>
       </c>
       <c r="B34" s="4"/>
       <c r="C34" s="4"/>
@@ -4909,7 +4945,7 @@
     </row>
     <row r="35" spans="1:4">
       <c r="A35" s="4" t="s">
-        <v>962</v>
+        <v>974</v>
       </c>
       <c r="B35" s="4"/>
       <c r="C35" s="4"/>
@@ -4917,7 +4953,7 @@
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="4" t="s">
-        <v>963</v>
+        <v>975</v>
       </c>
       <c r="B36" s="4"/>
       <c r="C36" s="4"/>
@@ -4925,7 +4961,7 @@
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="4" t="s">
-        <v>964</v>
+        <v>976</v>
       </c>
       <c r="B37" s="4"/>
       <c r="C37" s="4"/>
@@ -9153,7 +9189,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q92"/>
+  <dimension ref="A1:Q103"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -13040,6 +13076,476 @@
       </c>
       <c r="Q92" s="6">
         <f>IF($B92="","",$B92&amp;"_W"&amp;$C92)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93" spans="1:17">
+      <c r="A93" s="25">
+        <v>46242</v>
+      </c>
+      <c r="B93" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C93" s="6">
+        <v>3</v>
+      </c>
+      <c r="D93" s="6" t="s">
+        <v>641</v>
+      </c>
+      <c r="E93" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D93,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F93" s="6" t="s">
+        <v>686</v>
+      </c>
+      <c r="G93" s="6">
+        <v>3</v>
+      </c>
+      <c r="I93" s="6">
+        <v>0</v>
+      </c>
+      <c r="L93" s="6">
+        <v>3</v>
+      </c>
+      <c r="M93" s="6">
+        <v>5</v>
+      </c>
+      <c r="O93" s="6">
+        <v>3</v>
+      </c>
+      <c r="P93" s="4" t="s">
+        <v>780</v>
+      </c>
+      <c r="Q93" s="6">
+        <f>IF($B93="","",$B93&amp;"_W"&amp;$C93)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94" spans="1:17">
+      <c r="A94" s="25">
+        <v>46242</v>
+      </c>
+      <c r="B94" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C94" s="6">
+        <v>3</v>
+      </c>
+      <c r="D94" s="6" t="s">
+        <v>641</v>
+      </c>
+      <c r="E94" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D94,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F94" s="6" t="s">
+        <v>688</v>
+      </c>
+      <c r="G94" s="6">
+        <v>3</v>
+      </c>
+      <c r="I94" s="6">
+        <v>0</v>
+      </c>
+      <c r="L94" s="6">
+        <v>2</v>
+      </c>
+      <c r="M94" s="6">
+        <v>5</v>
+      </c>
+      <c r="O94" s="6">
+        <v>3</v>
+      </c>
+      <c r="P94" s="4" t="s">
+        <v>781</v>
+      </c>
+      <c r="Q94" s="6">
+        <f>IF($B94="","",$B94&amp;"_W"&amp;$C94)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="95" spans="1:17">
+      <c r="A95" s="25">
+        <v>46242</v>
+      </c>
+      <c r="B95" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C95" s="6">
+        <v>3</v>
+      </c>
+      <c r="D95" s="6" t="s">
+        <v>647</v>
+      </c>
+      <c r="E95" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D95,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F95" s="6" t="s">
+        <v>686</v>
+      </c>
+      <c r="G95" s="6">
+        <v>3</v>
+      </c>
+      <c r="I95" s="6">
+        <v>0</v>
+      </c>
+      <c r="L95" s="6">
+        <v>3</v>
+      </c>
+      <c r="M95" s="6">
+        <v>4</v>
+      </c>
+      <c r="O95" s="6">
+        <v>3</v>
+      </c>
+      <c r="P95" s="4" t="s">
+        <v>782</v>
+      </c>
+      <c r="Q95" s="6">
+        <f>IF($B95="","",$B95&amp;"_W"&amp;$C95)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="96" spans="1:17">
+      <c r="A96" s="25">
+        <v>46242</v>
+      </c>
+      <c r="B96" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C96" s="6">
+        <v>3</v>
+      </c>
+      <c r="D96" s="6" t="s">
+        <v>647</v>
+      </c>
+      <c r="E96" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D96,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F96" s="6" t="s">
+        <v>688</v>
+      </c>
+      <c r="G96" s="6">
+        <v>3</v>
+      </c>
+      <c r="I96" s="6">
+        <v>0</v>
+      </c>
+      <c r="L96" s="6">
+        <v>2</v>
+      </c>
+      <c r="M96" s="6">
+        <v>2</v>
+      </c>
+      <c r="O96" s="6">
+        <v>3</v>
+      </c>
+      <c r="P96" s="4" t="s">
+        <v>783</v>
+      </c>
+      <c r="Q96" s="6">
+        <f>IF($B96="","",$B96&amp;"_W"&amp;$C96)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="97" spans="1:17">
+      <c r="A97" s="25">
+        <v>46242</v>
+      </c>
+      <c r="B97" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C97" s="6">
+        <v>3</v>
+      </c>
+      <c r="D97" s="6" t="s">
+        <v>644</v>
+      </c>
+      <c r="E97" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D97,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F97" s="6" t="s">
+        <v>686</v>
+      </c>
+      <c r="G97" s="6">
+        <v>3</v>
+      </c>
+      <c r="I97" s="6">
+        <v>0</v>
+      </c>
+      <c r="L97" s="6">
+        <v>3</v>
+      </c>
+      <c r="M97" s="6">
+        <v>5</v>
+      </c>
+      <c r="O97" s="6">
+        <v>3</v>
+      </c>
+      <c r="P97" s="4" t="s">
+        <v>784</v>
+      </c>
+      <c r="Q97" s="6">
+        <f>IF($B97="","",$B97&amp;"_W"&amp;$C97)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="98" spans="1:17">
+      <c r="A98" s="25">
+        <v>46242</v>
+      </c>
+      <c r="B98" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C98" s="6">
+        <v>3</v>
+      </c>
+      <c r="D98" s="6" t="s">
+        <v>644</v>
+      </c>
+      <c r="E98" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D98,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F98" s="6" t="s">
+        <v>688</v>
+      </c>
+      <c r="G98" s="6">
+        <v>3</v>
+      </c>
+      <c r="I98" s="6">
+        <v>0</v>
+      </c>
+      <c r="L98" s="6">
+        <v>2</v>
+      </c>
+      <c r="M98" s="6">
+        <v>5</v>
+      </c>
+      <c r="O98" s="6">
+        <v>3</v>
+      </c>
+      <c r="P98" s="4" t="s">
+        <v>785</v>
+      </c>
+      <c r="Q98" s="6">
+        <f>IF($B98="","",$B98&amp;"_W"&amp;$C98)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="99" spans="1:17">
+      <c r="A99" s="25">
+        <v>46242</v>
+      </c>
+      <c r="B99" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C99" s="6">
+        <v>3</v>
+      </c>
+      <c r="D99" s="6" t="s">
+        <v>539</v>
+      </c>
+      <c r="E99" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D99,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F99" s="6" t="s">
+        <v>693</v>
+      </c>
+      <c r="G99" s="6">
+        <v>3</v>
+      </c>
+      <c r="H99" s="4" t="s">
+        <v>709</v>
+      </c>
+      <c r="I99" s="6">
+        <v>80</v>
+      </c>
+      <c r="J99" s="6">
+        <v>7</v>
+      </c>
+      <c r="O99" s="6">
+        <v>3</v>
+      </c>
+      <c r="P99" s="4" t="s">
+        <v>786</v>
+      </c>
+      <c r="Q99" s="6">
+        <f>IF($B99="","",$B99&amp;"_W"&amp;$C99)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="100" spans="1:17">
+      <c r="A100" s="25">
+        <v>46242</v>
+      </c>
+      <c r="B100" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C100" s="6">
+        <v>3</v>
+      </c>
+      <c r="D100" s="6" t="s">
+        <v>536</v>
+      </c>
+      <c r="E100" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D100,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F100" s="6" t="s">
+        <v>693</v>
+      </c>
+      <c r="G100" s="6">
+        <v>3</v>
+      </c>
+      <c r="H100" s="4" t="s">
+        <v>787</v>
+      </c>
+      <c r="I100" s="6">
+        <v>75</v>
+      </c>
+      <c r="J100" s="6">
+        <v>7</v>
+      </c>
+      <c r="O100" s="6">
+        <v>3</v>
+      </c>
+      <c r="P100" s="4" t="s">
+        <v>788</v>
+      </c>
+      <c r="Q100" s="6">
+        <f>IF($B100="","",$B100&amp;"_W"&amp;$C100)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="101" spans="1:17">
+      <c r="A101" s="25">
+        <v>46242</v>
+      </c>
+      <c r="B101" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C101" s="6">
+        <v>3</v>
+      </c>
+      <c r="D101" s="6" t="s">
+        <v>546</v>
+      </c>
+      <c r="E101" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D101,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F101" s="6" t="s">
+        <v>693</v>
+      </c>
+      <c r="G101" s="6">
+        <v>2</v>
+      </c>
+      <c r="H101" s="4" t="s">
+        <v>698</v>
+      </c>
+      <c r="I101" s="6">
+        <v>30</v>
+      </c>
+      <c r="J101" s="6">
+        <v>6</v>
+      </c>
+      <c r="O101" s="6">
+        <v>3</v>
+      </c>
+      <c r="P101" s="4" t="s">
+        <v>789</v>
+      </c>
+      <c r="Q101" s="6">
+        <f>IF($B101="","",$B101&amp;"_W"&amp;$C101)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="102" spans="1:17">
+      <c r="A102" s="25">
+        <v>46242</v>
+      </c>
+      <c r="B102" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C102" s="6">
+        <v>3</v>
+      </c>
+      <c r="D102" s="6" t="s">
+        <v>550</v>
+      </c>
+      <c r="E102" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D102,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F102" s="6" t="s">
+        <v>693</v>
+      </c>
+      <c r="G102" s="6">
+        <v>2</v>
+      </c>
+      <c r="H102" s="4" t="s">
+        <v>698</v>
+      </c>
+      <c r="I102" s="6">
+        <v>30</v>
+      </c>
+      <c r="J102" s="6">
+        <v>7</v>
+      </c>
+      <c r="O102" s="6">
+        <v>3</v>
+      </c>
+      <c r="Q102" s="6">
+        <f>IF($B102="","",$B102&amp;"_W"&amp;$C102)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="103" spans="1:17">
+      <c r="A103" s="25">
+        <v>46242</v>
+      </c>
+      <c r="B103" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C103" s="6">
+        <v>3</v>
+      </c>
+      <c r="D103" s="6" t="s">
+        <v>622</v>
+      </c>
+      <c r="E103" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D103,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F103" s="6" t="s">
+        <v>693</v>
+      </c>
+      <c r="G103" s="6">
+        <v>3</v>
+      </c>
+      <c r="H103" s="4" t="s">
+        <v>790</v>
+      </c>
+      <c r="J103" s="6">
+        <v>8</v>
+      </c>
+      <c r="M103" s="6">
+        <v>35</v>
+      </c>
+      <c r="O103" s="6">
+        <v>3</v>
+      </c>
+      <c r="P103" s="4" t="s">
+        <v>791</v>
+      </c>
+      <c r="Q103" s="6">
+        <f>IF($B103="","",$B103&amp;"_W"&amp;$C103)</f>
         <v>0</v>
       </c>
     </row>
@@ -13117,7 +13623,7 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>780</v>
+        <v>792</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -13128,20 +13634,20 @@
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="5" t="s">
-        <v>781</v>
+        <v>793</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="9" t="s">
-        <v>782</v>
+        <v>794</v>
       </c>
       <c r="B4" s="11">
         <v>81</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>790</v>
+        <v>802</v>
       </c>
       <c r="D4" s="4"/>
       <c r="E4" s="4"/>
@@ -13150,21 +13656,21 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="9" t="s">
-        <v>783</v>
+        <v>795</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>784</v>
+        <v>796</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="9" t="s">
-        <v>785</v>
+        <v>797</v>
       </c>
       <c r="B6" s="11">
         <v>2.2</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>791</v>
+        <v>803</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
@@ -13173,7 +13679,7 @@
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="9" t="s">
-        <v>786</v>
+        <v>798</v>
       </c>
       <c r="B7" s="11">
         <v>0.9</v>
@@ -13181,7 +13687,7 @@
     </row>
     <row r="8" spans="1:7">
       <c r="A8" s="9" t="s">
-        <v>787</v>
+        <v>799</v>
       </c>
       <c r="B8" s="10">
         <v>2700</v>
@@ -13189,7 +13695,7 @@
     </row>
     <row r="9" spans="1:7">
       <c r="A9" s="9" t="s">
-        <v>788</v>
+        <v>800</v>
       </c>
       <c r="B9" s="10">
         <f>ROUND(BW*B6,0)</f>
@@ -13198,7 +13704,7 @@
     </row>
     <row r="10" spans="1:7">
       <c r="A10" s="9" t="s">
-        <v>789</v>
+        <v>801</v>
       </c>
       <c r="B10" s="10">
         <f>ROUND(BW*B7,0)</f>
@@ -13207,7 +13713,7 @@
     </row>
     <row r="12" spans="1:7">
       <c r="A12" s="5" t="s">
-        <v>792</v>
+        <v>804</v>
       </c>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -13221,27 +13727,27 @@
         <v>87</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>793</v>
+        <v>805</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>794</v>
+        <v>806</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>795</v>
+        <v>807</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>796</v>
+        <v>808</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>797</v>
+        <v>809</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>798</v>
+        <v>810</v>
       </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" s="9" t="s">
-        <v>799</v>
+        <v>811</v>
       </c>
       <c r="B14" s="26">
         <v>250</v>
@@ -13263,7 +13769,7 @@
         <v>0</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>800</v>
+        <v>812</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -13290,12 +13796,12 @@
         <v>0</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>801</v>
+        <v>813</v>
       </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" s="9" t="s">
-        <v>802</v>
+        <v>814</v>
       </c>
       <c r="B16" s="26">
         <v>200</v>
@@ -13317,12 +13823,12 @@
         <v>0</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>803</v>
+        <v>815</v>
       </c>
     </row>
     <row r="17" spans="1:7">
       <c r="A17" s="9" t="s">
-        <v>804</v>
+        <v>816</v>
       </c>
       <c r="B17" s="26">
         <v>150</v>
@@ -13344,12 +13850,12 @@
         <v>0</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>805</v>
+        <v>817</v>
       </c>
     </row>
     <row r="18" spans="1:7">
       <c r="A18" s="9" t="s">
-        <v>806</v>
+        <v>818</v>
       </c>
       <c r="B18" s="26">
         <v>100</v>
@@ -13371,7 +13877,7 @@
         <v>0</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>807</v>
+        <v>819</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -13398,12 +13904,12 @@
         <v>0</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>808</v>
+        <v>820</v>
       </c>
     </row>
     <row r="21" spans="1:7">
       <c r="A21" s="5" t="s">
-        <v>809</v>
+        <v>821</v>
       </c>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
@@ -13414,7 +13920,7 @@
     </row>
     <row r="22" spans="1:7">
       <c r="A22" s="4" t="s">
-        <v>810</v>
+        <v>822</v>
       </c>
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
@@ -13425,7 +13931,7 @@
     </row>
     <row r="23" spans="1:7">
       <c r="A23" s="4" t="s">
-        <v>811</v>
+        <v>823</v>
       </c>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
@@ -13436,7 +13942,7 @@
     </row>
     <row r="24" spans="1:7">
       <c r="A24" s="4" t="s">
-        <v>812</v>
+        <v>824</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -13447,7 +13953,7 @@
     </row>
     <row r="25" spans="1:7">
       <c r="A25" s="4" t="s">
-        <v>813</v>
+        <v>825</v>
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -13492,7 +13998,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>814</v>
+        <v>826</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -13501,7 +14007,7 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="5" t="s">
-        <v>815</v>
+        <v>827</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
@@ -13510,126 +14016,126 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="7" t="s">
-        <v>816</v>
+        <v>828</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>817</v>
+        <v>829</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>818</v>
+        <v>830</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>819</v>
+        <v>831</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>820</v>
+        <v>832</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="9" t="s">
-        <v>821</v>
+        <v>833</v>
       </c>
       <c r="B5" s="22" t="s">
-        <v>822</v>
+        <v>834</v>
       </c>
       <c r="C5" s="27" t="s">
-        <v>823</v>
+        <v>835</v>
       </c>
       <c r="D5" s="28" t="s">
-        <v>824</v>
+        <v>836</v>
       </c>
       <c r="E5" s="29" t="s">
-        <v>825</v>
+        <v>837</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="9" t="s">
-        <v>826</v>
+        <v>838</v>
       </c>
       <c r="B6" s="22" t="s">
-        <v>827</v>
+        <v>839</v>
       </c>
       <c r="C6" s="27" t="s">
-        <v>828</v>
+        <v>840</v>
       </c>
       <c r="D6" s="28" t="s">
-        <v>829</v>
+        <v>841</v>
       </c>
       <c r="E6" s="29" t="s">
-        <v>830</v>
+        <v>842</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="9" t="s">
-        <v>831</v>
+        <v>843</v>
       </c>
       <c r="B7" s="22" t="s">
-        <v>832</v>
+        <v>844</v>
       </c>
       <c r="C7" s="27" t="s">
-        <v>833</v>
+        <v>845</v>
       </c>
       <c r="D7" s="28" t="s">
-        <v>834</v>
+        <v>846</v>
       </c>
       <c r="E7" s="29" t="s">
-        <v>835</v>
+        <v>847</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="9" t="s">
-        <v>836</v>
+        <v>848</v>
       </c>
       <c r="B8" s="22" t="s">
-        <v>837</v>
+        <v>849</v>
       </c>
       <c r="C8" s="27" t="s">
-        <v>838</v>
+        <v>850</v>
       </c>
       <c r="D8" s="28" t="s">
-        <v>839</v>
+        <v>851</v>
       </c>
       <c r="E8" s="29" t="s">
-        <v>840</v>
+        <v>852</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="9" t="s">
-        <v>841</v>
+        <v>853</v>
       </c>
       <c r="B9" s="22" t="s">
-        <v>842</v>
+        <v>854</v>
       </c>
       <c r="C9" s="27" t="s">
-        <v>843</v>
+        <v>855</v>
       </c>
       <c r="D9" s="28" t="s">
-        <v>844</v>
+        <v>856</v>
       </c>
       <c r="E9" s="29" t="s">
-        <v>845</v>
+        <v>857</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="9" t="s">
-        <v>846</v>
+        <v>858</v>
       </c>
       <c r="B10" s="22" t="s">
-        <v>847</v>
+        <v>859</v>
       </c>
       <c r="C10" s="27" t="s">
-        <v>848</v>
+        <v>860</v>
       </c>
       <c r="D10" s="28" t="s">
-        <v>849</v>
+        <v>861</v>
       </c>
       <c r="E10" s="29" t="s">
-        <v>850</v>
+        <v>862</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="5" t="s">
-        <v>851</v>
+        <v>863</v>
       </c>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -13701,7 +14207,7 @@
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="5" t="s">
-        <v>852</v>
+        <v>864</v>
       </c>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
@@ -13710,36 +14216,36 @@
     </row>
     <row r="22" spans="1:5">
       <c r="A22" s="7" t="s">
-        <v>853</v>
+        <v>865</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>854</v>
+        <v>866</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>855</v>
+        <v>867</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>856</v>
+        <v>868</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>857</v>
+        <v>869</v>
       </c>
     </row>
     <row r="23" spans="1:5">
       <c r="A23" s="14" t="s">
-        <v>858</v>
+        <v>870</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>859</v>
+        <v>871</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>860</v>
+        <v>872</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>861</v>
+        <v>873</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>862</v>
+        <v>874</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -13747,16 +14253,16 @@
         <v>48</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>863</v>
+        <v>875</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>864</v>
+        <v>876</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>865</v>
+        <v>877</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>866</v>
+        <v>878</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -13764,16 +14270,16 @@
         <v>35</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>867</v>
+        <v>879</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>868</v>
+        <v>880</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>869</v>
+        <v>881</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>870</v>
+        <v>882</v>
       </c>
     </row>
     <row r="26" spans="1:5">
@@ -13781,21 +14287,21 @@
         <v>38</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>871</v>
+        <v>883</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>872</v>
+        <v>884</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>873</v>
+        <v>885</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>874</v>
+        <v>886</v>
       </c>
     </row>
     <row r="28" spans="1:5">
       <c r="A28" s="5" t="s">
-        <v>875</v>
+        <v>887</v>
       </c>
       <c r="B28" s="5"/>
       <c r="C28" s="5"/>
@@ -13804,7 +14310,7 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" s="4" t="s">
-        <v>876</v>
+        <v>888</v>
       </c>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -13813,7 +14319,7 @@
     </row>
     <row r="30" spans="1:5">
       <c r="A30" s="4" t="s">
-        <v>877</v>
+        <v>889</v>
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -13822,7 +14328,7 @@
     </row>
     <row r="31" spans="1:5">
       <c r="A31" s="4" t="s">
-        <v>878</v>
+        <v>890</v>
       </c>
       <c r="B31" s="4"/>
       <c r="C31" s="4"/>
@@ -13831,7 +14337,7 @@
     </row>
     <row r="32" spans="1:5">
       <c r="A32" s="4" t="s">
-        <v>879</v>
+        <v>891</v>
       </c>
       <c r="B32" s="4"/>
       <c r="C32" s="4"/>
@@ -13840,7 +14346,7 @@
     </row>
     <row r="33" spans="1:5">
       <c r="A33" s="4" t="s">
-        <v>880</v>
+        <v>892</v>
       </c>
       <c r="B33" s="4"/>
       <c r="C33" s="4"/>
@@ -13864,98 +14370,98 @@
         <v>462</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>881</v>
+        <v>893</v>
       </c>
       <c r="D36" s="7"/>
       <c r="E36" s="7"/>
     </row>
     <row r="37" spans="1:5">
       <c r="A37" s="4" t="s">
-        <v>882</v>
+        <v>894</v>
       </c>
       <c r="B37" s="24" t="s">
-        <v>883</v>
+        <v>895</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>884</v>
+        <v>896</v>
       </c>
       <c r="D37" s="4"/>
       <c r="E37" s="4"/>
     </row>
     <row r="38" spans="1:5">
       <c r="A38" s="4" t="s">
-        <v>885</v>
+        <v>897</v>
       </c>
       <c r="B38" s="24" t="s">
-        <v>886</v>
+        <v>898</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>887</v>
+        <v>899</v>
       </c>
       <c r="D38" s="4"/>
       <c r="E38" s="4"/>
     </row>
     <row r="39" spans="1:5">
       <c r="A39" s="4" t="s">
-        <v>888</v>
+        <v>900</v>
       </c>
       <c r="B39" s="24" t="s">
         <v>470</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>889</v>
+        <v>901</v>
       </c>
       <c r="D39" s="4"/>
       <c r="E39" s="4"/>
     </row>
     <row r="40" spans="1:5">
       <c r="A40" s="4" t="s">
-        <v>890</v>
+        <v>902</v>
       </c>
       <c r="B40" s="24" t="s">
-        <v>891</v>
+        <v>903</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>892</v>
+        <v>904</v>
       </c>
       <c r="D40" s="4"/>
       <c r="E40" s="4"/>
     </row>
     <row r="41" spans="1:5">
       <c r="A41" s="4" t="s">
-        <v>890</v>
+        <v>902</v>
       </c>
       <c r="B41" s="24" t="s">
-        <v>893</v>
+        <v>905</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>894</v>
+        <v>906</v>
       </c>
       <c r="D41" s="4"/>
       <c r="E41" s="4"/>
     </row>
     <row r="42" spans="1:5">
       <c r="A42" s="4" t="s">
-        <v>895</v>
+        <v>907</v>
       </c>
       <c r="B42" s="24" t="s">
-        <v>896</v>
+        <v>908</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>897</v>
+        <v>909</v>
       </c>
       <c r="D42" s="4"/>
       <c r="E42" s="4"/>
     </row>
     <row r="43" spans="1:5">
       <c r="A43" s="4" t="s">
-        <v>898</v>
+        <v>910</v>
       </c>
       <c r="B43" s="24" t="s">
-        <v>899</v>
+        <v>911</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>900</v>
+        <v>912</v>
       </c>
       <c r="D43" s="4"/>
       <c r="E43" s="4"/>

</xml_diff>

<commit_message>
Log B7 W3 T3 (Recovery 4): leg progressions (BSS 42.5, ham 45x12, calves 90); LOW-BACK flag on leg press
</commit_message>
<xml_diff>
--- a/Training_3_B7.xlsx
+++ b/Training_3_B7.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1974" uniqueCount="977">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2011" uniqueCount="986">
   <si>
     <t>B7 — Performance-Block Dashboard (Advanced OAHS)</t>
   </si>
@@ -2406,6 +2406,33 @@
   </si>
   <si>
     <t>Zeit-Progress 30-&gt;35s</t>
+  </si>
+  <si>
+    <t>Mikrodosis Legs-together, ging recht gut</t>
+  </si>
+  <si>
+    <t>PROGRESS 40-&gt;42,5 @RPE7</t>
+  </si>
+  <si>
+    <t>RUECKEN: ab Satz 2-3 unterer Ruecken (nie zuvor bei Beinpresse); naechster Morgen Druck oberhalb Huefte, flexions-empfindlich, KEIN Ruck/kein scharfer Schmerz, ging schnell weg. Wahrsch. Bottom-Range Lumbalflexion unter Last</t>
+  </si>
+  <si>
+    <t>PROGRESS Reps 10-&gt;12 @45</t>
+  </si>
+  <si>
+    <t>80-&gt;90 (nur der Sprung verfuegbar), gut machbar</t>
+  </si>
+  <si>
+    <t>Endurance 3x60s (im Zirkel)</t>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
+    <t>liegende Bauchuebung 3x9 (im Zirkel); Pallof weggelassen</t>
+  </si>
+  <si>
+    <t>3x40s/Seite (im Zirkel) - Progress</t>
   </si>
   <si>
     <t>B7 — Nutrition Targets (Maintenance, KEIN Defizit)</t>
@@ -4216,7 +4243,7 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>913</v>
+        <v>922</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4226,7 +4253,7 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="12" t="s">
-        <v>914</v>
+        <v>923</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -4251,12 +4278,12 @@
         <v>155</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>915</v>
+        <v>924</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="9" t="s">
-        <v>916</v>
+        <v>925</v>
       </c>
       <c r="B4" s="11">
         <f>SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Skill90",'B7_Training_Log'!$C$2:$C$1000,1)+SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Planche",'B7_Training_Log'!$C$2:$C$1000,1)+SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Push",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4281,7 +4308,7 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="9" t="s">
-        <v>917</v>
+        <v>926</v>
       </c>
       <c r="B5" s="11">
         <f>SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Pull",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4306,7 +4333,7 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="9" t="s">
-        <v>918</v>
+        <v>927</v>
       </c>
       <c r="B6" s="11">
         <f>SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Legs",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4331,7 +4358,7 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="9" t="s">
-        <v>919</v>
+        <v>928</v>
       </c>
       <c r="B7" s="10">
         <f>SUMIFS('B7_Training_Log'!$N$2:$N$1000,'B7_Training_Log'!$D$2:$D$1000,"90",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4356,7 +4383,7 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="9" t="s">
-        <v>920</v>
+        <v>929</v>
       </c>
       <c r="B8" s="10">
         <f>COUNTIFS('B7_Training_Log'!$E$2:$E$1000,"SkillOAHS",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4381,7 +4408,7 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="9" t="s">
-        <v>921</v>
+        <v>930</v>
       </c>
       <c r="B9" s="10">
         <f>MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_straddle",'B7_Training_Log'!$F$2:$F$1000,"L",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4406,7 +4433,7 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="9" t="s">
-        <v>922</v>
+        <v>931</v>
       </c>
       <c r="B10" s="10">
         <f>MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_straddle",'B7_Training_Log'!$F$2:$F$1000,"R",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4431,7 +4458,7 @@
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="9" t="s">
-        <v>923</v>
+        <v>932</v>
       </c>
       <c r="B11" s="10">
         <f>MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_diamond",'B7_Training_Log'!$F$2:$F$1000,"L",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4456,7 +4483,7 @@
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="9" t="s">
-        <v>924</v>
+        <v>933</v>
       </c>
       <c r="B12" s="10">
         <f>MAX(MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_flag",'B7_Training_Log'!$C$2:$C$1000,1),MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_figa",'B7_Training_Log'!$C$2:$C$1000,1))</f>
@@ -4481,7 +4508,7 @@
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="9" t="s">
-        <v>925</v>
+        <v>934</v>
       </c>
       <c r="B13" s="11">
         <f>IFERROR(AVERAGEIFS('B7_Training_Log'!$J$2:$J$1000,'B7_Training_Log'!$C$2:$C$1000,1),0)</f>
@@ -4556,7 +4583,7 @@
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="9" t="s">
-        <v>926</v>
+        <v>935</v>
       </c>
       <c r="B16" s="10">
         <f>COUNTIFS('B7_Training_Log'!$K$2:$K$1000,"&gt;=4",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4581,7 +4608,7 @@
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="9" t="s">
-        <v>927</v>
+        <v>936</v>
       </c>
       <c r="B17" s="10">
         <f>COUNTIFS('B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4625,7 +4652,7 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
-        <v>928</v>
+        <v>937</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4633,7 +4660,7 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="5" t="s">
-        <v>929</v>
+        <v>938</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
@@ -4641,13 +4668,13 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="7" t="s">
-        <v>930</v>
+        <v>939</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>931</v>
+        <v>940</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>932</v>
+        <v>941</v>
       </c>
       <c r="D4" s="7"/>
     </row>
@@ -4656,10 +4683,10 @@
         <v>672</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>933</v>
+        <v>942</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>934</v>
+        <v>943</v>
       </c>
       <c r="D5" s="4"/>
     </row>
@@ -4668,10 +4695,10 @@
         <v>673</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>935</v>
+        <v>944</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>936</v>
+        <v>945</v>
       </c>
       <c r="D6" s="4"/>
     </row>
@@ -4680,10 +4707,10 @@
         <v>674</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>937</v>
+        <v>946</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>938</v>
+        <v>947</v>
       </c>
       <c r="D7" s="4"/>
     </row>
@@ -4692,10 +4719,10 @@
         <v>481</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>939</v>
+        <v>948</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>940</v>
+        <v>949</v>
       </c>
       <c r="D8" s="4"/>
     </row>
@@ -4704,10 +4731,10 @@
         <v>484</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>941</v>
+        <v>950</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>942</v>
+        <v>951</v>
       </c>
       <c r="D9" s="4"/>
     </row>
@@ -4716,10 +4743,10 @@
         <v>675</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>943</v>
+        <v>952</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>944</v>
+        <v>953</v>
       </c>
       <c r="D10" s="4"/>
     </row>
@@ -4728,10 +4755,10 @@
         <v>676</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>945</v>
+        <v>954</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>946</v>
+        <v>955</v>
       </c>
       <c r="D11" s="4"/>
     </row>
@@ -4740,10 +4767,10 @@
         <v>677</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>947</v>
+        <v>956</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>948</v>
+        <v>957</v>
       </c>
       <c r="D12" s="4"/>
     </row>
@@ -4752,10 +4779,10 @@
         <v>678</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>945</v>
+        <v>954</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>949</v>
+        <v>958</v>
       </c>
       <c r="D13" s="4"/>
     </row>
@@ -4764,10 +4791,10 @@
         <v>679</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>950</v>
+        <v>959</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>951</v>
+        <v>960</v>
       </c>
       <c r="D14" s="4"/>
     </row>
@@ -4776,10 +4803,10 @@
         <v>680</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>952</v>
+        <v>961</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>953</v>
+        <v>962</v>
       </c>
       <c r="D15" s="4"/>
     </row>
@@ -4788,10 +4815,10 @@
         <v>681</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>954</v>
+        <v>963</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>955</v>
+        <v>964</v>
       </c>
       <c r="D16" s="4"/>
     </row>
@@ -4800,10 +4827,10 @@
         <v>682</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>945</v>
+        <v>954</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>956</v>
+        <v>965</v>
       </c>
       <c r="D17" s="4"/>
     </row>
@@ -4812,10 +4839,10 @@
         <v>683</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>945</v>
+        <v>954</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>957</v>
+        <v>966</v>
       </c>
       <c r="D18" s="4"/>
     </row>
@@ -4824,10 +4851,10 @@
         <v>684</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>958</v>
+        <v>967</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>959</v>
+        <v>968</v>
       </c>
       <c r="D19" s="4"/>
     </row>
@@ -4836,10 +4863,10 @@
         <v>94</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>947</v>
+        <v>956</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>960</v>
+        <v>969</v>
       </c>
       <c r="D20" s="4"/>
     </row>
@@ -4848,16 +4875,16 @@
         <v>685</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>961</v>
+        <v>970</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>962</v>
+        <v>971</v>
       </c>
       <c r="D21" s="4"/>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="5" t="s">
-        <v>963</v>
+        <v>972</v>
       </c>
       <c r="B23" s="5"/>
       <c r="C23" s="5"/>
@@ -4865,7 +4892,7 @@
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="4" t="s">
-        <v>964</v>
+        <v>973</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -4873,7 +4900,7 @@
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="4" t="s">
-        <v>965</v>
+        <v>974</v>
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -4881,7 +4908,7 @@
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="4" t="s">
-        <v>966</v>
+        <v>975</v>
       </c>
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
@@ -4889,7 +4916,7 @@
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="4" t="s">
-        <v>967</v>
+        <v>976</v>
       </c>
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
@@ -4897,7 +4924,7 @@
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="4" t="s">
-        <v>968</v>
+        <v>977</v>
       </c>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
@@ -4905,7 +4932,7 @@
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="4" t="s">
-        <v>969</v>
+        <v>978</v>
       </c>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -4913,7 +4940,7 @@
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="4" t="s">
-        <v>970</v>
+        <v>979</v>
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -4921,7 +4948,7 @@
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="5" t="s">
-        <v>971</v>
+        <v>980</v>
       </c>
       <c r="B32" s="5"/>
       <c r="C32" s="5"/>
@@ -4929,7 +4956,7 @@
     </row>
     <row r="33" spans="1:4">
       <c r="A33" s="4" t="s">
-        <v>972</v>
+        <v>981</v>
       </c>
       <c r="B33" s="4"/>
       <c r="C33" s="4"/>
@@ -4937,7 +4964,7 @@
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="4" t="s">
-        <v>973</v>
+        <v>982</v>
       </c>
       <c r="B34" s="4"/>
       <c r="C34" s="4"/>
@@ -4945,7 +4972,7 @@
     </row>
     <row r="35" spans="1:4">
       <c r="A35" s="4" t="s">
-        <v>974</v>
+        <v>983</v>
       </c>
       <c r="B35" s="4"/>
       <c r="C35" s="4"/>
@@ -4953,7 +4980,7 @@
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="4" t="s">
-        <v>975</v>
+        <v>984</v>
       </c>
       <c r="B36" s="4"/>
       <c r="C36" s="4"/>
@@ -4961,7 +4988,7 @@
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="4" t="s">
-        <v>976</v>
+        <v>985</v>
       </c>
       <c r="B37" s="4"/>
       <c r="C37" s="4"/>
@@ -9189,7 +9216,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q103"/>
+  <dimension ref="A1:Q111"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -13546,6 +13573,338 @@
       </c>
       <c r="Q103" s="6">
         <f>IF($B103="","",$B103&amp;"_W"&amp;$C103)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="104" spans="1:17">
+      <c r="A104" s="25">
+        <v>46244</v>
+      </c>
+      <c r="B104" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="C104" s="6">
+        <v>3</v>
+      </c>
+      <c r="D104" s="6" t="s">
+        <v>653</v>
+      </c>
+      <c r="E104" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D104,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F104" s="6" t="s">
+        <v>693</v>
+      </c>
+      <c r="G104" s="6">
+        <v>2</v>
+      </c>
+      <c r="I104" s="6">
+        <v>0</v>
+      </c>
+      <c r="L104" s="6">
+        <v>3</v>
+      </c>
+      <c r="O104" s="6">
+        <v>4</v>
+      </c>
+      <c r="P104" s="4" t="s">
+        <v>792</v>
+      </c>
+      <c r="Q104" s="6">
+        <f>IF($B104="","",$B104&amp;"_W"&amp;$C104)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="105" spans="1:17">
+      <c r="A105" s="25">
+        <v>46244</v>
+      </c>
+      <c r="B105" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="C105" s="6">
+        <v>3</v>
+      </c>
+      <c r="D105" s="6" t="s">
+        <v>589</v>
+      </c>
+      <c r="E105" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D105,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F105" s="6" t="s">
+        <v>693</v>
+      </c>
+      <c r="G105" s="6">
+        <v>3</v>
+      </c>
+      <c r="H105" s="4" t="s">
+        <v>709</v>
+      </c>
+      <c r="I105" s="6">
+        <v>42.5</v>
+      </c>
+      <c r="J105" s="6">
+        <v>7</v>
+      </c>
+      <c r="O105" s="6">
+        <v>4</v>
+      </c>
+      <c r="P105" s="4" t="s">
+        <v>793</v>
+      </c>
+      <c r="Q105" s="6">
+        <f>IF($B105="","",$B105&amp;"_W"&amp;$C105)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="106" spans="1:17">
+      <c r="A106" s="25">
+        <v>46244</v>
+      </c>
+      <c r="B106" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="C106" s="6">
+        <v>3</v>
+      </c>
+      <c r="D106" s="6" t="s">
+        <v>592</v>
+      </c>
+      <c r="E106" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D106,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F106" s="6" t="s">
+        <v>693</v>
+      </c>
+      <c r="G106" s="6">
+        <v>3</v>
+      </c>
+      <c r="H106" s="4" t="s">
+        <v>698</v>
+      </c>
+      <c r="I106" s="6">
+        <v>80</v>
+      </c>
+      <c r="J106" s="6">
+        <v>8</v>
+      </c>
+      <c r="K106" s="6">
+        <v>3</v>
+      </c>
+      <c r="O106" s="6">
+        <v>4</v>
+      </c>
+      <c r="P106" s="4" t="s">
+        <v>794</v>
+      </c>
+      <c r="Q106" s="6">
+        <f>IF($B106="","",$B106&amp;"_W"&amp;$C106)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="107" spans="1:17">
+      <c r="A107" s="25">
+        <v>46244</v>
+      </c>
+      <c r="B107" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="C107" s="6">
+        <v>3</v>
+      </c>
+      <c r="D107" s="6" t="s">
+        <v>595</v>
+      </c>
+      <c r="E107" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D107,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F107" s="6" t="s">
+        <v>693</v>
+      </c>
+      <c r="G107" s="6">
+        <v>3</v>
+      </c>
+      <c r="H107" s="4" t="s">
+        <v>698</v>
+      </c>
+      <c r="I107" s="6">
+        <v>45</v>
+      </c>
+      <c r="J107" s="6">
+        <v>7</v>
+      </c>
+      <c r="O107" s="6">
+        <v>4</v>
+      </c>
+      <c r="P107" s="4" t="s">
+        <v>795</v>
+      </c>
+      <c r="Q107" s="6">
+        <f>IF($B107="","",$B107&amp;"_W"&amp;$C107)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="108" spans="1:17">
+      <c r="A108" s="25">
+        <v>46244</v>
+      </c>
+      <c r="B108" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="C108" s="6">
+        <v>3</v>
+      </c>
+      <c r="D108" s="6" t="s">
+        <v>605</v>
+      </c>
+      <c r="E108" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D108,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F108" s="6" t="s">
+        <v>693</v>
+      </c>
+      <c r="G108" s="6">
+        <v>3</v>
+      </c>
+      <c r="H108" s="4" t="s">
+        <v>698</v>
+      </c>
+      <c r="I108" s="6">
+        <v>90</v>
+      </c>
+      <c r="J108" s="6">
+        <v>7</v>
+      </c>
+      <c r="O108" s="6">
+        <v>4</v>
+      </c>
+      <c r="P108" s="4" t="s">
+        <v>796</v>
+      </c>
+      <c r="Q108" s="6">
+        <f>IF($B108="","",$B108&amp;"_W"&amp;$C108)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="109" spans="1:17">
+      <c r="A109" s="25">
+        <v>46244</v>
+      </c>
+      <c r="B109" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="C109" s="6">
+        <v>3</v>
+      </c>
+      <c r="D109" s="6" t="s">
+        <v>504</v>
+      </c>
+      <c r="E109" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D109,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F109" s="6" t="s">
+        <v>693</v>
+      </c>
+      <c r="G109" s="6">
+        <v>3</v>
+      </c>
+      <c r="I109" s="6">
+        <v>0</v>
+      </c>
+      <c r="L109" s="6">
+        <v>4</v>
+      </c>
+      <c r="M109" s="6">
+        <v>60</v>
+      </c>
+      <c r="O109" s="6">
+        <v>4</v>
+      </c>
+      <c r="P109" s="4" t="s">
+        <v>797</v>
+      </c>
+      <c r="Q109" s="6">
+        <f>IF($B109="","",$B109&amp;"_W"&amp;$C109)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="110" spans="1:17">
+      <c r="A110" s="25">
+        <v>46244</v>
+      </c>
+      <c r="B110" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="C110" s="6">
+        <v>3</v>
+      </c>
+      <c r="D110" s="6" t="s">
+        <v>614</v>
+      </c>
+      <c r="E110" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D110,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F110" s="6" t="s">
+        <v>693</v>
+      </c>
+      <c r="G110" s="6">
+        <v>3</v>
+      </c>
+      <c r="H110" s="4" t="s">
+        <v>798</v>
+      </c>
+      <c r="O110" s="6">
+        <v>4</v>
+      </c>
+      <c r="P110" s="4" t="s">
+        <v>799</v>
+      </c>
+      <c r="Q110" s="6">
+        <f>IF($B110="","",$B110&amp;"_W"&amp;$C110)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="111" spans="1:17">
+      <c r="A111" s="25">
+        <v>46244</v>
+      </c>
+      <c r="B111" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="C111" s="6">
+        <v>3</v>
+      </c>
+      <c r="D111" s="6" t="s">
+        <v>618</v>
+      </c>
+      <c r="E111" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D111,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F111" s="6" t="s">
+        <v>693</v>
+      </c>
+      <c r="G111" s="6">
+        <v>3</v>
+      </c>
+      <c r="M111" s="6">
+        <v>40</v>
+      </c>
+      <c r="O111" s="6">
+        <v>4</v>
+      </c>
+      <c r="P111" s="4" t="s">
+        <v>800</v>
+      </c>
+      <c r="Q111" s="6">
+        <f>IF($B111="","",$B111&amp;"_W"&amp;$C111)</f>
         <v>0</v>
       </c>
     </row>
@@ -13623,7 +13982,7 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>792</v>
+        <v>801</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -13634,20 +13993,20 @@
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="5" t="s">
-        <v>793</v>
+        <v>802</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="9" t="s">
-        <v>794</v>
+        <v>803</v>
       </c>
       <c r="B4" s="11">
         <v>81</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>802</v>
+        <v>811</v>
       </c>
       <c r="D4" s="4"/>
       <c r="E4" s="4"/>
@@ -13656,21 +14015,21 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="9" t="s">
-        <v>795</v>
+        <v>804</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>796</v>
+        <v>805</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="9" t="s">
-        <v>797</v>
+        <v>806</v>
       </c>
       <c r="B6" s="11">
         <v>2.2</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>803</v>
+        <v>812</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
@@ -13679,7 +14038,7 @@
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="9" t="s">
-        <v>798</v>
+        <v>807</v>
       </c>
       <c r="B7" s="11">
         <v>0.9</v>
@@ -13687,7 +14046,7 @@
     </row>
     <row r="8" spans="1:7">
       <c r="A8" s="9" t="s">
-        <v>799</v>
+        <v>808</v>
       </c>
       <c r="B8" s="10">
         <v>2700</v>
@@ -13695,7 +14054,7 @@
     </row>
     <row r="9" spans="1:7">
       <c r="A9" s="9" t="s">
-        <v>800</v>
+        <v>809</v>
       </c>
       <c r="B9" s="10">
         <f>ROUND(BW*B6,0)</f>
@@ -13704,7 +14063,7 @@
     </row>
     <row r="10" spans="1:7">
       <c r="A10" s="9" t="s">
-        <v>801</v>
+        <v>810</v>
       </c>
       <c r="B10" s="10">
         <f>ROUND(BW*B7,0)</f>
@@ -13713,7 +14072,7 @@
     </row>
     <row r="12" spans="1:7">
       <c r="A12" s="5" t="s">
-        <v>804</v>
+        <v>813</v>
       </c>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -13727,27 +14086,27 @@
         <v>87</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>805</v>
+        <v>814</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>806</v>
+        <v>815</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>807</v>
+        <v>816</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>808</v>
+        <v>817</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>809</v>
+        <v>818</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>810</v>
+        <v>819</v>
       </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" s="9" t="s">
-        <v>811</v>
+        <v>820</v>
       </c>
       <c r="B14" s="26">
         <v>250</v>
@@ -13769,7 +14128,7 @@
         <v>0</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>812</v>
+        <v>821</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -13796,12 +14155,12 @@
         <v>0</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>813</v>
+        <v>822</v>
       </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" s="9" t="s">
-        <v>814</v>
+        <v>823</v>
       </c>
       <c r="B16" s="26">
         <v>200</v>
@@ -13823,12 +14182,12 @@
         <v>0</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>815</v>
+        <v>824</v>
       </c>
     </row>
     <row r="17" spans="1:7">
       <c r="A17" s="9" t="s">
-        <v>816</v>
+        <v>825</v>
       </c>
       <c r="B17" s="26">
         <v>150</v>
@@ -13850,12 +14209,12 @@
         <v>0</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>817</v>
+        <v>826</v>
       </c>
     </row>
     <row r="18" spans="1:7">
       <c r="A18" s="9" t="s">
-        <v>818</v>
+        <v>827</v>
       </c>
       <c r="B18" s="26">
         <v>100</v>
@@ -13877,7 +14236,7 @@
         <v>0</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>819</v>
+        <v>828</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -13904,12 +14263,12 @@
         <v>0</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>820</v>
+        <v>829</v>
       </c>
     </row>
     <row r="21" spans="1:7">
       <c r="A21" s="5" t="s">
-        <v>821</v>
+        <v>830</v>
       </c>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
@@ -13920,7 +14279,7 @@
     </row>
     <row r="22" spans="1:7">
       <c r="A22" s="4" t="s">
-        <v>822</v>
+        <v>831</v>
       </c>
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
@@ -13931,7 +14290,7 @@
     </row>
     <row r="23" spans="1:7">
       <c r="A23" s="4" t="s">
-        <v>823</v>
+        <v>832</v>
       </c>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
@@ -13942,7 +14301,7 @@
     </row>
     <row r="24" spans="1:7">
       <c r="A24" s="4" t="s">
-        <v>824</v>
+        <v>833</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -13953,7 +14312,7 @@
     </row>
     <row r="25" spans="1:7">
       <c r="A25" s="4" t="s">
-        <v>825</v>
+        <v>834</v>
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -13998,7 +14357,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>826</v>
+        <v>835</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -14007,7 +14366,7 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="5" t="s">
-        <v>827</v>
+        <v>836</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
@@ -14016,126 +14375,126 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="7" t="s">
-        <v>828</v>
+        <v>837</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>829</v>
+        <v>838</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>830</v>
+        <v>839</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>831</v>
+        <v>840</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>832</v>
+        <v>841</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="9" t="s">
-        <v>833</v>
+        <v>842</v>
       </c>
       <c r="B5" s="22" t="s">
-        <v>834</v>
+        <v>843</v>
       </c>
       <c r="C5" s="27" t="s">
-        <v>835</v>
+        <v>844</v>
       </c>
       <c r="D5" s="28" t="s">
-        <v>836</v>
+        <v>845</v>
       </c>
       <c r="E5" s="29" t="s">
-        <v>837</v>
+        <v>846</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="9" t="s">
-        <v>838</v>
+        <v>847</v>
       </c>
       <c r="B6" s="22" t="s">
-        <v>839</v>
+        <v>848</v>
       </c>
       <c r="C6" s="27" t="s">
-        <v>840</v>
+        <v>849</v>
       </c>
       <c r="D6" s="28" t="s">
-        <v>841</v>
+        <v>850</v>
       </c>
       <c r="E6" s="29" t="s">
-        <v>842</v>
+        <v>851</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="9" t="s">
-        <v>843</v>
+        <v>852</v>
       </c>
       <c r="B7" s="22" t="s">
-        <v>844</v>
+        <v>853</v>
       </c>
       <c r="C7" s="27" t="s">
-        <v>845</v>
+        <v>854</v>
       </c>
       <c r="D7" s="28" t="s">
-        <v>846</v>
+        <v>855</v>
       </c>
       <c r="E7" s="29" t="s">
-        <v>847</v>
+        <v>856</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="9" t="s">
-        <v>848</v>
+        <v>857</v>
       </c>
       <c r="B8" s="22" t="s">
-        <v>849</v>
+        <v>858</v>
       </c>
       <c r="C8" s="27" t="s">
-        <v>850</v>
+        <v>859</v>
       </c>
       <c r="D8" s="28" t="s">
-        <v>851</v>
+        <v>860</v>
       </c>
       <c r="E8" s="29" t="s">
-        <v>852</v>
+        <v>861</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="9" t="s">
-        <v>853</v>
+        <v>862</v>
       </c>
       <c r="B9" s="22" t="s">
-        <v>854</v>
+        <v>863</v>
       </c>
       <c r="C9" s="27" t="s">
-        <v>855</v>
+        <v>864</v>
       </c>
       <c r="D9" s="28" t="s">
-        <v>856</v>
+        <v>865</v>
       </c>
       <c r="E9" s="29" t="s">
-        <v>857</v>
+        <v>866</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="9" t="s">
-        <v>858</v>
+        <v>867</v>
       </c>
       <c r="B10" s="22" t="s">
-        <v>859</v>
+        <v>868</v>
       </c>
       <c r="C10" s="27" t="s">
-        <v>860</v>
+        <v>869</v>
       </c>
       <c r="D10" s="28" t="s">
-        <v>861</v>
+        <v>870</v>
       </c>
       <c r="E10" s="29" t="s">
-        <v>862</v>
+        <v>871</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="5" t="s">
-        <v>863</v>
+        <v>872</v>
       </c>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -14207,7 +14566,7 @@
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="5" t="s">
-        <v>864</v>
+        <v>873</v>
       </c>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
@@ -14216,36 +14575,36 @@
     </row>
     <row r="22" spans="1:5">
       <c r="A22" s="7" t="s">
-        <v>865</v>
+        <v>874</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>866</v>
+        <v>875</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>867</v>
+        <v>876</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>868</v>
+        <v>877</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>869</v>
+        <v>878</v>
       </c>
     </row>
     <row r="23" spans="1:5">
       <c r="A23" s="14" t="s">
-        <v>870</v>
+        <v>879</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>871</v>
+        <v>880</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>872</v>
+        <v>881</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>873</v>
+        <v>882</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>874</v>
+        <v>883</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -14253,16 +14612,16 @@
         <v>48</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>875</v>
+        <v>884</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>876</v>
+        <v>885</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>877</v>
+        <v>886</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>878</v>
+        <v>887</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -14270,16 +14629,16 @@
         <v>35</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>879</v>
+        <v>888</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>880</v>
+        <v>889</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>881</v>
+        <v>890</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>882</v>
+        <v>891</v>
       </c>
     </row>
     <row r="26" spans="1:5">
@@ -14287,21 +14646,21 @@
         <v>38</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>883</v>
+        <v>892</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>884</v>
+        <v>893</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>885</v>
+        <v>894</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>886</v>
+        <v>895</v>
       </c>
     </row>
     <row r="28" spans="1:5">
       <c r="A28" s="5" t="s">
-        <v>887</v>
+        <v>896</v>
       </c>
       <c r="B28" s="5"/>
       <c r="C28" s="5"/>
@@ -14310,7 +14669,7 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" s="4" t="s">
-        <v>888</v>
+        <v>897</v>
       </c>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -14319,7 +14678,7 @@
     </row>
     <row r="30" spans="1:5">
       <c r="A30" s="4" t="s">
-        <v>889</v>
+        <v>898</v>
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -14328,7 +14687,7 @@
     </row>
     <row r="31" spans="1:5">
       <c r="A31" s="4" t="s">
-        <v>890</v>
+        <v>899</v>
       </c>
       <c r="B31" s="4"/>
       <c r="C31" s="4"/>
@@ -14337,7 +14696,7 @@
     </row>
     <row r="32" spans="1:5">
       <c r="A32" s="4" t="s">
-        <v>891</v>
+        <v>900</v>
       </c>
       <c r="B32" s="4"/>
       <c r="C32" s="4"/>
@@ -14346,7 +14705,7 @@
     </row>
     <row r="33" spans="1:5">
       <c r="A33" s="4" t="s">
-        <v>892</v>
+        <v>901</v>
       </c>
       <c r="B33" s="4"/>
       <c r="C33" s="4"/>
@@ -14370,98 +14729,98 @@
         <v>462</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>893</v>
+        <v>902</v>
       </c>
       <c r="D36" s="7"/>
       <c r="E36" s="7"/>
     </row>
     <row r="37" spans="1:5">
       <c r="A37" s="4" t="s">
-        <v>894</v>
+        <v>903</v>
       </c>
       <c r="B37" s="24" t="s">
-        <v>895</v>
+        <v>904</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>896</v>
+        <v>905</v>
       </c>
       <c r="D37" s="4"/>
       <c r="E37" s="4"/>
     </row>
     <row r="38" spans="1:5">
       <c r="A38" s="4" t="s">
-        <v>897</v>
+        <v>906</v>
       </c>
       <c r="B38" s="24" t="s">
-        <v>898</v>
+        <v>907</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>899</v>
+        <v>908</v>
       </c>
       <c r="D38" s="4"/>
       <c r="E38" s="4"/>
     </row>
     <row r="39" spans="1:5">
       <c r="A39" s="4" t="s">
-        <v>900</v>
+        <v>909</v>
       </c>
       <c r="B39" s="24" t="s">
         <v>470</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>901</v>
+        <v>910</v>
       </c>
       <c r="D39" s="4"/>
       <c r="E39" s="4"/>
     </row>
     <row r="40" spans="1:5">
       <c r="A40" s="4" t="s">
-        <v>902</v>
+        <v>911</v>
       </c>
       <c r="B40" s="24" t="s">
-        <v>903</v>
+        <v>912</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>904</v>
+        <v>913</v>
       </c>
       <c r="D40" s="4"/>
       <c r="E40" s="4"/>
     </row>
     <row r="41" spans="1:5">
       <c r="A41" s="4" t="s">
-        <v>902</v>
+        <v>911</v>
       </c>
       <c r="B41" s="24" t="s">
-        <v>905</v>
+        <v>914</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>906</v>
+        <v>915</v>
       </c>
       <c r="D41" s="4"/>
       <c r="E41" s="4"/>
     </row>
     <row r="42" spans="1:5">
       <c r="A42" s="4" t="s">
-        <v>907</v>
+        <v>916</v>
       </c>
       <c r="B42" s="24" t="s">
-        <v>908</v>
+        <v>917</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>909</v>
+        <v>918</v>
       </c>
       <c r="D42" s="4"/>
       <c r="E42" s="4"/>
     </row>
     <row r="43" spans="1:5">
       <c r="A43" s="4" t="s">
-        <v>910</v>
+        <v>919</v>
       </c>
       <c r="B43" s="24" t="s">
-        <v>911</v>
+        <v>920</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>912</v>
+        <v>921</v>
       </c>
       <c r="D43" s="4"/>
       <c r="E43" s="4"/>

</xml_diff>

<commit_message>
Log B7 W3 T4 (back-safe): flag clean, R up to 2-3s, no back pain; 90 neg quality restored
</commit_message>
<xml_diff>
--- a/Training_3_B7.xlsx
+++ b/Training_3_B7.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2011" uniqueCount="986">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2041" uniqueCount="993">
   <si>
     <t>B7 — Performance-Block Dashboard (Advanced OAHS)</t>
   </si>
@@ -2433,6 +2433,27 @@
   </si>
   <si>
     <t>3x40s/Seite (im Zirkel) - Progress</t>
+  </si>
+  <si>
+    <t>Flag-Lean+Return, bis 3s Freeze, teils gehalten; KEIN Rueckenziehen</t>
+  </si>
+  <si>
+    <t>Lean+Return: Balance im Center verloren, aber 2-3s gehalten (Trash-Tag war 1s)</t>
+  </si>
+  <si>
+    <t>Straddle Flag Hold 3-4s alle Saetze</t>
+  </si>
+  <si>
+    <t>Straddle Flag Hold ~3s</t>
+  </si>
+  <si>
+    <t>gute Spannung, ribs down; Koerper schwer, NS aber gut</t>
+  </si>
+  <si>
+    <t>Deep/High Push-ups (statt Pike)</t>
+  </si>
+  <si>
+    <t>Ring Rows horizontal, rueckenschonend (statt Kabelzug); Zahlen ca.</t>
   </si>
   <si>
     <t>B7 — Nutrition Targets (Maintenance, KEIN Defizit)</t>
@@ -4243,7 +4264,7 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>922</v>
+        <v>929</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4253,7 +4274,7 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="12" t="s">
-        <v>923</v>
+        <v>930</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -4278,12 +4299,12 @@
         <v>155</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>924</v>
+        <v>931</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="9" t="s">
-        <v>925</v>
+        <v>932</v>
       </c>
       <c r="B4" s="11">
         <f>SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Skill90",'B7_Training_Log'!$C$2:$C$1000,1)+SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Planche",'B7_Training_Log'!$C$2:$C$1000,1)+SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Push",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4308,7 +4329,7 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="9" t="s">
-        <v>926</v>
+        <v>933</v>
       </c>
       <c r="B5" s="11">
         <f>SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Pull",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4333,7 +4354,7 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="9" t="s">
-        <v>927</v>
+        <v>934</v>
       </c>
       <c r="B6" s="11">
         <f>SUMIFS('B7_Training_Log'!$G$2:$G$1000,'B7_Training_Log'!$E$2:$E$1000,"Legs",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4358,7 +4379,7 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="9" t="s">
-        <v>928</v>
+        <v>935</v>
       </c>
       <c r="B7" s="10">
         <f>SUMIFS('B7_Training_Log'!$N$2:$N$1000,'B7_Training_Log'!$D$2:$D$1000,"90",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4383,7 +4404,7 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="9" t="s">
-        <v>929</v>
+        <v>936</v>
       </c>
       <c r="B8" s="10">
         <f>COUNTIFS('B7_Training_Log'!$E$2:$E$1000,"SkillOAHS",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4408,7 +4429,7 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="9" t="s">
-        <v>930</v>
+        <v>937</v>
       </c>
       <c r="B9" s="10">
         <f>MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_straddle",'B7_Training_Log'!$F$2:$F$1000,"L",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4433,7 +4454,7 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="9" t="s">
-        <v>931</v>
+        <v>938</v>
       </c>
       <c r="B10" s="10">
         <f>MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_straddle",'B7_Training_Log'!$F$2:$F$1000,"R",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4458,7 +4479,7 @@
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="9" t="s">
-        <v>932</v>
+        <v>939</v>
       </c>
       <c r="B11" s="10">
         <f>MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_diamond",'B7_Training_Log'!$F$2:$F$1000,"L",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4483,7 +4504,7 @@
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="9" t="s">
-        <v>933</v>
+        <v>940</v>
       </c>
       <c r="B12" s="10">
         <f>MAX(MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_flag",'B7_Training_Log'!$C$2:$C$1000,1),MAXIFS('B7_Training_Log'!$M$2:$M$1000,'B7_Training_Log'!$D$2:$D$1000,"oahs_figa",'B7_Training_Log'!$C$2:$C$1000,1))</f>
@@ -4508,7 +4529,7 @@
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="9" t="s">
-        <v>934</v>
+        <v>941</v>
       </c>
       <c r="B13" s="11">
         <f>IFERROR(AVERAGEIFS('B7_Training_Log'!$J$2:$J$1000,'B7_Training_Log'!$C$2:$C$1000,1),0)</f>
@@ -4583,7 +4604,7 @@
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="9" t="s">
-        <v>935</v>
+        <v>942</v>
       </c>
       <c r="B16" s="10">
         <f>COUNTIFS('B7_Training_Log'!$K$2:$K$1000,"&gt;=4",'B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4608,7 +4629,7 @@
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="9" t="s">
-        <v>936</v>
+        <v>943</v>
       </c>
       <c r="B17" s="10">
         <f>COUNTIFS('B7_Training_Log'!$C$2:$C$1000,1)</f>
@@ -4652,7 +4673,7 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
-        <v>937</v>
+        <v>944</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4660,7 +4681,7 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="5" t="s">
-        <v>938</v>
+        <v>945</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
@@ -4668,13 +4689,13 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="7" t="s">
-        <v>939</v>
+        <v>946</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>940</v>
+        <v>947</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>941</v>
+        <v>948</v>
       </c>
       <c r="D4" s="7"/>
     </row>
@@ -4683,10 +4704,10 @@
         <v>672</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>942</v>
+        <v>949</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>943</v>
+        <v>950</v>
       </c>
       <c r="D5" s="4"/>
     </row>
@@ -4695,10 +4716,10 @@
         <v>673</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>944</v>
+        <v>951</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>945</v>
+        <v>952</v>
       </c>
       <c r="D6" s="4"/>
     </row>
@@ -4707,10 +4728,10 @@
         <v>674</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>946</v>
+        <v>953</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>947</v>
+        <v>954</v>
       </c>
       <c r="D7" s="4"/>
     </row>
@@ -4719,10 +4740,10 @@
         <v>481</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>948</v>
+        <v>955</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>949</v>
+        <v>956</v>
       </c>
       <c r="D8" s="4"/>
     </row>
@@ -4731,10 +4752,10 @@
         <v>484</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>950</v>
+        <v>957</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>951</v>
+        <v>958</v>
       </c>
       <c r="D9" s="4"/>
     </row>
@@ -4743,10 +4764,10 @@
         <v>675</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>952</v>
+        <v>959</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>953</v>
+        <v>960</v>
       </c>
       <c r="D10" s="4"/>
     </row>
@@ -4755,10 +4776,10 @@
         <v>676</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>954</v>
+        <v>961</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>955</v>
+        <v>962</v>
       </c>
       <c r="D11" s="4"/>
     </row>
@@ -4767,10 +4788,10 @@
         <v>677</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>956</v>
+        <v>963</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>957</v>
+        <v>964</v>
       </c>
       <c r="D12" s="4"/>
     </row>
@@ -4779,10 +4800,10 @@
         <v>678</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>954</v>
+        <v>961</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>958</v>
+        <v>965</v>
       </c>
       <c r="D13" s="4"/>
     </row>
@@ -4791,10 +4812,10 @@
         <v>679</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>959</v>
+        <v>966</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>960</v>
+        <v>967</v>
       </c>
       <c r="D14" s="4"/>
     </row>
@@ -4803,10 +4824,10 @@
         <v>680</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>961</v>
+        <v>968</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>962</v>
+        <v>969</v>
       </c>
       <c r="D15" s="4"/>
     </row>
@@ -4815,10 +4836,10 @@
         <v>681</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>963</v>
+        <v>970</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>964</v>
+        <v>971</v>
       </c>
       <c r="D16" s="4"/>
     </row>
@@ -4827,10 +4848,10 @@
         <v>682</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>954</v>
+        <v>961</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>965</v>
+        <v>972</v>
       </c>
       <c r="D17" s="4"/>
     </row>
@@ -4839,10 +4860,10 @@
         <v>683</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>954</v>
+        <v>961</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>966</v>
+        <v>973</v>
       </c>
       <c r="D18" s="4"/>
     </row>
@@ -4851,10 +4872,10 @@
         <v>684</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>967</v>
+        <v>974</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>968</v>
+        <v>975</v>
       </c>
       <c r="D19" s="4"/>
     </row>
@@ -4863,10 +4884,10 @@
         <v>94</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>956</v>
+        <v>963</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>969</v>
+        <v>976</v>
       </c>
       <c r="D20" s="4"/>
     </row>
@@ -4875,16 +4896,16 @@
         <v>685</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>970</v>
+        <v>977</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>971</v>
+        <v>978</v>
       </c>
       <c r="D21" s="4"/>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="5" t="s">
-        <v>972</v>
+        <v>979</v>
       </c>
       <c r="B23" s="5"/>
       <c r="C23" s="5"/>
@@ -4892,7 +4913,7 @@
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="4" t="s">
-        <v>973</v>
+        <v>980</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -4900,7 +4921,7 @@
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="4" t="s">
-        <v>974</v>
+        <v>981</v>
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -4908,7 +4929,7 @@
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="4" t="s">
-        <v>975</v>
+        <v>982</v>
       </c>
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
@@ -4916,7 +4937,7 @@
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="4" t="s">
-        <v>976</v>
+        <v>983</v>
       </c>
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
@@ -4924,7 +4945,7 @@
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="4" t="s">
-        <v>977</v>
+        <v>984</v>
       </c>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
@@ -4932,7 +4953,7 @@
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="4" t="s">
-        <v>978</v>
+        <v>985</v>
       </c>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -4940,7 +4961,7 @@
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="4" t="s">
-        <v>979</v>
+        <v>986</v>
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -4948,7 +4969,7 @@
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="5" t="s">
-        <v>980</v>
+        <v>987</v>
       </c>
       <c r="B32" s="5"/>
       <c r="C32" s="5"/>
@@ -4956,7 +4977,7 @@
     </row>
     <row r="33" spans="1:4">
       <c r="A33" s="4" t="s">
-        <v>981</v>
+        <v>988</v>
       </c>
       <c r="B33" s="4"/>
       <c r="C33" s="4"/>
@@ -4964,7 +4985,7 @@
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="4" t="s">
-        <v>982</v>
+        <v>989</v>
       </c>
       <c r="B34" s="4"/>
       <c r="C34" s="4"/>
@@ -4972,7 +4993,7 @@
     </row>
     <row r="35" spans="1:4">
       <c r="A35" s="4" t="s">
-        <v>983</v>
+        <v>990</v>
       </c>
       <c r="B35" s="4"/>
       <c r="C35" s="4"/>
@@ -4980,7 +5001,7 @@
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="4" t="s">
-        <v>984</v>
+        <v>991</v>
       </c>
       <c r="B36" s="4"/>
       <c r="C36" s="4"/>
@@ -4988,7 +5009,7 @@
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="4" t="s">
-        <v>985</v>
+        <v>992</v>
       </c>
       <c r="B37" s="4"/>
       <c r="C37" s="4"/>
@@ -9216,7 +9237,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q111"/>
+  <dimension ref="A1:Q118"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -13905,6 +13926,301 @@
       </c>
       <c r="Q111" s="6">
         <f>IF($B111="","",$B111&amp;"_W"&amp;$C111)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="112" spans="1:17">
+      <c r="A112" s="25">
+        <v>46247</v>
+      </c>
+      <c r="B112" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="C112" s="6">
+        <v>3</v>
+      </c>
+      <c r="D112" s="6" t="s">
+        <v>668</v>
+      </c>
+      <c r="E112" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D112,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F112" s="6" t="s">
+        <v>686</v>
+      </c>
+      <c r="G112" s="6">
+        <v>3</v>
+      </c>
+      <c r="I112" s="6">
+        <v>0</v>
+      </c>
+      <c r="L112" s="6">
+        <v>3</v>
+      </c>
+      <c r="M112" s="6">
+        <v>3</v>
+      </c>
+      <c r="O112" s="6">
+        <v>4</v>
+      </c>
+      <c r="P112" s="4" t="s">
+        <v>801</v>
+      </c>
+      <c r="Q112" s="6">
+        <f>IF($B112="","",$B112&amp;"_W"&amp;$C112)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="113" spans="1:17">
+      <c r="A113" s="25">
+        <v>46247</v>
+      </c>
+      <c r="B113" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="C113" s="6">
+        <v>3</v>
+      </c>
+      <c r="D113" s="6" t="s">
+        <v>668</v>
+      </c>
+      <c r="E113" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D113,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F113" s="6" t="s">
+        <v>688</v>
+      </c>
+      <c r="G113" s="6">
+        <v>3</v>
+      </c>
+      <c r="I113" s="6">
+        <v>0</v>
+      </c>
+      <c r="L113" s="6">
+        <v>2</v>
+      </c>
+      <c r="M113" s="6">
+        <v>3</v>
+      </c>
+      <c r="O113" s="6">
+        <v>4</v>
+      </c>
+      <c r="P113" s="4" t="s">
+        <v>802</v>
+      </c>
+      <c r="Q113" s="6">
+        <f>IF($B113="","",$B113&amp;"_W"&amp;$C113)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="114" spans="1:17">
+      <c r="A114" s="25">
+        <v>46247</v>
+      </c>
+      <c r="B114" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="C114" s="6">
+        <v>3</v>
+      </c>
+      <c r="D114" s="6" t="s">
+        <v>668</v>
+      </c>
+      <c r="E114" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D114,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F114" s="6" t="s">
+        <v>686</v>
+      </c>
+      <c r="G114" s="6">
+        <v>3</v>
+      </c>
+      <c r="I114" s="6">
+        <v>0</v>
+      </c>
+      <c r="L114" s="6">
+        <v>3</v>
+      </c>
+      <c r="M114" s="6">
+        <v>4</v>
+      </c>
+      <c r="O114" s="6">
+        <v>4</v>
+      </c>
+      <c r="P114" s="4" t="s">
+        <v>803</v>
+      </c>
+      <c r="Q114" s="6">
+        <f>IF($B114="","",$B114&amp;"_W"&amp;$C114)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="115" spans="1:17">
+      <c r="A115" s="25">
+        <v>46247</v>
+      </c>
+      <c r="B115" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="C115" s="6">
+        <v>3</v>
+      </c>
+      <c r="D115" s="6" t="s">
+        <v>668</v>
+      </c>
+      <c r="E115" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D115,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F115" s="6" t="s">
+        <v>688</v>
+      </c>
+      <c r="G115" s="6">
+        <v>3</v>
+      </c>
+      <c r="I115" s="6">
+        <v>0</v>
+      </c>
+      <c r="L115" s="6">
+        <v>3</v>
+      </c>
+      <c r="M115" s="6">
+        <v>3</v>
+      </c>
+      <c r="O115" s="6">
+        <v>4</v>
+      </c>
+      <c r="P115" s="4" t="s">
+        <v>804</v>
+      </c>
+      <c r="Q115" s="6">
+        <f>IF($B115="","",$B115&amp;"_W"&amp;$C115)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="116" spans="1:17">
+      <c r="A116" s="25">
+        <v>46247</v>
+      </c>
+      <c r="B116" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="C116" s="6">
+        <v>3</v>
+      </c>
+      <c r="D116" s="6" t="s">
+        <v>489</v>
+      </c>
+      <c r="E116" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D116,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F116" s="6" t="s">
+        <v>693</v>
+      </c>
+      <c r="G116" s="6">
+        <v>3</v>
+      </c>
+      <c r="H116" s="4" t="s">
+        <v>694</v>
+      </c>
+      <c r="I116" s="6">
+        <v>0</v>
+      </c>
+      <c r="J116" s="6">
+        <v>7</v>
+      </c>
+      <c r="O116" s="6">
+        <v>4</v>
+      </c>
+      <c r="P116" s="4" t="s">
+        <v>805</v>
+      </c>
+      <c r="Q116" s="6">
+        <f>IF($B116="","",$B116&amp;"_W"&amp;$C116)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="117" spans="1:17">
+      <c r="A117" s="25">
+        <v>46247</v>
+      </c>
+      <c r="B117" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="C117" s="6">
+        <v>3</v>
+      </c>
+      <c r="D117" s="6" t="s">
+        <v>574</v>
+      </c>
+      <c r="E117" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D117,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F117" s="6" t="s">
+        <v>693</v>
+      </c>
+      <c r="G117" s="6">
+        <v>3</v>
+      </c>
+      <c r="H117" s="4" t="s">
+        <v>787</v>
+      </c>
+      <c r="I117" s="6">
+        <v>0</v>
+      </c>
+      <c r="J117" s="6">
+        <v>7</v>
+      </c>
+      <c r="O117" s="6">
+        <v>4</v>
+      </c>
+      <c r="P117" s="4" t="s">
+        <v>806</v>
+      </c>
+      <c r="Q117" s="6">
+        <f>IF($B117="","",$B117&amp;"_W"&amp;$C117)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="118" spans="1:17">
+      <c r="A118" s="25">
+        <v>46247</v>
+      </c>
+      <c r="B118" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="C118" s="6">
+        <v>3</v>
+      </c>
+      <c r="D118" s="6" t="s">
+        <v>539</v>
+      </c>
+      <c r="E118" s="6">
+        <f>IFERROR(INDEX('B7_Exercise_Library'!$D$4:$D$54,MATCH($D118,'B7_Exercise_Library'!$A$4:$A$54,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F118" s="6" t="s">
+        <v>693</v>
+      </c>
+      <c r="G118" s="6">
+        <v>3</v>
+      </c>
+      <c r="I118" s="6">
+        <v>0</v>
+      </c>
+      <c r="O118" s="6">
+        <v>4</v>
+      </c>
+      <c r="P118" s="4" t="s">
+        <v>807</v>
+      </c>
+      <c r="Q118" s="6">
+        <f>IF($B118="","",$B118&amp;"_W"&amp;$C118)</f>
         <v>0</v>
       </c>
     </row>
@@ -13982,7 +14298,7 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>801</v>
+        <v>808</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -13993,20 +14309,20 @@
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="5" t="s">
-        <v>802</v>
+        <v>809</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="9" t="s">
-        <v>803</v>
+        <v>810</v>
       </c>
       <c r="B4" s="11">
         <v>81</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>811</v>
+        <v>818</v>
       </c>
       <c r="D4" s="4"/>
       <c r="E4" s="4"/>
@@ -14015,21 +14331,21 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="9" t="s">
-        <v>804</v>
+        <v>811</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>805</v>
+        <v>812</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="9" t="s">
-        <v>806</v>
+        <v>813</v>
       </c>
       <c r="B6" s="11">
         <v>2.2</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>812</v>
+        <v>819</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
@@ -14038,7 +14354,7 @@
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="9" t="s">
-        <v>807</v>
+        <v>814</v>
       </c>
       <c r="B7" s="11">
         <v>0.9</v>
@@ -14046,7 +14362,7 @@
     </row>
     <row r="8" spans="1:7">
       <c r="A8" s="9" t="s">
-        <v>808</v>
+        <v>815</v>
       </c>
       <c r="B8" s="10">
         <v>2700</v>
@@ -14054,7 +14370,7 @@
     </row>
     <row r="9" spans="1:7">
       <c r="A9" s="9" t="s">
-        <v>809</v>
+        <v>816</v>
       </c>
       <c r="B9" s="10">
         <f>ROUND(BW*B6,0)</f>
@@ -14063,7 +14379,7 @@
     </row>
     <row r="10" spans="1:7">
       <c r="A10" s="9" t="s">
-        <v>810</v>
+        <v>817</v>
       </c>
       <c r="B10" s="10">
         <f>ROUND(BW*B7,0)</f>
@@ -14072,7 +14388,7 @@
     </row>
     <row r="12" spans="1:7">
       <c r="A12" s="5" t="s">
-        <v>813</v>
+        <v>820</v>
       </c>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -14086,27 +14402,27 @@
         <v>87</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>814</v>
+        <v>821</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>815</v>
+        <v>822</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>816</v>
+        <v>823</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>817</v>
+        <v>824</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>818</v>
+        <v>825</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>819</v>
+        <v>826</v>
       </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" s="9" t="s">
-        <v>820</v>
+        <v>827</v>
       </c>
       <c r="B14" s="26">
         <v>250</v>
@@ -14128,7 +14444,7 @@
         <v>0</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>821</v>
+        <v>828</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -14155,12 +14471,12 @@
         <v>0</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>822</v>
+        <v>829</v>
       </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" s="9" t="s">
-        <v>823</v>
+        <v>830</v>
       </c>
       <c r="B16" s="26">
         <v>200</v>
@@ -14182,12 +14498,12 @@
         <v>0</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>824</v>
+        <v>831</v>
       </c>
     </row>
     <row r="17" spans="1:7">
       <c r="A17" s="9" t="s">
-        <v>825</v>
+        <v>832</v>
       </c>
       <c r="B17" s="26">
         <v>150</v>
@@ -14209,12 +14525,12 @@
         <v>0</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>826</v>
+        <v>833</v>
       </c>
     </row>
     <row r="18" spans="1:7">
       <c r="A18" s="9" t="s">
-        <v>827</v>
+        <v>834</v>
       </c>
       <c r="B18" s="26">
         <v>100</v>
@@ -14236,7 +14552,7 @@
         <v>0</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>828</v>
+        <v>835</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -14263,12 +14579,12 @@
         <v>0</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>829</v>
+        <v>836</v>
       </c>
     </row>
     <row r="21" spans="1:7">
       <c r="A21" s="5" t="s">
-        <v>830</v>
+        <v>837</v>
       </c>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
@@ -14279,7 +14595,7 @@
     </row>
     <row r="22" spans="1:7">
       <c r="A22" s="4" t="s">
-        <v>831</v>
+        <v>838</v>
       </c>
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
@@ -14290,7 +14606,7 @@
     </row>
     <row r="23" spans="1:7">
       <c r="A23" s="4" t="s">
-        <v>832</v>
+        <v>839</v>
       </c>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
@@ -14301,7 +14617,7 @@
     </row>
     <row r="24" spans="1:7">
       <c r="A24" s="4" t="s">
-        <v>833</v>
+        <v>840</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -14312,7 +14628,7 @@
     </row>
     <row r="25" spans="1:7">
       <c r="A25" s="4" t="s">
-        <v>834</v>
+        <v>841</v>
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -14357,7 +14673,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>835</v>
+        <v>842</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -14366,7 +14682,7 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="5" t="s">
-        <v>836</v>
+        <v>843</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
@@ -14375,126 +14691,126 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="7" t="s">
-        <v>837</v>
+        <v>844</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>838</v>
+        <v>845</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>839</v>
+        <v>846</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>840</v>
+        <v>847</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>841</v>
+        <v>848</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="9" t="s">
-        <v>842</v>
+        <v>849</v>
       </c>
       <c r="B5" s="22" t="s">
-        <v>843</v>
+        <v>850</v>
       </c>
       <c r="C5" s="27" t="s">
-        <v>844</v>
+        <v>851</v>
       </c>
       <c r="D5" s="28" t="s">
-        <v>845</v>
+        <v>852</v>
       </c>
       <c r="E5" s="29" t="s">
-        <v>846</v>
+        <v>853</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="9" t="s">
-        <v>847</v>
+        <v>854</v>
       </c>
       <c r="B6" s="22" t="s">
-        <v>848</v>
+        <v>855</v>
       </c>
       <c r="C6" s="27" t="s">
-        <v>849</v>
+        <v>856</v>
       </c>
       <c r="D6" s="28" t="s">
-        <v>850</v>
+        <v>857</v>
       </c>
       <c r="E6" s="29" t="s">
-        <v>851</v>
+        <v>858</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="9" t="s">
-        <v>852</v>
+        <v>859</v>
       </c>
       <c r="B7" s="22" t="s">
-        <v>853</v>
+        <v>860</v>
       </c>
       <c r="C7" s="27" t="s">
-        <v>854</v>
+        <v>861</v>
       </c>
       <c r="D7" s="28" t="s">
-        <v>855</v>
+        <v>862</v>
       </c>
       <c r="E7" s="29" t="s">
-        <v>856</v>
+        <v>863</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="9" t="s">
-        <v>857</v>
+        <v>864</v>
       </c>
       <c r="B8" s="22" t="s">
-        <v>858</v>
+        <v>865</v>
       </c>
       <c r="C8" s="27" t="s">
-        <v>859</v>
+        <v>866</v>
       </c>
       <c r="D8" s="28" t="s">
-        <v>860</v>
+        <v>867</v>
       </c>
       <c r="E8" s="29" t="s">
-        <v>861</v>
+        <v>868</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="9" t="s">
-        <v>862</v>
+        <v>869</v>
       </c>
       <c r="B9" s="22" t="s">
-        <v>863</v>
+        <v>870</v>
       </c>
       <c r="C9" s="27" t="s">
-        <v>864</v>
+        <v>871</v>
       </c>
       <c r="D9" s="28" t="s">
-        <v>865</v>
+        <v>872</v>
       </c>
       <c r="E9" s="29" t="s">
-        <v>866</v>
+        <v>873</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="9" t="s">
-        <v>867</v>
+        <v>874</v>
       </c>
       <c r="B10" s="22" t="s">
-        <v>868</v>
+        <v>875</v>
       </c>
       <c r="C10" s="27" t="s">
-        <v>869</v>
+        <v>876</v>
       </c>
       <c r="D10" s="28" t="s">
-        <v>870</v>
+        <v>877</v>
       </c>
       <c r="E10" s="29" t="s">
-        <v>871</v>
+        <v>878</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="5" t="s">
-        <v>872</v>
+        <v>879</v>
       </c>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -14566,7 +14882,7 @@
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="5" t="s">
-        <v>873</v>
+        <v>880</v>
       </c>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
@@ -14575,36 +14891,36 @@
     </row>
     <row r="22" spans="1:5">
       <c r="A22" s="7" t="s">
-        <v>874</v>
+        <v>881</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>875</v>
+        <v>882</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>876</v>
+        <v>883</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>877</v>
+        <v>884</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>878</v>
+        <v>885</v>
       </c>
     </row>
     <row r="23" spans="1:5">
       <c r="A23" s="14" t="s">
-        <v>879</v>
+        <v>886</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>880</v>
+        <v>887</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>881</v>
+        <v>888</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>882</v>
+        <v>889</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>883</v>
+        <v>890</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -14612,16 +14928,16 @@
         <v>48</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>884</v>
+        <v>891</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>885</v>
+        <v>892</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>886</v>
+        <v>893</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>887</v>
+        <v>894</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -14629,16 +14945,16 @@
         <v>35</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>888</v>
+        <v>895</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>889</v>
+        <v>896</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>890</v>
+        <v>897</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>891</v>
+        <v>898</v>
       </c>
     </row>
     <row r="26" spans="1:5">
@@ -14646,21 +14962,21 @@
         <v>38</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>892</v>
+        <v>899</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>893</v>
+        <v>900</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>894</v>
+        <v>901</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>895</v>
+        <v>902</v>
       </c>
     </row>
     <row r="28" spans="1:5">
       <c r="A28" s="5" t="s">
-        <v>896</v>
+        <v>903</v>
       </c>
       <c r="B28" s="5"/>
       <c r="C28" s="5"/>
@@ -14669,7 +14985,7 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" s="4" t="s">
-        <v>897</v>
+        <v>904</v>
       </c>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -14678,7 +14994,7 @@
     </row>
     <row r="30" spans="1:5">
       <c r="A30" s="4" t="s">
-        <v>898</v>
+        <v>905</v>
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -14687,7 +15003,7 @@
     </row>
     <row r="31" spans="1:5">
       <c r="A31" s="4" t="s">
-        <v>899</v>
+        <v>906</v>
       </c>
       <c r="B31" s="4"/>
       <c r="C31" s="4"/>
@@ -14696,7 +15012,7 @@
     </row>
     <row r="32" spans="1:5">
       <c r="A32" s="4" t="s">
-        <v>900</v>
+        <v>907</v>
       </c>
       <c r="B32" s="4"/>
       <c r="C32" s="4"/>
@@ -14705,7 +15021,7 @@
     </row>
     <row r="33" spans="1:5">
       <c r="A33" s="4" t="s">
-        <v>901</v>
+        <v>908</v>
       </c>
       <c r="B33" s="4"/>
       <c r="C33" s="4"/>
@@ -14729,98 +15045,98 @@
         <v>462</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>902</v>
+        <v>909</v>
       </c>
       <c r="D36" s="7"/>
       <c r="E36" s="7"/>
     </row>
     <row r="37" spans="1:5">
       <c r="A37" s="4" t="s">
-        <v>903</v>
+        <v>910</v>
       </c>
       <c r="B37" s="24" t="s">
-        <v>904</v>
+        <v>911</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>905</v>
+        <v>912</v>
       </c>
       <c r="D37" s="4"/>
       <c r="E37" s="4"/>
     </row>
     <row r="38" spans="1:5">
       <c r="A38" s="4" t="s">
-        <v>906</v>
+        <v>913</v>
       </c>
       <c r="B38" s="24" t="s">
-        <v>907</v>
+        <v>914</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>908</v>
+        <v>915</v>
       </c>
       <c r="D38" s="4"/>
       <c r="E38" s="4"/>
     </row>
     <row r="39" spans="1:5">
       <c r="A39" s="4" t="s">
-        <v>909</v>
+        <v>916</v>
       </c>
       <c r="B39" s="24" t="s">
         <v>470</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>910</v>
+        <v>917</v>
       </c>
       <c r="D39" s="4"/>
       <c r="E39" s="4"/>
     </row>
     <row r="40" spans="1:5">
       <c r="A40" s="4" t="s">
-        <v>911</v>
+        <v>918</v>
       </c>
       <c r="B40" s="24" t="s">
-        <v>912</v>
+        <v>919</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>913</v>
+        <v>920</v>
       </c>
       <c r="D40" s="4"/>
       <c r="E40" s="4"/>
     </row>
     <row r="41" spans="1:5">
       <c r="A41" s="4" t="s">
-        <v>911</v>
+        <v>918</v>
       </c>
       <c r="B41" s="24" t="s">
-        <v>914</v>
+        <v>921</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>915</v>
+        <v>922</v>
       </c>
       <c r="D41" s="4"/>
       <c r="E41" s="4"/>
     </row>
     <row r="42" spans="1:5">
       <c r="A42" s="4" t="s">
-        <v>916</v>
+        <v>923</v>
       </c>
       <c r="B42" s="24" t="s">
-        <v>917</v>
+        <v>924</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>918</v>
+        <v>925</v>
       </c>
       <c r="D42" s="4"/>
       <c r="E42" s="4"/>
     </row>
     <row r="43" spans="1:5">
       <c r="A43" s="4" t="s">
-        <v>919</v>
+        <v>926</v>
       </c>
       <c r="B43" s="24" t="s">
-        <v>920</v>
+        <v>927</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>921</v>
+        <v>928</v>
       </c>
       <c r="D43" s="4"/>
       <c r="E43" s="4"/>

</xml_diff>